<commit_message>
File Updated on 06/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A9D8CC-B08F-44D6-A9BA-350EACD9031F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58B8A00F-948A-4FF5-B86B-9B8724486156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1873,27 +1873,51 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="15" t="str">
+    <row r="24" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="13">
+        <v>46271</v>
+      </c>
+      <c r="B24" s="14">
+        <v>480</v>
+      </c>
+      <c r="C24" s="14">
+        <v>0</v>
+      </c>
+      <c r="D24" s="14">
+        <v>120</v>
+      </c>
+      <c r="E24" s="14">
+        <v>0</v>
+      </c>
+      <c r="F24" s="14">
+        <v>0</v>
+      </c>
+      <c r="G24" s="14">
+        <v>0</v>
+      </c>
+      <c r="H24" s="14">
+        <v>180</v>
+      </c>
+      <c r="I24" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="15" t="str">
+        <v>780</v>
+      </c>
+      <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="17"/>
+        <v>660</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L24" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N24" s="17" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="13"/>

</xml_diff>

<commit_message>
File Updated on 08/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58B8A00F-948A-4FF5-B86B-9B8724486156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94EF2651-3891-491D-ABD2-0631734FF0FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -236,6 +236,9 @@
   </si>
   <si>
     <t>Productive, but not efficient</t>
+  </si>
+  <si>
+    <t>20266-09-07</t>
   </si>
 </sst>
 </file>
@@ -1920,48 +1923,96 @@
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="13"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="15" t="str">
+      <c r="A25" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" s="14">
+        <v>360</v>
+      </c>
+      <c r="C25" s="14">
+        <v>0</v>
+      </c>
+      <c r="D25" s="14">
+        <v>90</v>
+      </c>
+      <c r="E25" s="14">
+        <v>0</v>
+      </c>
+      <c r="F25" s="14">
+        <v>250</v>
+      </c>
+      <c r="G25" s="14">
+        <v>5</v>
+      </c>
+      <c r="H25" s="14">
+        <v>60</v>
+      </c>
+      <c r="I25" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="15" t="str">
+        <v>760</v>
+      </c>
+      <c r="J25" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="17"/>
+        <v>680</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L25" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N25" s="17" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="15" t="str">
+      <c r="A26" s="13">
+        <v>46273</v>
+      </c>
+      <c r="B26" s="14">
+        <v>360</v>
+      </c>
+      <c r="C26" s="14">
+        <v>0</v>
+      </c>
+      <c r="D26" s="14">
+        <v>120</v>
+      </c>
+      <c r="E26" s="14">
+        <v>0</v>
+      </c>
+      <c r="F26" s="14">
+        <v>400</v>
+      </c>
+      <c r="G26" s="14">
+        <v>8</v>
+      </c>
+      <c r="H26" s="14">
+        <v>90</v>
+      </c>
+      <c r="I26" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="15" t="str">
+        <v>970</v>
+      </c>
+      <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="16"/>
-      <c r="N26" s="17"/>
+        <v>470</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L26" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N26" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="13"/>

</xml_diff>

<commit_message>
File Updated on 09/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94EF2651-3891-491D-ABD2-0631734FF0FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE26305F-8320-40CC-B9D8-2306A5A30C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2014,27 +2014,51 @@
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="15" t="str">
+    <row r="27" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="13">
+        <v>46274</v>
+      </c>
+      <c r="B27" s="14">
+        <v>360</v>
+      </c>
+      <c r="C27" s="14">
+        <v>0</v>
+      </c>
+      <c r="D27" s="14">
+        <v>45</v>
+      </c>
+      <c r="E27" s="14">
+        <v>0</v>
+      </c>
+      <c r="F27" s="14">
+        <v>350</v>
+      </c>
+      <c r="G27" s="14">
+        <v>7</v>
+      </c>
+      <c r="H27" s="14">
+        <v>60</v>
+      </c>
+      <c r="I27" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="15" t="str">
+        <v>815</v>
+      </c>
+      <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="17"/>
+        <v>625</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="N27" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="13"/>

</xml_diff>

<commit_message>
File Updated on 11/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE26305F-8320-40CC-B9D8-2306A5A30C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C2E7CF5-0F5A-465A-B0F6-0BB4C648EB9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2061,48 +2061,96 @@
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+      <c r="A28" s="13">
+        <v>46275</v>
+      </c>
+      <c r="B28" s="14">
+        <v>420</v>
+      </c>
+      <c r="C28" s="14">
+        <v>0</v>
+      </c>
+      <c r="D28" s="14">
+        <v>45</v>
+      </c>
+      <c r="E28" s="14">
+        <v>30</v>
+      </c>
+      <c r="F28" s="14">
+        <v>100</v>
+      </c>
+      <c r="G28" s="14">
+        <v>2</v>
+      </c>
+      <c r="H28" s="14">
+        <v>90</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>685</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="17"/>
+        <v>755</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N28" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15" t="str">
+      <c r="A29" s="13">
+        <v>46276</v>
+      </c>
+      <c r="B29" s="14">
+        <v>360</v>
+      </c>
+      <c r="C29" s="14">
+        <v>0</v>
+      </c>
+      <c r="D29" s="14">
+        <v>60</v>
+      </c>
+      <c r="E29" s="14">
+        <v>0</v>
+      </c>
+      <c r="F29" s="14">
+        <v>150</v>
+      </c>
+      <c r="G29" s="14">
+        <v>3</v>
+      </c>
+      <c r="H29" s="14">
+        <v>75</v>
+      </c>
+      <c r="I29" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
+        <v>645</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="17"/>
+        <v>795</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N29" s="17" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="13"/>

</xml_diff>

<commit_message>
File Updated on 13/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C2E7CF5-0F5A-465A-B0F6-0BB4C648EB9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{924688BB-715D-4FF2-A959-D1CD62602784}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2153,48 +2153,96 @@
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15" t="str">
+      <c r="A30" s="13">
+        <v>46277</v>
+      </c>
+      <c r="B30" s="14">
+        <v>480</v>
+      </c>
+      <c r="C30" s="14">
+        <v>0</v>
+      </c>
+      <c r="D30" s="14">
+        <v>180</v>
+      </c>
+      <c r="E30" s="14">
+        <v>0</v>
+      </c>
+      <c r="F30" s="14">
+        <v>0</v>
+      </c>
+      <c r="G30" s="14">
+        <v>0</v>
+      </c>
+      <c r="H30" s="14">
+        <v>90</v>
+      </c>
+      <c r="I30" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="15" t="str">
+        <v>750</v>
+      </c>
+      <c r="J30" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="17"/>
+        <v>690</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M30" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N30" s="17" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="13"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="15" t="str">
+      <c r="A31" s="13">
+        <v>46278</v>
+      </c>
+      <c r="B31" s="14">
+        <v>540</v>
+      </c>
+      <c r="C31" s="14">
+        <v>0</v>
+      </c>
+      <c r="D31" s="14">
+        <v>180</v>
+      </c>
+      <c r="E31" s="14">
+        <v>0</v>
+      </c>
+      <c r="F31" s="14">
+        <v>0</v>
+      </c>
+      <c r="G31" s="14">
+        <v>0</v>
+      </c>
+      <c r="H31" s="14">
+        <v>120</v>
+      </c>
+      <c r="I31" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="15" t="str">
+        <v>840</v>
+      </c>
+      <c r="J31" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="17"/>
+        <v>600</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M31" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N31" s="17" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="13"/>

</xml_diff>

<commit_message>
File Updated on 14/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{924688BB-715D-4FF2-A959-D1CD62602784}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B104A31-AFE7-4D42-B8B3-616DE6A8EB6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -731,186 +731,186 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A39"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="105" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="23.25" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" ht="22.8" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" s="4"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" s="4"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" s="5"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" s="4"/>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
     </row>
   </sheetData>
@@ -922,7 +922,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:N401"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="6" width="11" customWidth="1"/>
@@ -935,7 +935,7 @@
     <col min="14" max="14" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>29</v>
       </c>
@@ -953,7 +953,7 @@
       <c r="M1" s="19"/>
       <c r="N1" s="19"/>
     </row>
-    <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>30</v>
       </c>
@@ -970,7 +970,7 @@
       </c>
       <c r="G2" s="22"/>
     </row>
-    <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>32</v>
       </c>
@@ -987,7 +987,7 @@
       </c>
       <c r="G3" s="22"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
         <v>34</v>
       </c>
@@ -1005,7 +1005,7 @@
       <c r="M4" s="18"/>
       <c r="N4" s="18"/>
     </row>
-    <row r="5" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>35</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>46252</v>
       </c>
@@ -1094,7 +1094,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="13">
         <v>46253</v>
       </c>
@@ -1140,7 +1140,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="13">
         <v>46254</v>
       </c>
@@ -1186,7 +1186,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="13">
         <v>46256</v>
       </c>
@@ -1232,7 +1232,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="13">
         <v>46257</v>
       </c>
@@ -1278,7 +1278,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="13">
         <v>46258</v>
       </c>
@@ -1324,7 +1324,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="13">
         <v>46259</v>
       </c>
@@ -1370,7 +1370,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="13">
         <v>46260</v>
       </c>
@@ -1416,7 +1416,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="13">
         <v>46261</v>
       </c>
@@ -1462,7 +1462,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="13">
         <v>46262</v>
       </c>
@@ -1508,7 +1508,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="13">
         <v>46263</v>
       </c>
@@ -1554,7 +1554,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="13">
         <v>46264</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="13">
         <v>46265</v>
       </c>
@@ -1646,7 +1646,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="13">
         <v>46266</v>
       </c>
@@ -1692,7 +1692,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="13">
         <v>46267</v>
       </c>
@@ -1738,7 +1738,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="13">
         <v>46268</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="13">
         <v>46269</v>
       </c>
@@ -1830,7 +1830,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="13">
         <v>46270</v>
       </c>
@@ -1876,7 +1876,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="13">
         <v>46271</v>
       </c>
@@ -1922,7 +1922,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="13" t="s">
         <v>67</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="13">
         <v>46273</v>
       </c>
@@ -2014,7 +2014,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="13">
         <v>46274</v>
       </c>
@@ -2060,7 +2060,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" s="13">
         <v>46275</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="13">
         <v>46276</v>
       </c>
@@ -2152,7 +2152,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="13">
         <v>46277</v>
       </c>
@@ -2198,7 +2198,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" s="13">
         <v>46278</v>
       </c>
@@ -2244,29 +2244,53 @@
         <v>66</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="13"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="15" t="str">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A32" s="13">
+        <v>46279</v>
+      </c>
+      <c r="B32" s="14">
+        <v>420</v>
+      </c>
+      <c r="C32" s="14">
+        <v>0</v>
+      </c>
+      <c r="D32" s="14">
+        <v>120</v>
+      </c>
+      <c r="E32" s="14">
+        <v>0</v>
+      </c>
+      <c r="F32" s="14">
+        <v>250</v>
+      </c>
+      <c r="G32" s="14">
+        <v>5</v>
+      </c>
+      <c r="H32" s="14">
+        <v>70</v>
+      </c>
+      <c r="I32" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J32" s="15" t="str">
+        <v>860</v>
+      </c>
+      <c r="J32" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16"/>
-      <c r="M32" s="16"/>
-      <c r="N32" s="17"/>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+        <v>580</v>
+      </c>
+      <c r="K32" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L32" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M32" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="N32" s="17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="13"/>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -2288,7 +2312,7 @@
       <c r="M33" s="16"/>
       <c r="N33" s="17"/>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="13"/>
       <c r="B34" s="14"/>
       <c r="C34" s="14"/>
@@ -2310,7 +2334,7 @@
       <c r="M34" s="16"/>
       <c r="N34" s="17"/>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="13"/>
       <c r="B35" s="14"/>
       <c r="C35" s="14"/>
@@ -2332,7 +2356,7 @@
       <c r="M35" s="16"/>
       <c r="N35" s="17"/>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" s="13"/>
       <c r="B36" s="14"/>
       <c r="C36" s="14"/>
@@ -2354,7 +2378,7 @@
       <c r="M36" s="16"/>
       <c r="N36" s="17"/>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" s="13"/>
       <c r="B37" s="14"/>
       <c r="C37" s="14"/>
@@ -2376,7 +2400,7 @@
       <c r="M37" s="16"/>
       <c r="N37" s="17"/>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" s="13"/>
       <c r="B38" s="14"/>
       <c r="C38" s="14"/>
@@ -2398,7 +2422,7 @@
       <c r="M38" s="16"/>
       <c r="N38" s="17"/>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" s="13"/>
       <c r="B39" s="14"/>
       <c r="C39" s="14"/>
@@ -2420,7 +2444,7 @@
       <c r="M39" s="16"/>
       <c r="N39" s="17"/>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" s="13"/>
       <c r="B40" s="14"/>
       <c r="C40" s="14"/>
@@ -2442,7 +2466,7 @@
       <c r="M40" s="16"/>
       <c r="N40" s="17"/>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="13"/>
       <c r="B41" s="14"/>
       <c r="C41" s="14"/>
@@ -2464,7 +2488,7 @@
       <c r="M41" s="16"/>
       <c r="N41" s="17"/>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" s="13"/>
       <c r="B42" s="14"/>
       <c r="C42" s="14"/>
@@ -2486,7 +2510,7 @@
       <c r="M42" s="16"/>
       <c r="N42" s="17"/>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" s="13"/>
       <c r="B43" s="14"/>
       <c r="C43" s="14"/>
@@ -2508,7 +2532,7 @@
       <c r="M43" s="16"/>
       <c r="N43" s="17"/>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" s="13"/>
       <c r="B44" s="14"/>
       <c r="C44" s="14"/>
@@ -2530,7 +2554,7 @@
       <c r="M44" s="16"/>
       <c r="N44" s="17"/>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" s="13"/>
       <c r="B45" s="14"/>
       <c r="C45" s="14"/>
@@ -2552,7 +2576,7 @@
       <c r="M45" s="16"/>
       <c r="N45" s="17"/>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" s="13"/>
       <c r="B46" s="14"/>
       <c r="C46" s="14"/>
@@ -2574,7 +2598,7 @@
       <c r="M46" s="16"/>
       <c r="N46" s="17"/>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" s="13"/>
       <c r="B47" s="14"/>
       <c r="C47" s="14"/>
@@ -2596,7 +2620,7 @@
       <c r="M47" s="16"/>
       <c r="N47" s="17"/>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" s="13"/>
       <c r="B48" s="14"/>
       <c r="C48" s="14"/>
@@ -2618,7 +2642,7 @@
       <c r="M48" s="16"/>
       <c r="N48" s="17"/>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" s="13"/>
       <c r="B49" s="14"/>
       <c r="C49" s="14"/>
@@ -2640,7 +2664,7 @@
       <c r="M49" s="16"/>
       <c r="N49" s="17"/>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" s="13"/>
       <c r="B50" s="14"/>
       <c r="C50" s="14"/>
@@ -2662,7 +2686,7 @@
       <c r="M50" s="16"/>
       <c r="N50" s="17"/>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" s="13"/>
       <c r="B51" s="14"/>
       <c r="C51" s="14"/>
@@ -2684,7 +2708,7 @@
       <c r="M51" s="16"/>
       <c r="N51" s="17"/>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" s="13"/>
       <c r="B52" s="14"/>
       <c r="C52" s="14"/>
@@ -2706,7 +2730,7 @@
       <c r="M52" s="16"/>
       <c r="N52" s="17"/>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" s="13"/>
       <c r="B53" s="14"/>
       <c r="C53" s="14"/>
@@ -2728,7 +2752,7 @@
       <c r="M53" s="16"/>
       <c r="N53" s="17"/>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" s="13"/>
       <c r="B54" s="14"/>
       <c r="C54" s="14"/>
@@ -2750,7 +2774,7 @@
       <c r="M54" s="16"/>
       <c r="N54" s="17"/>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" s="13"/>
       <c r="B55" s="14"/>
       <c r="C55" s="14"/>
@@ -2772,7 +2796,7 @@
       <c r="M55" s="16"/>
       <c r="N55" s="17"/>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" s="13"/>
       <c r="B56" s="14"/>
       <c r="C56" s="14"/>
@@ -2794,7 +2818,7 @@
       <c r="M56" s="16"/>
       <c r="N56" s="17"/>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" s="13"/>
       <c r="B57" s="14"/>
       <c r="C57" s="14"/>
@@ -2816,7 +2840,7 @@
       <c r="M57" s="16"/>
       <c r="N57" s="17"/>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" s="13"/>
       <c r="B58" s="14"/>
       <c r="C58" s="14"/>
@@ -2838,7 +2862,7 @@
       <c r="M58" s="16"/>
       <c r="N58" s="17"/>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" s="13"/>
       <c r="B59" s="14"/>
       <c r="C59" s="14"/>
@@ -2860,7 +2884,7 @@
       <c r="M59" s="16"/>
       <c r="N59" s="17"/>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" s="13"/>
       <c r="B60" s="14"/>
       <c r="C60" s="14"/>
@@ -2882,7 +2906,7 @@
       <c r="M60" s="16"/>
       <c r="N60" s="17"/>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" s="13"/>
       <c r="B61" s="14"/>
       <c r="C61" s="14"/>
@@ -2904,7 +2928,7 @@
       <c r="M61" s="16"/>
       <c r="N61" s="17"/>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" s="13"/>
       <c r="B62" s="14"/>
       <c r="C62" s="14"/>
@@ -2926,7 +2950,7 @@
       <c r="M62" s="16"/>
       <c r="N62" s="17"/>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" s="13"/>
       <c r="B63" s="14"/>
       <c r="C63" s="14"/>
@@ -2948,7 +2972,7 @@
       <c r="M63" s="16"/>
       <c r="N63" s="17"/>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="13"/>
       <c r="B64" s="14"/>
       <c r="C64" s="14"/>
@@ -2970,7 +2994,7 @@
       <c r="M64" s="16"/>
       <c r="N64" s="17"/>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" s="13"/>
       <c r="B65" s="14"/>
       <c r="C65" s="14"/>
@@ -2992,7 +3016,7 @@
       <c r="M65" s="16"/>
       <c r="N65" s="17"/>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" s="13"/>
       <c r="B66" s="14"/>
       <c r="C66" s="14"/>
@@ -3014,7 +3038,7 @@
       <c r="M66" s="16"/>
       <c r="N66" s="17"/>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" s="13"/>
       <c r="B67" s="14"/>
       <c r="C67" s="14"/>
@@ -3036,7 +3060,7 @@
       <c r="M67" s="16"/>
       <c r="N67" s="17"/>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" s="13"/>
       <c r="B68" s="14"/>
       <c r="C68" s="14"/>
@@ -3058,7 +3082,7 @@
       <c r="M68" s="16"/>
       <c r="N68" s="17"/>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69" s="13"/>
       <c r="B69" s="14"/>
       <c r="C69" s="14"/>
@@ -3080,7 +3104,7 @@
       <c r="M69" s="16"/>
       <c r="N69" s="17"/>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70" s="13"/>
       <c r="B70" s="14"/>
       <c r="C70" s="14"/>
@@ -3102,7 +3126,7 @@
       <c r="M70" s="16"/>
       <c r="N70" s="17"/>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71" s="13"/>
       <c r="B71" s="14"/>
       <c r="C71" s="14"/>
@@ -3124,7 +3148,7 @@
       <c r="M71" s="16"/>
       <c r="N71" s="17"/>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" s="13"/>
       <c r="B72" s="14"/>
       <c r="C72" s="14"/>
@@ -3146,7 +3170,7 @@
       <c r="M72" s="16"/>
       <c r="N72" s="17"/>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73" s="13"/>
       <c r="B73" s="14"/>
       <c r="C73" s="14"/>
@@ -3168,7 +3192,7 @@
       <c r="M73" s="16"/>
       <c r="N73" s="17"/>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74" s="13"/>
       <c r="B74" s="14"/>
       <c r="C74" s="14"/>
@@ -3190,7 +3214,7 @@
       <c r="M74" s="16"/>
       <c r="N74" s="17"/>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75" s="13"/>
       <c r="B75" s="14"/>
       <c r="C75" s="14"/>
@@ -3212,7 +3236,7 @@
       <c r="M75" s="16"/>
       <c r="N75" s="17"/>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76" s="13"/>
       <c r="B76" s="14"/>
       <c r="C76" s="14"/>
@@ -3234,7 +3258,7 @@
       <c r="M76" s="16"/>
       <c r="N76" s="17"/>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77" s="13"/>
       <c r="B77" s="14"/>
       <c r="C77" s="14"/>
@@ -3256,7 +3280,7 @@
       <c r="M77" s="16"/>
       <c r="N77" s="17"/>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A78" s="13"/>
       <c r="B78" s="14"/>
       <c r="C78" s="14"/>
@@ -3278,7 +3302,7 @@
       <c r="M78" s="16"/>
       <c r="N78" s="17"/>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A79" s="13"/>
       <c r="B79" s="14"/>
       <c r="C79" s="14"/>
@@ -3300,7 +3324,7 @@
       <c r="M79" s="16"/>
       <c r="N79" s="17"/>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A80" s="13"/>
       <c r="B80" s="14"/>
       <c r="C80" s="14"/>
@@ -3322,7 +3346,7 @@
       <c r="M80" s="16"/>
       <c r="N80" s="17"/>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A81" s="13"/>
       <c r="B81" s="14"/>
       <c r="C81" s="14"/>
@@ -3344,7 +3368,7 @@
       <c r="M81" s="16"/>
       <c r="N81" s="17"/>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A82" s="13"/>
       <c r="B82" s="14"/>
       <c r="C82" s="14"/>
@@ -3366,7 +3390,7 @@
       <c r="M82" s="16"/>
       <c r="N82" s="17"/>
     </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A83" s="13"/>
       <c r="B83" s="14"/>
       <c r="C83" s="14"/>
@@ -3388,7 +3412,7 @@
       <c r="M83" s="16"/>
       <c r="N83" s="17"/>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A84" s="13"/>
       <c r="B84" s="14"/>
       <c r="C84" s="14"/>
@@ -3410,7 +3434,7 @@
       <c r="M84" s="16"/>
       <c r="N84" s="17"/>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A85" s="13"/>
       <c r="B85" s="14"/>
       <c r="C85" s="14"/>
@@ -3432,7 +3456,7 @@
       <c r="M85" s="16"/>
       <c r="N85" s="17"/>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A86" s="13"/>
       <c r="B86" s="14"/>
       <c r="C86" s="14"/>
@@ -3454,7 +3478,7 @@
       <c r="M86" s="16"/>
       <c r="N86" s="17"/>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A87" s="13"/>
       <c r="B87" s="14"/>
       <c r="C87" s="14"/>
@@ -3476,7 +3500,7 @@
       <c r="M87" s="16"/>
       <c r="N87" s="17"/>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A88" s="13"/>
       <c r="B88" s="14"/>
       <c r="C88" s="14"/>
@@ -3498,7 +3522,7 @@
       <c r="M88" s="16"/>
       <c r="N88" s="17"/>
     </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A89" s="13"/>
       <c r="B89" s="14"/>
       <c r="C89" s="14"/>
@@ -3520,7 +3544,7 @@
       <c r="M89" s="16"/>
       <c r="N89" s="17"/>
     </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A90" s="13"/>
       <c r="B90" s="14"/>
       <c r="C90" s="14"/>
@@ -3542,7 +3566,7 @@
       <c r="M90" s="16"/>
       <c r="N90" s="17"/>
     </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A91" s="13"/>
       <c r="B91" s="14"/>
       <c r="C91" s="14"/>
@@ -3564,7 +3588,7 @@
       <c r="M91" s="16"/>
       <c r="N91" s="17"/>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A92" s="13"/>
       <c r="B92" s="14"/>
       <c r="C92" s="14"/>
@@ -3586,7 +3610,7 @@
       <c r="M92" s="16"/>
       <c r="N92" s="17"/>
     </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A93" s="13"/>
       <c r="B93" s="14"/>
       <c r="C93" s="14"/>
@@ -3608,7 +3632,7 @@
       <c r="M93" s="16"/>
       <c r="N93" s="17"/>
     </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A94" s="13"/>
       <c r="B94" s="14"/>
       <c r="C94" s="14"/>
@@ -3630,7 +3654,7 @@
       <c r="M94" s="16"/>
       <c r="N94" s="17"/>
     </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A95" s="13"/>
       <c r="B95" s="14"/>
       <c r="C95" s="14"/>
@@ -3652,7 +3676,7 @@
       <c r="M95" s="16"/>
       <c r="N95" s="17"/>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A96" s="13"/>
       <c r="B96" s="14"/>
       <c r="C96" s="14"/>
@@ -3674,7 +3698,7 @@
       <c r="M96" s="16"/>
       <c r="N96" s="17"/>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A97" s="13"/>
       <c r="B97" s="14"/>
       <c r="C97" s="14"/>
@@ -3696,7 +3720,7 @@
       <c r="M97" s="16"/>
       <c r="N97" s="17"/>
     </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A98" s="13"/>
       <c r="B98" s="14"/>
       <c r="C98" s="14"/>
@@ -3718,7 +3742,7 @@
       <c r="M98" s="16"/>
       <c r="N98" s="17"/>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A99" s="13"/>
       <c r="B99" s="14"/>
       <c r="C99" s="14"/>
@@ -3740,7 +3764,7 @@
       <c r="M99" s="16"/>
       <c r="N99" s="17"/>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A100" s="13"/>
       <c r="B100" s="14"/>
       <c r="C100" s="14"/>
@@ -3762,7 +3786,7 @@
       <c r="M100" s="16"/>
       <c r="N100" s="17"/>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A101" s="13"/>
       <c r="B101" s="14"/>
       <c r="C101" s="14"/>
@@ -3784,7 +3808,7 @@
       <c r="M101" s="16"/>
       <c r="N101" s="17"/>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A102" s="13"/>
       <c r="B102" s="14"/>
       <c r="C102" s="14"/>
@@ -3806,7 +3830,7 @@
       <c r="M102" s="16"/>
       <c r="N102" s="17"/>
     </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A103" s="13"/>
       <c r="B103" s="14"/>
       <c r="C103" s="14"/>
@@ -3828,7 +3852,7 @@
       <c r="M103" s="16"/>
       <c r="N103" s="17"/>
     </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A104" s="13"/>
       <c r="B104" s="14"/>
       <c r="C104" s="14"/>
@@ -3850,7 +3874,7 @@
       <c r="M104" s="16"/>
       <c r="N104" s="17"/>
     </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A105" s="13"/>
       <c r="B105" s="14"/>
       <c r="C105" s="14"/>
@@ -3872,7 +3896,7 @@
       <c r="M105" s="16"/>
       <c r="N105" s="17"/>
     </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A106" s="13"/>
       <c r="B106" s="14"/>
       <c r="C106" s="14"/>
@@ -3894,7 +3918,7 @@
       <c r="M106" s="16"/>
       <c r="N106" s="17"/>
     </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A107" s="13"/>
       <c r="B107" s="14"/>
       <c r="C107" s="14"/>
@@ -3916,7 +3940,7 @@
       <c r="M107" s="16"/>
       <c r="N107" s="17"/>
     </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A108" s="13"/>
       <c r="B108" s="14"/>
       <c r="C108" s="14"/>
@@ -3938,7 +3962,7 @@
       <c r="M108" s="16"/>
       <c r="N108" s="17"/>
     </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A109" s="13"/>
       <c r="B109" s="14"/>
       <c r="C109" s="14"/>
@@ -3960,7 +3984,7 @@
       <c r="M109" s="16"/>
       <c r="N109" s="17"/>
     </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A110" s="13"/>
       <c r="B110" s="14"/>
       <c r="C110" s="14"/>
@@ -3982,7 +4006,7 @@
       <c r="M110" s="16"/>
       <c r="N110" s="17"/>
     </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A111" s="13"/>
       <c r="B111" s="14"/>
       <c r="C111" s="14"/>
@@ -4004,7 +4028,7 @@
       <c r="M111" s="16"/>
       <c r="N111" s="17"/>
     </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A112" s="13"/>
       <c r="B112" s="14"/>
       <c r="C112" s="14"/>
@@ -4026,7 +4050,7 @@
       <c r="M112" s="16"/>
       <c r="N112" s="17"/>
     </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A113" s="13"/>
       <c r="B113" s="14"/>
       <c r="C113" s="14"/>
@@ -4048,7 +4072,7 @@
       <c r="M113" s="16"/>
       <c r="N113" s="17"/>
     </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A114" s="13"/>
       <c r="B114" s="14"/>
       <c r="C114" s="14"/>
@@ -4070,7 +4094,7 @@
       <c r="M114" s="16"/>
       <c r="N114" s="17"/>
     </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A115" s="13"/>
       <c r="B115" s="14"/>
       <c r="C115" s="14"/>
@@ -4092,7 +4116,7 @@
       <c r="M115" s="16"/>
       <c r="N115" s="17"/>
     </row>
-    <row r="116" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A116" s="13"/>
       <c r="B116" s="14"/>
       <c r="C116" s="14"/>
@@ -4114,7 +4138,7 @@
       <c r="M116" s="16"/>
       <c r="N116" s="17"/>
     </row>
-    <row r="117" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A117" s="13"/>
       <c r="B117" s="14"/>
       <c r="C117" s="14"/>
@@ -4136,7 +4160,7 @@
       <c r="M117" s="16"/>
       <c r="N117" s="17"/>
     </row>
-    <row r="118" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A118" s="13"/>
       <c r="B118" s="14"/>
       <c r="C118" s="14"/>
@@ -4158,7 +4182,7 @@
       <c r="M118" s="16"/>
       <c r="N118" s="17"/>
     </row>
-    <row r="119" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A119" s="13"/>
       <c r="B119" s="14"/>
       <c r="C119" s="14"/>
@@ -4180,7 +4204,7 @@
       <c r="M119" s="16"/>
       <c r="N119" s="17"/>
     </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A120" s="13"/>
       <c r="B120" s="14"/>
       <c r="C120" s="14"/>
@@ -4202,7 +4226,7 @@
       <c r="M120" s="16"/>
       <c r="N120" s="17"/>
     </row>
-    <row r="121" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A121" s="13"/>
       <c r="B121" s="14"/>
       <c r="C121" s="14"/>
@@ -4224,7 +4248,7 @@
       <c r="M121" s="16"/>
       <c r="N121" s="17"/>
     </row>
-    <row r="122" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A122" s="13"/>
       <c r="B122" s="14"/>
       <c r="C122" s="14"/>
@@ -4246,7 +4270,7 @@
       <c r="M122" s="16"/>
       <c r="N122" s="17"/>
     </row>
-    <row r="123" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A123" s="13"/>
       <c r="B123" s="14"/>
       <c r="C123" s="14"/>
@@ -4268,7 +4292,7 @@
       <c r="M123" s="16"/>
       <c r="N123" s="17"/>
     </row>
-    <row r="124" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A124" s="13"/>
       <c r="B124" s="14"/>
       <c r="C124" s="14"/>
@@ -4290,7 +4314,7 @@
       <c r="M124" s="16"/>
       <c r="N124" s="17"/>
     </row>
-    <row r="125" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A125" s="13"/>
       <c r="B125" s="14"/>
       <c r="C125" s="14"/>
@@ -4312,7 +4336,7 @@
       <c r="M125" s="16"/>
       <c r="N125" s="17"/>
     </row>
-    <row r="126" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A126" s="13"/>
       <c r="B126" s="14"/>
       <c r="C126" s="14"/>
@@ -4334,7 +4358,7 @@
       <c r="M126" s="16"/>
       <c r="N126" s="17"/>
     </row>
-    <row r="127" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A127" s="13"/>
       <c r="B127" s="14"/>
       <c r="C127" s="14"/>
@@ -4356,7 +4380,7 @@
       <c r="M127" s="16"/>
       <c r="N127" s="17"/>
     </row>
-    <row r="128" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A128" s="13"/>
       <c r="B128" s="14"/>
       <c r="C128" s="14"/>
@@ -4378,7 +4402,7 @@
       <c r="M128" s="16"/>
       <c r="N128" s="17"/>
     </row>
-    <row r="129" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A129" s="13"/>
       <c r="B129" s="14"/>
       <c r="C129" s="14"/>
@@ -4400,7 +4424,7 @@
       <c r="M129" s="16"/>
       <c r="N129" s="17"/>
     </row>
-    <row r="130" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A130" s="13"/>
       <c r="B130" s="14"/>
       <c r="C130" s="14"/>
@@ -4422,7 +4446,7 @@
       <c r="M130" s="16"/>
       <c r="N130" s="17"/>
     </row>
-    <row r="131" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A131" s="13"/>
       <c r="B131" s="14"/>
       <c r="C131" s="14"/>
@@ -4444,7 +4468,7 @@
       <c r="M131" s="16"/>
       <c r="N131" s="17"/>
     </row>
-    <row r="132" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A132" s="13"/>
       <c r="B132" s="14"/>
       <c r="C132" s="14"/>
@@ -4466,7 +4490,7 @@
       <c r="M132" s="16"/>
       <c r="N132" s="17"/>
     </row>
-    <row r="133" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A133" s="13"/>
       <c r="B133" s="14"/>
       <c r="C133" s="14"/>
@@ -4488,7 +4512,7 @@
       <c r="M133" s="16"/>
       <c r="N133" s="17"/>
     </row>
-    <row r="134" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A134" s="13"/>
       <c r="B134" s="14"/>
       <c r="C134" s="14"/>
@@ -4510,7 +4534,7 @@
       <c r="M134" s="16"/>
       <c r="N134" s="17"/>
     </row>
-    <row r="135" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A135" s="13"/>
       <c r="B135" s="14"/>
       <c r="C135" s="14"/>
@@ -4532,7 +4556,7 @@
       <c r="M135" s="16"/>
       <c r="N135" s="17"/>
     </row>
-    <row r="136" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A136" s="13"/>
       <c r="B136" s="14"/>
       <c r="C136" s="14"/>
@@ -4554,7 +4578,7 @@
       <c r="M136" s="16"/>
       <c r="N136" s="17"/>
     </row>
-    <row r="137" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A137" s="13"/>
       <c r="B137" s="14"/>
       <c r="C137" s="14"/>
@@ -4576,7 +4600,7 @@
       <c r="M137" s="16"/>
       <c r="N137" s="17"/>
     </row>
-    <row r="138" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A138" s="13"/>
       <c r="B138" s="14"/>
       <c r="C138" s="14"/>
@@ -4598,7 +4622,7 @@
       <c r="M138" s="16"/>
       <c r="N138" s="17"/>
     </row>
-    <row r="139" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A139" s="13"/>
       <c r="B139" s="14"/>
       <c r="C139" s="14"/>
@@ -4620,7 +4644,7 @@
       <c r="M139" s="16"/>
       <c r="N139" s="17"/>
     </row>
-    <row r="140" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A140" s="13"/>
       <c r="B140" s="14"/>
       <c r="C140" s="14"/>
@@ -4642,7 +4666,7 @@
       <c r="M140" s="16"/>
       <c r="N140" s="17"/>
     </row>
-    <row r="141" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A141" s="13"/>
       <c r="B141" s="14"/>
       <c r="C141" s="14"/>
@@ -4664,7 +4688,7 @@
       <c r="M141" s="16"/>
       <c r="N141" s="17"/>
     </row>
-    <row r="142" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A142" s="13"/>
       <c r="B142" s="14"/>
       <c r="C142" s="14"/>
@@ -4686,7 +4710,7 @@
       <c r="M142" s="16"/>
       <c r="N142" s="17"/>
     </row>
-    <row r="143" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A143" s="13"/>
       <c r="B143" s="14"/>
       <c r="C143" s="14"/>
@@ -4708,7 +4732,7 @@
       <c r="M143" s="16"/>
       <c r="N143" s="17"/>
     </row>
-    <row r="144" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A144" s="13"/>
       <c r="B144" s="14"/>
       <c r="C144" s="14"/>
@@ -4730,7 +4754,7 @@
       <c r="M144" s="16"/>
       <c r="N144" s="17"/>
     </row>
-    <row r="145" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A145" s="13"/>
       <c r="B145" s="14"/>
       <c r="C145" s="14"/>
@@ -4752,7 +4776,7 @@
       <c r="M145" s="16"/>
       <c r="N145" s="17"/>
     </row>
-    <row r="146" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A146" s="13"/>
       <c r="B146" s="14"/>
       <c r="C146" s="14"/>
@@ -4774,7 +4798,7 @@
       <c r="M146" s="16"/>
       <c r="N146" s="17"/>
     </row>
-    <row r="147" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A147" s="13"/>
       <c r="B147" s="14"/>
       <c r="C147" s="14"/>
@@ -4796,7 +4820,7 @@
       <c r="M147" s="16"/>
       <c r="N147" s="17"/>
     </row>
-    <row r="148" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A148" s="13"/>
       <c r="B148" s="14"/>
       <c r="C148" s="14"/>
@@ -4818,7 +4842,7 @@
       <c r="M148" s="16"/>
       <c r="N148" s="17"/>
     </row>
-    <row r="149" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A149" s="13"/>
       <c r="B149" s="14"/>
       <c r="C149" s="14"/>
@@ -4840,7 +4864,7 @@
       <c r="M149" s="16"/>
       <c r="N149" s="17"/>
     </row>
-    <row r="150" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A150" s="13"/>
       <c r="B150" s="14"/>
       <c r="C150" s="14"/>
@@ -4862,7 +4886,7 @@
       <c r="M150" s="16"/>
       <c r="N150" s="17"/>
     </row>
-    <row r="151" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A151" s="13"/>
       <c r="B151" s="14"/>
       <c r="C151" s="14"/>
@@ -4884,7 +4908,7 @@
       <c r="M151" s="16"/>
       <c r="N151" s="17"/>
     </row>
-    <row r="152" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A152" s="13"/>
       <c r="B152" s="14"/>
       <c r="C152" s="14"/>
@@ -4906,7 +4930,7 @@
       <c r="M152" s="16"/>
       <c r="N152" s="17"/>
     </row>
-    <row r="153" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A153" s="13"/>
       <c r="B153" s="14"/>
       <c r="C153" s="14"/>
@@ -4928,7 +4952,7 @@
       <c r="M153" s="16"/>
       <c r="N153" s="17"/>
     </row>
-    <row r="154" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A154" s="13"/>
       <c r="B154" s="14"/>
       <c r="C154" s="14"/>
@@ -4950,7 +4974,7 @@
       <c r="M154" s="16"/>
       <c r="N154" s="17"/>
     </row>
-    <row r="155" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A155" s="13"/>
       <c r="B155" s="14"/>
       <c r="C155" s="14"/>
@@ -4972,7 +4996,7 @@
       <c r="M155" s="16"/>
       <c r="N155" s="17"/>
     </row>
-    <row r="156" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A156" s="13"/>
       <c r="B156" s="14"/>
       <c r="C156" s="14"/>
@@ -4994,7 +5018,7 @@
       <c r="M156" s="16"/>
       <c r="N156" s="17"/>
     </row>
-    <row r="157" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A157" s="13"/>
       <c r="B157" s="14"/>
       <c r="C157" s="14"/>
@@ -5016,7 +5040,7 @@
       <c r="M157" s="16"/>
       <c r="N157" s="17"/>
     </row>
-    <row r="158" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A158" s="13"/>
       <c r="B158" s="14"/>
       <c r="C158" s="14"/>
@@ -5038,7 +5062,7 @@
       <c r="M158" s="16"/>
       <c r="N158" s="17"/>
     </row>
-    <row r="159" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A159" s="13"/>
       <c r="B159" s="14"/>
       <c r="C159" s="14"/>
@@ -5060,7 +5084,7 @@
       <c r="M159" s="16"/>
       <c r="N159" s="17"/>
     </row>
-    <row r="160" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A160" s="13"/>
       <c r="B160" s="14"/>
       <c r="C160" s="14"/>
@@ -5082,7 +5106,7 @@
       <c r="M160" s="16"/>
       <c r="N160" s="17"/>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A161" s="13"/>
       <c r="B161" s="14"/>
       <c r="C161" s="14"/>
@@ -5104,7 +5128,7 @@
       <c r="M161" s="16"/>
       <c r="N161" s="17"/>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A162" s="13"/>
       <c r="B162" s="14"/>
       <c r="C162" s="14"/>
@@ -5126,7 +5150,7 @@
       <c r="M162" s="16"/>
       <c r="N162" s="17"/>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A163" s="13"/>
       <c r="B163" s="14"/>
       <c r="C163" s="14"/>
@@ -5148,7 +5172,7 @@
       <c r="M163" s="16"/>
       <c r="N163" s="17"/>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A164" s="13"/>
       <c r="B164" s="14"/>
       <c r="C164" s="14"/>
@@ -5170,7 +5194,7 @@
       <c r="M164" s="16"/>
       <c r="N164" s="17"/>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A165" s="13"/>
       <c r="B165" s="14"/>
       <c r="C165" s="14"/>
@@ -5192,7 +5216,7 @@
       <c r="M165" s="16"/>
       <c r="N165" s="17"/>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A166" s="13"/>
       <c r="B166" s="14"/>
       <c r="C166" s="14"/>
@@ -5214,7 +5238,7 @@
       <c r="M166" s="16"/>
       <c r="N166" s="17"/>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A167" s="13"/>
       <c r="B167" s="14"/>
       <c r="C167" s="14"/>
@@ -5236,7 +5260,7 @@
       <c r="M167" s="16"/>
       <c r="N167" s="17"/>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A168" s="13"/>
       <c r="B168" s="14"/>
       <c r="C168" s="14"/>
@@ -5258,7 +5282,7 @@
       <c r="M168" s="16"/>
       <c r="N168" s="17"/>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A169" s="13"/>
       <c r="B169" s="14"/>
       <c r="C169" s="14"/>
@@ -5280,7 +5304,7 @@
       <c r="M169" s="16"/>
       <c r="N169" s="17"/>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A170" s="13"/>
       <c r="B170" s="14"/>
       <c r="C170" s="14"/>
@@ -5302,7 +5326,7 @@
       <c r="M170" s="16"/>
       <c r="N170" s="17"/>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A171" s="13"/>
       <c r="B171" s="14"/>
       <c r="C171" s="14"/>
@@ -5324,7 +5348,7 @@
       <c r="M171" s="16"/>
       <c r="N171" s="17"/>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A172" s="13"/>
       <c r="B172" s="14"/>
       <c r="C172" s="14"/>
@@ -5346,7 +5370,7 @@
       <c r="M172" s="16"/>
       <c r="N172" s="17"/>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A173" s="13"/>
       <c r="B173" s="14"/>
       <c r="C173" s="14"/>
@@ -5368,7 +5392,7 @@
       <c r="M173" s="16"/>
       <c r="N173" s="17"/>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A174" s="13"/>
       <c r="B174" s="14"/>
       <c r="C174" s="14"/>
@@ -5390,7 +5414,7 @@
       <c r="M174" s="16"/>
       <c r="N174" s="17"/>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A175" s="13"/>
       <c r="B175" s="14"/>
       <c r="C175" s="14"/>
@@ -5412,7 +5436,7 @@
       <c r="M175" s="16"/>
       <c r="N175" s="17"/>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A176" s="13"/>
       <c r="B176" s="14"/>
       <c r="C176" s="14"/>
@@ -5434,7 +5458,7 @@
       <c r="M176" s="16"/>
       <c r="N176" s="17"/>
     </row>
-    <row r="177" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A177" s="13"/>
       <c r="B177" s="14"/>
       <c r="C177" s="14"/>
@@ -5456,7 +5480,7 @@
       <c r="M177" s="16"/>
       <c r="N177" s="17"/>
     </row>
-    <row r="178" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A178" s="13"/>
       <c r="B178" s="14"/>
       <c r="C178" s="14"/>
@@ -5478,7 +5502,7 @@
       <c r="M178" s="16"/>
       <c r="N178" s="17"/>
     </row>
-    <row r="179" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A179" s="13"/>
       <c r="B179" s="14"/>
       <c r="C179" s="14"/>
@@ -5500,7 +5524,7 @@
       <c r="M179" s="16"/>
       <c r="N179" s="17"/>
     </row>
-    <row r="180" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A180" s="13"/>
       <c r="B180" s="14"/>
       <c r="C180" s="14"/>
@@ -5522,7 +5546,7 @@
       <c r="M180" s="16"/>
       <c r="N180" s="17"/>
     </row>
-    <row r="181" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A181" s="13"/>
       <c r="B181" s="14"/>
       <c r="C181" s="14"/>
@@ -5544,7 +5568,7 @@
       <c r="M181" s="16"/>
       <c r="N181" s="17"/>
     </row>
-    <row r="182" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A182" s="13"/>
       <c r="B182" s="14"/>
       <c r="C182" s="14"/>
@@ -5566,7 +5590,7 @@
       <c r="M182" s="16"/>
       <c r="N182" s="17"/>
     </row>
-    <row r="183" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A183" s="13"/>
       <c r="B183" s="14"/>
       <c r="C183" s="14"/>
@@ -5588,7 +5612,7 @@
       <c r="M183" s="16"/>
       <c r="N183" s="17"/>
     </row>
-    <row r="184" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A184" s="13"/>
       <c r="B184" s="14"/>
       <c r="C184" s="14"/>
@@ -5610,7 +5634,7 @@
       <c r="M184" s="16"/>
       <c r="N184" s="17"/>
     </row>
-    <row r="185" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A185" s="13"/>
       <c r="B185" s="14"/>
       <c r="C185" s="14"/>
@@ -5632,7 +5656,7 @@
       <c r="M185" s="16"/>
       <c r="N185" s="17"/>
     </row>
-    <row r="186" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A186" s="13"/>
       <c r="B186" s="14"/>
       <c r="C186" s="14"/>
@@ -5654,7 +5678,7 @@
       <c r="M186" s="16"/>
       <c r="N186" s="17"/>
     </row>
-    <row r="187" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A187" s="13"/>
       <c r="B187" s="14"/>
       <c r="C187" s="14"/>
@@ -5676,7 +5700,7 @@
       <c r="M187" s="16"/>
       <c r="N187" s="17"/>
     </row>
-    <row r="188" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A188" s="13"/>
       <c r="B188" s="14"/>
       <c r="C188" s="14"/>
@@ -5698,7 +5722,7 @@
       <c r="M188" s="16"/>
       <c r="N188" s="17"/>
     </row>
-    <row r="189" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A189" s="13"/>
       <c r="B189" s="14"/>
       <c r="C189" s="14"/>
@@ -5720,7 +5744,7 @@
       <c r="M189" s="16"/>
       <c r="N189" s="17"/>
     </row>
-    <row r="190" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A190" s="13"/>
       <c r="B190" s="14"/>
       <c r="C190" s="14"/>
@@ -5742,7 +5766,7 @@
       <c r="M190" s="16"/>
       <c r="N190" s="17"/>
     </row>
-    <row r="191" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A191" s="13"/>
       <c r="B191" s="14"/>
       <c r="C191" s="14"/>
@@ -5764,7 +5788,7 @@
       <c r="M191" s="16"/>
       <c r="N191" s="17"/>
     </row>
-    <row r="192" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A192" s="13"/>
       <c r="B192" s="14"/>
       <c r="C192" s="14"/>
@@ -5786,7 +5810,7 @@
       <c r="M192" s="16"/>
       <c r="N192" s="17"/>
     </row>
-    <row r="193" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A193" s="13"/>
       <c r="B193" s="14"/>
       <c r="C193" s="14"/>
@@ -5808,7 +5832,7 @@
       <c r="M193" s="16"/>
       <c r="N193" s="17"/>
     </row>
-    <row r="194" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A194" s="13"/>
       <c r="B194" s="14"/>
       <c r="C194" s="14"/>
@@ -5830,7 +5854,7 @@
       <c r="M194" s="16"/>
       <c r="N194" s="17"/>
     </row>
-    <row r="195" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A195" s="13"/>
       <c r="B195" s="14"/>
       <c r="C195" s="14"/>
@@ -5852,7 +5876,7 @@
       <c r="M195" s="16"/>
       <c r="N195" s="17"/>
     </row>
-    <row r="196" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A196" s="13"/>
       <c r="B196" s="14"/>
       <c r="C196" s="14"/>
@@ -5874,7 +5898,7 @@
       <c r="M196" s="16"/>
       <c r="N196" s="17"/>
     </row>
-    <row r="197" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A197" s="13"/>
       <c r="B197" s="14"/>
       <c r="C197" s="14"/>
@@ -5896,7 +5920,7 @@
       <c r="M197" s="16"/>
       <c r="N197" s="17"/>
     </row>
-    <row r="198" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A198" s="13"/>
       <c r="B198" s="14"/>
       <c r="C198" s="14"/>
@@ -5918,7 +5942,7 @@
       <c r="M198" s="16"/>
       <c r="N198" s="17"/>
     </row>
-    <row r="199" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A199" s="13"/>
       <c r="B199" s="14"/>
       <c r="C199" s="14"/>
@@ -5940,7 +5964,7 @@
       <c r="M199" s="16"/>
       <c r="N199" s="17"/>
     </row>
-    <row r="200" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A200" s="13"/>
       <c r="B200" s="14"/>
       <c r="C200" s="14"/>
@@ -5962,7 +5986,7 @@
       <c r="M200" s="16"/>
       <c r="N200" s="17"/>
     </row>
-    <row r="201" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A201" s="13"/>
       <c r="B201" s="14"/>
       <c r="C201" s="14"/>
@@ -5984,7 +6008,7 @@
       <c r="M201" s="16"/>
       <c r="N201" s="17"/>
     </row>
-    <row r="202" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A202" s="13"/>
       <c r="B202" s="14"/>
       <c r="C202" s="14"/>
@@ -6006,7 +6030,7 @@
       <c r="M202" s="16"/>
       <c r="N202" s="17"/>
     </row>
-    <row r="203" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A203" s="13"/>
       <c r="B203" s="14"/>
       <c r="C203" s="14"/>
@@ -6028,7 +6052,7 @@
       <c r="M203" s="16"/>
       <c r="N203" s="17"/>
     </row>
-    <row r="204" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A204" s="13"/>
       <c r="B204" s="14"/>
       <c r="C204" s="14"/>
@@ -6050,7 +6074,7 @@
       <c r="M204" s="16"/>
       <c r="N204" s="17"/>
     </row>
-    <row r="205" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A205" s="13"/>
       <c r="B205" s="14"/>
       <c r="C205" s="14"/>
@@ -6072,7 +6096,7 @@
       <c r="M205" s="16"/>
       <c r="N205" s="17"/>
     </row>
-    <row r="206" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A206" s="13"/>
       <c r="B206" s="14"/>
       <c r="C206" s="14"/>
@@ -6094,7 +6118,7 @@
       <c r="M206" s="16"/>
       <c r="N206" s="17"/>
     </row>
-    <row r="207" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A207" s="13"/>
       <c r="B207" s="14"/>
       <c r="C207" s="14"/>
@@ -6116,7 +6140,7 @@
       <c r="M207" s="16"/>
       <c r="N207" s="17"/>
     </row>
-    <row r="208" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A208" s="13"/>
       <c r="B208" s="14"/>
       <c r="C208" s="14"/>
@@ -6138,7 +6162,7 @@
       <c r="M208" s="16"/>
       <c r="N208" s="17"/>
     </row>
-    <row r="209" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A209" s="13"/>
       <c r="B209" s="14"/>
       <c r="C209" s="14"/>
@@ -6160,7 +6184,7 @@
       <c r="M209" s="16"/>
       <c r="N209" s="17"/>
     </row>
-    <row r="210" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A210" s="13"/>
       <c r="B210" s="14"/>
       <c r="C210" s="14"/>
@@ -6182,7 +6206,7 @@
       <c r="M210" s="16"/>
       <c r="N210" s="17"/>
     </row>
-    <row r="211" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A211" s="13"/>
       <c r="B211" s="14"/>
       <c r="C211" s="14"/>
@@ -6204,7 +6228,7 @@
       <c r="M211" s="16"/>
       <c r="N211" s="17"/>
     </row>
-    <row r="212" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A212" s="13"/>
       <c r="B212" s="14"/>
       <c r="C212" s="14"/>
@@ -6226,7 +6250,7 @@
       <c r="M212" s="16"/>
       <c r="N212" s="17"/>
     </row>
-    <row r="213" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A213" s="13"/>
       <c r="B213" s="14"/>
       <c r="C213" s="14"/>
@@ -6248,7 +6272,7 @@
       <c r="M213" s="16"/>
       <c r="N213" s="17"/>
     </row>
-    <row r="214" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A214" s="13"/>
       <c r="B214" s="14"/>
       <c r="C214" s="14"/>
@@ -6270,7 +6294,7 @@
       <c r="M214" s="16"/>
       <c r="N214" s="17"/>
     </row>
-    <row r="215" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A215" s="13"/>
       <c r="B215" s="14"/>
       <c r="C215" s="14"/>
@@ -6292,7 +6316,7 @@
       <c r="M215" s="16"/>
       <c r="N215" s="17"/>
     </row>
-    <row r="216" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A216" s="13"/>
       <c r="B216" s="14"/>
       <c r="C216" s="14"/>
@@ -6314,7 +6338,7 @@
       <c r="M216" s="16"/>
       <c r="N216" s="17"/>
     </row>
-    <row r="217" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A217" s="13"/>
       <c r="B217" s="14"/>
       <c r="C217" s="14"/>
@@ -6336,7 +6360,7 @@
       <c r="M217" s="16"/>
       <c r="N217" s="17"/>
     </row>
-    <row r="218" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A218" s="13"/>
       <c r="B218" s="14"/>
       <c r="C218" s="14"/>
@@ -6358,7 +6382,7 @@
       <c r="M218" s="16"/>
       <c r="N218" s="17"/>
     </row>
-    <row r="219" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A219" s="13"/>
       <c r="B219" s="14"/>
       <c r="C219" s="14"/>
@@ -6380,7 +6404,7 @@
       <c r="M219" s="16"/>
       <c r="N219" s="17"/>
     </row>
-    <row r="220" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A220" s="13"/>
       <c r="B220" s="14"/>
       <c r="C220" s="14"/>
@@ -6402,7 +6426,7 @@
       <c r="M220" s="16"/>
       <c r="N220" s="17"/>
     </row>
-    <row r="221" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A221" s="13"/>
       <c r="B221" s="14"/>
       <c r="C221" s="14"/>
@@ -6424,7 +6448,7 @@
       <c r="M221" s="16"/>
       <c r="N221" s="17"/>
     </row>
-    <row r="222" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A222" s="13"/>
       <c r="B222" s="14"/>
       <c r="C222" s="14"/>
@@ -6446,7 +6470,7 @@
       <c r="M222" s="16"/>
       <c r="N222" s="17"/>
     </row>
-    <row r="223" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A223" s="13"/>
       <c r="B223" s="14"/>
       <c r="C223" s="14"/>
@@ -6468,7 +6492,7 @@
       <c r="M223" s="16"/>
       <c r="N223" s="17"/>
     </row>
-    <row r="224" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A224" s="13"/>
       <c r="B224" s="14"/>
       <c r="C224" s="14"/>
@@ -6490,7 +6514,7 @@
       <c r="M224" s="16"/>
       <c r="N224" s="17"/>
     </row>
-    <row r="225" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A225" s="13"/>
       <c r="B225" s="14"/>
       <c r="C225" s="14"/>
@@ -6512,7 +6536,7 @@
       <c r="M225" s="16"/>
       <c r="N225" s="17"/>
     </row>
-    <row r="226" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A226" s="13"/>
       <c r="B226" s="14"/>
       <c r="C226" s="14"/>
@@ -6534,7 +6558,7 @@
       <c r="M226" s="16"/>
       <c r="N226" s="17"/>
     </row>
-    <row r="227" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A227" s="13"/>
       <c r="B227" s="14"/>
       <c r="C227" s="14"/>
@@ -6556,7 +6580,7 @@
       <c r="M227" s="16"/>
       <c r="N227" s="17"/>
     </row>
-    <row r="228" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A228" s="13"/>
       <c r="B228" s="14"/>
       <c r="C228" s="14"/>
@@ -6578,7 +6602,7 @@
       <c r="M228" s="16"/>
       <c r="N228" s="17"/>
     </row>
-    <row r="229" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A229" s="13"/>
       <c r="B229" s="14"/>
       <c r="C229" s="14"/>
@@ -6600,7 +6624,7 @@
       <c r="M229" s="16"/>
       <c r="N229" s="17"/>
     </row>
-    <row r="230" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A230" s="13"/>
       <c r="B230" s="14"/>
       <c r="C230" s="14"/>
@@ -6622,7 +6646,7 @@
       <c r="M230" s="16"/>
       <c r="N230" s="17"/>
     </row>
-    <row r="231" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A231" s="13"/>
       <c r="B231" s="14"/>
       <c r="C231" s="14"/>
@@ -6644,7 +6668,7 @@
       <c r="M231" s="16"/>
       <c r="N231" s="17"/>
     </row>
-    <row r="232" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A232" s="13"/>
       <c r="B232" s="14"/>
       <c r="C232" s="14"/>
@@ -6666,7 +6690,7 @@
       <c r="M232" s="16"/>
       <c r="N232" s="17"/>
     </row>
-    <row r="233" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A233" s="13"/>
       <c r="B233" s="14"/>
       <c r="C233" s="14"/>
@@ -6688,7 +6712,7 @@
       <c r="M233" s="16"/>
       <c r="N233" s="17"/>
     </row>
-    <row r="234" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A234" s="13"/>
       <c r="B234" s="14"/>
       <c r="C234" s="14"/>
@@ -6710,7 +6734,7 @@
       <c r="M234" s="16"/>
       <c r="N234" s="17"/>
     </row>
-    <row r="235" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A235" s="13"/>
       <c r="B235" s="14"/>
       <c r="C235" s="14"/>
@@ -6732,7 +6756,7 @@
       <c r="M235" s="16"/>
       <c r="N235" s="17"/>
     </row>
-    <row r="236" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A236" s="13"/>
       <c r="B236" s="14"/>
       <c r="C236" s="14"/>
@@ -6754,7 +6778,7 @@
       <c r="M236" s="16"/>
       <c r="N236" s="17"/>
     </row>
-    <row r="237" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A237" s="13"/>
       <c r="B237" s="14"/>
       <c r="C237" s="14"/>
@@ -6776,7 +6800,7 @@
       <c r="M237" s="16"/>
       <c r="N237" s="17"/>
     </row>
-    <row r="238" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A238" s="13"/>
       <c r="B238" s="14"/>
       <c r="C238" s="14"/>
@@ -6798,7 +6822,7 @@
       <c r="M238" s="16"/>
       <c r="N238" s="17"/>
     </row>
-    <row r="239" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A239" s="13"/>
       <c r="B239" s="14"/>
       <c r="C239" s="14"/>
@@ -6820,7 +6844,7 @@
       <c r="M239" s="16"/>
       <c r="N239" s="17"/>
     </row>
-    <row r="240" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A240" s="13"/>
       <c r="B240" s="14"/>
       <c r="C240" s="14"/>
@@ -6842,7 +6866,7 @@
       <c r="M240" s="16"/>
       <c r="N240" s="17"/>
     </row>
-    <row r="241" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A241" s="13"/>
       <c r="B241" s="14"/>
       <c r="C241" s="14"/>
@@ -6864,7 +6888,7 @@
       <c r="M241" s="16"/>
       <c r="N241" s="17"/>
     </row>
-    <row r="242" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A242" s="13"/>
       <c r="B242" s="14"/>
       <c r="C242" s="14"/>
@@ -6886,7 +6910,7 @@
       <c r="M242" s="16"/>
       <c r="N242" s="17"/>
     </row>
-    <row r="243" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A243" s="13"/>
       <c r="B243" s="14"/>
       <c r="C243" s="14"/>
@@ -6908,7 +6932,7 @@
       <c r="M243" s="16"/>
       <c r="N243" s="17"/>
     </row>
-    <row r="244" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A244" s="13"/>
       <c r="B244" s="14"/>
       <c r="C244" s="14"/>
@@ -6930,7 +6954,7 @@
       <c r="M244" s="16"/>
       <c r="N244" s="17"/>
     </row>
-    <row r="245" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A245" s="13"/>
       <c r="B245" s="14"/>
       <c r="C245" s="14"/>
@@ -6952,7 +6976,7 @@
       <c r="M245" s="16"/>
       <c r="N245" s="17"/>
     </row>
-    <row r="246" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A246" s="13"/>
       <c r="B246" s="14"/>
       <c r="C246" s="14"/>
@@ -6974,7 +6998,7 @@
       <c r="M246" s="16"/>
       <c r="N246" s="17"/>
     </row>
-    <row r="247" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A247" s="13"/>
       <c r="B247" s="14"/>
       <c r="C247" s="14"/>
@@ -6996,7 +7020,7 @@
       <c r="M247" s="16"/>
       <c r="N247" s="17"/>
     </row>
-    <row r="248" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A248" s="13"/>
       <c r="B248" s="14"/>
       <c r="C248" s="14"/>
@@ -7018,7 +7042,7 @@
       <c r="M248" s="16"/>
       <c r="N248" s="17"/>
     </row>
-    <row r="249" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A249" s="13"/>
       <c r="B249" s="14"/>
       <c r="C249" s="14"/>
@@ -7040,7 +7064,7 @@
       <c r="M249" s="16"/>
       <c r="N249" s="17"/>
     </row>
-    <row r="250" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A250" s="13"/>
       <c r="B250" s="14"/>
       <c r="C250" s="14"/>
@@ -7062,7 +7086,7 @@
       <c r="M250" s="16"/>
       <c r="N250" s="17"/>
     </row>
-    <row r="251" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A251" s="13"/>
       <c r="B251" s="14"/>
       <c r="C251" s="14"/>
@@ -7084,7 +7108,7 @@
       <c r="M251" s="16"/>
       <c r="N251" s="17"/>
     </row>
-    <row r="252" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A252" s="13"/>
       <c r="B252" s="14"/>
       <c r="C252" s="14"/>
@@ -7106,7 +7130,7 @@
       <c r="M252" s="16"/>
       <c r="N252" s="17"/>
     </row>
-    <row r="253" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A253" s="13"/>
       <c r="B253" s="14"/>
       <c r="C253" s="14"/>
@@ -7128,7 +7152,7 @@
       <c r="M253" s="16"/>
       <c r="N253" s="17"/>
     </row>
-    <row r="254" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A254" s="13"/>
       <c r="B254" s="14"/>
       <c r="C254" s="14"/>
@@ -7150,7 +7174,7 @@
       <c r="M254" s="16"/>
       <c r="N254" s="17"/>
     </row>
-    <row r="255" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A255" s="13"/>
       <c r="B255" s="14"/>
       <c r="C255" s="14"/>
@@ -7172,7 +7196,7 @@
       <c r="M255" s="16"/>
       <c r="N255" s="17"/>
     </row>
-    <row r="256" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A256" s="13"/>
       <c r="B256" s="14"/>
       <c r="C256" s="14"/>
@@ -7194,7 +7218,7 @@
       <c r="M256" s="16"/>
       <c r="N256" s="17"/>
     </row>
-    <row r="257" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A257" s="13"/>
       <c r="B257" s="14"/>
       <c r="C257" s="14"/>
@@ -7216,7 +7240,7 @@
       <c r="M257" s="16"/>
       <c r="N257" s="17"/>
     </row>
-    <row r="258" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A258" s="13"/>
       <c r="B258" s="14"/>
       <c r="C258" s="14"/>
@@ -7238,7 +7262,7 @@
       <c r="M258" s="16"/>
       <c r="N258" s="17"/>
     </row>
-    <row r="259" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A259" s="13"/>
       <c r="B259" s="14"/>
       <c r="C259" s="14"/>
@@ -7260,7 +7284,7 @@
       <c r="M259" s="16"/>
       <c r="N259" s="17"/>
     </row>
-    <row r="260" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A260" s="13"/>
       <c r="B260" s="14"/>
       <c r="C260" s="14"/>
@@ -7282,7 +7306,7 @@
       <c r="M260" s="16"/>
       <c r="N260" s="17"/>
     </row>
-    <row r="261" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A261" s="13"/>
       <c r="B261" s="14"/>
       <c r="C261" s="14"/>
@@ -7304,7 +7328,7 @@
       <c r="M261" s="16"/>
       <c r="N261" s="17"/>
     </row>
-    <row r="262" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A262" s="13"/>
       <c r="B262" s="14"/>
       <c r="C262" s="14"/>
@@ -7326,7 +7350,7 @@
       <c r="M262" s="16"/>
       <c r="N262" s="17"/>
     </row>
-    <row r="263" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A263" s="13"/>
       <c r="B263" s="14"/>
       <c r="C263" s="14"/>
@@ -7348,7 +7372,7 @@
       <c r="M263" s="16"/>
       <c r="N263" s="17"/>
     </row>
-    <row r="264" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A264" s="13"/>
       <c r="B264" s="14"/>
       <c r="C264" s="14"/>
@@ -7370,7 +7394,7 @@
       <c r="M264" s="16"/>
       <c r="N264" s="17"/>
     </row>
-    <row r="265" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A265" s="13"/>
       <c r="B265" s="14"/>
       <c r="C265" s="14"/>
@@ -7392,7 +7416,7 @@
       <c r="M265" s="16"/>
       <c r="N265" s="17"/>
     </row>
-    <row r="266" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A266" s="13"/>
       <c r="B266" s="14"/>
       <c r="C266" s="14"/>
@@ -7414,7 +7438,7 @@
       <c r="M266" s="16"/>
       <c r="N266" s="17"/>
     </row>
-    <row r="267" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A267" s="13"/>
       <c r="B267" s="14"/>
       <c r="C267" s="14"/>
@@ -7436,7 +7460,7 @@
       <c r="M267" s="16"/>
       <c r="N267" s="17"/>
     </row>
-    <row r="268" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A268" s="13"/>
       <c r="B268" s="14"/>
       <c r="C268" s="14"/>
@@ -7458,7 +7482,7 @@
       <c r="M268" s="16"/>
       <c r="N268" s="17"/>
     </row>
-    <row r="269" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A269" s="13"/>
       <c r="B269" s="14"/>
       <c r="C269" s="14"/>
@@ -7480,7 +7504,7 @@
       <c r="M269" s="16"/>
       <c r="N269" s="17"/>
     </row>
-    <row r="270" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A270" s="13"/>
       <c r="B270" s="14"/>
       <c r="C270" s="14"/>
@@ -7502,7 +7526,7 @@
       <c r="M270" s="16"/>
       <c r="N270" s="17"/>
     </row>
-    <row r="271" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A271" s="13"/>
       <c r="B271" s="14"/>
       <c r="C271" s="14"/>
@@ -7524,7 +7548,7 @@
       <c r="M271" s="16"/>
       <c r="N271" s="17"/>
     </row>
-    <row r="272" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A272" s="13"/>
       <c r="B272" s="14"/>
       <c r="C272" s="14"/>
@@ -7546,7 +7570,7 @@
       <c r="M272" s="16"/>
       <c r="N272" s="17"/>
     </row>
-    <row r="273" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A273" s="13"/>
       <c r="B273" s="14"/>
       <c r="C273" s="14"/>
@@ -7568,7 +7592,7 @@
       <c r="M273" s="16"/>
       <c r="N273" s="17"/>
     </row>
-    <row r="274" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A274" s="13"/>
       <c r="B274" s="14"/>
       <c r="C274" s="14"/>
@@ -7590,7 +7614,7 @@
       <c r="M274" s="16"/>
       <c r="N274" s="17"/>
     </row>
-    <row r="275" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A275" s="13"/>
       <c r="B275" s="14"/>
       <c r="C275" s="14"/>
@@ -7612,7 +7636,7 @@
       <c r="M275" s="16"/>
       <c r="N275" s="17"/>
     </row>
-    <row r="276" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A276" s="13"/>
       <c r="B276" s="14"/>
       <c r="C276" s="14"/>
@@ -7634,7 +7658,7 @@
       <c r="M276" s="16"/>
       <c r="N276" s="17"/>
     </row>
-    <row r="277" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A277" s="13"/>
       <c r="B277" s="14"/>
       <c r="C277" s="14"/>
@@ -7656,7 +7680,7 @@
       <c r="M277" s="16"/>
       <c r="N277" s="17"/>
     </row>
-    <row r="278" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A278" s="13"/>
       <c r="B278" s="14"/>
       <c r="C278" s="14"/>
@@ -7678,7 +7702,7 @@
       <c r="M278" s="16"/>
       <c r="N278" s="17"/>
     </row>
-    <row r="279" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A279" s="13"/>
       <c r="B279" s="14"/>
       <c r="C279" s="14"/>
@@ -7700,7 +7724,7 @@
       <c r="M279" s="16"/>
       <c r="N279" s="17"/>
     </row>
-    <row r="280" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A280" s="13"/>
       <c r="B280" s="14"/>
       <c r="C280" s="14"/>
@@ -7722,7 +7746,7 @@
       <c r="M280" s="16"/>
       <c r="N280" s="17"/>
     </row>
-    <row r="281" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A281" s="13"/>
       <c r="B281" s="14"/>
       <c r="C281" s="14"/>
@@ -7744,7 +7768,7 @@
       <c r="M281" s="16"/>
       <c r="N281" s="17"/>
     </row>
-    <row r="282" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A282" s="13"/>
       <c r="B282" s="14"/>
       <c r="C282" s="14"/>
@@ -7766,7 +7790,7 @@
       <c r="M282" s="16"/>
       <c r="N282" s="17"/>
     </row>
-    <row r="283" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A283" s="13"/>
       <c r="B283" s="14"/>
       <c r="C283" s="14"/>
@@ -7788,7 +7812,7 @@
       <c r="M283" s="16"/>
       <c r="N283" s="17"/>
     </row>
-    <row r="284" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A284" s="13"/>
       <c r="B284" s="14"/>
       <c r="C284" s="14"/>
@@ -7810,7 +7834,7 @@
       <c r="M284" s="16"/>
       <c r="N284" s="17"/>
     </row>
-    <row r="285" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A285" s="13"/>
       <c r="B285" s="14"/>
       <c r="C285" s="14"/>
@@ -7832,7 +7856,7 @@
       <c r="M285" s="16"/>
       <c r="N285" s="17"/>
     </row>
-    <row r="286" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A286" s="13"/>
       <c r="B286" s="14"/>
       <c r="C286" s="14"/>
@@ -7854,7 +7878,7 @@
       <c r="M286" s="16"/>
       <c r="N286" s="17"/>
     </row>
-    <row r="287" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A287" s="13"/>
       <c r="B287" s="14"/>
       <c r="C287" s="14"/>
@@ -7876,7 +7900,7 @@
       <c r="M287" s="16"/>
       <c r="N287" s="17"/>
     </row>
-    <row r="288" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A288" s="13"/>
       <c r="B288" s="14"/>
       <c r="C288" s="14"/>
@@ -7898,7 +7922,7 @@
       <c r="M288" s="16"/>
       <c r="N288" s="17"/>
     </row>
-    <row r="289" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A289" s="13"/>
       <c r="B289" s="14"/>
       <c r="C289" s="14"/>
@@ -7920,7 +7944,7 @@
       <c r="M289" s="16"/>
       <c r="N289" s="17"/>
     </row>
-    <row r="290" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A290" s="13"/>
       <c r="B290" s="14"/>
       <c r="C290" s="14"/>
@@ -7942,7 +7966,7 @@
       <c r="M290" s="16"/>
       <c r="N290" s="17"/>
     </row>
-    <row r="291" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A291" s="13"/>
       <c r="B291" s="14"/>
       <c r="C291" s="14"/>
@@ -7964,7 +7988,7 @@
       <c r="M291" s="16"/>
       <c r="N291" s="17"/>
     </row>
-    <row r="292" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A292" s="13"/>
       <c r="B292" s="14"/>
       <c r="C292" s="14"/>
@@ -7986,7 +8010,7 @@
       <c r="M292" s="16"/>
       <c r="N292" s="17"/>
     </row>
-    <row r="293" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A293" s="13"/>
       <c r="B293" s="14"/>
       <c r="C293" s="14"/>
@@ -8008,7 +8032,7 @@
       <c r="M293" s="16"/>
       <c r="N293" s="17"/>
     </row>
-    <row r="294" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A294" s="13"/>
       <c r="B294" s="14"/>
       <c r="C294" s="14"/>
@@ -8030,7 +8054,7 @@
       <c r="M294" s="16"/>
       <c r="N294" s="17"/>
     </row>
-    <row r="295" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A295" s="13"/>
       <c r="B295" s="14"/>
       <c r="C295" s="14"/>
@@ -8052,7 +8076,7 @@
       <c r="M295" s="16"/>
       <c r="N295" s="17"/>
     </row>
-    <row r="296" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A296" s="13"/>
       <c r="B296" s="14"/>
       <c r="C296" s="14"/>
@@ -8074,7 +8098,7 @@
       <c r="M296" s="16"/>
       <c r="N296" s="17"/>
     </row>
-    <row r="297" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A297" s="13"/>
       <c r="B297" s="14"/>
       <c r="C297" s="14"/>
@@ -8096,7 +8120,7 @@
       <c r="M297" s="16"/>
       <c r="N297" s="17"/>
     </row>
-    <row r="298" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A298" s="13"/>
       <c r="B298" s="14"/>
       <c r="C298" s="14"/>
@@ -8118,7 +8142,7 @@
       <c r="M298" s="16"/>
       <c r="N298" s="17"/>
     </row>
-    <row r="299" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A299" s="13"/>
       <c r="B299" s="14"/>
       <c r="C299" s="14"/>
@@ -8140,7 +8164,7 @@
       <c r="M299" s="16"/>
       <c r="N299" s="17"/>
     </row>
-    <row r="300" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A300" s="13"/>
       <c r="B300" s="14"/>
       <c r="C300" s="14"/>
@@ -8162,7 +8186,7 @@
       <c r="M300" s="16"/>
       <c r="N300" s="17"/>
     </row>
-    <row r="301" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A301" s="13"/>
       <c r="B301" s="14"/>
       <c r="C301" s="14"/>
@@ -8184,7 +8208,7 @@
       <c r="M301" s="16"/>
       <c r="N301" s="17"/>
     </row>
-    <row r="302" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A302" s="13"/>
       <c r="B302" s="14"/>
       <c r="C302" s="14"/>
@@ -8206,7 +8230,7 @@
       <c r="M302" s="16"/>
       <c r="N302" s="17"/>
     </row>
-    <row r="303" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A303" s="13"/>
       <c r="B303" s="14"/>
       <c r="C303" s="14"/>
@@ -8228,7 +8252,7 @@
       <c r="M303" s="16"/>
       <c r="N303" s="17"/>
     </row>
-    <row r="304" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A304" s="13"/>
       <c r="B304" s="14"/>
       <c r="C304" s="14"/>
@@ -8250,7 +8274,7 @@
       <c r="M304" s="16"/>
       <c r="N304" s="17"/>
     </row>
-    <row r="305" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A305" s="13"/>
       <c r="B305" s="14"/>
       <c r="C305" s="14"/>
@@ -8272,7 +8296,7 @@
       <c r="M305" s="16"/>
       <c r="N305" s="17"/>
     </row>
-    <row r="306" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A306" s="13"/>
       <c r="B306" s="14"/>
       <c r="C306" s="14"/>
@@ -8294,7 +8318,7 @@
       <c r="M306" s="16"/>
       <c r="N306" s="17"/>
     </row>
-    <row r="307" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A307" s="13"/>
       <c r="B307" s="14"/>
       <c r="C307" s="14"/>
@@ -8316,7 +8340,7 @@
       <c r="M307" s="16"/>
       <c r="N307" s="17"/>
     </row>
-    <row r="308" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A308" s="13"/>
       <c r="B308" s="14"/>
       <c r="C308" s="14"/>
@@ -8338,7 +8362,7 @@
       <c r="M308" s="16"/>
       <c r="N308" s="17"/>
     </row>
-    <row r="309" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A309" s="13"/>
       <c r="B309" s="14"/>
       <c r="C309" s="14"/>
@@ -8360,7 +8384,7 @@
       <c r="M309" s="16"/>
       <c r="N309" s="17"/>
     </row>
-    <row r="310" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A310" s="13"/>
       <c r="B310" s="14"/>
       <c r="C310" s="14"/>
@@ -8382,7 +8406,7 @@
       <c r="M310" s="16"/>
       <c r="N310" s="17"/>
     </row>
-    <row r="311" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A311" s="13"/>
       <c r="B311" s="14"/>
       <c r="C311" s="14"/>
@@ -8404,7 +8428,7 @@
       <c r="M311" s="16"/>
       <c r="N311" s="17"/>
     </row>
-    <row r="312" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A312" s="13"/>
       <c r="B312" s="14"/>
       <c r="C312" s="14"/>
@@ -8426,7 +8450,7 @@
       <c r="M312" s="16"/>
       <c r="N312" s="17"/>
     </row>
-    <row r="313" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A313" s="13"/>
       <c r="B313" s="14"/>
       <c r="C313" s="14"/>
@@ -8448,7 +8472,7 @@
       <c r="M313" s="16"/>
       <c r="N313" s="17"/>
     </row>
-    <row r="314" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A314" s="13"/>
       <c r="B314" s="14"/>
       <c r="C314" s="14"/>
@@ -8470,7 +8494,7 @@
       <c r="M314" s="16"/>
       <c r="N314" s="17"/>
     </row>
-    <row r="315" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A315" s="13"/>
       <c r="B315" s="14"/>
       <c r="C315" s="14"/>
@@ -8492,7 +8516,7 @@
       <c r="M315" s="16"/>
       <c r="N315" s="17"/>
     </row>
-    <row r="316" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A316" s="13"/>
       <c r="B316" s="14"/>
       <c r="C316" s="14"/>
@@ -8514,7 +8538,7 @@
       <c r="M316" s="16"/>
       <c r="N316" s="17"/>
     </row>
-    <row r="317" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A317" s="13"/>
       <c r="B317" s="14"/>
       <c r="C317" s="14"/>
@@ -8536,7 +8560,7 @@
       <c r="M317" s="16"/>
       <c r="N317" s="17"/>
     </row>
-    <row r="318" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A318" s="13"/>
       <c r="B318" s="14"/>
       <c r="C318" s="14"/>
@@ -8558,7 +8582,7 @@
       <c r="M318" s="16"/>
       <c r="N318" s="17"/>
     </row>
-    <row r="319" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A319" s="13"/>
       <c r="B319" s="14"/>
       <c r="C319" s="14"/>
@@ -8580,7 +8604,7 @@
       <c r="M319" s="16"/>
       <c r="N319" s="17"/>
     </row>
-    <row r="320" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A320" s="13"/>
       <c r="B320" s="14"/>
       <c r="C320" s="14"/>
@@ -8602,7 +8626,7 @@
       <c r="M320" s="16"/>
       <c r="N320" s="17"/>
     </row>
-    <row r="321" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A321" s="13"/>
       <c r="B321" s="14"/>
       <c r="C321" s="14"/>
@@ -8624,7 +8648,7 @@
       <c r="M321" s="16"/>
       <c r="N321" s="17"/>
     </row>
-    <row r="322" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A322" s="13"/>
       <c r="B322" s="14"/>
       <c r="C322" s="14"/>
@@ -8646,7 +8670,7 @@
       <c r="M322" s="16"/>
       <c r="N322" s="17"/>
     </row>
-    <row r="323" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A323" s="13"/>
       <c r="B323" s="14"/>
       <c r="C323" s="14"/>
@@ -8668,7 +8692,7 @@
       <c r="M323" s="16"/>
       <c r="N323" s="17"/>
     </row>
-    <row r="324" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A324" s="13"/>
       <c r="B324" s="14"/>
       <c r="C324" s="14"/>
@@ -8690,7 +8714,7 @@
       <c r="M324" s="16"/>
       <c r="N324" s="17"/>
     </row>
-    <row r="325" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A325" s="13"/>
       <c r="B325" s="14"/>
       <c r="C325" s="14"/>
@@ -8712,7 +8736,7 @@
       <c r="M325" s="16"/>
       <c r="N325" s="17"/>
     </row>
-    <row r="326" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A326" s="13"/>
       <c r="B326" s="14"/>
       <c r="C326" s="14"/>
@@ -8734,7 +8758,7 @@
       <c r="M326" s="16"/>
       <c r="N326" s="17"/>
     </row>
-    <row r="327" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A327" s="13"/>
       <c r="B327" s="14"/>
       <c r="C327" s="14"/>
@@ -8756,7 +8780,7 @@
       <c r="M327" s="16"/>
       <c r="N327" s="17"/>
     </row>
-    <row r="328" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A328" s="13"/>
       <c r="B328" s="14"/>
       <c r="C328" s="14"/>
@@ -8778,7 +8802,7 @@
       <c r="M328" s="16"/>
       <c r="N328" s="17"/>
     </row>
-    <row r="329" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A329" s="13"/>
       <c r="B329" s="14"/>
       <c r="C329" s="14"/>
@@ -8800,7 +8824,7 @@
       <c r="M329" s="16"/>
       <c r="N329" s="17"/>
     </row>
-    <row r="330" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A330" s="13"/>
       <c r="B330" s="14"/>
       <c r="C330" s="14"/>
@@ -8822,7 +8846,7 @@
       <c r="M330" s="16"/>
       <c r="N330" s="17"/>
     </row>
-    <row r="331" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A331" s="13"/>
       <c r="B331" s="14"/>
       <c r="C331" s="14"/>
@@ -8844,7 +8868,7 @@
       <c r="M331" s="16"/>
       <c r="N331" s="17"/>
     </row>
-    <row r="332" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A332" s="13"/>
       <c r="B332" s="14"/>
       <c r="C332" s="14"/>
@@ -8866,7 +8890,7 @@
       <c r="M332" s="16"/>
       <c r="N332" s="17"/>
     </row>
-    <row r="333" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A333" s="13"/>
       <c r="B333" s="14"/>
       <c r="C333" s="14"/>
@@ -8888,7 +8912,7 @@
       <c r="M333" s="16"/>
       <c r="N333" s="17"/>
     </row>
-    <row r="334" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A334" s="13"/>
       <c r="B334" s="14"/>
       <c r="C334" s="14"/>
@@ -8910,7 +8934,7 @@
       <c r="M334" s="16"/>
       <c r="N334" s="17"/>
     </row>
-    <row r="335" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A335" s="13"/>
       <c r="B335" s="14"/>
       <c r="C335" s="14"/>
@@ -8932,7 +8956,7 @@
       <c r="M335" s="16"/>
       <c r="N335" s="17"/>
     </row>
-    <row r="336" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A336" s="13"/>
       <c r="B336" s="14"/>
       <c r="C336" s="14"/>
@@ -8954,7 +8978,7 @@
       <c r="M336" s="16"/>
       <c r="N336" s="17"/>
     </row>
-    <row r="337" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A337" s="13"/>
       <c r="B337" s="14"/>
       <c r="C337" s="14"/>
@@ -8976,7 +9000,7 @@
       <c r="M337" s="16"/>
       <c r="N337" s="17"/>
     </row>
-    <row r="338" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A338" s="13"/>
       <c r="B338" s="14"/>
       <c r="C338" s="14"/>
@@ -8998,7 +9022,7 @@
       <c r="M338" s="16"/>
       <c r="N338" s="17"/>
     </row>
-    <row r="339" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A339" s="13"/>
       <c r="B339" s="14"/>
       <c r="C339" s="14"/>
@@ -9020,7 +9044,7 @@
       <c r="M339" s="16"/>
       <c r="N339" s="17"/>
     </row>
-    <row r="340" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A340" s="13"/>
       <c r="B340" s="14"/>
       <c r="C340" s="14"/>
@@ -9042,7 +9066,7 @@
       <c r="M340" s="16"/>
       <c r="N340" s="17"/>
     </row>
-    <row r="341" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A341" s="13"/>
       <c r="B341" s="14"/>
       <c r="C341" s="14"/>
@@ -9064,7 +9088,7 @@
       <c r="M341" s="16"/>
       <c r="N341" s="17"/>
     </row>
-    <row r="342" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A342" s="13"/>
       <c r="B342" s="14"/>
       <c r="C342" s="14"/>
@@ -9086,7 +9110,7 @@
       <c r="M342" s="16"/>
       <c r="N342" s="17"/>
     </row>
-    <row r="343" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A343" s="13"/>
       <c r="B343" s="14"/>
       <c r="C343" s="14"/>
@@ -9108,7 +9132,7 @@
       <c r="M343" s="16"/>
       <c r="N343" s="17"/>
     </row>
-    <row r="344" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A344" s="13"/>
       <c r="B344" s="14"/>
       <c r="C344" s="14"/>
@@ -9130,7 +9154,7 @@
       <c r="M344" s="16"/>
       <c r="N344" s="17"/>
     </row>
-    <row r="345" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A345" s="13"/>
       <c r="B345" s="14"/>
       <c r="C345" s="14"/>
@@ -9152,7 +9176,7 @@
       <c r="M345" s="16"/>
       <c r="N345" s="17"/>
     </row>
-    <row r="346" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A346" s="13"/>
       <c r="B346" s="14"/>
       <c r="C346" s="14"/>
@@ -9174,7 +9198,7 @@
       <c r="M346" s="16"/>
       <c r="N346" s="17"/>
     </row>
-    <row r="347" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A347" s="13"/>
       <c r="B347" s="14"/>
       <c r="C347" s="14"/>
@@ -9196,7 +9220,7 @@
       <c r="M347" s="16"/>
       <c r="N347" s="17"/>
     </row>
-    <row r="348" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A348" s="13"/>
       <c r="B348" s="14"/>
       <c r="C348" s="14"/>
@@ -9218,7 +9242,7 @@
       <c r="M348" s="16"/>
       <c r="N348" s="17"/>
     </row>
-    <row r="349" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A349" s="13"/>
       <c r="B349" s="14"/>
       <c r="C349" s="14"/>
@@ -9240,7 +9264,7 @@
       <c r="M349" s="16"/>
       <c r="N349" s="17"/>
     </row>
-    <row r="350" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A350" s="13"/>
       <c r="B350" s="14"/>
       <c r="C350" s="14"/>
@@ -9262,7 +9286,7 @@
       <c r="M350" s="16"/>
       <c r="N350" s="17"/>
     </row>
-    <row r="351" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A351" s="13"/>
       <c r="B351" s="14"/>
       <c r="C351" s="14"/>
@@ -9284,7 +9308,7 @@
       <c r="M351" s="16"/>
       <c r="N351" s="17"/>
     </row>
-    <row r="352" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A352" s="13"/>
       <c r="B352" s="14"/>
       <c r="C352" s="14"/>
@@ -9306,7 +9330,7 @@
       <c r="M352" s="16"/>
       <c r="N352" s="17"/>
     </row>
-    <row r="353" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A353" s="13"/>
       <c r="B353" s="14"/>
       <c r="C353" s="14"/>
@@ -9328,7 +9352,7 @@
       <c r="M353" s="16"/>
       <c r="N353" s="17"/>
     </row>
-    <row r="354" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A354" s="13"/>
       <c r="B354" s="14"/>
       <c r="C354" s="14"/>
@@ -9350,7 +9374,7 @@
       <c r="M354" s="16"/>
       <c r="N354" s="17"/>
     </row>
-    <row r="355" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A355" s="13"/>
       <c r="B355" s="14"/>
       <c r="C355" s="14"/>
@@ -9372,7 +9396,7 @@
       <c r="M355" s="16"/>
       <c r="N355" s="17"/>
     </row>
-    <row r="356" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A356" s="13"/>
       <c r="B356" s="14"/>
       <c r="C356" s="14"/>
@@ -9394,7 +9418,7 @@
       <c r="M356" s="16"/>
       <c r="N356" s="17"/>
     </row>
-    <row r="357" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A357" s="13"/>
       <c r="B357" s="14"/>
       <c r="C357" s="14"/>
@@ -9416,7 +9440,7 @@
       <c r="M357" s="16"/>
       <c r="N357" s="17"/>
     </row>
-    <row r="358" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A358" s="13"/>
       <c r="B358" s="14"/>
       <c r="C358" s="14"/>
@@ -9438,7 +9462,7 @@
       <c r="M358" s="16"/>
       <c r="N358" s="17"/>
     </row>
-    <row r="359" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A359" s="13"/>
       <c r="B359" s="14"/>
       <c r="C359" s="14"/>
@@ -9460,7 +9484,7 @@
       <c r="M359" s="16"/>
       <c r="N359" s="17"/>
     </row>
-    <row r="360" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A360" s="13"/>
       <c r="B360" s="14"/>
       <c r="C360" s="14"/>
@@ -9482,7 +9506,7 @@
       <c r="M360" s="16"/>
       <c r="N360" s="17"/>
     </row>
-    <row r="361" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A361" s="13"/>
       <c r="B361" s="14"/>
       <c r="C361" s="14"/>
@@ -9504,7 +9528,7 @@
       <c r="M361" s="16"/>
       <c r="N361" s="17"/>
     </row>
-    <row r="362" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A362" s="13"/>
       <c r="B362" s="14"/>
       <c r="C362" s="14"/>
@@ -9526,7 +9550,7 @@
       <c r="M362" s="16"/>
       <c r="N362" s="17"/>
     </row>
-    <row r="363" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A363" s="13"/>
       <c r="B363" s="14"/>
       <c r="C363" s="14"/>
@@ -9548,7 +9572,7 @@
       <c r="M363" s="16"/>
       <c r="N363" s="17"/>
     </row>
-    <row r="364" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A364" s="13"/>
       <c r="B364" s="14"/>
       <c r="C364" s="14"/>
@@ -9570,7 +9594,7 @@
       <c r="M364" s="16"/>
       <c r="N364" s="17"/>
     </row>
-    <row r="365" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A365" s="13"/>
       <c r="B365" s="14"/>
       <c r="C365" s="14"/>
@@ -9592,7 +9616,7 @@
       <c r="M365" s="16"/>
       <c r="N365" s="17"/>
     </row>
-    <row r="366" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A366" s="13"/>
       <c r="B366" s="14"/>
       <c r="C366" s="14"/>
@@ -9614,7 +9638,7 @@
       <c r="M366" s="16"/>
       <c r="N366" s="17"/>
     </row>
-    <row r="367" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A367" s="13"/>
       <c r="B367" s="14"/>
       <c r="C367" s="14"/>
@@ -9636,7 +9660,7 @@
       <c r="M367" s="16"/>
       <c r="N367" s="17"/>
     </row>
-    <row r="368" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A368" s="13"/>
       <c r="B368" s="14"/>
       <c r="C368" s="14"/>
@@ -9658,7 +9682,7 @@
       <c r="M368" s="16"/>
       <c r="N368" s="17"/>
     </row>
-    <row r="369" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A369" s="13"/>
       <c r="B369" s="14"/>
       <c r="C369" s="14"/>
@@ -9680,7 +9704,7 @@
       <c r="M369" s="16"/>
       <c r="N369" s="17"/>
     </row>
-    <row r="370" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A370" s="13"/>
       <c r="B370" s="14"/>
       <c r="C370" s="14"/>
@@ -9702,7 +9726,7 @@
       <c r="M370" s="16"/>
       <c r="N370" s="17"/>
     </row>
-    <row r="371" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A371" s="13"/>
       <c r="B371" s="14"/>
       <c r="C371" s="14"/>
@@ -9724,7 +9748,7 @@
       <c r="M371" s="16"/>
       <c r="N371" s="17"/>
     </row>
-    <row r="372" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A372" s="13"/>
       <c r="B372" s="14"/>
       <c r="C372" s="14"/>
@@ -9746,7 +9770,7 @@
       <c r="M372" s="16"/>
       <c r="N372" s="17"/>
     </row>
-    <row r="373" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A373" s="13"/>
       <c r="B373" s="14"/>
       <c r="C373" s="14"/>
@@ -9768,7 +9792,7 @@
       <c r="M373" s="16"/>
       <c r="N373" s="17"/>
     </row>
-    <row r="374" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A374" s="13"/>
       <c r="B374" s="14"/>
       <c r="C374" s="14"/>
@@ -9790,7 +9814,7 @@
       <c r="M374" s="16"/>
       <c r="N374" s="17"/>
     </row>
-    <row r="375" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A375" s="13"/>
       <c r="B375" s="14"/>
       <c r="C375" s="14"/>
@@ -9812,7 +9836,7 @@
       <c r="M375" s="16"/>
       <c r="N375" s="17"/>
     </row>
-    <row r="376" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A376" s="13"/>
       <c r="B376" s="14"/>
       <c r="C376" s="14"/>
@@ -9834,7 +9858,7 @@
       <c r="M376" s="16"/>
       <c r="N376" s="17"/>
     </row>
-    <row r="377" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A377" s="13"/>
       <c r="B377" s="14"/>
       <c r="C377" s="14"/>
@@ -9856,7 +9880,7 @@
       <c r="M377" s="16"/>
       <c r="N377" s="17"/>
     </row>
-    <row r="378" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A378" s="13"/>
       <c r="B378" s="14"/>
       <c r="C378" s="14"/>
@@ -9878,7 +9902,7 @@
       <c r="M378" s="16"/>
       <c r="N378" s="17"/>
     </row>
-    <row r="379" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A379" s="13"/>
       <c r="B379" s="14"/>
       <c r="C379" s="14"/>
@@ -9900,7 +9924,7 @@
       <c r="M379" s="16"/>
       <c r="N379" s="17"/>
     </row>
-    <row r="380" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A380" s="13"/>
       <c r="B380" s="14"/>
       <c r="C380" s="14"/>
@@ -9922,7 +9946,7 @@
       <c r="M380" s="16"/>
       <c r="N380" s="17"/>
     </row>
-    <row r="381" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A381" s="13"/>
       <c r="B381" s="14"/>
       <c r="C381" s="14"/>
@@ -9944,7 +9968,7 @@
       <c r="M381" s="16"/>
       <c r="N381" s="17"/>
     </row>
-    <row r="382" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A382" s="13"/>
       <c r="B382" s="14"/>
       <c r="C382" s="14"/>
@@ -9966,7 +9990,7 @@
       <c r="M382" s="16"/>
       <c r="N382" s="17"/>
     </row>
-    <row r="383" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A383" s="13"/>
       <c r="B383" s="14"/>
       <c r="C383" s="14"/>
@@ -9988,7 +10012,7 @@
       <c r="M383" s="16"/>
       <c r="N383" s="17"/>
     </row>
-    <row r="384" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A384" s="13"/>
       <c r="B384" s="14"/>
       <c r="C384" s="14"/>
@@ -10010,7 +10034,7 @@
       <c r="M384" s="16"/>
       <c r="N384" s="17"/>
     </row>
-    <row r="385" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A385" s="13"/>
       <c r="B385" s="14"/>
       <c r="C385" s="14"/>
@@ -10032,7 +10056,7 @@
       <c r="M385" s="16"/>
       <c r="N385" s="17"/>
     </row>
-    <row r="386" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A386" s="13"/>
       <c r="B386" s="14"/>
       <c r="C386" s="14"/>
@@ -10054,7 +10078,7 @@
       <c r="M386" s="16"/>
       <c r="N386" s="17"/>
     </row>
-    <row r="387" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A387" s="13"/>
       <c r="B387" s="14"/>
       <c r="C387" s="14"/>
@@ -10076,7 +10100,7 @@
       <c r="M387" s="16"/>
       <c r="N387" s="17"/>
     </row>
-    <row r="388" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A388" s="13"/>
       <c r="B388" s="14"/>
       <c r="C388" s="14"/>
@@ -10098,7 +10122,7 @@
       <c r="M388" s="16"/>
       <c r="N388" s="17"/>
     </row>
-    <row r="389" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A389" s="13"/>
       <c r="B389" s="14"/>
       <c r="C389" s="14"/>
@@ -10120,7 +10144,7 @@
       <c r="M389" s="16"/>
       <c r="N389" s="17"/>
     </row>
-    <row r="390" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A390" s="13"/>
       <c r="B390" s="14"/>
       <c r="C390" s="14"/>
@@ -10142,7 +10166,7 @@
       <c r="M390" s="16"/>
       <c r="N390" s="17"/>
     </row>
-    <row r="391" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A391" s="13"/>
       <c r="B391" s="14"/>
       <c r="C391" s="14"/>
@@ -10164,7 +10188,7 @@
       <c r="M391" s="16"/>
       <c r="N391" s="17"/>
     </row>
-    <row r="392" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A392" s="13"/>
       <c r="B392" s="14"/>
       <c r="C392" s="14"/>
@@ -10186,7 +10210,7 @@
       <c r="M392" s="16"/>
       <c r="N392" s="17"/>
     </row>
-    <row r="393" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A393" s="13"/>
       <c r="B393" s="14"/>
       <c r="C393" s="14"/>
@@ -10208,7 +10232,7 @@
       <c r="M393" s="16"/>
       <c r="N393" s="17"/>
     </row>
-    <row r="394" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A394" s="13"/>
       <c r="B394" s="14"/>
       <c r="C394" s="14"/>
@@ -10230,7 +10254,7 @@
       <c r="M394" s="16"/>
       <c r="N394" s="17"/>
     </row>
-    <row r="395" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A395" s="13"/>
       <c r="B395" s="14"/>
       <c r="C395" s="14"/>
@@ -10252,7 +10276,7 @@
       <c r="M395" s="16"/>
       <c r="N395" s="17"/>
     </row>
-    <row r="396" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A396" s="13"/>
       <c r="B396" s="14"/>
       <c r="C396" s="14"/>
@@ -10274,7 +10298,7 @@
       <c r="M396" s="16"/>
       <c r="N396" s="17"/>
     </row>
-    <row r="397" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A397" s="13"/>
       <c r="B397" s="14"/>
       <c r="C397" s="14"/>
@@ -10296,7 +10320,7 @@
       <c r="M397" s="16"/>
       <c r="N397" s="17"/>
     </row>
-    <row r="398" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A398" s="13"/>
       <c r="B398" s="14"/>
       <c r="C398" s="14"/>
@@ -10318,7 +10342,7 @@
       <c r="M398" s="16"/>
       <c r="N398" s="17"/>
     </row>
-    <row r="399" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A399" s="13"/>
       <c r="B399" s="14"/>
       <c r="C399" s="14"/>
@@ -10340,7 +10364,7 @@
       <c r="M399" s="16"/>
       <c r="N399" s="17"/>
     </row>
-    <row r="400" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A400" s="13"/>
       <c r="B400" s="14"/>
       <c r="C400" s="14"/>
@@ -10362,7 +10386,7 @@
       <c r="M400" s="16"/>
       <c r="N400" s="17"/>
     </row>
-    <row r="401" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A401" s="13"/>
       <c r="B401" s="14"/>
       <c r="C401" s="14"/>

</xml_diff>

<commit_message>
File Updated on 15/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python\Project Data\776\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B104A31-AFE7-4D42-B8B3-616DE6A8EB6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FD7FDDB-CEA3-484C-A5B2-D44D18172ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="69">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -239,6 +239,9 @@
   </si>
   <si>
     <t>20266-09-07</t>
+  </si>
+  <si>
+    <t>Bad</t>
   </si>
 </sst>
 </file>
@@ -2291,26 +2294,50 @@
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="13"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="15" t="str">
+      <c r="A33" s="13">
+        <v>46280</v>
+      </c>
+      <c r="B33" s="14">
+        <v>420</v>
+      </c>
+      <c r="C33" s="14">
+        <v>0</v>
+      </c>
+      <c r="D33" s="14">
+        <v>150</v>
+      </c>
+      <c r="E33" s="14">
+        <v>30</v>
+      </c>
+      <c r="F33" s="14">
+        <v>400</v>
+      </c>
+      <c r="G33" s="14">
+        <v>8</v>
+      </c>
+      <c r="H33" s="14">
+        <v>50</v>
+      </c>
+      <c r="I33" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J33" s="15" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J33" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16"/>
-      <c r="M33" s="16"/>
-      <c r="N33" s="17"/>
+        <v>390</v>
+      </c>
+      <c r="K33" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="L33" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M33" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="N33" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="13"/>

</xml_diff>

<commit_message>
File Updated on 16/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FD7FDDB-CEA3-484C-A5B2-D44D18172ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B119B42D-0501-4E7B-9175-81ED1E612E44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="70">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -242,6 +242,9 @@
   </si>
   <si>
     <t>Bad</t>
+  </si>
+  <si>
+    <t>Sleepy all day</t>
   </si>
 </sst>
 </file>
@@ -2340,26 +2343,50 @@
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A34" s="13"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="15" t="str">
+      <c r="A34" s="13">
+        <v>46281</v>
+      </c>
+      <c r="B34" s="14">
+        <v>480</v>
+      </c>
+      <c r="C34" s="14">
+        <v>0</v>
+      </c>
+      <c r="D34" s="14">
+        <v>0</v>
+      </c>
+      <c r="E34" s="14">
+        <v>0</v>
+      </c>
+      <c r="F34" s="14">
+        <v>350</v>
+      </c>
+      <c r="G34" s="14">
+        <v>7</v>
+      </c>
+      <c r="H34" s="14">
+        <v>45</v>
+      </c>
+      <c r="I34" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J34" s="15" t="str">
+        <v>875</v>
+      </c>
+      <c r="J34" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
-      <c r="M34" s="16"/>
-      <c r="N34" s="17"/>
+        <v>565</v>
+      </c>
+      <c r="K34" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L34" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M34" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N34" s="17" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="13"/>

</xml_diff>

<commit_message>
File Updated on 19/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B119B42D-0501-4E7B-9175-81ED1E612E44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B4C92D-1A4C-4E14-8CCB-3CBDB488EA5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="612" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="70">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -193,9 +193,6 @@
     <t>D1P2632</t>
   </si>
   <si>
-    <t>August</t>
-  </si>
-  <si>
     <t>Low</t>
   </si>
   <si>
@@ -245,6 +242,9 @@
   </si>
   <si>
     <t>Sleepy all day</t>
+  </si>
+  <si>
+    <t>September</t>
   </si>
 </sst>
 </file>
@@ -989,7 +989,7 @@
         <v>33</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="G3" s="22"/>
     </row>
@@ -1088,16 +1088,16 @@
         <v>540</v>
       </c>
       <c r="K6" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="L6" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="M6" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="N6" s="12" t="s">
         <v>55</v>
-      </c>
-      <c r="L6" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="M6" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="N6" s="12" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -1134,16 +1134,16 @@
         <v>610</v>
       </c>
       <c r="K7" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L7" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M7" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="M7" s="16" t="s">
+      <c r="N7" s="17" t="s">
         <v>58</v>
-      </c>
-      <c r="N7" s="17" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
@@ -1180,16 +1180,16 @@
         <v>750</v>
       </c>
       <c r="K8" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N8" s="17" t="s">
         <v>60</v>
-      </c>
-      <c r="L8" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="M8" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="N8" s="17" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -1226,16 +1226,16 @@
         <v>660</v>
       </c>
       <c r="K9" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L9" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N9" s="17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1272,16 +1272,16 @@
         <v>675</v>
       </c>
       <c r="K10" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L10" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N10" s="17" t="s">
         <v>64</v>
-      </c>
-      <c r="L10" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="M10" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="N10" s="17" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1318,16 +1318,16 @@
         <v>600</v>
       </c>
       <c r="K11" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L11" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N11" s="17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -1364,16 +1364,16 @@
         <v>400</v>
       </c>
       <c r="K12" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L12" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M12" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N12" s="17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1410,16 +1410,16 @@
         <v>515</v>
       </c>
       <c r="K13" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L13" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M13" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N13" s="17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -1456,16 +1456,16 @@
         <v>430</v>
       </c>
       <c r="K14" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L14" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M14" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N14" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -1502,16 +1502,16 @@
         <v>690</v>
       </c>
       <c r="K15" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L15" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M15" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N15" s="17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1548,16 +1548,16 @@
         <v>620</v>
       </c>
       <c r="K16" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L16" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M16" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N16" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1594,16 +1594,16 @@
         <v>610</v>
       </c>
       <c r="K17" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L17" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M17" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N17" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
@@ -1640,16 +1640,16 @@
         <v>480</v>
       </c>
       <c r="K18" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L18" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M18" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N18" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
@@ -1686,16 +1686,16 @@
         <v>505</v>
       </c>
       <c r="K19" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L19" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M19" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N19" s="17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
@@ -1732,16 +1732,16 @@
         <v>520</v>
       </c>
       <c r="K20" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L20" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N20" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
@@ -1778,16 +1778,16 @@
         <v>610</v>
       </c>
       <c r="K21" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L21" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M21" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="M21" s="16" t="s">
-        <v>58</v>
-      </c>
       <c r="N21" s="17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
@@ -1824,16 +1824,16 @@
         <v>700</v>
       </c>
       <c r="K22" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L22" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M22" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N22" s="17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1870,16 +1870,16 @@
         <v>840</v>
       </c>
       <c r="K23" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L23" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M23" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N23" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1916,21 +1916,21 @@
         <v>660</v>
       </c>
       <c r="K24" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L24" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M24" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N24" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B25" s="14">
         <v>360</v>
@@ -1962,16 +1962,16 @@
         <v>680</v>
       </c>
       <c r="K25" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L25" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M25" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N25" s="17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
@@ -2008,16 +2008,16 @@
         <v>470</v>
       </c>
       <c r="K26" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L26" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M26" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N26" s="17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -2054,16 +2054,16 @@
         <v>625</v>
       </c>
       <c r="K27" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L27" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M27" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N27" s="17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
@@ -2100,16 +2100,16 @@
         <v>755</v>
       </c>
       <c r="K28" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L28" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M28" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N28" s="17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
@@ -2146,16 +2146,16 @@
         <v>795</v>
       </c>
       <c r="K29" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L29" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M29" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N29" s="17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
@@ -2192,16 +2192,16 @@
         <v>690</v>
       </c>
       <c r="K30" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L30" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M30" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N30" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
@@ -2238,16 +2238,16 @@
         <v>600</v>
       </c>
       <c r="K31" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L31" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M31" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N31" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
@@ -2284,16 +2284,16 @@
         <v>580</v>
       </c>
       <c r="K32" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L32" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M32" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N32" s="17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
@@ -2330,16 +2330,16 @@
         <v>390</v>
       </c>
       <c r="K33" s="16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="L33" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M33" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N33" s="17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
@@ -2376,83 +2376,155 @@
         <v>565</v>
       </c>
       <c r="K34" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L34" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M34" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N34" s="17" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A35" s="13">
+        <v>46282</v>
+      </c>
+      <c r="B35" s="14">
+        <v>480</v>
+      </c>
+      <c r="C35" s="14">
+        <v>0</v>
+      </c>
+      <c r="D35" s="14">
+        <v>120</v>
+      </c>
+      <c r="E35" s="14">
+        <v>0</v>
+      </c>
+      <c r="F35" s="14">
+        <v>150</v>
+      </c>
+      <c r="G35" s="14">
+        <v>3</v>
+      </c>
+      <c r="H35" s="14">
+        <v>70</v>
+      </c>
+      <c r="I35" s="15">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J35" s="15">
+        <f t="shared" si="1"/>
+        <v>620</v>
+      </c>
+      <c r="K35" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="M34" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="N34" s="17" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="13"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="15" t="str">
+      <c r="L35" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M35" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N35" s="17" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A36" s="13">
+        <v>46283</v>
+      </c>
+      <c r="B36" s="14">
+        <v>420</v>
+      </c>
+      <c r="C36" s="14">
+        <v>0</v>
+      </c>
+      <c r="D36" s="14">
+        <v>180</v>
+      </c>
+      <c r="E36" s="14">
+        <v>0</v>
+      </c>
+      <c r="F36" s="14">
+        <v>200</v>
+      </c>
+      <c r="G36" s="14">
+        <v>4</v>
+      </c>
+      <c r="H36" s="14">
+        <v>75</v>
+      </c>
+      <c r="I36" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J35" s="15" t="str">
+        <v>875</v>
+      </c>
+      <c r="J36" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="17"/>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A36" s="13"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="15" t="str">
+        <v>565</v>
+      </c>
+      <c r="K36" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L36" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M36" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N36" s="17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A37" s="13">
+        <v>46284</v>
+      </c>
+      <c r="B37" s="14">
+        <v>360</v>
+      </c>
+      <c r="C37" s="14">
+        <v>0</v>
+      </c>
+      <c r="D37" s="14">
+        <v>150</v>
+      </c>
+      <c r="E37" s="14">
+        <v>0</v>
+      </c>
+      <c r="F37" s="14">
+        <v>0</v>
+      </c>
+      <c r="G37" s="14">
+        <v>0</v>
+      </c>
+      <c r="H37" s="14">
+        <v>140</v>
+      </c>
+      <c r="I37" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J36" s="15" t="str">
+        <v>650</v>
+      </c>
+      <c r="J37" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K36" s="16"/>
-      <c r="L36" s="16"/>
-      <c r="M36" s="16"/>
-      <c r="N36" s="17"/>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="13"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16"/>
-      <c r="M37" s="16"/>
-      <c r="N37" s="17"/>
+        <v>790</v>
+      </c>
+      <c r="K37" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L37" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M37" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N37" s="17" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" s="13"/>

</xml_diff>

<commit_message>
File Upated on 20/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B4C92D-1A4C-4E14-8CCB-3CBDB488EA5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91EB6113-EE9F-4EAB-B932-0FF2462EBDBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="612" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="70">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2526,27 +2526,51 @@
         <v>61</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="13"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="15" t="str">
+    <row r="38" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="13">
+        <v>47381</v>
+      </c>
+      <c r="B38" s="14">
+        <v>720</v>
+      </c>
+      <c r="C38" s="14">
+        <v>0</v>
+      </c>
+      <c r="D38" s="14">
+        <v>0</v>
+      </c>
+      <c r="E38" s="14">
+        <v>0</v>
+      </c>
+      <c r="F38" s="14">
+        <v>0</v>
+      </c>
+      <c r="G38" s="14">
+        <v>0</v>
+      </c>
+      <c r="H38" s="14">
+        <v>120</v>
+      </c>
+      <c r="I38" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="15" t="str">
+        <v>840</v>
+      </c>
+      <c r="J38" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
-      <c r="N38" s="17"/>
+        <v>600</v>
+      </c>
+      <c r="K38" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L38" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M38" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N38" s="17" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" s="13"/>

</xml_diff>

<commit_message>
File Updated on 22/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91EB6113-EE9F-4EAB-B932-0FF2462EBDBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DB999A0-35E1-455D-AA22-6957B3029ED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="612" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="72">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -245,6 +245,12 @@
   </si>
   <si>
     <t>September</t>
+  </si>
+  <si>
+    <t>Sleepy after classes</t>
+  </si>
+  <si>
+    <t>Tired after classes and faced delayed output in vs code with c++ code</t>
   </si>
 </sst>
 </file>
@@ -2528,7 +2534,7 @@
     </row>
     <row r="38" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A38" s="13">
-        <v>47381</v>
+        <v>46285</v>
       </c>
       <c r="B38" s="14">
         <v>720</v>
@@ -2572,49 +2578,97 @@
         <v>61</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A39" s="13"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="15" t="str">
+    <row r="39" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A39" s="13">
+        <v>46286</v>
+      </c>
+      <c r="B39" s="14">
+        <v>420</v>
+      </c>
+      <c r="C39" s="14">
+        <v>0</v>
+      </c>
+      <c r="D39" s="14">
+        <v>150</v>
+      </c>
+      <c r="E39" s="14">
+        <v>0</v>
+      </c>
+      <c r="F39" s="14">
+        <v>250</v>
+      </c>
+      <c r="G39" s="14">
+        <v>5</v>
+      </c>
+      <c r="H39" s="14">
+        <v>100</v>
+      </c>
+      <c r="I39" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="15" t="str">
+        <v>920</v>
+      </c>
+      <c r="J39" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
-      <c r="N39" s="17"/>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="13"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="15" t="str">
+        <v>520</v>
+      </c>
+      <c r="K39" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L39" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M39" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N39" s="17" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A40" s="13">
+        <v>46287</v>
+      </c>
+      <c r="B40" s="14">
+        <v>420</v>
+      </c>
+      <c r="C40" s="14">
+        <v>0</v>
+      </c>
+      <c r="D40" s="14">
+        <v>140</v>
+      </c>
+      <c r="E40" s="14">
+        <v>0</v>
+      </c>
+      <c r="F40" s="14">
+        <v>400</v>
+      </c>
+      <c r="G40" s="14">
+        <v>8</v>
+      </c>
+      <c r="H40" s="14">
+        <v>70</v>
+      </c>
+      <c r="I40" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="15" t="str">
+        <v>1030</v>
+      </c>
+      <c r="J40" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16"/>
-      <c r="M40" s="16"/>
-      <c r="N40" s="17"/>
+        <v>410</v>
+      </c>
+      <c r="K40" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L40" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M40" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N40" s="17" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="13"/>

</xml_diff>

<commit_message>
File Updated on 23/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DB999A0-35E1-455D-AA22-6957B3029ED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1FE7092-CF26-4463-970B-8AFBEBA5FBDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="612" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="73">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -251,6 +251,9 @@
   </si>
   <si>
     <t>Tired after classes and faced delayed output in vs code with c++ code</t>
+  </si>
+  <si>
+    <t>Tired after classes and worked on the python project</t>
   </si>
 </sst>
 </file>
@@ -2670,27 +2673,51 @@
         <v>71</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A41" s="13"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="15" t="str">
+    <row r="41" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A41" s="13">
+        <v>46288</v>
+      </c>
+      <c r="B41" s="14">
+        <v>450</v>
+      </c>
+      <c r="C41" s="14">
+        <v>0</v>
+      </c>
+      <c r="D41" s="14">
+        <v>130</v>
+      </c>
+      <c r="E41" s="14">
+        <v>0</v>
+      </c>
+      <c r="F41" s="14">
+        <v>350</v>
+      </c>
+      <c r="G41" s="14">
+        <v>7</v>
+      </c>
+      <c r="H41" s="14">
+        <v>50</v>
+      </c>
+      <c r="I41" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J41" s="15" t="str">
+        <v>980</v>
+      </c>
+      <c r="J41" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K41" s="16"/>
-      <c r="L41" s="16"/>
-      <c r="M41" s="16"/>
-      <c r="N41" s="17"/>
+        <v>460</v>
+      </c>
+      <c r="K41" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L41" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M41" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N41" s="17" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" s="13"/>

</xml_diff>

<commit_message>
File Updated On 24/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1FE7092-CF26-4463-970B-8AFBEBA5FBDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30452763-8320-4B7A-A73F-557A759A75BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="612" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="73">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2720,26 +2720,50 @@
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A42" s="13"/>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
-      <c r="G42" s="14"/>
-      <c r="H42" s="14"/>
-      <c r="I42" s="15" t="str">
+      <c r="A42" s="13">
+        <v>46289</v>
+      </c>
+      <c r="B42" s="14">
+        <v>510</v>
+      </c>
+      <c r="C42" s="14">
+        <v>0</v>
+      </c>
+      <c r="D42" s="14">
+        <v>110</v>
+      </c>
+      <c r="E42" s="14">
+        <v>0</v>
+      </c>
+      <c r="F42" s="14">
+        <v>100</v>
+      </c>
+      <c r="G42" s="14">
+        <v>2</v>
+      </c>
+      <c r="H42" s="14">
+        <v>55</v>
+      </c>
+      <c r="I42" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J42" s="15" t="str">
+        <v>775</v>
+      </c>
+      <c r="J42" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K42" s="16"/>
-      <c r="L42" s="16"/>
-      <c r="M42" s="16"/>
-      <c r="N42" s="17"/>
+        <v>665</v>
+      </c>
+      <c r="K42" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L42" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M42" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N42" s="17" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" s="13"/>

</xml_diff>

<commit_message>
File Updated On 25/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30452763-8320-4B7A-A73F-557A759A75BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEFBB86D-5512-4E78-838B-D6046C398D40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="612" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="73">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2766,26 +2766,50 @@
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A43" s="13"/>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="15" t="str">
+      <c r="A43" s="13">
+        <v>46290</v>
+      </c>
+      <c r="B43" s="14">
+        <v>420</v>
+      </c>
+      <c r="C43" s="14">
+        <v>0</v>
+      </c>
+      <c r="D43" s="14">
+        <v>120</v>
+      </c>
+      <c r="E43" s="14">
+        <v>0</v>
+      </c>
+      <c r="F43" s="14">
+        <v>200</v>
+      </c>
+      <c r="G43" s="14">
+        <v>4</v>
+      </c>
+      <c r="H43" s="14">
+        <v>60</v>
+      </c>
+      <c r="I43" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J43" s="15" t="str">
+        <v>800</v>
+      </c>
+      <c r="J43" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K43" s="16"/>
-      <c r="L43" s="16"/>
-      <c r="M43" s="16"/>
-      <c r="N43" s="17"/>
+        <v>640</v>
+      </c>
+      <c r="K43" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L43" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M43" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N43" s="17" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" s="13"/>

</xml_diff>

<commit_message>
File Updated On 30/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEFBB86D-5512-4E78-838B-D6046C398D40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44DB24BB-6B61-4B0C-BA8C-BABC1117C416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="612" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="76">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -196,12 +196,6 @@
     <t>Low</t>
   </si>
   <si>
-    <t>Not Satisfied</t>
-  </si>
-  <si>
-    <t>Average</t>
-  </si>
-  <si>
     <t>Feeling very tired after classes</t>
   </si>
   <si>
@@ -223,12 +217,6 @@
     <t>Not productive</t>
   </si>
   <si>
-    <t>Below Average</t>
-  </si>
-  <si>
-    <t>Above Average</t>
-  </si>
-  <si>
     <t>Not productive enough</t>
   </si>
   <si>
@@ -238,13 +226,7 @@
     <t>20266-09-07</t>
   </si>
   <si>
-    <t>Bad</t>
-  </si>
-  <si>
     <t>Sleepy all day</t>
-  </si>
-  <si>
-    <t>September</t>
   </si>
   <si>
     <t>Sleepy after classes</t>
@@ -254,6 +236,33 @@
   </si>
   <si>
     <t>Tired after classes and worked on the python project</t>
+  </si>
+  <si>
+    <t>Neutral</t>
+  </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>Stressed</t>
+  </si>
+  <si>
+    <t>Very Unsatisfied</t>
+  </si>
+  <si>
+    <t>Unsatisfied</t>
+  </si>
+  <si>
+    <t>Septmeber</t>
+  </si>
+  <si>
+    <t>Attended Makeup classes</t>
+  </si>
+  <si>
+    <t>Travelled</t>
+  </si>
+  <si>
+    <t>Sleepy all day because of travel fatigue</t>
   </si>
 </sst>
 </file>
@@ -998,7 +1007,7 @@
         <v>33</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G3" s="22"/>
     </row>
@@ -1097,16 +1106,16 @@
         <v>540</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L6" s="11" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="M6" s="11" t="s">
         <v>52</v>
       </c>
       <c r="N6" s="12" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -1143,16 +1152,16 @@
         <v>610</v>
       </c>
       <c r="K7" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L7" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M7" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N7" s="17" t="s">
         <v>56</v>
-      </c>
-      <c r="M7" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N7" s="17" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
@@ -1189,16 +1198,16 @@
         <v>750</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="L8" s="16" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N8" s="17" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -1235,19 +1244,19 @@
         <v>660</v>
       </c>
       <c r="K9" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L9" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M9" s="16" t="s">
         <v>52</v>
       </c>
       <c r="N9" s="17" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="13">
         <v>46257</v>
       </c>
@@ -1281,19 +1290,19 @@
         <v>675</v>
       </c>
       <c r="K10" s="16" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="L10" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M10" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N10" s="17" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="13">
         <v>46258</v>
       </c>
@@ -1327,16 +1336,16 @@
         <v>600</v>
       </c>
       <c r="K11" s="16" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="L11" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N11" s="17" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -1373,19 +1382,19 @@
         <v>400</v>
       </c>
       <c r="K12" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L12" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M12" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N12" s="17" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="13">
         <v>46260</v>
       </c>
@@ -1419,16 +1428,16 @@
         <v>515</v>
       </c>
       <c r="K13" s="16" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="L13" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M13" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N13" s="17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -1465,16 +1474,16 @@
         <v>430</v>
       </c>
       <c r="K14" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L14" s="16" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="M14" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N14" s="17" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -1511,19 +1520,19 @@
         <v>690</v>
       </c>
       <c r="K15" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L15" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M15" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N15" s="17" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="13">
         <v>46263</v>
       </c>
@@ -1557,19 +1566,19 @@
         <v>620</v>
       </c>
       <c r="K16" s="16" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="L16" s="16" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="M16" s="16" t="s">
         <v>52</v>
       </c>
       <c r="N16" s="17" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="13">
         <v>46264</v>
       </c>
@@ -1603,16 +1612,16 @@
         <v>610</v>
       </c>
       <c r="K17" s="16" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="L17" s="16" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="M17" s="16" t="s">
         <v>52</v>
       </c>
       <c r="N17" s="17" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
@@ -1649,16 +1658,16 @@
         <v>480</v>
       </c>
       <c r="K18" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L18" s="16" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="M18" s="16" t="s">
         <v>52</v>
       </c>
       <c r="N18" s="17" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
@@ -1695,16 +1704,16 @@
         <v>505</v>
       </c>
       <c r="K19" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L19" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M19" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N19" s="17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
@@ -1741,16 +1750,16 @@
         <v>520</v>
       </c>
       <c r="K20" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L20" s="16" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N20" s="17" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
@@ -1787,16 +1796,16 @@
         <v>610</v>
       </c>
       <c r="K21" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L21" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="L21" s="16" t="s">
-        <v>56</v>
-      </c>
       <c r="M21" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N21" s="17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
@@ -1833,19 +1842,19 @@
         <v>700</v>
       </c>
       <c r="K22" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L22" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M22" s="16" t="s">
         <v>52</v>
       </c>
       <c r="N22" s="17" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="13">
         <v>46270</v>
       </c>
@@ -1879,19 +1888,19 @@
         <v>840</v>
       </c>
       <c r="K23" s="16" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="L23" s="16" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="M23" s="16" t="s">
         <v>52</v>
       </c>
       <c r="N23" s="17" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="13">
         <v>46271</v>
       </c>
@@ -1925,21 +1934,21 @@
         <v>660</v>
       </c>
       <c r="K24" s="16" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="L24" s="16" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="M24" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N24" s="17" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="13" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B25" s="14">
         <v>360</v>
@@ -1971,16 +1980,16 @@
         <v>680</v>
       </c>
       <c r="K25" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L25" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M25" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N25" s="17" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
@@ -2017,19 +2026,19 @@
         <v>470</v>
       </c>
       <c r="K26" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L26" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M26" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N26" s="17" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="13">
         <v>46274</v>
       </c>
@@ -2063,16 +2072,16 @@
         <v>625</v>
       </c>
       <c r="K27" s="16" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="L27" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M27" s="16" t="s">
         <v>52</v>
       </c>
       <c r="N27" s="17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
@@ -2109,16 +2118,16 @@
         <v>755</v>
       </c>
       <c r="K28" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L28" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M28" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N28" s="17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
@@ -2155,16 +2164,16 @@
         <v>795</v>
       </c>
       <c r="K29" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L29" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M29" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N29" s="17" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
@@ -2201,16 +2210,16 @@
         <v>690</v>
       </c>
       <c r="K30" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L30" s="16" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="M30" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N30" s="17" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
@@ -2247,16 +2256,16 @@
         <v>600</v>
       </c>
       <c r="K31" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L31" s="16" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="M31" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N31" s="17" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
@@ -2293,16 +2302,16 @@
         <v>580</v>
       </c>
       <c r="K32" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L32" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M32" s="16" t="s">
         <v>52</v>
       </c>
       <c r="N32" s="17" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
@@ -2339,16 +2348,16 @@
         <v>390</v>
       </c>
       <c r="K33" s="16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L33" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M33" s="16" t="s">
         <v>52</v>
       </c>
       <c r="N33" s="17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
@@ -2385,16 +2394,16 @@
         <v>565</v>
       </c>
       <c r="K34" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L34" s="16" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="M34" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N34" s="17" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
@@ -2431,16 +2440,16 @@
         <v>620</v>
       </c>
       <c r="K35" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L35" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M35" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N35" s="17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
@@ -2477,16 +2486,16 @@
         <v>565</v>
       </c>
       <c r="K36" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L36" s="16" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="M36" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N36" s="17" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
@@ -2523,19 +2532,19 @@
         <v>790</v>
       </c>
       <c r="K37" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L37" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M37" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N37" s="17" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" s="13">
         <v>46285</v>
       </c>
@@ -2569,19 +2578,19 @@
         <v>600</v>
       </c>
       <c r="K38" s="16" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="L38" s="16" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="M38" s="16" t="s">
         <v>52</v>
       </c>
       <c r="N38" s="17" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" s="13">
         <v>46286</v>
       </c>
@@ -2615,16 +2624,16 @@
         <v>520</v>
       </c>
       <c r="K39" s="16" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="L39" s="16" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="M39" s="16" t="s">
         <v>52</v>
       </c>
       <c r="N39" s="17" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
@@ -2661,16 +2670,16 @@
         <v>410</v>
       </c>
       <c r="K40" s="16" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="L40" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M40" s="16" t="s">
         <v>52</v>
       </c>
       <c r="N40" s="17" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -2707,16 +2716,16 @@
         <v>460</v>
       </c>
       <c r="K41" s="16" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="L41" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M41" s="16" t="s">
         <v>52</v>
       </c>
       <c r="N41" s="17" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
@@ -2753,16 +2762,16 @@
         <v>665</v>
       </c>
       <c r="K42" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L42" s="16" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="M42" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N42" s="17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
@@ -2799,127 +2808,247 @@
         <v>640</v>
       </c>
       <c r="K43" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="L43" s="16" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="M43" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N43" s="17" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A44" s="13"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="14"/>
-      <c r="G44" s="14"/>
-      <c r="H44" s="14"/>
-      <c r="I44" s="15" t="str">
+      <c r="A44" s="13">
+        <v>46291</v>
+      </c>
+      <c r="B44" s="14">
+        <v>300</v>
+      </c>
+      <c r="C44" s="14">
+        <v>0</v>
+      </c>
+      <c r="D44" s="14">
+        <v>75</v>
+      </c>
+      <c r="E44" s="14">
+        <v>0</v>
+      </c>
+      <c r="F44" s="14">
+        <v>150</v>
+      </c>
+      <c r="G44" s="14">
+        <v>3</v>
+      </c>
+      <c r="H44" s="14">
+        <v>45</v>
+      </c>
+      <c r="I44" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J44" s="15" t="str">
+        <v>570</v>
+      </c>
+      <c r="J44" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K44" s="16"/>
-      <c r="L44" s="16"/>
-      <c r="M44" s="16"/>
-      <c r="N44" s="17"/>
+        <v>870</v>
+      </c>
+      <c r="K44" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L44" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M44" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N44" s="17" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A45" s="13"/>
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="14"/>
-      <c r="G45" s="14"/>
-      <c r="H45" s="14"/>
-      <c r="I45" s="15" t="str">
+      <c r="A45" s="13">
+        <v>46292</v>
+      </c>
+      <c r="B45" s="14">
+        <v>420</v>
+      </c>
+      <c r="C45" s="14">
+        <v>0</v>
+      </c>
+      <c r="D45" s="14">
+        <v>0</v>
+      </c>
+      <c r="E45" s="14">
+        <v>0</v>
+      </c>
+      <c r="F45" s="14">
+        <v>0</v>
+      </c>
+      <c r="G45" s="14">
+        <v>0</v>
+      </c>
+      <c r="H45" s="14">
+        <v>90</v>
+      </c>
+      <c r="I45" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J45" s="15" t="str">
+        <v>510</v>
+      </c>
+      <c r="J45" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K45" s="16"/>
-      <c r="L45" s="16"/>
-      <c r="M45" s="16"/>
-      <c r="N45" s="17"/>
+        <v>930</v>
+      </c>
+      <c r="K45" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L45" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M45" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N45" s="17" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A46" s="13"/>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="14"/>
-      <c r="G46" s="14"/>
-      <c r="H46" s="14"/>
-      <c r="I46" s="15" t="str">
+      <c r="A46" s="13">
+        <v>46293</v>
+      </c>
+      <c r="B46" s="14">
+        <v>360</v>
+      </c>
+      <c r="C46" s="14">
+        <v>0</v>
+      </c>
+      <c r="D46" s="14">
+        <v>0</v>
+      </c>
+      <c r="E46" s="14">
+        <v>0</v>
+      </c>
+      <c r="F46" s="14">
+        <v>0</v>
+      </c>
+      <c r="G46" s="14">
+        <v>0</v>
+      </c>
+      <c r="H46" s="14">
+        <v>720</v>
+      </c>
+      <c r="I46" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J46" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J46" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K46" s="16"/>
-      <c r="L46" s="16"/>
-      <c r="M46" s="16"/>
-      <c r="N46" s="17"/>
+        <v>360</v>
+      </c>
+      <c r="K46" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="L46" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M46" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N46" s="17" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A47" s="13"/>
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="14"/>
-      <c r="G47" s="14"/>
-      <c r="H47" s="14"/>
-      <c r="I47" s="15" t="str">
+      <c r="A47" s="13">
+        <v>46294</v>
+      </c>
+      <c r="B47" s="14">
+        <v>120</v>
+      </c>
+      <c r="C47" s="14">
+        <v>0</v>
+      </c>
+      <c r="D47" s="14">
+        <v>0</v>
+      </c>
+      <c r="E47" s="14">
+        <v>0</v>
+      </c>
+      <c r="F47" s="14">
+        <v>0</v>
+      </c>
+      <c r="G47" s="14">
+        <v>0</v>
+      </c>
+      <c r="H47" s="14">
+        <v>360</v>
+      </c>
+      <c r="I47" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J47" s="15" t="str">
+        <v>480</v>
+      </c>
+      <c r="J47" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K47" s="16"/>
-      <c r="L47" s="16"/>
-      <c r="M47" s="16"/>
-      <c r="N47" s="17"/>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A48" s="13"/>
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="14"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="15" t="str">
+        <v>960</v>
+      </c>
+      <c r="K47" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L47" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M47" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N47" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A48" s="13">
+        <v>46295</v>
+      </c>
+      <c r="B48" s="14">
+        <v>480</v>
+      </c>
+      <c r="C48" s="14">
+        <v>0</v>
+      </c>
+      <c r="D48" s="14">
+        <v>0</v>
+      </c>
+      <c r="E48" s="14">
+        <v>0</v>
+      </c>
+      <c r="F48" s="14">
+        <v>0</v>
+      </c>
+      <c r="G48" s="14">
+        <v>0</v>
+      </c>
+      <c r="H48" s="14">
+        <v>260</v>
+      </c>
+      <c r="I48" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J48" s="15" t="str">
+        <v>740</v>
+      </c>
+      <c r="J48" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K48" s="16"/>
-      <c r="L48" s="16"/>
-      <c r="M48" s="16"/>
-      <c r="N48" s="17"/>
+        <v>700</v>
+      </c>
+      <c r="K48" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L48" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M48" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N48" s="17" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" s="13"/>

</xml_diff>

<commit_message>
File Updated On 04/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44DB24BB-6B61-4B0C-BA8C-BABC1117C416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2CFEBE0-10BB-4550-A652-5C2A05922490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="612" yWindow="-108" windowWidth="22536" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="81">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -263,6 +263,21 @@
   </si>
   <si>
     <t>Sleepy all day because of travel fatigue</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Made a plan for studies but didn't follow</t>
+  </si>
+  <si>
+    <t>Feeling good because of high energy</t>
+  </si>
+  <si>
+    <t>Tried studying but couldn't because of headache</t>
+  </si>
+  <si>
+    <t>Was feeling sleepy today</t>
   </si>
 </sst>
 </file>
@@ -3050,93 +3065,189 @@
         <v>75</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" s="13"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="14"/>
-      <c r="G49" s="14"/>
-      <c r="H49" s="14"/>
-      <c r="I49" s="15" t="str">
+    <row r="49" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A49" s="13">
+        <v>46296</v>
+      </c>
+      <c r="B49" s="14">
+        <v>480</v>
+      </c>
+      <c r="C49" s="14">
+        <v>0</v>
+      </c>
+      <c r="D49" s="14">
+        <v>0</v>
+      </c>
+      <c r="E49" s="14">
+        <v>0</v>
+      </c>
+      <c r="F49" s="14">
+        <v>0</v>
+      </c>
+      <c r="G49" s="14">
+        <v>0</v>
+      </c>
+      <c r="H49" s="14">
+        <v>300</v>
+      </c>
+      <c r="I49" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J49" s="15" t="str">
+        <v>780</v>
+      </c>
+      <c r="J49" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K49" s="16"/>
-      <c r="L49" s="16"/>
-      <c r="M49" s="16"/>
-      <c r="N49" s="17"/>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A50" s="13"/>
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="14"/>
-      <c r="F50" s="14"/>
-      <c r="G50" s="14"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="15" t="str">
+        <v>660</v>
+      </c>
+      <c r="K49" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L49" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M49" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N49" s="17" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A50" s="13">
+        <v>46297</v>
+      </c>
+      <c r="B50" s="14">
+        <v>480</v>
+      </c>
+      <c r="C50" s="14">
+        <v>0</v>
+      </c>
+      <c r="D50" s="14">
+        <v>15</v>
+      </c>
+      <c r="E50" s="14">
+        <v>0</v>
+      </c>
+      <c r="F50" s="14">
+        <v>0</v>
+      </c>
+      <c r="G50" s="14">
+        <v>0</v>
+      </c>
+      <c r="H50" s="14">
+        <v>340</v>
+      </c>
+      <c r="I50" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J50" s="15" t="str">
+        <v>835</v>
+      </c>
+      <c r="J50" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K50" s="16"/>
-      <c r="L50" s="16"/>
-      <c r="M50" s="16"/>
-      <c r="N50" s="17"/>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A51" s="13"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="14"/>
-      <c r="F51" s="14"/>
-      <c r="G51" s="14"/>
-      <c r="H51" s="14"/>
-      <c r="I51" s="15" t="str">
+        <v>605</v>
+      </c>
+      <c r="K50" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L50" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="M50" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="N50" s="17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A51" s="13">
+        <v>46298</v>
+      </c>
+      <c r="B51" s="14">
+        <v>480</v>
+      </c>
+      <c r="C51" s="14">
+        <v>0</v>
+      </c>
+      <c r="D51" s="14">
+        <v>30</v>
+      </c>
+      <c r="E51" s="14">
+        <v>0</v>
+      </c>
+      <c r="F51" s="14">
+        <v>0</v>
+      </c>
+      <c r="G51" s="14">
+        <v>0</v>
+      </c>
+      <c r="H51" s="14">
+        <v>280</v>
+      </c>
+      <c r="I51" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J51" s="15" t="str">
+        <v>790</v>
+      </c>
+      <c r="J51" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K51" s="16"/>
-      <c r="L51" s="16"/>
-      <c r="M51" s="16"/>
-      <c r="N51" s="17"/>
+        <v>650</v>
+      </c>
+      <c r="K51" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L51" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M51" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="N51" s="17" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A52" s="13"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="14"/>
-      <c r="F52" s="14"/>
-      <c r="G52" s="14"/>
-      <c r="H52" s="14"/>
-      <c r="I52" s="15" t="str">
+      <c r="A52" s="13">
+        <v>46299</v>
+      </c>
+      <c r="B52" s="14">
+        <v>480</v>
+      </c>
+      <c r="C52" s="14">
+        <v>0</v>
+      </c>
+      <c r="D52" s="14">
+        <v>75</v>
+      </c>
+      <c r="E52" s="14">
+        <v>0</v>
+      </c>
+      <c r="F52" s="14">
+        <v>0</v>
+      </c>
+      <c r="G52" s="14">
+        <v>0</v>
+      </c>
+      <c r="H52" s="14">
+        <v>250</v>
+      </c>
+      <c r="I52" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J52" s="15" t="str">
+        <v>805</v>
+      </c>
+      <c r="J52" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K52" s="16"/>
-      <c r="L52" s="16"/>
-      <c r="M52" s="16"/>
-      <c r="N52" s="17"/>
+        <v>635</v>
+      </c>
+      <c r="K52" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L52" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M52" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N52" s="17" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" s="13"/>

</xml_diff>

<commit_message>
File Updated On 05/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2CFEBE0-10BB-4550-A652-5C2A05922490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{530162D4-BF91-45A6-BC6F-E29D9F695625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="612" yWindow="-108" windowWidth="22536" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="81">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3250,26 +3250,50 @@
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A53" s="13"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="14"/>
-      <c r="F53" s="14"/>
-      <c r="G53" s="14"/>
-      <c r="H53" s="14"/>
-      <c r="I53" s="15" t="str">
+      <c r="A53" s="13">
+        <v>46300</v>
+      </c>
+      <c r="B53" s="14">
+        <v>480</v>
+      </c>
+      <c r="C53" s="14">
+        <v>0</v>
+      </c>
+      <c r="D53" s="14">
+        <v>120</v>
+      </c>
+      <c r="E53" s="14">
+        <v>0</v>
+      </c>
+      <c r="F53" s="14">
+        <v>250</v>
+      </c>
+      <c r="G53" s="14">
+        <v>5</v>
+      </c>
+      <c r="H53" s="14">
+        <v>160</v>
+      </c>
+      <c r="I53" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J53" s="15" t="str">
+        <v>1010</v>
+      </c>
+      <c r="J53" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K53" s="16"/>
-      <c r="L53" s="16"/>
-      <c r="M53" s="16"/>
-      <c r="N53" s="17"/>
+        <v>430</v>
+      </c>
+      <c r="K53" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L53" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M53" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N53" s="17" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" s="13"/>

</xml_diff>

<commit_message>
File Updated On 06/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{530162D4-BF91-45A6-BC6F-E29D9F695625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F16463E7-CF8E-4AFD-97FF-D6B11BF81616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="82">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -253,9 +253,6 @@
     <t>Unsatisfied</t>
   </si>
   <si>
-    <t>Septmeber</t>
-  </si>
-  <si>
     <t>Attended Makeup classes</t>
   </si>
   <si>
@@ -278,6 +275,12 @@
   </si>
   <si>
     <t>Was feeling sleepy today</t>
+  </si>
+  <si>
+    <t>August</t>
+  </si>
+  <si>
+    <t>Attended classes and solved mcqs</t>
   </si>
 </sst>
 </file>
@@ -1022,7 +1025,7 @@
         <v>33</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="G3" s="22"/>
     </row>
@@ -2878,7 +2881,7 @@
         <v>55</v>
       </c>
       <c r="N44" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
@@ -2970,7 +2973,7 @@
         <v>52</v>
       </c>
       <c r="N46" s="17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
@@ -3016,7 +3019,7 @@
         <v>52</v>
       </c>
       <c r="N47" s="17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="48" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -3062,7 +3065,7 @@
         <v>52</v>
       </c>
       <c r="N48" s="17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="49" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -3108,7 +3111,7 @@
         <v>55</v>
       </c>
       <c r="N49" s="17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="50" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -3151,10 +3154,10 @@
         <v>70</v>
       </c>
       <c r="M50" s="16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N50" s="17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="51" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -3197,10 +3200,10 @@
         <v>54</v>
       </c>
       <c r="M51" s="16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N51" s="17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
@@ -3246,7 +3249,7 @@
         <v>55</v>
       </c>
       <c r="N52" s="17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
@@ -3295,27 +3298,51 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A54" s="13"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="14"/>
-      <c r="F54" s="14"/>
-      <c r="G54" s="14"/>
-      <c r="H54" s="14"/>
-      <c r="I54" s="15" t="str">
+    <row r="54" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A54" s="13">
+        <v>46301</v>
+      </c>
+      <c r="B54" s="14">
+        <v>480</v>
+      </c>
+      <c r="C54" s="14">
+        <v>0</v>
+      </c>
+      <c r="D54" s="14">
+        <v>200</v>
+      </c>
+      <c r="E54" s="14">
+        <v>30</v>
+      </c>
+      <c r="F54" s="14">
+        <v>400</v>
+      </c>
+      <c r="G54" s="14">
+        <v>8</v>
+      </c>
+      <c r="H54" s="14">
+        <v>180</v>
+      </c>
+      <c r="I54" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J54" s="15" t="str">
+        <v>1290</v>
+      </c>
+      <c r="J54" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K54" s="16"/>
-      <c r="L54" s="16"/>
-      <c r="M54" s="16"/>
-      <c r="N54" s="17"/>
+        <v>150</v>
+      </c>
+      <c r="K54" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L54" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M54" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N54" s="17" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" s="13"/>

</xml_diff>

<commit_message>
File Updated On 07/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F16463E7-CF8E-4AFD-97FF-D6B11BF81616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6DAA19-4CFF-49C2-93CB-FC231C164030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="83">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -281,6 +281,9 @@
   </si>
   <si>
     <t>Attended classes and solved mcqs</t>
+  </si>
+  <si>
+    <t>No notes  today</t>
   </si>
 </sst>
 </file>
@@ -3345,26 +3348,50 @@
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A55" s="13"/>
-      <c r="B55" s="14"/>
-      <c r="C55" s="14"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="14"/>
-      <c r="F55" s="14"/>
-      <c r="G55" s="14"/>
-      <c r="H55" s="14"/>
-      <c r="I55" s="15" t="str">
+      <c r="A55" s="13">
+        <v>46302</v>
+      </c>
+      <c r="B55" s="14">
+        <v>480</v>
+      </c>
+      <c r="C55" s="14">
+        <v>0</v>
+      </c>
+      <c r="D55" s="14">
+        <v>160</v>
+      </c>
+      <c r="E55" s="14">
+        <v>15</v>
+      </c>
+      <c r="F55" s="14">
+        <v>350</v>
+      </c>
+      <c r="G55" s="14">
+        <v>7</v>
+      </c>
+      <c r="H55" s="14">
+        <v>150</v>
+      </c>
+      <c r="I55" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J55" s="15" t="str">
+        <v>1155</v>
+      </c>
+      <c r="J55" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K55" s="16"/>
-      <c r="L55" s="16"/>
-      <c r="M55" s="16"/>
-      <c r="N55" s="17"/>
+        <v>285</v>
+      </c>
+      <c r="K55" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L55" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M55" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N55" s="17" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" s="13"/>

</xml_diff>

<commit_message>
File Updated On 08/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6DAA19-4CFF-49C2-93CB-FC231C164030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91C07D52-F08C-4A2C-9BE1-543DAAD08ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="83">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3394,26 +3394,50 @@
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A56" s="13"/>
-      <c r="B56" s="14"/>
-      <c r="C56" s="14"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="14"/>
-      <c r="F56" s="14"/>
-      <c r="G56" s="14"/>
-      <c r="H56" s="14"/>
-      <c r="I56" s="15" t="str">
+      <c r="A56" s="13">
+        <v>46303</v>
+      </c>
+      <c r="B56" s="14">
+        <v>480</v>
+      </c>
+      <c r="C56" s="14">
+        <v>0</v>
+      </c>
+      <c r="D56" s="14">
+        <v>100</v>
+      </c>
+      <c r="E56" s="14">
+        <v>0</v>
+      </c>
+      <c r="F56" s="14">
+        <v>150</v>
+      </c>
+      <c r="G56" s="14">
+        <v>3</v>
+      </c>
+      <c r="H56" s="14">
+        <v>180</v>
+      </c>
+      <c r="I56" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J56" s="15" t="str">
+        <v>910</v>
+      </c>
+      <c r="J56" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K56" s="16"/>
-      <c r="L56" s="16"/>
-      <c r="M56" s="16"/>
-      <c r="N56" s="17"/>
+        <v>530</v>
+      </c>
+      <c r="K56" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="L56" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="M56" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N56" s="17" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" s="13"/>

</xml_diff>

<commit_message>
File Updated On 11/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91C07D52-F08C-4A2C-9BE1-543DAAD08ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1513893C-697F-4C22-BF51-3B956D834C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="84">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -284,6 +284,9 @@
   </si>
   <si>
     <t>No notes  today</t>
+  </si>
+  <si>
+    <t>Attended doubt sessions</t>
   </si>
 </sst>
 </file>
@@ -3440,70 +3443,142 @@
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A57" s="13"/>
-      <c r="B57" s="14"/>
-      <c r="C57" s="14"/>
-      <c r="D57" s="14"/>
-      <c r="E57" s="14"/>
-      <c r="F57" s="14"/>
-      <c r="G57" s="14"/>
-      <c r="H57" s="14"/>
-      <c r="I57" s="15" t="str">
+      <c r="A57" s="13">
+        <v>46304</v>
+      </c>
+      <c r="B57" s="14">
+        <v>489</v>
+      </c>
+      <c r="C57" s="14">
+        <v>0</v>
+      </c>
+      <c r="D57" s="14">
+        <v>0</v>
+      </c>
+      <c r="E57" s="14">
+        <v>0</v>
+      </c>
+      <c r="F57" s="14">
+        <v>100</v>
+      </c>
+      <c r="G57" s="14">
+        <v>2</v>
+      </c>
+      <c r="H57" s="14">
+        <v>160</v>
+      </c>
+      <c r="I57" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J57" s="15" t="str">
+        <v>749</v>
+      </c>
+      <c r="J57" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K57" s="16"/>
-      <c r="L57" s="16"/>
-      <c r="M57" s="16"/>
-      <c r="N57" s="17"/>
+        <v>691</v>
+      </c>
+      <c r="K57" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L57" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M57" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N57" s="17" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A58" s="13"/>
-      <c r="B58" s="14"/>
-      <c r="C58" s="14"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="14"/>
-      <c r="F58" s="14"/>
-      <c r="G58" s="14"/>
-      <c r="H58" s="14"/>
-      <c r="I58" s="15" t="str">
+      <c r="A58" s="13">
+        <v>46305</v>
+      </c>
+      <c r="B58" s="14">
+        <v>480</v>
+      </c>
+      <c r="C58" s="14">
+        <v>0</v>
+      </c>
+      <c r="D58" s="14">
+        <v>0</v>
+      </c>
+      <c r="E58" s="14">
+        <v>0</v>
+      </c>
+      <c r="F58" s="14">
+        <v>0</v>
+      </c>
+      <c r="G58" s="14">
+        <v>0</v>
+      </c>
+      <c r="H58" s="14">
+        <v>145</v>
+      </c>
+      <c r="I58" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J58" s="15" t="str">
+        <v>625</v>
+      </c>
+      <c r="J58" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K58" s="16"/>
-      <c r="L58" s="16"/>
-      <c r="M58" s="16"/>
-      <c r="N58" s="17"/>
+        <v>815</v>
+      </c>
+      <c r="K58" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L58" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M58" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N58" s="17" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A59" s="13"/>
-      <c r="B59" s="14"/>
-      <c r="C59" s="14"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="14"/>
-      <c r="F59" s="14"/>
-      <c r="G59" s="14"/>
-      <c r="H59" s="14"/>
-      <c r="I59" s="15" t="str">
+      <c r="A59" s="13">
+        <v>46306</v>
+      </c>
+      <c r="B59" s="14">
+        <v>240</v>
+      </c>
+      <c r="C59" s="14">
+        <v>0</v>
+      </c>
+      <c r="D59" s="14">
+        <v>50</v>
+      </c>
+      <c r="E59" s="14">
+        <v>0</v>
+      </c>
+      <c r="F59" s="14">
+        <v>0</v>
+      </c>
+      <c r="G59" s="14">
+        <v>0</v>
+      </c>
+      <c r="H59" s="14">
+        <v>250</v>
+      </c>
+      <c r="I59" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J59" s="15" t="str">
+        <v>540</v>
+      </c>
+      <c r="J59" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K59" s="16"/>
-      <c r="L59" s="16"/>
-      <c r="M59" s="16"/>
-      <c r="N59" s="17"/>
+        <v>900</v>
+      </c>
+      <c r="K59" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="L59" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M59" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N59" s="17" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" s="13"/>

</xml_diff>

<commit_message>
File Updated On 12/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1513893C-697F-4C22-BF51-3B956D834C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CF267A7-9FCE-4B77-A44F-DF05D083ED39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="85">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -287,6 +287,9 @@
   </si>
   <si>
     <t>Attended doubt sessions</t>
+  </si>
+  <si>
+    <t>1st mid term exam</t>
   </si>
 </sst>
 </file>
@@ -3581,26 +3584,50 @@
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A60" s="13"/>
-      <c r="B60" s="14"/>
-      <c r="C60" s="14"/>
-      <c r="D60" s="14"/>
-      <c r="E60" s="14"/>
-      <c r="F60" s="14"/>
-      <c r="G60" s="14"/>
-      <c r="H60" s="14"/>
-      <c r="I60" s="15" t="str">
+      <c r="A60" s="13">
+        <v>46307</v>
+      </c>
+      <c r="B60" s="14">
+        <v>300</v>
+      </c>
+      <c r="C60" s="14">
+        <v>0</v>
+      </c>
+      <c r="D60" s="14">
+        <v>200</v>
+      </c>
+      <c r="E60" s="14">
+        <v>0</v>
+      </c>
+      <c r="F60" s="14">
+        <v>0</v>
+      </c>
+      <c r="G60" s="14">
+        <v>0</v>
+      </c>
+      <c r="H60" s="14">
+        <v>170</v>
+      </c>
+      <c r="I60" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J60" s="15" t="str">
+        <v>670</v>
+      </c>
+      <c r="J60" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K60" s="16"/>
-      <c r="L60" s="16"/>
-      <c r="M60" s="16"/>
-      <c r="N60" s="17"/>
+        <v>770</v>
+      </c>
+      <c r="K60" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L60" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M60" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="N60" s="17" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" s="13"/>

</xml_diff>

<commit_message>
File Updated On 14/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CF267A7-9FCE-4B77-A44F-DF05D083ED39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4CC53BF-EC77-4128-BFE0-4A587EAD326B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="87">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -291,6 +291,12 @@
   <si>
     <t>1st mid term exam</t>
   </si>
+  <si>
+    <t>2nd mid term exam</t>
+  </si>
+  <si>
+    <t>3rd mid term exam</t>
+  </si>
 </sst>
 </file>
 
@@ -299,7 +305,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -378,6 +384,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -3630,48 +3642,96 @@
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A61" s="13"/>
-      <c r="B61" s="14"/>
-      <c r="C61" s="14"/>
-      <c r="D61" s="14"/>
-      <c r="E61" s="14"/>
-      <c r="F61" s="14"/>
-      <c r="G61" s="14"/>
-      <c r="H61" s="14"/>
-      <c r="I61" s="15" t="str">
+      <c r="A61" s="13">
+        <v>46308</v>
+      </c>
+      <c r="B61" s="14">
+        <v>300</v>
+      </c>
+      <c r="C61" s="14">
+        <v>0</v>
+      </c>
+      <c r="D61" s="14">
+        <v>220</v>
+      </c>
+      <c r="E61" s="14">
+        <v>0</v>
+      </c>
+      <c r="F61" s="14">
+        <v>0</v>
+      </c>
+      <c r="G61" s="14">
+        <v>0</v>
+      </c>
+      <c r="H61" s="14">
+        <v>140</v>
+      </c>
+      <c r="I61" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J61" s="15" t="str">
+        <v>660</v>
+      </c>
+      <c r="J61" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K61" s="16"/>
-      <c r="L61" s="16"/>
-      <c r="M61" s="16"/>
-      <c r="N61" s="17"/>
+        <v>780</v>
+      </c>
+      <c r="K61" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L61" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M61" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N61" s="17" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A62" s="13"/>
-      <c r="B62" s="14"/>
-      <c r="C62" s="14"/>
-      <c r="D62" s="14"/>
-      <c r="E62" s="14"/>
-      <c r="F62" s="14"/>
-      <c r="G62" s="14"/>
-      <c r="H62" s="14"/>
-      <c r="I62" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J62" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K62" s="16"/>
-      <c r="L62" s="16"/>
-      <c r="M62" s="16"/>
-      <c r="N62" s="17"/>
+      <c r="A62" s="13">
+        <v>46309</v>
+      </c>
+      <c r="B62" s="14">
+        <v>300</v>
+      </c>
+      <c r="C62" s="14">
+        <v>0</v>
+      </c>
+      <c r="D62" s="14">
+        <v>250</v>
+      </c>
+      <c r="E62" s="14">
+        <v>0</v>
+      </c>
+      <c r="F62" s="14">
+        <v>0</v>
+      </c>
+      <c r="G62" s="14">
+        <v>0</v>
+      </c>
+      <c r="H62" s="14">
+        <v>150</v>
+      </c>
+      <c r="I62" s="15">
+        <f t="shared" ref="I62" si="4">IF(SUM(B62:F62,H62)=0,"",SUM(B62:F62,H62))</f>
+        <v>700</v>
+      </c>
+      <c r="J62" s="15">
+        <f t="shared" ref="J62" si="5">IF(I62="","",1440-I62)</f>
+        <v>740</v>
+      </c>
+      <c r="K62" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L62" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M62" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="N62" s="17" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" s="13"/>
@@ -3837,11 +3897,11 @@
       <c r="G70" s="14"/>
       <c r="H70" s="14"/>
       <c r="I70" s="15" t="str">
-        <f t="shared" ref="I70:I133" si="4">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
+        <f t="shared" ref="I70:I133" si="6">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
         <v/>
       </c>
       <c r="J70" s="15" t="str">
-        <f t="shared" ref="J70:J133" si="5">IF(I70="","",1440-I70)</f>
+        <f t="shared" ref="J70:J133" si="7">IF(I70="","",1440-I70)</f>
         <v/>
       </c>
       <c r="K70" s="16"/>
@@ -3859,11 +3919,11 @@
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
       <c r="I71" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J71" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K71" s="16"/>
@@ -3881,11 +3941,11 @@
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
       <c r="I72" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J72" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K72" s="16"/>
@@ -3903,11 +3963,11 @@
       <c r="G73" s="14"/>
       <c r="H73" s="14"/>
       <c r="I73" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J73" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K73" s="16"/>
@@ -3925,11 +3985,11 @@
       <c r="G74" s="14"/>
       <c r="H74" s="14"/>
       <c r="I74" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J74" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K74" s="16"/>
@@ -3947,11 +4007,11 @@
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
       <c r="I75" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J75" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K75" s="16"/>
@@ -3969,11 +4029,11 @@
       <c r="G76" s="14"/>
       <c r="H76" s="14"/>
       <c r="I76" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J76" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K76" s="16"/>
@@ -3991,11 +4051,11 @@
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
       <c r="I77" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J77" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K77" s="16"/>
@@ -4013,11 +4073,11 @@
       <c r="G78" s="14"/>
       <c r="H78" s="14"/>
       <c r="I78" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J78" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K78" s="16"/>
@@ -4035,11 +4095,11 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J79" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K79" s="16"/>
@@ -4057,11 +4117,11 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J80" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K80" s="16"/>
@@ -4079,11 +4139,11 @@
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J81" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K81" s="16"/>
@@ -4101,11 +4161,11 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J82" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K82" s="16"/>
@@ -4123,11 +4183,11 @@
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
       <c r="I83" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J83" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K83" s="16"/>
@@ -4145,11 +4205,11 @@
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
       <c r="I84" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J84" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K84" s="16"/>
@@ -4167,11 +4227,11 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J85" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K85" s="16"/>
@@ -4189,11 +4249,11 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J86" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K86" s="16"/>
@@ -4211,11 +4271,11 @@
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
       <c r="I87" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J87" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K87" s="16"/>
@@ -4233,11 +4293,11 @@
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
       <c r="I88" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J88" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K88" s="16"/>
@@ -4255,11 +4315,11 @@
       <c r="G89" s="14"/>
       <c r="H89" s="14"/>
       <c r="I89" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J89" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K89" s="16"/>
@@ -4277,11 +4337,11 @@
       <c r="G90" s="14"/>
       <c r="H90" s="14"/>
       <c r="I90" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J90" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K90" s="16"/>
@@ -4299,11 +4359,11 @@
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
       <c r="I91" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J91" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K91" s="16"/>
@@ -4321,11 +4381,11 @@
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
       <c r="I92" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J92" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K92" s="16"/>
@@ -4343,11 +4403,11 @@
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J93" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K93" s="16"/>
@@ -4365,11 +4425,11 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J94" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K94" s="16"/>
@@ -4387,11 +4447,11 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J95" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K95" s="16"/>
@@ -4409,11 +4469,11 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J96" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K96" s="16"/>
@@ -4431,11 +4491,11 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J97" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K97" s="16"/>
@@ -4453,11 +4513,11 @@
       <c r="G98" s="14"/>
       <c r="H98" s="14"/>
       <c r="I98" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J98" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K98" s="16"/>
@@ -4475,11 +4535,11 @@
       <c r="G99" s="14"/>
       <c r="H99" s="14"/>
       <c r="I99" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J99" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K99" s="16"/>
@@ -4497,11 +4557,11 @@
       <c r="G100" s="14"/>
       <c r="H100" s="14"/>
       <c r="I100" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J100" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K100" s="16"/>
@@ -4519,11 +4579,11 @@
       <c r="G101" s="14"/>
       <c r="H101" s="14"/>
       <c r="I101" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J101" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K101" s="16"/>
@@ -4541,11 +4601,11 @@
       <c r="G102" s="14"/>
       <c r="H102" s="14"/>
       <c r="I102" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J102" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K102" s="16"/>
@@ -4563,11 +4623,11 @@
       <c r="G103" s="14"/>
       <c r="H103" s="14"/>
       <c r="I103" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J103" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K103" s="16"/>
@@ -4585,11 +4645,11 @@
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
       <c r="I104" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J104" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K104" s="16"/>
@@ -4607,11 +4667,11 @@
       <c r="G105" s="14"/>
       <c r="H105" s="14"/>
       <c r="I105" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J105" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K105" s="16"/>
@@ -4629,11 +4689,11 @@
       <c r="G106" s="14"/>
       <c r="H106" s="14"/>
       <c r="I106" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J106" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K106" s="16"/>
@@ -4651,11 +4711,11 @@
       <c r="G107" s="14"/>
       <c r="H107" s="14"/>
       <c r="I107" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J107" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K107" s="16"/>
@@ -4673,11 +4733,11 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J108" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K108" s="16"/>
@@ -4695,11 +4755,11 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J109" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K109" s="16"/>
@@ -4717,11 +4777,11 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J110" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K110" s="16"/>
@@ -4739,11 +4799,11 @@
       <c r="G111" s="14"/>
       <c r="H111" s="14"/>
       <c r="I111" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J111" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K111" s="16"/>
@@ -4761,11 +4821,11 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J112" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K112" s="16"/>
@@ -4783,11 +4843,11 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J113" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K113" s="16"/>
@@ -4805,11 +4865,11 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J114" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K114" s="16"/>
@@ -4827,11 +4887,11 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J115" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K115" s="16"/>
@@ -4849,11 +4909,11 @@
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
       <c r="I116" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J116" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K116" s="16"/>
@@ -4871,11 +4931,11 @@
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
       <c r="I117" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J117" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K117" s="16"/>
@@ -4893,11 +4953,11 @@
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
       <c r="I118" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J118" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K118" s="16"/>
@@ -4915,11 +4975,11 @@
       <c r="G119" s="14"/>
       <c r="H119" s="14"/>
       <c r="I119" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J119" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K119" s="16"/>
@@ -4937,11 +4997,11 @@
       <c r="G120" s="14"/>
       <c r="H120" s="14"/>
       <c r="I120" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J120" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K120" s="16"/>
@@ -4959,11 +5019,11 @@
       <c r="G121" s="14"/>
       <c r="H121" s="14"/>
       <c r="I121" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J121" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K121" s="16"/>
@@ -4981,11 +5041,11 @@
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
       <c r="I122" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J122" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K122" s="16"/>
@@ -5003,11 +5063,11 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J123" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K123" s="16"/>
@@ -5025,11 +5085,11 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J124" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K124" s="16"/>
@@ -5047,11 +5107,11 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J125" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K125" s="16"/>
@@ -5069,11 +5129,11 @@
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
       <c r="I126" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J126" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K126" s="16"/>
@@ -5091,11 +5151,11 @@
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J127" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K127" s="16"/>
@@ -5113,11 +5173,11 @@
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
       <c r="I128" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J128" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K128" s="16"/>
@@ -5135,11 +5195,11 @@
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
       <c r="I129" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J129" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K129" s="16"/>
@@ -5157,11 +5217,11 @@
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
       <c r="I130" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J130" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K130" s="16"/>
@@ -5179,11 +5239,11 @@
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
       <c r="I131" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J131" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K131" s="16"/>
@@ -5201,11 +5261,11 @@
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
       <c r="I132" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J132" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K132" s="16"/>
@@ -5223,11 +5283,11 @@
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
       <c r="I133" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J133" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K133" s="16"/>
@@ -5245,11 +5305,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="6">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" ref="I134:I197" si="8">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="7">IF(I134="","",1440-I134)</f>
+        <f t="shared" ref="J134:J197" si="9">IF(I134="","",1440-I134)</f>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -5267,11 +5327,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5289,11 +5349,11 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J136" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K136" s="16"/>
@@ -5311,11 +5371,11 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J137" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K137" s="16"/>
@@ -5333,11 +5393,11 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J138" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K138" s="16"/>
@@ -5355,11 +5415,11 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J139" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K139" s="16"/>
@@ -5377,11 +5437,11 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J140" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K140" s="16"/>
@@ -5399,11 +5459,11 @@
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J141" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K141" s="16"/>
@@ -5421,11 +5481,11 @@
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J142" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K142" s="16"/>
@@ -5443,11 +5503,11 @@
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J143" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K143" s="16"/>
@@ -5465,11 +5525,11 @@
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J144" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K144" s="16"/>
@@ -5487,11 +5547,11 @@
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J145" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K145" s="16"/>
@@ -5509,11 +5569,11 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J146" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K146" s="16"/>
@@ -5531,11 +5591,11 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J147" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K147" s="16"/>
@@ -5553,11 +5613,11 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J148" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K148" s="16"/>
@@ -5575,11 +5635,11 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J149" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K149" s="16"/>
@@ -5597,11 +5657,11 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J150" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K150" s="16"/>
@@ -5619,11 +5679,11 @@
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
       <c r="I151" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J151" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K151" s="16"/>
@@ -5641,11 +5701,11 @@
       <c r="G152" s="14"/>
       <c r="H152" s="14"/>
       <c r="I152" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J152" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K152" s="16"/>
@@ -5663,11 +5723,11 @@
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J153" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K153" s="16"/>
@@ -5685,11 +5745,11 @@
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J154" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K154" s="16"/>
@@ -5707,11 +5767,11 @@
       <c r="G155" s="14"/>
       <c r="H155" s="14"/>
       <c r="I155" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J155" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K155" s="16"/>
@@ -5729,11 +5789,11 @@
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
       <c r="I156" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J156" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K156" s="16"/>
@@ -5751,11 +5811,11 @@
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J157" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K157" s="16"/>
@@ -5773,11 +5833,11 @@
       <c r="G158" s="14"/>
       <c r="H158" s="14"/>
       <c r="I158" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J158" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K158" s="16"/>
@@ -5795,11 +5855,11 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J159" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K159" s="16"/>
@@ -5817,11 +5877,11 @@
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
       <c r="I160" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J160" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K160" s="16"/>
@@ -5839,11 +5899,11 @@
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
       <c r="I161" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J161" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K161" s="16"/>
@@ -5861,11 +5921,11 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J162" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K162" s="16"/>
@@ -5883,11 +5943,11 @@
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
       <c r="I163" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J163" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K163" s="16"/>
@@ -5905,11 +5965,11 @@
       <c r="G164" s="14"/>
       <c r="H164" s="14"/>
       <c r="I164" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J164" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K164" s="16"/>
@@ -5927,11 +5987,11 @@
       <c r="G165" s="14"/>
       <c r="H165" s="14"/>
       <c r="I165" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J165" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K165" s="16"/>
@@ -5949,11 +6009,11 @@
       <c r="G166" s="14"/>
       <c r="H166" s="14"/>
       <c r="I166" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J166" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K166" s="16"/>
@@ -5971,11 +6031,11 @@
       <c r="G167" s="14"/>
       <c r="H167" s="14"/>
       <c r="I167" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J167" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K167" s="16"/>
@@ -5993,11 +6053,11 @@
       <c r="G168" s="14"/>
       <c r="H168" s="14"/>
       <c r="I168" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J168" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K168" s="16"/>
@@ -6015,11 +6075,11 @@
       <c r="G169" s="14"/>
       <c r="H169" s="14"/>
       <c r="I169" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J169" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K169" s="16"/>
@@ -6037,11 +6097,11 @@
       <c r="G170" s="14"/>
       <c r="H170" s="14"/>
       <c r="I170" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J170" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K170" s="16"/>
@@ -6059,11 +6119,11 @@
       <c r="G171" s="14"/>
       <c r="H171" s="14"/>
       <c r="I171" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J171" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K171" s="16"/>
@@ -6081,11 +6141,11 @@
       <c r="G172" s="14"/>
       <c r="H172" s="14"/>
       <c r="I172" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J172" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K172" s="16"/>
@@ -6103,11 +6163,11 @@
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
       <c r="I173" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J173" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K173" s="16"/>
@@ -6125,11 +6185,11 @@
       <c r="G174" s="14"/>
       <c r="H174" s="14"/>
       <c r="I174" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J174" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K174" s="16"/>
@@ -6147,11 +6207,11 @@
       <c r="G175" s="14"/>
       <c r="H175" s="14"/>
       <c r="I175" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J175" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K175" s="16"/>
@@ -6169,11 +6229,11 @@
       <c r="G176" s="14"/>
       <c r="H176" s="14"/>
       <c r="I176" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J176" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K176" s="16"/>
@@ -6191,11 +6251,11 @@
       <c r="G177" s="14"/>
       <c r="H177" s="14"/>
       <c r="I177" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J177" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K177" s="16"/>
@@ -6213,11 +6273,11 @@
       <c r="G178" s="14"/>
       <c r="H178" s="14"/>
       <c r="I178" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J178" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K178" s="16"/>
@@ -6235,11 +6295,11 @@
       <c r="G179" s="14"/>
       <c r="H179" s="14"/>
       <c r="I179" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J179" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K179" s="16"/>
@@ -6257,11 +6317,11 @@
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
       <c r="I180" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J180" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K180" s="16"/>
@@ -6279,11 +6339,11 @@
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J181" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K181" s="16"/>
@@ -6301,11 +6361,11 @@
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J182" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K182" s="16"/>
@@ -6323,11 +6383,11 @@
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J183" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K183" s="16"/>
@@ -6345,11 +6405,11 @@
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
       <c r="I184" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J184" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K184" s="16"/>
@@ -6367,11 +6427,11 @@
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
       <c r="I185" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J185" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K185" s="16"/>
@@ -6389,11 +6449,11 @@
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J186" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K186" s="16"/>
@@ -6411,11 +6471,11 @@
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J187" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K187" s="16"/>
@@ -6433,11 +6493,11 @@
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
       <c r="I188" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J188" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K188" s="16"/>
@@ -6455,11 +6515,11 @@
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
       <c r="I189" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J189" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K189" s="16"/>
@@ -6477,11 +6537,11 @@
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J190" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K190" s="16"/>
@@ -6499,11 +6559,11 @@
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J191" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K191" s="16"/>
@@ -6521,11 +6581,11 @@
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J192" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K192" s="16"/>
@@ -6543,11 +6603,11 @@
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
       <c r="I193" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J193" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K193" s="16"/>
@@ -6565,11 +6625,11 @@
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
       <c r="I194" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J194" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K194" s="16"/>
@@ -6587,11 +6647,11 @@
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J195" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K195" s="16"/>
@@ -6609,11 +6669,11 @@
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J196" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K196" s="16"/>
@@ -6631,11 +6691,11 @@
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J197" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K197" s="16"/>
@@ -6653,11 +6713,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="8">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" ref="I198:I261" si="10">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="9">IF(I198="","",1440-I198)</f>
+        <f t="shared" ref="J198:J261" si="11">IF(I198="","",1440-I198)</f>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -6675,11 +6735,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -6697,11 +6757,11 @@
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J200" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K200" s="16"/>
@@ -6719,11 +6779,11 @@
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
       <c r="I201" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J201" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K201" s="16"/>
@@ -6741,11 +6801,11 @@
       <c r="G202" s="14"/>
       <c r="H202" s="14"/>
       <c r="I202" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J202" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K202" s="16"/>
@@ -6763,11 +6823,11 @@
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
       <c r="I203" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J203" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K203" s="16"/>
@@ -6785,11 +6845,11 @@
       <c r="G204" s="14"/>
       <c r="H204" s="14"/>
       <c r="I204" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J204" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K204" s="16"/>
@@ -6807,11 +6867,11 @@
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J205" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K205" s="16"/>
@@ -6829,11 +6889,11 @@
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J206" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K206" s="16"/>
@@ -6851,11 +6911,11 @@
       <c r="G207" s="14"/>
       <c r="H207" s="14"/>
       <c r="I207" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J207" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K207" s="16"/>
@@ -6873,11 +6933,11 @@
       <c r="G208" s="14"/>
       <c r="H208" s="14"/>
       <c r="I208" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J208" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K208" s="16"/>
@@ -6895,11 +6955,11 @@
       <c r="G209" s="14"/>
       <c r="H209" s="14"/>
       <c r="I209" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J209" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K209" s="16"/>
@@ -6917,11 +6977,11 @@
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J210" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K210" s="16"/>
@@ -6939,11 +6999,11 @@
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J211" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K211" s="16"/>
@@ -6961,11 +7021,11 @@
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J212" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K212" s="16"/>
@@ -6983,11 +7043,11 @@
       <c r="G213" s="14"/>
       <c r="H213" s="14"/>
       <c r="I213" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J213" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K213" s="16"/>
@@ -7005,11 +7065,11 @@
       <c r="G214" s="14"/>
       <c r="H214" s="14"/>
       <c r="I214" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J214" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K214" s="16"/>
@@ -7027,11 +7087,11 @@
       <c r="G215" s="14"/>
       <c r="H215" s="14"/>
       <c r="I215" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J215" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K215" s="16"/>
@@ -7049,11 +7109,11 @@
       <c r="G216" s="14"/>
       <c r="H216" s="14"/>
       <c r="I216" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J216" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K216" s="16"/>
@@ -7071,11 +7131,11 @@
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J217" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K217" s="16"/>
@@ -7093,11 +7153,11 @@
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J218" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K218" s="16"/>
@@ -7115,11 +7175,11 @@
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J219" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K219" s="16"/>
@@ -7137,11 +7197,11 @@
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J220" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K220" s="16"/>
@@ -7159,11 +7219,11 @@
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J221" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K221" s="16"/>
@@ -7181,11 +7241,11 @@
       <c r="G222" s="14"/>
       <c r="H222" s="14"/>
       <c r="I222" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J222" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K222" s="16"/>
@@ -7203,11 +7263,11 @@
       <c r="G223" s="14"/>
       <c r="H223" s="14"/>
       <c r="I223" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J223" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K223" s="16"/>
@@ -7225,11 +7285,11 @@
       <c r="G224" s="14"/>
       <c r="H224" s="14"/>
       <c r="I224" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J224" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K224" s="16"/>
@@ -7247,11 +7307,11 @@
       <c r="G225" s="14"/>
       <c r="H225" s="14"/>
       <c r="I225" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J225" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K225" s="16"/>
@@ -7269,11 +7329,11 @@
       <c r="G226" s="14"/>
       <c r="H226" s="14"/>
       <c r="I226" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J226" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K226" s="16"/>
@@ -7291,11 +7351,11 @@
       <c r="G227" s="14"/>
       <c r="H227" s="14"/>
       <c r="I227" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J227" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K227" s="16"/>
@@ -7313,11 +7373,11 @@
       <c r="G228" s="14"/>
       <c r="H228" s="14"/>
       <c r="I228" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J228" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K228" s="16"/>
@@ -7335,11 +7395,11 @@
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J229" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K229" s="16"/>
@@ -7357,11 +7417,11 @@
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J230" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K230" s="16"/>
@@ -7379,11 +7439,11 @@
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
       <c r="I231" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J231" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K231" s="16"/>
@@ -7401,11 +7461,11 @@
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
       <c r="I232" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J232" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K232" s="16"/>
@@ -7423,11 +7483,11 @@
       <c r="G233" s="14"/>
       <c r="H233" s="14"/>
       <c r="I233" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J233" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K233" s="16"/>
@@ -7445,11 +7505,11 @@
       <c r="G234" s="14"/>
       <c r="H234" s="14"/>
       <c r="I234" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J234" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K234" s="16"/>
@@ -7467,11 +7527,11 @@
       <c r="G235" s="14"/>
       <c r="H235" s="14"/>
       <c r="I235" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J235" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K235" s="16"/>
@@ -7489,11 +7549,11 @@
       <c r="G236" s="14"/>
       <c r="H236" s="14"/>
       <c r="I236" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J236" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K236" s="16"/>
@@ -7511,11 +7571,11 @@
       <c r="G237" s="14"/>
       <c r="H237" s="14"/>
       <c r="I237" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J237" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K237" s="16"/>
@@ -7533,11 +7593,11 @@
       <c r="G238" s="14"/>
       <c r="H238" s="14"/>
       <c r="I238" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J238" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K238" s="16"/>
@@ -7555,11 +7615,11 @@
       <c r="G239" s="14"/>
       <c r="H239" s="14"/>
       <c r="I239" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J239" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K239" s="16"/>
@@ -7577,11 +7637,11 @@
       <c r="G240" s="14"/>
       <c r="H240" s="14"/>
       <c r="I240" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J240" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K240" s="16"/>
@@ -7599,11 +7659,11 @@
       <c r="G241" s="14"/>
       <c r="H241" s="14"/>
       <c r="I241" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J241" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K241" s="16"/>
@@ -7621,11 +7681,11 @@
       <c r="G242" s="14"/>
       <c r="H242" s="14"/>
       <c r="I242" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J242" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K242" s="16"/>
@@ -7643,11 +7703,11 @@
       <c r="G243" s="14"/>
       <c r="H243" s="14"/>
       <c r="I243" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J243" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K243" s="16"/>
@@ -7665,11 +7725,11 @@
       <c r="G244" s="14"/>
       <c r="H244" s="14"/>
       <c r="I244" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J244" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K244" s="16"/>
@@ -7687,11 +7747,11 @@
       <c r="G245" s="14"/>
       <c r="H245" s="14"/>
       <c r="I245" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J245" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K245" s="16"/>
@@ -7709,11 +7769,11 @@
       <c r="G246" s="14"/>
       <c r="H246" s="14"/>
       <c r="I246" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J246" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K246" s="16"/>
@@ -7731,11 +7791,11 @@
       <c r="G247" s="14"/>
       <c r="H247" s="14"/>
       <c r="I247" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J247" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K247" s="16"/>
@@ -7753,11 +7813,11 @@
       <c r="G248" s="14"/>
       <c r="H248" s="14"/>
       <c r="I248" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J248" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K248" s="16"/>
@@ -7775,11 +7835,11 @@
       <c r="G249" s="14"/>
       <c r="H249" s="14"/>
       <c r="I249" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J249" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K249" s="16"/>
@@ -7797,11 +7857,11 @@
       <c r="G250" s="14"/>
       <c r="H250" s="14"/>
       <c r="I250" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J250" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K250" s="16"/>
@@ -7819,11 +7879,11 @@
       <c r="G251" s="14"/>
       <c r="H251" s="14"/>
       <c r="I251" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J251" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K251" s="16"/>
@@ -7841,11 +7901,11 @@
       <c r="G252" s="14"/>
       <c r="H252" s="14"/>
       <c r="I252" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J252" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K252" s="16"/>
@@ -7863,11 +7923,11 @@
       <c r="G253" s="14"/>
       <c r="H253" s="14"/>
       <c r="I253" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J253" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K253" s="16"/>
@@ -7885,11 +7945,11 @@
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
       <c r="I254" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J254" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K254" s="16"/>
@@ -7907,11 +7967,11 @@
       <c r="G255" s="14"/>
       <c r="H255" s="14"/>
       <c r="I255" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J255" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K255" s="16"/>
@@ -7929,11 +7989,11 @@
       <c r="G256" s="14"/>
       <c r="H256" s="14"/>
       <c r="I256" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J256" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K256" s="16"/>
@@ -7951,11 +8011,11 @@
       <c r="G257" s="14"/>
       <c r="H257" s="14"/>
       <c r="I257" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J257" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K257" s="16"/>
@@ -7973,11 +8033,11 @@
       <c r="G258" s="14"/>
       <c r="H258" s="14"/>
       <c r="I258" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J258" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K258" s="16"/>
@@ -7995,11 +8055,11 @@
       <c r="G259" s="14"/>
       <c r="H259" s="14"/>
       <c r="I259" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J259" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K259" s="16"/>
@@ -8017,11 +8077,11 @@
       <c r="G260" s="14"/>
       <c r="H260" s="14"/>
       <c r="I260" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J260" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K260" s="16"/>
@@ -8039,11 +8099,11 @@
       <c r="G261" s="14"/>
       <c r="H261" s="14"/>
       <c r="I261" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J261" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K261" s="16"/>
@@ -8061,11 +8121,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="10">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" ref="I262:I325" si="12">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="11">IF(I262="","",1440-I262)</f>
+        <f t="shared" ref="J262:J325" si="13">IF(I262="","",1440-I262)</f>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -8083,11 +8143,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8105,11 +8165,11 @@
       <c r="G264" s="14"/>
       <c r="H264" s="14"/>
       <c r="I264" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J264" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K264" s="16"/>
@@ -8127,11 +8187,11 @@
       <c r="G265" s="14"/>
       <c r="H265" s="14"/>
       <c r="I265" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J265" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K265" s="16"/>
@@ -8149,11 +8209,11 @@
       <c r="G266" s="14"/>
       <c r="H266" s="14"/>
       <c r="I266" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J266" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K266" s="16"/>
@@ -8171,11 +8231,11 @@
       <c r="G267" s="14"/>
       <c r="H267" s="14"/>
       <c r="I267" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J267" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K267" s="16"/>
@@ -8193,11 +8253,11 @@
       <c r="G268" s="14"/>
       <c r="H268" s="14"/>
       <c r="I268" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J268" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K268" s="16"/>
@@ -8215,11 +8275,11 @@
       <c r="G269" s="14"/>
       <c r="H269" s="14"/>
       <c r="I269" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J269" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K269" s="16"/>
@@ -8237,11 +8297,11 @@
       <c r="G270" s="14"/>
       <c r="H270" s="14"/>
       <c r="I270" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J270" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K270" s="16"/>
@@ -8259,11 +8319,11 @@
       <c r="G271" s="14"/>
       <c r="H271" s="14"/>
       <c r="I271" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J271" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K271" s="16"/>
@@ -8281,11 +8341,11 @@
       <c r="G272" s="14"/>
       <c r="H272" s="14"/>
       <c r="I272" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J272" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K272" s="16"/>
@@ -8303,11 +8363,11 @@
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
       <c r="I273" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J273" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K273" s="16"/>
@@ -8325,11 +8385,11 @@
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
       <c r="I274" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J274" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K274" s="16"/>
@@ -8347,11 +8407,11 @@
       <c r="G275" s="14"/>
       <c r="H275" s="14"/>
       <c r="I275" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J275" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K275" s="16"/>
@@ -8369,11 +8429,11 @@
       <c r="G276" s="14"/>
       <c r="H276" s="14"/>
       <c r="I276" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J276" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K276" s="16"/>
@@ -8391,11 +8451,11 @@
       <c r="G277" s="14"/>
       <c r="H277" s="14"/>
       <c r="I277" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J277" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K277" s="16"/>
@@ -8413,11 +8473,11 @@
       <c r="G278" s="14"/>
       <c r="H278" s="14"/>
       <c r="I278" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J278" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K278" s="16"/>
@@ -8435,11 +8495,11 @@
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
       <c r="I279" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J279" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K279" s="16"/>
@@ -8457,11 +8517,11 @@
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
       <c r="I280" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J280" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K280" s="16"/>
@@ -8479,11 +8539,11 @@
       <c r="G281" s="14"/>
       <c r="H281" s="14"/>
       <c r="I281" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J281" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K281" s="16"/>
@@ -8501,11 +8561,11 @@
       <c r="G282" s="14"/>
       <c r="H282" s="14"/>
       <c r="I282" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J282" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K282" s="16"/>
@@ -8523,11 +8583,11 @@
       <c r="G283" s="14"/>
       <c r="H283" s="14"/>
       <c r="I283" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J283" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K283" s="16"/>
@@ -8545,11 +8605,11 @@
       <c r="G284" s="14"/>
       <c r="H284" s="14"/>
       <c r="I284" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J284" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K284" s="16"/>
@@ -8567,11 +8627,11 @@
       <c r="G285" s="14"/>
       <c r="H285" s="14"/>
       <c r="I285" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J285" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K285" s="16"/>
@@ -8589,11 +8649,11 @@
       <c r="G286" s="14"/>
       <c r="H286" s="14"/>
       <c r="I286" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J286" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K286" s="16"/>
@@ -8611,11 +8671,11 @@
       <c r="G287" s="14"/>
       <c r="H287" s="14"/>
       <c r="I287" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J287" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K287" s="16"/>
@@ -8633,11 +8693,11 @@
       <c r="G288" s="14"/>
       <c r="H288" s="14"/>
       <c r="I288" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J288" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K288" s="16"/>
@@ -8655,11 +8715,11 @@
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
       <c r="I289" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J289" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K289" s="16"/>
@@ -8677,11 +8737,11 @@
       <c r="G290" s="14"/>
       <c r="H290" s="14"/>
       <c r="I290" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J290" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K290" s="16"/>
@@ -8699,11 +8759,11 @@
       <c r="G291" s="14"/>
       <c r="H291" s="14"/>
       <c r="I291" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J291" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K291" s="16"/>
@@ -8721,11 +8781,11 @@
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
       <c r="I292" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J292" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K292" s="16"/>
@@ -8743,11 +8803,11 @@
       <c r="G293" s="14"/>
       <c r="H293" s="14"/>
       <c r="I293" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J293" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K293" s="16"/>
@@ -8765,11 +8825,11 @@
       <c r="G294" s="14"/>
       <c r="H294" s="14"/>
       <c r="I294" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J294" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K294" s="16"/>
@@ -8787,11 +8847,11 @@
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
       <c r="I295" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J295" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K295" s="16"/>
@@ -8809,11 +8869,11 @@
       <c r="G296" s="14"/>
       <c r="H296" s="14"/>
       <c r="I296" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J296" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K296" s="16"/>
@@ -8831,11 +8891,11 @@
       <c r="G297" s="14"/>
       <c r="H297" s="14"/>
       <c r="I297" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J297" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K297" s="16"/>
@@ -8853,11 +8913,11 @@
       <c r="G298" s="14"/>
       <c r="H298" s="14"/>
       <c r="I298" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J298" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K298" s="16"/>
@@ -8875,11 +8935,11 @@
       <c r="G299" s="14"/>
       <c r="H299" s="14"/>
       <c r="I299" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J299" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K299" s="16"/>
@@ -8897,11 +8957,11 @@
       <c r="G300" s="14"/>
       <c r="H300" s="14"/>
       <c r="I300" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J300" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K300" s="16"/>
@@ -8919,11 +8979,11 @@
       <c r="G301" s="14"/>
       <c r="H301" s="14"/>
       <c r="I301" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J301" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K301" s="16"/>
@@ -8941,11 +9001,11 @@
       <c r="G302" s="14"/>
       <c r="H302" s="14"/>
       <c r="I302" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J302" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K302" s="16"/>
@@ -8963,11 +9023,11 @@
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
       <c r="I303" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J303" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K303" s="16"/>
@@ -8985,11 +9045,11 @@
       <c r="G304" s="14"/>
       <c r="H304" s="14"/>
       <c r="I304" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J304" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K304" s="16"/>
@@ -9007,11 +9067,11 @@
       <c r="G305" s="14"/>
       <c r="H305" s="14"/>
       <c r="I305" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J305" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K305" s="16"/>
@@ -9029,11 +9089,11 @@
       <c r="G306" s="14"/>
       <c r="H306" s="14"/>
       <c r="I306" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J306" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K306" s="16"/>
@@ -9051,11 +9111,11 @@
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
       <c r="I307" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J307" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K307" s="16"/>
@@ -9073,11 +9133,11 @@
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
       <c r="I308" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J308" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K308" s="16"/>
@@ -9095,11 +9155,11 @@
       <c r="G309" s="14"/>
       <c r="H309" s="14"/>
       <c r="I309" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J309" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K309" s="16"/>
@@ -9117,11 +9177,11 @@
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
       <c r="I310" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J310" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K310" s="16"/>
@@ -9139,11 +9199,11 @@
       <c r="G311" s="14"/>
       <c r="H311" s="14"/>
       <c r="I311" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J311" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K311" s="16"/>
@@ -9161,11 +9221,11 @@
       <c r="G312" s="14"/>
       <c r="H312" s="14"/>
       <c r="I312" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J312" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K312" s="16"/>
@@ -9183,11 +9243,11 @@
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
       <c r="I313" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J313" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K313" s="16"/>
@@ -9205,11 +9265,11 @@
       <c r="G314" s="14"/>
       <c r="H314" s="14"/>
       <c r="I314" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J314" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K314" s="16"/>
@@ -9227,11 +9287,11 @@
       <c r="G315" s="14"/>
       <c r="H315" s="14"/>
       <c r="I315" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J315" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K315" s="16"/>
@@ -9249,11 +9309,11 @@
       <c r="G316" s="14"/>
       <c r="H316" s="14"/>
       <c r="I316" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J316" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K316" s="16"/>
@@ -9271,11 +9331,11 @@
       <c r="G317" s="14"/>
       <c r="H317" s="14"/>
       <c r="I317" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J317" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K317" s="16"/>
@@ -9293,11 +9353,11 @@
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
       <c r="I318" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J318" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K318" s="16"/>
@@ -9315,11 +9375,11 @@
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
       <c r="I319" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J319" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K319" s="16"/>
@@ -9337,11 +9397,11 @@
       <c r="G320" s="14"/>
       <c r="H320" s="14"/>
       <c r="I320" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J320" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K320" s="16"/>
@@ -9359,11 +9419,11 @@
       <c r="G321" s="14"/>
       <c r="H321" s="14"/>
       <c r="I321" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J321" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K321" s="16"/>
@@ -9381,11 +9441,11 @@
       <c r="G322" s="14"/>
       <c r="H322" s="14"/>
       <c r="I322" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J322" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K322" s="16"/>
@@ -9403,11 +9463,11 @@
       <c r="G323" s="14"/>
       <c r="H323" s="14"/>
       <c r="I323" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J323" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K323" s="16"/>
@@ -9425,11 +9485,11 @@
       <c r="G324" s="14"/>
       <c r="H324" s="14"/>
       <c r="I324" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J324" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K324" s="16"/>
@@ -9447,11 +9507,11 @@
       <c r="G325" s="14"/>
       <c r="H325" s="14"/>
       <c r="I325" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J325" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K325" s="16"/>
@@ -9469,11 +9529,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="12">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" ref="I326:I389" si="14">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="13">IF(I326="","",1440-I326)</f>
+        <f t="shared" ref="J326:J389" si="15">IF(I326="","",1440-I326)</f>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -9491,11 +9551,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -9513,11 +9573,11 @@
       <c r="G328" s="14"/>
       <c r="H328" s="14"/>
       <c r="I328" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J328" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K328" s="16"/>
@@ -9535,11 +9595,11 @@
       <c r="G329" s="14"/>
       <c r="H329" s="14"/>
       <c r="I329" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J329" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K329" s="16"/>
@@ -9557,11 +9617,11 @@
       <c r="G330" s="14"/>
       <c r="H330" s="14"/>
       <c r="I330" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J330" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K330" s="16"/>
@@ -9579,11 +9639,11 @@
       <c r="G331" s="14"/>
       <c r="H331" s="14"/>
       <c r="I331" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J331" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K331" s="16"/>
@@ -9601,11 +9661,11 @@
       <c r="G332" s="14"/>
       <c r="H332" s="14"/>
       <c r="I332" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J332" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K332" s="16"/>
@@ -9623,11 +9683,11 @@
       <c r="G333" s="14"/>
       <c r="H333" s="14"/>
       <c r="I333" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J333" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K333" s="16"/>
@@ -9645,11 +9705,11 @@
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
       <c r="I334" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J334" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K334" s="16"/>
@@ -9667,11 +9727,11 @@
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
       <c r="I335" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J335" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K335" s="16"/>
@@ -9689,11 +9749,11 @@
       <c r="G336" s="14"/>
       <c r="H336" s="14"/>
       <c r="I336" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J336" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K336" s="16"/>
@@ -9711,11 +9771,11 @@
       <c r="G337" s="14"/>
       <c r="H337" s="14"/>
       <c r="I337" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J337" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K337" s="16"/>
@@ -9733,11 +9793,11 @@
       <c r="G338" s="14"/>
       <c r="H338" s="14"/>
       <c r="I338" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J338" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K338" s="16"/>
@@ -9755,11 +9815,11 @@
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
       <c r="I339" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J339" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K339" s="16"/>
@@ -9777,11 +9837,11 @@
       <c r="G340" s="14"/>
       <c r="H340" s="14"/>
       <c r="I340" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J340" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K340" s="16"/>
@@ -9799,11 +9859,11 @@
       <c r="G341" s="14"/>
       <c r="H341" s="14"/>
       <c r="I341" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J341" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K341" s="16"/>
@@ -9821,11 +9881,11 @@
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
       <c r="I342" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J342" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K342" s="16"/>
@@ -9843,11 +9903,11 @@
       <c r="G343" s="14"/>
       <c r="H343" s="14"/>
       <c r="I343" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J343" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K343" s="16"/>
@@ -9865,11 +9925,11 @@
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
       <c r="I344" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J344" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K344" s="16"/>
@@ -9887,11 +9947,11 @@
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
       <c r="I345" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J345" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K345" s="16"/>
@@ -9909,11 +9969,11 @@
       <c r="G346" s="14"/>
       <c r="H346" s="14"/>
       <c r="I346" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J346" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K346" s="16"/>
@@ -9931,11 +9991,11 @@
       <c r="G347" s="14"/>
       <c r="H347" s="14"/>
       <c r="I347" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J347" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K347" s="16"/>
@@ -9953,11 +10013,11 @@
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
       <c r="I348" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J348" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K348" s="16"/>
@@ -9975,11 +10035,11 @@
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
       <c r="I349" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J349" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K349" s="16"/>
@@ -9997,11 +10057,11 @@
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
       <c r="I350" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J350" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K350" s="16"/>
@@ -10019,11 +10079,11 @@
       <c r="G351" s="14"/>
       <c r="H351" s="14"/>
       <c r="I351" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J351" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K351" s="16"/>
@@ -10041,11 +10101,11 @@
       <c r="G352" s="14"/>
       <c r="H352" s="14"/>
       <c r="I352" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J352" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K352" s="16"/>
@@ -10063,11 +10123,11 @@
       <c r="G353" s="14"/>
       <c r="H353" s="14"/>
       <c r="I353" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J353" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K353" s="16"/>
@@ -10085,11 +10145,11 @@
       <c r="G354" s="14"/>
       <c r="H354" s="14"/>
       <c r="I354" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J354" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K354" s="16"/>
@@ -10107,11 +10167,11 @@
       <c r="G355" s="14"/>
       <c r="H355" s="14"/>
       <c r="I355" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J355" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K355" s="16"/>
@@ -10129,11 +10189,11 @@
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
       <c r="I356" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J356" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K356" s="16"/>
@@ -10151,11 +10211,11 @@
       <c r="G357" s="14"/>
       <c r="H357" s="14"/>
       <c r="I357" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J357" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K357" s="16"/>
@@ -10173,11 +10233,11 @@
       <c r="G358" s="14"/>
       <c r="H358" s="14"/>
       <c r="I358" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J358" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K358" s="16"/>
@@ -10195,11 +10255,11 @@
       <c r="G359" s="14"/>
       <c r="H359" s="14"/>
       <c r="I359" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J359" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K359" s="16"/>
@@ -10217,11 +10277,11 @@
       <c r="G360" s="14"/>
       <c r="H360" s="14"/>
       <c r="I360" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J360" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K360" s="16"/>
@@ -10239,11 +10299,11 @@
       <c r="G361" s="14"/>
       <c r="H361" s="14"/>
       <c r="I361" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J361" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K361" s="16"/>
@@ -10261,11 +10321,11 @@
       <c r="G362" s="14"/>
       <c r="H362" s="14"/>
       <c r="I362" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J362" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K362" s="16"/>
@@ -10283,11 +10343,11 @@
       <c r="G363" s="14"/>
       <c r="H363" s="14"/>
       <c r="I363" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J363" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K363" s="16"/>
@@ -10305,11 +10365,11 @@
       <c r="G364" s="14"/>
       <c r="H364" s="14"/>
       <c r="I364" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J364" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K364" s="16"/>
@@ -10327,11 +10387,11 @@
       <c r="G365" s="14"/>
       <c r="H365" s="14"/>
       <c r="I365" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J365" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K365" s="16"/>
@@ -10349,11 +10409,11 @@
       <c r="G366" s="14"/>
       <c r="H366" s="14"/>
       <c r="I366" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J366" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K366" s="16"/>
@@ -10371,11 +10431,11 @@
       <c r="G367" s="14"/>
       <c r="H367" s="14"/>
       <c r="I367" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J367" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K367" s="16"/>
@@ -10393,11 +10453,11 @@
       <c r="G368" s="14"/>
       <c r="H368" s="14"/>
       <c r="I368" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J368" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K368" s="16"/>
@@ -10415,11 +10475,11 @@
       <c r="G369" s="14"/>
       <c r="H369" s="14"/>
       <c r="I369" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J369" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K369" s="16"/>
@@ -10437,11 +10497,11 @@
       <c r="G370" s="14"/>
       <c r="H370" s="14"/>
       <c r="I370" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J370" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K370" s="16"/>
@@ -10459,11 +10519,11 @@
       <c r="G371" s="14"/>
       <c r="H371" s="14"/>
       <c r="I371" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J371" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K371" s="16"/>
@@ -10481,11 +10541,11 @@
       <c r="G372" s="14"/>
       <c r="H372" s="14"/>
       <c r="I372" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J372" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K372" s="16"/>
@@ -10503,11 +10563,11 @@
       <c r="G373" s="14"/>
       <c r="H373" s="14"/>
       <c r="I373" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J373" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K373" s="16"/>
@@ -10525,11 +10585,11 @@
       <c r="G374" s="14"/>
       <c r="H374" s="14"/>
       <c r="I374" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J374" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K374" s="16"/>
@@ -10547,11 +10607,11 @@
       <c r="G375" s="14"/>
       <c r="H375" s="14"/>
       <c r="I375" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J375" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K375" s="16"/>
@@ -10569,11 +10629,11 @@
       <c r="G376" s="14"/>
       <c r="H376" s="14"/>
       <c r="I376" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J376" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K376" s="16"/>
@@ -10591,11 +10651,11 @@
       <c r="G377" s="14"/>
       <c r="H377" s="14"/>
       <c r="I377" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J377" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K377" s="16"/>
@@ -10613,11 +10673,11 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K378" s="16"/>
@@ -10635,11 +10695,11 @@
       <c r="G379" s="14"/>
       <c r="H379" s="14"/>
       <c r="I379" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J379" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K379" s="16"/>
@@ -10657,11 +10717,11 @@
       <c r="G380" s="14"/>
       <c r="H380" s="14"/>
       <c r="I380" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J380" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K380" s="16"/>
@@ -10679,11 +10739,11 @@
       <c r="G381" s="14"/>
       <c r="H381" s="14"/>
       <c r="I381" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J381" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K381" s="16"/>
@@ -10701,11 +10761,11 @@
       <c r="G382" s="14"/>
       <c r="H382" s="14"/>
       <c r="I382" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J382" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K382" s="16"/>
@@ -10723,11 +10783,11 @@
       <c r="G383" s="14"/>
       <c r="H383" s="14"/>
       <c r="I383" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J383" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K383" s="16"/>
@@ -10745,11 +10805,11 @@
       <c r="G384" s="14"/>
       <c r="H384" s="14"/>
       <c r="I384" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J384" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K384" s="16"/>
@@ -10767,11 +10827,11 @@
       <c r="G385" s="14"/>
       <c r="H385" s="14"/>
       <c r="I385" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J385" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K385" s="16"/>
@@ -10789,11 +10849,11 @@
       <c r="G386" s="14"/>
       <c r="H386" s="14"/>
       <c r="I386" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J386" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K386" s="16"/>
@@ -10811,11 +10871,11 @@
       <c r="G387" s="14"/>
       <c r="H387" s="14"/>
       <c r="I387" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J387" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K387" s="16"/>
@@ -10833,11 +10893,11 @@
       <c r="G388" s="14"/>
       <c r="H388" s="14"/>
       <c r="I388" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J388" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K388" s="16"/>
@@ -10855,11 +10915,11 @@
       <c r="G389" s="14"/>
       <c r="H389" s="14"/>
       <c r="I389" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J389" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K389" s="16"/>
@@ -10877,11 +10937,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="14">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="16">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="15">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="17">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -10899,11 +10959,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -10921,11 +10981,11 @@
       <c r="G392" s="14"/>
       <c r="H392" s="14"/>
       <c r="I392" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J392" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K392" s="16"/>
@@ -10943,11 +11003,11 @@
       <c r="G393" s="14"/>
       <c r="H393" s="14"/>
       <c r="I393" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J393" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K393" s="16"/>
@@ -10965,11 +11025,11 @@
       <c r="G394" s="14"/>
       <c r="H394" s="14"/>
       <c r="I394" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J394" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K394" s="16"/>
@@ -10987,11 +11047,11 @@
       <c r="G395" s="14"/>
       <c r="H395" s="14"/>
       <c r="I395" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J395" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K395" s="16"/>
@@ -11009,11 +11069,11 @@
       <c r="G396" s="14"/>
       <c r="H396" s="14"/>
       <c r="I396" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J396" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K396" s="16"/>
@@ -11031,11 +11091,11 @@
       <c r="G397" s="14"/>
       <c r="H397" s="14"/>
       <c r="I397" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J397" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K397" s="16"/>
@@ -11053,11 +11113,11 @@
       <c r="G398" s="14"/>
       <c r="H398" s="14"/>
       <c r="I398" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J398" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K398" s="16"/>
@@ -11075,11 +11135,11 @@
       <c r="G399" s="14"/>
       <c r="H399" s="14"/>
       <c r="I399" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J399" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K399" s="16"/>
@@ -11097,11 +11157,11 @@
       <c r="G400" s="14"/>
       <c r="H400" s="14"/>
       <c r="I400" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J400" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K400" s="16"/>
@@ -11119,11 +11179,11 @@
       <c r="G401" s="14"/>
       <c r="H401" s="14"/>
       <c r="I401" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J401" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K401" s="16"/>
@@ -11140,6 +11200,7 @@
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="F3:G3"/>
   </mergeCells>
+  <phoneticPr fontId="12" type="noConversion"/>
   <conditionalFormatting sqref="J6:J401">
     <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
       <formula>0</formula>

</xml_diff>

<commit_message>
File Updated On 15/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4CC53BF-EC77-4128-BFE0-4A587EAD326B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95F270BB-016F-4E77-AF19-6E199FBED1AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="87">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -520,7 +520,19 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3734,26 +3746,50 @@
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A63" s="13"/>
-      <c r="B63" s="14"/>
-      <c r="C63" s="14"/>
-      <c r="D63" s="14"/>
-      <c r="E63" s="14"/>
-      <c r="F63" s="14"/>
-      <c r="G63" s="14"/>
-      <c r="H63" s="14"/>
-      <c r="I63" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J63" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K63" s="16"/>
-      <c r="L63" s="16"/>
-      <c r="M63" s="16"/>
-      <c r="N63" s="17"/>
+      <c r="A63" s="13">
+        <v>46310</v>
+      </c>
+      <c r="B63" s="14">
+        <v>480</v>
+      </c>
+      <c r="C63" s="14">
+        <v>0</v>
+      </c>
+      <c r="D63" s="14">
+        <v>150</v>
+      </c>
+      <c r="E63" s="14">
+        <v>0</v>
+      </c>
+      <c r="F63" s="14">
+        <v>0</v>
+      </c>
+      <c r="G63" s="14">
+        <v>0</v>
+      </c>
+      <c r="H63" s="14">
+        <v>250</v>
+      </c>
+      <c r="I63" s="15">
+        <f t="shared" ref="I63" si="6">IF(SUM(B63:F63,H63)=0,"",SUM(B63:F63,H63))</f>
+        <v>880</v>
+      </c>
+      <c r="J63" s="15">
+        <f t="shared" ref="J63" si="7">IF(I63="","",1440-I63)</f>
+        <v>560</v>
+      </c>
+      <c r="K63" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L63" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M63" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="N63" s="17" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="13"/>
@@ -3897,11 +3933,11 @@
       <c r="G70" s="14"/>
       <c r="H70" s="14"/>
       <c r="I70" s="15" t="str">
-        <f t="shared" ref="I70:I133" si="6">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
+        <f t="shared" ref="I70:I133" si="8">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
         <v/>
       </c>
       <c r="J70" s="15" t="str">
-        <f t="shared" ref="J70:J133" si="7">IF(I70="","",1440-I70)</f>
+        <f t="shared" ref="J70:J133" si="9">IF(I70="","",1440-I70)</f>
         <v/>
       </c>
       <c r="K70" s="16"/>
@@ -3919,11 +3955,11 @@
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
       <c r="I71" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J71" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K71" s="16"/>
@@ -3941,11 +3977,11 @@
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
       <c r="I72" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J72" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K72" s="16"/>
@@ -3963,11 +3999,11 @@
       <c r="G73" s="14"/>
       <c r="H73" s="14"/>
       <c r="I73" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J73" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K73" s="16"/>
@@ -3985,11 +4021,11 @@
       <c r="G74" s="14"/>
       <c r="H74" s="14"/>
       <c r="I74" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J74" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K74" s="16"/>
@@ -4007,11 +4043,11 @@
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
       <c r="I75" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J75" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K75" s="16"/>
@@ -4029,11 +4065,11 @@
       <c r="G76" s="14"/>
       <c r="H76" s="14"/>
       <c r="I76" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J76" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K76" s="16"/>
@@ -4051,11 +4087,11 @@
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
       <c r="I77" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J77" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K77" s="16"/>
@@ -4073,11 +4109,11 @@
       <c r="G78" s="14"/>
       <c r="H78" s="14"/>
       <c r="I78" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J78" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K78" s="16"/>
@@ -4095,11 +4131,11 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J79" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K79" s="16"/>
@@ -4117,11 +4153,11 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J80" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K80" s="16"/>
@@ -4139,11 +4175,11 @@
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J81" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K81" s="16"/>
@@ -4161,11 +4197,11 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J82" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K82" s="16"/>
@@ -4183,11 +4219,11 @@
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
       <c r="I83" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J83" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K83" s="16"/>
@@ -4205,11 +4241,11 @@
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
       <c r="I84" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J84" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K84" s="16"/>
@@ -4227,11 +4263,11 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J85" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K85" s="16"/>
@@ -4249,11 +4285,11 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J86" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K86" s="16"/>
@@ -4271,11 +4307,11 @@
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
       <c r="I87" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J87" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K87" s="16"/>
@@ -4293,11 +4329,11 @@
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
       <c r="I88" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J88" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K88" s="16"/>
@@ -4315,11 +4351,11 @@
       <c r="G89" s="14"/>
       <c r="H89" s="14"/>
       <c r="I89" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J89" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K89" s="16"/>
@@ -4337,11 +4373,11 @@
       <c r="G90" s="14"/>
       <c r="H90" s="14"/>
       <c r="I90" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J90" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K90" s="16"/>
@@ -4359,11 +4395,11 @@
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
       <c r="I91" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J91" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K91" s="16"/>
@@ -4381,11 +4417,11 @@
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
       <c r="I92" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J92" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K92" s="16"/>
@@ -4403,11 +4439,11 @@
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J93" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K93" s="16"/>
@@ -4425,11 +4461,11 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J94" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K94" s="16"/>
@@ -4447,11 +4483,11 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J95" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K95" s="16"/>
@@ -4469,11 +4505,11 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J96" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K96" s="16"/>
@@ -4491,11 +4527,11 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J97" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K97" s="16"/>
@@ -4513,11 +4549,11 @@
       <c r="G98" s="14"/>
       <c r="H98" s="14"/>
       <c r="I98" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J98" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K98" s="16"/>
@@ -4535,11 +4571,11 @@
       <c r="G99" s="14"/>
       <c r="H99" s="14"/>
       <c r="I99" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J99" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K99" s="16"/>
@@ -4557,11 +4593,11 @@
       <c r="G100" s="14"/>
       <c r="H100" s="14"/>
       <c r="I100" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J100" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K100" s="16"/>
@@ -4579,11 +4615,11 @@
       <c r="G101" s="14"/>
       <c r="H101" s="14"/>
       <c r="I101" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J101" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K101" s="16"/>
@@ -4601,11 +4637,11 @@
       <c r="G102" s="14"/>
       <c r="H102" s="14"/>
       <c r="I102" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J102" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K102" s="16"/>
@@ -4623,11 +4659,11 @@
       <c r="G103" s="14"/>
       <c r="H103" s="14"/>
       <c r="I103" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J103" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K103" s="16"/>
@@ -4645,11 +4681,11 @@
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
       <c r="I104" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J104" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K104" s="16"/>
@@ -4667,11 +4703,11 @@
       <c r="G105" s="14"/>
       <c r="H105" s="14"/>
       <c r="I105" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J105" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K105" s="16"/>
@@ -4689,11 +4725,11 @@
       <c r="G106" s="14"/>
       <c r="H106" s="14"/>
       <c r="I106" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J106" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K106" s="16"/>
@@ -4711,11 +4747,11 @@
       <c r="G107" s="14"/>
       <c r="H107" s="14"/>
       <c r="I107" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J107" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K107" s="16"/>
@@ -4733,11 +4769,11 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J108" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K108" s="16"/>
@@ -4755,11 +4791,11 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J109" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K109" s="16"/>
@@ -4777,11 +4813,11 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J110" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K110" s="16"/>
@@ -4799,11 +4835,11 @@
       <c r="G111" s="14"/>
       <c r="H111" s="14"/>
       <c r="I111" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J111" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K111" s="16"/>
@@ -4821,11 +4857,11 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J112" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K112" s="16"/>
@@ -4843,11 +4879,11 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J113" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K113" s="16"/>
@@ -4865,11 +4901,11 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J114" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K114" s="16"/>
@@ -4887,11 +4923,11 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J115" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K115" s="16"/>
@@ -4909,11 +4945,11 @@
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
       <c r="I116" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J116" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K116" s="16"/>
@@ -4931,11 +4967,11 @@
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
       <c r="I117" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J117" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K117" s="16"/>
@@ -4953,11 +4989,11 @@
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
       <c r="I118" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J118" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K118" s="16"/>
@@ -4975,11 +5011,11 @@
       <c r="G119" s="14"/>
       <c r="H119" s="14"/>
       <c r="I119" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J119" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K119" s="16"/>
@@ -4997,11 +5033,11 @@
       <c r="G120" s="14"/>
       <c r="H120" s="14"/>
       <c r="I120" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J120" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K120" s="16"/>
@@ -5019,11 +5055,11 @@
       <c r="G121" s="14"/>
       <c r="H121" s="14"/>
       <c r="I121" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J121" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K121" s="16"/>
@@ -5041,11 +5077,11 @@
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
       <c r="I122" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J122" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K122" s="16"/>
@@ -5063,11 +5099,11 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J123" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K123" s="16"/>
@@ -5085,11 +5121,11 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J124" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K124" s="16"/>
@@ -5107,11 +5143,11 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J125" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K125" s="16"/>
@@ -5129,11 +5165,11 @@
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
       <c r="I126" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J126" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K126" s="16"/>
@@ -5151,11 +5187,11 @@
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J127" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K127" s="16"/>
@@ -5173,11 +5209,11 @@
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
       <c r="I128" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J128" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K128" s="16"/>
@@ -5195,11 +5231,11 @@
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
       <c r="I129" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J129" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K129" s="16"/>
@@ -5217,11 +5253,11 @@
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
       <c r="I130" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J130" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K130" s="16"/>
@@ -5239,11 +5275,11 @@
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
       <c r="I131" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J131" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K131" s="16"/>
@@ -5261,11 +5297,11 @@
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
       <c r="I132" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J132" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K132" s="16"/>
@@ -5283,11 +5319,11 @@
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
       <c r="I133" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J133" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K133" s="16"/>
@@ -5305,11 +5341,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="8">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" ref="I134:I197" si="10">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="9">IF(I134="","",1440-I134)</f>
+        <f t="shared" ref="J134:J197" si="11">IF(I134="","",1440-I134)</f>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -5327,11 +5363,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5349,11 +5385,11 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J136" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K136" s="16"/>
@@ -5371,11 +5407,11 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J137" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K137" s="16"/>
@@ -5393,11 +5429,11 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J138" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K138" s="16"/>
@@ -5415,11 +5451,11 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J139" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K139" s="16"/>
@@ -5437,11 +5473,11 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J140" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K140" s="16"/>
@@ -5459,11 +5495,11 @@
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J141" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K141" s="16"/>
@@ -5481,11 +5517,11 @@
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J142" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K142" s="16"/>
@@ -5503,11 +5539,11 @@
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J143" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K143" s="16"/>
@@ -5525,11 +5561,11 @@
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J144" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K144" s="16"/>
@@ -5547,11 +5583,11 @@
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J145" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K145" s="16"/>
@@ -5569,11 +5605,11 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J146" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K146" s="16"/>
@@ -5591,11 +5627,11 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J147" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K147" s="16"/>
@@ -5613,11 +5649,11 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J148" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K148" s="16"/>
@@ -5635,11 +5671,11 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J149" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K149" s="16"/>
@@ -5657,11 +5693,11 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J150" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K150" s="16"/>
@@ -5679,11 +5715,11 @@
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
       <c r="I151" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J151" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K151" s="16"/>
@@ -5701,11 +5737,11 @@
       <c r="G152" s="14"/>
       <c r="H152" s="14"/>
       <c r="I152" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J152" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K152" s="16"/>
@@ -5723,11 +5759,11 @@
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J153" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K153" s="16"/>
@@ -5745,11 +5781,11 @@
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J154" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K154" s="16"/>
@@ -5767,11 +5803,11 @@
       <c r="G155" s="14"/>
       <c r="H155" s="14"/>
       <c r="I155" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J155" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K155" s="16"/>
@@ -5789,11 +5825,11 @@
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
       <c r="I156" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J156" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K156" s="16"/>
@@ -5811,11 +5847,11 @@
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J157" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K157" s="16"/>
@@ -5833,11 +5869,11 @@
       <c r="G158" s="14"/>
       <c r="H158" s="14"/>
       <c r="I158" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J158" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K158" s="16"/>
@@ -5855,11 +5891,11 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J159" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K159" s="16"/>
@@ -5877,11 +5913,11 @@
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
       <c r="I160" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J160" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K160" s="16"/>
@@ -5899,11 +5935,11 @@
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
       <c r="I161" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J161" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K161" s="16"/>
@@ -5921,11 +5957,11 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J162" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K162" s="16"/>
@@ -5943,11 +5979,11 @@
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
       <c r="I163" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J163" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K163" s="16"/>
@@ -5965,11 +6001,11 @@
       <c r="G164" s="14"/>
       <c r="H164" s="14"/>
       <c r="I164" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J164" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K164" s="16"/>
@@ -5987,11 +6023,11 @@
       <c r="G165" s="14"/>
       <c r="H165" s="14"/>
       <c r="I165" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J165" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K165" s="16"/>
@@ -6009,11 +6045,11 @@
       <c r="G166" s="14"/>
       <c r="H166" s="14"/>
       <c r="I166" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J166" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K166" s="16"/>
@@ -6031,11 +6067,11 @@
       <c r="G167" s="14"/>
       <c r="H167" s="14"/>
       <c r="I167" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J167" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K167" s="16"/>
@@ -6053,11 +6089,11 @@
       <c r="G168" s="14"/>
       <c r="H168" s="14"/>
       <c r="I168" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J168" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K168" s="16"/>
@@ -6075,11 +6111,11 @@
       <c r="G169" s="14"/>
       <c r="H169" s="14"/>
       <c r="I169" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J169" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K169" s="16"/>
@@ -6097,11 +6133,11 @@
       <c r="G170" s="14"/>
       <c r="H170" s="14"/>
       <c r="I170" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J170" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K170" s="16"/>
@@ -6119,11 +6155,11 @@
       <c r="G171" s="14"/>
       <c r="H171" s="14"/>
       <c r="I171" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J171" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K171" s="16"/>
@@ -6141,11 +6177,11 @@
       <c r="G172" s="14"/>
       <c r="H172" s="14"/>
       <c r="I172" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J172" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K172" s="16"/>
@@ -6163,11 +6199,11 @@
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
       <c r="I173" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J173" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K173" s="16"/>
@@ -6185,11 +6221,11 @@
       <c r="G174" s="14"/>
       <c r="H174" s="14"/>
       <c r="I174" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J174" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K174" s="16"/>
@@ -6207,11 +6243,11 @@
       <c r="G175" s="14"/>
       <c r="H175" s="14"/>
       <c r="I175" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J175" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K175" s="16"/>
@@ -6229,11 +6265,11 @@
       <c r="G176" s="14"/>
       <c r="H176" s="14"/>
       <c r="I176" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J176" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K176" s="16"/>
@@ -6251,11 +6287,11 @@
       <c r="G177" s="14"/>
       <c r="H177" s="14"/>
       <c r="I177" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J177" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K177" s="16"/>
@@ -6273,11 +6309,11 @@
       <c r="G178" s="14"/>
       <c r="H178" s="14"/>
       <c r="I178" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J178" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K178" s="16"/>
@@ -6295,11 +6331,11 @@
       <c r="G179" s="14"/>
       <c r="H179" s="14"/>
       <c r="I179" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J179" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K179" s="16"/>
@@ -6317,11 +6353,11 @@
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
       <c r="I180" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J180" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K180" s="16"/>
@@ -6339,11 +6375,11 @@
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J181" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K181" s="16"/>
@@ -6361,11 +6397,11 @@
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J182" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K182" s="16"/>
@@ -6383,11 +6419,11 @@
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J183" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K183" s="16"/>
@@ -6405,11 +6441,11 @@
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
       <c r="I184" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J184" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K184" s="16"/>
@@ -6427,11 +6463,11 @@
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
       <c r="I185" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J185" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K185" s="16"/>
@@ -6449,11 +6485,11 @@
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J186" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K186" s="16"/>
@@ -6471,11 +6507,11 @@
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J187" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K187" s="16"/>
@@ -6493,11 +6529,11 @@
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
       <c r="I188" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J188" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K188" s="16"/>
@@ -6515,11 +6551,11 @@
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
       <c r="I189" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J189" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K189" s="16"/>
@@ -6537,11 +6573,11 @@
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J190" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K190" s="16"/>
@@ -6559,11 +6595,11 @@
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J191" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K191" s="16"/>
@@ -6581,11 +6617,11 @@
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J192" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K192" s="16"/>
@@ -6603,11 +6639,11 @@
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
       <c r="I193" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J193" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K193" s="16"/>
@@ -6625,11 +6661,11 @@
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
       <c r="I194" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J194" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K194" s="16"/>
@@ -6647,11 +6683,11 @@
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J195" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K195" s="16"/>
@@ -6669,11 +6705,11 @@
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J196" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K196" s="16"/>
@@ -6691,11 +6727,11 @@
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J197" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K197" s="16"/>
@@ -6713,11 +6749,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="10">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" ref="I198:I261" si="12">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="11">IF(I198="","",1440-I198)</f>
+        <f t="shared" ref="J198:J261" si="13">IF(I198="","",1440-I198)</f>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -6735,11 +6771,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -6757,11 +6793,11 @@
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J200" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K200" s="16"/>
@@ -6779,11 +6815,11 @@
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
       <c r="I201" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J201" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K201" s="16"/>
@@ -6801,11 +6837,11 @@
       <c r="G202" s="14"/>
       <c r="H202" s="14"/>
       <c r="I202" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J202" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K202" s="16"/>
@@ -6823,11 +6859,11 @@
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
       <c r="I203" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J203" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K203" s="16"/>
@@ -6845,11 +6881,11 @@
       <c r="G204" s="14"/>
       <c r="H204" s="14"/>
       <c r="I204" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J204" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K204" s="16"/>
@@ -6867,11 +6903,11 @@
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J205" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K205" s="16"/>
@@ -6889,11 +6925,11 @@
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J206" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K206" s="16"/>
@@ -6911,11 +6947,11 @@
       <c r="G207" s="14"/>
       <c r="H207" s="14"/>
       <c r="I207" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J207" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K207" s="16"/>
@@ -6933,11 +6969,11 @@
       <c r="G208" s="14"/>
       <c r="H208" s="14"/>
       <c r="I208" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J208" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K208" s="16"/>
@@ -6955,11 +6991,11 @@
       <c r="G209" s="14"/>
       <c r="H209" s="14"/>
       <c r="I209" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J209" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K209" s="16"/>
@@ -6977,11 +7013,11 @@
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J210" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K210" s="16"/>
@@ -6999,11 +7035,11 @@
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J211" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K211" s="16"/>
@@ -7021,11 +7057,11 @@
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J212" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K212" s="16"/>
@@ -7043,11 +7079,11 @@
       <c r="G213" s="14"/>
       <c r="H213" s="14"/>
       <c r="I213" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J213" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K213" s="16"/>
@@ -7065,11 +7101,11 @@
       <c r="G214" s="14"/>
       <c r="H214" s="14"/>
       <c r="I214" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J214" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K214" s="16"/>
@@ -7087,11 +7123,11 @@
       <c r="G215" s="14"/>
       <c r="H215" s="14"/>
       <c r="I215" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J215" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K215" s="16"/>
@@ -7109,11 +7145,11 @@
       <c r="G216" s="14"/>
       <c r="H216" s="14"/>
       <c r="I216" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J216" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K216" s="16"/>
@@ -7131,11 +7167,11 @@
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J217" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K217" s="16"/>
@@ -7153,11 +7189,11 @@
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J218" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K218" s="16"/>
@@ -7175,11 +7211,11 @@
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J219" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K219" s="16"/>
@@ -7197,11 +7233,11 @@
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J220" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K220" s="16"/>
@@ -7219,11 +7255,11 @@
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J221" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K221" s="16"/>
@@ -7241,11 +7277,11 @@
       <c r="G222" s="14"/>
       <c r="H222" s="14"/>
       <c r="I222" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J222" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K222" s="16"/>
@@ -7263,11 +7299,11 @@
       <c r="G223" s="14"/>
       <c r="H223" s="14"/>
       <c r="I223" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J223" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K223" s="16"/>
@@ -7285,11 +7321,11 @@
       <c r="G224" s="14"/>
       <c r="H224" s="14"/>
       <c r="I224" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J224" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K224" s="16"/>
@@ -7307,11 +7343,11 @@
       <c r="G225" s="14"/>
       <c r="H225" s="14"/>
       <c r="I225" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J225" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K225" s="16"/>
@@ -7329,11 +7365,11 @@
       <c r="G226" s="14"/>
       <c r="H226" s="14"/>
       <c r="I226" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J226" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K226" s="16"/>
@@ -7351,11 +7387,11 @@
       <c r="G227" s="14"/>
       <c r="H227" s="14"/>
       <c r="I227" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J227" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K227" s="16"/>
@@ -7373,11 +7409,11 @@
       <c r="G228" s="14"/>
       <c r="H228" s="14"/>
       <c r="I228" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J228" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K228" s="16"/>
@@ -7395,11 +7431,11 @@
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J229" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K229" s="16"/>
@@ -7417,11 +7453,11 @@
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J230" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K230" s="16"/>
@@ -7439,11 +7475,11 @@
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
       <c r="I231" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J231" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K231" s="16"/>
@@ -7461,11 +7497,11 @@
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
       <c r="I232" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J232" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K232" s="16"/>
@@ -7483,11 +7519,11 @@
       <c r="G233" s="14"/>
       <c r="H233" s="14"/>
       <c r="I233" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J233" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K233" s="16"/>
@@ -7505,11 +7541,11 @@
       <c r="G234" s="14"/>
       <c r="H234" s="14"/>
       <c r="I234" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J234" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K234" s="16"/>
@@ -7527,11 +7563,11 @@
       <c r="G235" s="14"/>
       <c r="H235" s="14"/>
       <c r="I235" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J235" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K235" s="16"/>
@@ -7549,11 +7585,11 @@
       <c r="G236" s="14"/>
       <c r="H236" s="14"/>
       <c r="I236" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J236" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K236" s="16"/>
@@ -7571,11 +7607,11 @@
       <c r="G237" s="14"/>
       <c r="H237" s="14"/>
       <c r="I237" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J237" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K237" s="16"/>
@@ -7593,11 +7629,11 @@
       <c r="G238" s="14"/>
       <c r="H238" s="14"/>
       <c r="I238" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J238" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K238" s="16"/>
@@ -7615,11 +7651,11 @@
       <c r="G239" s="14"/>
       <c r="H239" s="14"/>
       <c r="I239" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J239" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K239" s="16"/>
@@ -7637,11 +7673,11 @@
       <c r="G240" s="14"/>
       <c r="H240" s="14"/>
       <c r="I240" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J240" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K240" s="16"/>
@@ -7659,11 +7695,11 @@
       <c r="G241" s="14"/>
       <c r="H241" s="14"/>
       <c r="I241" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J241" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K241" s="16"/>
@@ -7681,11 +7717,11 @@
       <c r="G242" s="14"/>
       <c r="H242" s="14"/>
       <c r="I242" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J242" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K242" s="16"/>
@@ -7703,11 +7739,11 @@
       <c r="G243" s="14"/>
       <c r="H243" s="14"/>
       <c r="I243" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J243" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K243" s="16"/>
@@ -7725,11 +7761,11 @@
       <c r="G244" s="14"/>
       <c r="H244" s="14"/>
       <c r="I244" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J244" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K244" s="16"/>
@@ -7747,11 +7783,11 @@
       <c r="G245" s="14"/>
       <c r="H245" s="14"/>
       <c r="I245" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J245" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K245" s="16"/>
@@ -7769,11 +7805,11 @@
       <c r="G246" s="14"/>
       <c r="H246" s="14"/>
       <c r="I246" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J246" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K246" s="16"/>
@@ -7791,11 +7827,11 @@
       <c r="G247" s="14"/>
       <c r="H247" s="14"/>
       <c r="I247" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J247" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K247" s="16"/>
@@ -7813,11 +7849,11 @@
       <c r="G248" s="14"/>
       <c r="H248" s="14"/>
       <c r="I248" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J248" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K248" s="16"/>
@@ -7835,11 +7871,11 @@
       <c r="G249" s="14"/>
       <c r="H249" s="14"/>
       <c r="I249" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J249" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K249" s="16"/>
@@ -7857,11 +7893,11 @@
       <c r="G250" s="14"/>
       <c r="H250" s="14"/>
       <c r="I250" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J250" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K250" s="16"/>
@@ -7879,11 +7915,11 @@
       <c r="G251" s="14"/>
       <c r="H251" s="14"/>
       <c r="I251" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J251" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K251" s="16"/>
@@ -7901,11 +7937,11 @@
       <c r="G252" s="14"/>
       <c r="H252" s="14"/>
       <c r="I252" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J252" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K252" s="16"/>
@@ -7923,11 +7959,11 @@
       <c r="G253" s="14"/>
       <c r="H253" s="14"/>
       <c r="I253" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J253" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K253" s="16"/>
@@ -7945,11 +7981,11 @@
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
       <c r="I254" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J254" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K254" s="16"/>
@@ -7967,11 +8003,11 @@
       <c r="G255" s="14"/>
       <c r="H255" s="14"/>
       <c r="I255" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J255" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K255" s="16"/>
@@ -7989,11 +8025,11 @@
       <c r="G256" s="14"/>
       <c r="H256" s="14"/>
       <c r="I256" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J256" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K256" s="16"/>
@@ -8011,11 +8047,11 @@
       <c r="G257" s="14"/>
       <c r="H257" s="14"/>
       <c r="I257" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J257" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K257" s="16"/>
@@ -8033,11 +8069,11 @@
       <c r="G258" s="14"/>
       <c r="H258" s="14"/>
       <c r="I258" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J258" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K258" s="16"/>
@@ -8055,11 +8091,11 @@
       <c r="G259" s="14"/>
       <c r="H259" s="14"/>
       <c r="I259" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J259" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K259" s="16"/>
@@ -8077,11 +8113,11 @@
       <c r="G260" s="14"/>
       <c r="H260" s="14"/>
       <c r="I260" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J260" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K260" s="16"/>
@@ -8099,11 +8135,11 @@
       <c r="G261" s="14"/>
       <c r="H261" s="14"/>
       <c r="I261" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J261" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K261" s="16"/>
@@ -8121,11 +8157,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="12">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" ref="I262:I325" si="14">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="13">IF(I262="","",1440-I262)</f>
+        <f t="shared" ref="J262:J325" si="15">IF(I262="","",1440-I262)</f>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -8143,11 +8179,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8165,11 +8201,11 @@
       <c r="G264" s="14"/>
       <c r="H264" s="14"/>
       <c r="I264" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J264" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K264" s="16"/>
@@ -8187,11 +8223,11 @@
       <c r="G265" s="14"/>
       <c r="H265" s="14"/>
       <c r="I265" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J265" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K265" s="16"/>
@@ -8209,11 +8245,11 @@
       <c r="G266" s="14"/>
       <c r="H266" s="14"/>
       <c r="I266" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J266" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K266" s="16"/>
@@ -8231,11 +8267,11 @@
       <c r="G267" s="14"/>
       <c r="H267" s="14"/>
       <c r="I267" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J267" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K267" s="16"/>
@@ -8253,11 +8289,11 @@
       <c r="G268" s="14"/>
       <c r="H268" s="14"/>
       <c r="I268" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J268" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K268" s="16"/>
@@ -8275,11 +8311,11 @@
       <c r="G269" s="14"/>
       <c r="H269" s="14"/>
       <c r="I269" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J269" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K269" s="16"/>
@@ -8297,11 +8333,11 @@
       <c r="G270" s="14"/>
       <c r="H270" s="14"/>
       <c r="I270" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J270" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K270" s="16"/>
@@ -8319,11 +8355,11 @@
       <c r="G271" s="14"/>
       <c r="H271" s="14"/>
       <c r="I271" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J271" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K271" s="16"/>
@@ -8341,11 +8377,11 @@
       <c r="G272" s="14"/>
       <c r="H272" s="14"/>
       <c r="I272" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J272" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K272" s="16"/>
@@ -8363,11 +8399,11 @@
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
       <c r="I273" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J273" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K273" s="16"/>
@@ -8385,11 +8421,11 @@
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
       <c r="I274" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J274" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K274" s="16"/>
@@ -8407,11 +8443,11 @@
       <c r="G275" s="14"/>
       <c r="H275" s="14"/>
       <c r="I275" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J275" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K275" s="16"/>
@@ -8429,11 +8465,11 @@
       <c r="G276" s="14"/>
       <c r="H276" s="14"/>
       <c r="I276" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J276" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K276" s="16"/>
@@ -8451,11 +8487,11 @@
       <c r="G277" s="14"/>
       <c r="H277" s="14"/>
       <c r="I277" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J277" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K277" s="16"/>
@@ -8473,11 +8509,11 @@
       <c r="G278" s="14"/>
       <c r="H278" s="14"/>
       <c r="I278" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J278" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K278" s="16"/>
@@ -8495,11 +8531,11 @@
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
       <c r="I279" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J279" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K279" s="16"/>
@@ -8517,11 +8553,11 @@
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
       <c r="I280" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J280" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K280" s="16"/>
@@ -8539,11 +8575,11 @@
       <c r="G281" s="14"/>
       <c r="H281" s="14"/>
       <c r="I281" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J281" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K281" s="16"/>
@@ -8561,11 +8597,11 @@
       <c r="G282" s="14"/>
       <c r="H282" s="14"/>
       <c r="I282" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J282" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K282" s="16"/>
@@ -8583,11 +8619,11 @@
       <c r="G283" s="14"/>
       <c r="H283" s="14"/>
       <c r="I283" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J283" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K283" s="16"/>
@@ -8605,11 +8641,11 @@
       <c r="G284" s="14"/>
       <c r="H284" s="14"/>
       <c r="I284" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J284" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K284" s="16"/>
@@ -8627,11 +8663,11 @@
       <c r="G285" s="14"/>
       <c r="H285" s="14"/>
       <c r="I285" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J285" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K285" s="16"/>
@@ -8649,11 +8685,11 @@
       <c r="G286" s="14"/>
       <c r="H286" s="14"/>
       <c r="I286" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J286" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K286" s="16"/>
@@ -8671,11 +8707,11 @@
       <c r="G287" s="14"/>
       <c r="H287" s="14"/>
       <c r="I287" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J287" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K287" s="16"/>
@@ -8693,11 +8729,11 @@
       <c r="G288" s="14"/>
       <c r="H288" s="14"/>
       <c r="I288" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J288" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K288" s="16"/>
@@ -8715,11 +8751,11 @@
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
       <c r="I289" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J289" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K289" s="16"/>
@@ -8737,11 +8773,11 @@
       <c r="G290" s="14"/>
       <c r="H290" s="14"/>
       <c r="I290" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J290" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K290" s="16"/>
@@ -8759,11 +8795,11 @@
       <c r="G291" s="14"/>
       <c r="H291" s="14"/>
       <c r="I291" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J291" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K291" s="16"/>
@@ -8781,11 +8817,11 @@
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
       <c r="I292" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J292" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K292" s="16"/>
@@ -8803,11 +8839,11 @@
       <c r="G293" s="14"/>
       <c r="H293" s="14"/>
       <c r="I293" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J293" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K293" s="16"/>
@@ -8825,11 +8861,11 @@
       <c r="G294" s="14"/>
       <c r="H294" s="14"/>
       <c r="I294" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J294" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K294" s="16"/>
@@ -8847,11 +8883,11 @@
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
       <c r="I295" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J295" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K295" s="16"/>
@@ -8869,11 +8905,11 @@
       <c r="G296" s="14"/>
       <c r="H296" s="14"/>
       <c r="I296" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J296" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K296" s="16"/>
@@ -8891,11 +8927,11 @@
       <c r="G297" s="14"/>
       <c r="H297" s="14"/>
       <c r="I297" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J297" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K297" s="16"/>
@@ -8913,11 +8949,11 @@
       <c r="G298" s="14"/>
       <c r="H298" s="14"/>
       <c r="I298" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J298" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K298" s="16"/>
@@ -8935,11 +8971,11 @@
       <c r="G299" s="14"/>
       <c r="H299" s="14"/>
       <c r="I299" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J299" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K299" s="16"/>
@@ -8957,11 +8993,11 @@
       <c r="G300" s="14"/>
       <c r="H300" s="14"/>
       <c r="I300" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J300" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K300" s="16"/>
@@ -8979,11 +9015,11 @@
       <c r="G301" s="14"/>
       <c r="H301" s="14"/>
       <c r="I301" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J301" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K301" s="16"/>
@@ -9001,11 +9037,11 @@
       <c r="G302" s="14"/>
       <c r="H302" s="14"/>
       <c r="I302" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J302" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K302" s="16"/>
@@ -9023,11 +9059,11 @@
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
       <c r="I303" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J303" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K303" s="16"/>
@@ -9045,11 +9081,11 @@
       <c r="G304" s="14"/>
       <c r="H304" s="14"/>
       <c r="I304" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J304" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K304" s="16"/>
@@ -9067,11 +9103,11 @@
       <c r="G305" s="14"/>
       <c r="H305" s="14"/>
       <c r="I305" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J305" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K305" s="16"/>
@@ -9089,11 +9125,11 @@
       <c r="G306" s="14"/>
       <c r="H306" s="14"/>
       <c r="I306" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J306" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K306" s="16"/>
@@ -9111,11 +9147,11 @@
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
       <c r="I307" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J307" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K307" s="16"/>
@@ -9133,11 +9169,11 @@
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
       <c r="I308" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J308" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K308" s="16"/>
@@ -9155,11 +9191,11 @@
       <c r="G309" s="14"/>
       <c r="H309" s="14"/>
       <c r="I309" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J309" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K309" s="16"/>
@@ -9177,11 +9213,11 @@
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
       <c r="I310" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J310" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K310" s="16"/>
@@ -9199,11 +9235,11 @@
       <c r="G311" s="14"/>
       <c r="H311" s="14"/>
       <c r="I311" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J311" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K311" s="16"/>
@@ -9221,11 +9257,11 @@
       <c r="G312" s="14"/>
       <c r="H312" s="14"/>
       <c r="I312" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J312" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K312" s="16"/>
@@ -9243,11 +9279,11 @@
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
       <c r="I313" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J313" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K313" s="16"/>
@@ -9265,11 +9301,11 @@
       <c r="G314" s="14"/>
       <c r="H314" s="14"/>
       <c r="I314" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J314" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K314" s="16"/>
@@ -9287,11 +9323,11 @@
       <c r="G315" s="14"/>
       <c r="H315" s="14"/>
       <c r="I315" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J315" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K315" s="16"/>
@@ -9309,11 +9345,11 @@
       <c r="G316" s="14"/>
       <c r="H316" s="14"/>
       <c r="I316" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J316" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K316" s="16"/>
@@ -9331,11 +9367,11 @@
       <c r="G317" s="14"/>
       <c r="H317" s="14"/>
       <c r="I317" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J317" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K317" s="16"/>
@@ -9353,11 +9389,11 @@
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
       <c r="I318" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J318" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K318" s="16"/>
@@ -9375,11 +9411,11 @@
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
       <c r="I319" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J319" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K319" s="16"/>
@@ -9397,11 +9433,11 @@
       <c r="G320" s="14"/>
       <c r="H320" s="14"/>
       <c r="I320" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J320" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K320" s="16"/>
@@ -9419,11 +9455,11 @@
       <c r="G321" s="14"/>
       <c r="H321" s="14"/>
       <c r="I321" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J321" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K321" s="16"/>
@@ -9441,11 +9477,11 @@
       <c r="G322" s="14"/>
       <c r="H322" s="14"/>
       <c r="I322" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J322" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K322" s="16"/>
@@ -9463,11 +9499,11 @@
       <c r="G323" s="14"/>
       <c r="H323" s="14"/>
       <c r="I323" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J323" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K323" s="16"/>
@@ -9485,11 +9521,11 @@
       <c r="G324" s="14"/>
       <c r="H324" s="14"/>
       <c r="I324" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J324" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K324" s="16"/>
@@ -9507,11 +9543,11 @@
       <c r="G325" s="14"/>
       <c r="H325" s="14"/>
       <c r="I325" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J325" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K325" s="16"/>
@@ -9529,11 +9565,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="14">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" ref="I326:I389" si="16">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="15">IF(I326="","",1440-I326)</f>
+        <f t="shared" ref="J326:J389" si="17">IF(I326="","",1440-I326)</f>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -9551,11 +9587,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -9573,11 +9609,11 @@
       <c r="G328" s="14"/>
       <c r="H328" s="14"/>
       <c r="I328" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J328" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K328" s="16"/>
@@ -9595,11 +9631,11 @@
       <c r="G329" s="14"/>
       <c r="H329" s="14"/>
       <c r="I329" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J329" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K329" s="16"/>
@@ -9617,11 +9653,11 @@
       <c r="G330" s="14"/>
       <c r="H330" s="14"/>
       <c r="I330" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J330" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K330" s="16"/>
@@ -9639,11 +9675,11 @@
       <c r="G331" s="14"/>
       <c r="H331" s="14"/>
       <c r="I331" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J331" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K331" s="16"/>
@@ -9661,11 +9697,11 @@
       <c r="G332" s="14"/>
       <c r="H332" s="14"/>
       <c r="I332" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J332" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K332" s="16"/>
@@ -9683,11 +9719,11 @@
       <c r="G333" s="14"/>
       <c r="H333" s="14"/>
       <c r="I333" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J333" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K333" s="16"/>
@@ -9705,11 +9741,11 @@
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
       <c r="I334" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J334" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K334" s="16"/>
@@ -9727,11 +9763,11 @@
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
       <c r="I335" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J335" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K335" s="16"/>
@@ -9749,11 +9785,11 @@
       <c r="G336" s="14"/>
       <c r="H336" s="14"/>
       <c r="I336" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J336" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K336" s="16"/>
@@ -9771,11 +9807,11 @@
       <c r="G337" s="14"/>
       <c r="H337" s="14"/>
       <c r="I337" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J337" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K337" s="16"/>
@@ -9793,11 +9829,11 @@
       <c r="G338" s="14"/>
       <c r="H338" s="14"/>
       <c r="I338" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J338" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K338" s="16"/>
@@ -9815,11 +9851,11 @@
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
       <c r="I339" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J339" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K339" s="16"/>
@@ -9837,11 +9873,11 @@
       <c r="G340" s="14"/>
       <c r="H340" s="14"/>
       <c r="I340" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J340" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K340" s="16"/>
@@ -9859,11 +9895,11 @@
       <c r="G341" s="14"/>
       <c r="H341" s="14"/>
       <c r="I341" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J341" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K341" s="16"/>
@@ -9881,11 +9917,11 @@
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
       <c r="I342" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J342" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K342" s="16"/>
@@ -9903,11 +9939,11 @@
       <c r="G343" s="14"/>
       <c r="H343" s="14"/>
       <c r="I343" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J343" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K343" s="16"/>
@@ -9925,11 +9961,11 @@
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
       <c r="I344" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J344" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K344" s="16"/>
@@ -9947,11 +9983,11 @@
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
       <c r="I345" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J345" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K345" s="16"/>
@@ -9969,11 +10005,11 @@
       <c r="G346" s="14"/>
       <c r="H346" s="14"/>
       <c r="I346" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J346" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K346" s="16"/>
@@ -9991,11 +10027,11 @@
       <c r="G347" s="14"/>
       <c r="H347" s="14"/>
       <c r="I347" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J347" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K347" s="16"/>
@@ -10013,11 +10049,11 @@
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
       <c r="I348" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J348" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K348" s="16"/>
@@ -10035,11 +10071,11 @@
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
       <c r="I349" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J349" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K349" s="16"/>
@@ -10057,11 +10093,11 @@
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
       <c r="I350" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J350" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K350" s="16"/>
@@ -10079,11 +10115,11 @@
       <c r="G351" s="14"/>
       <c r="H351" s="14"/>
       <c r="I351" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J351" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K351" s="16"/>
@@ -10101,11 +10137,11 @@
       <c r="G352" s="14"/>
       <c r="H352" s="14"/>
       <c r="I352" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J352" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K352" s="16"/>
@@ -10123,11 +10159,11 @@
       <c r="G353" s="14"/>
       <c r="H353" s="14"/>
       <c r="I353" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J353" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K353" s="16"/>
@@ -10145,11 +10181,11 @@
       <c r="G354" s="14"/>
       <c r="H354" s="14"/>
       <c r="I354" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J354" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K354" s="16"/>
@@ -10167,11 +10203,11 @@
       <c r="G355" s="14"/>
       <c r="H355" s="14"/>
       <c r="I355" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J355" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K355" s="16"/>
@@ -10189,11 +10225,11 @@
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
       <c r="I356" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J356" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K356" s="16"/>
@@ -10211,11 +10247,11 @@
       <c r="G357" s="14"/>
       <c r="H357" s="14"/>
       <c r="I357" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J357" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K357" s="16"/>
@@ -10233,11 +10269,11 @@
       <c r="G358" s="14"/>
       <c r="H358" s="14"/>
       <c r="I358" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J358" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K358" s="16"/>
@@ -10255,11 +10291,11 @@
       <c r="G359" s="14"/>
       <c r="H359" s="14"/>
       <c r="I359" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J359" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K359" s="16"/>
@@ -10277,11 +10313,11 @@
       <c r="G360" s="14"/>
       <c r="H360" s="14"/>
       <c r="I360" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J360" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K360" s="16"/>
@@ -10299,11 +10335,11 @@
       <c r="G361" s="14"/>
       <c r="H361" s="14"/>
       <c r="I361" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J361" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K361" s="16"/>
@@ -10321,11 +10357,11 @@
       <c r="G362" s="14"/>
       <c r="H362" s="14"/>
       <c r="I362" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J362" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K362" s="16"/>
@@ -10343,11 +10379,11 @@
       <c r="G363" s="14"/>
       <c r="H363" s="14"/>
       <c r="I363" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J363" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K363" s="16"/>
@@ -10365,11 +10401,11 @@
       <c r="G364" s="14"/>
       <c r="H364" s="14"/>
       <c r="I364" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J364" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K364" s="16"/>
@@ -10387,11 +10423,11 @@
       <c r="G365" s="14"/>
       <c r="H365" s="14"/>
       <c r="I365" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J365" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K365" s="16"/>
@@ -10409,11 +10445,11 @@
       <c r="G366" s="14"/>
       <c r="H366" s="14"/>
       <c r="I366" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J366" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K366" s="16"/>
@@ -10431,11 +10467,11 @@
       <c r="G367" s="14"/>
       <c r="H367" s="14"/>
       <c r="I367" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J367" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K367" s="16"/>
@@ -10453,11 +10489,11 @@
       <c r="G368" s="14"/>
       <c r="H368" s="14"/>
       <c r="I368" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J368" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K368" s="16"/>
@@ -10475,11 +10511,11 @@
       <c r="G369" s="14"/>
       <c r="H369" s="14"/>
       <c r="I369" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J369" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K369" s="16"/>
@@ -10497,11 +10533,11 @@
       <c r="G370" s="14"/>
       <c r="H370" s="14"/>
       <c r="I370" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J370" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K370" s="16"/>
@@ -10519,11 +10555,11 @@
       <c r="G371" s="14"/>
       <c r="H371" s="14"/>
       <c r="I371" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J371" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K371" s="16"/>
@@ -10541,11 +10577,11 @@
       <c r="G372" s="14"/>
       <c r="H372" s="14"/>
       <c r="I372" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J372" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K372" s="16"/>
@@ -10563,11 +10599,11 @@
       <c r="G373" s="14"/>
       <c r="H373" s="14"/>
       <c r="I373" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J373" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K373" s="16"/>
@@ -10585,11 +10621,11 @@
       <c r="G374" s="14"/>
       <c r="H374" s="14"/>
       <c r="I374" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J374" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K374" s="16"/>
@@ -10607,11 +10643,11 @@
       <c r="G375" s="14"/>
       <c r="H375" s="14"/>
       <c r="I375" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J375" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K375" s="16"/>
@@ -10629,11 +10665,11 @@
       <c r="G376" s="14"/>
       <c r="H376" s="14"/>
       <c r="I376" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J376" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K376" s="16"/>
@@ -10651,11 +10687,11 @@
       <c r="G377" s="14"/>
       <c r="H377" s="14"/>
       <c r="I377" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J377" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K377" s="16"/>
@@ -10673,11 +10709,11 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K378" s="16"/>
@@ -10695,11 +10731,11 @@
       <c r="G379" s="14"/>
       <c r="H379" s="14"/>
       <c r="I379" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J379" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K379" s="16"/>
@@ -10717,11 +10753,11 @@
       <c r="G380" s="14"/>
       <c r="H380" s="14"/>
       <c r="I380" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J380" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K380" s="16"/>
@@ -10739,11 +10775,11 @@
       <c r="G381" s="14"/>
       <c r="H381" s="14"/>
       <c r="I381" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J381" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K381" s="16"/>
@@ -10761,11 +10797,11 @@
       <c r="G382" s="14"/>
       <c r="H382" s="14"/>
       <c r="I382" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J382" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K382" s="16"/>
@@ -10783,11 +10819,11 @@
       <c r="G383" s="14"/>
       <c r="H383" s="14"/>
       <c r="I383" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J383" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K383" s="16"/>
@@ -10805,11 +10841,11 @@
       <c r="G384" s="14"/>
       <c r="H384" s="14"/>
       <c r="I384" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J384" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K384" s="16"/>
@@ -10827,11 +10863,11 @@
       <c r="G385" s="14"/>
       <c r="H385" s="14"/>
       <c r="I385" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J385" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K385" s="16"/>
@@ -10849,11 +10885,11 @@
       <c r="G386" s="14"/>
       <c r="H386" s="14"/>
       <c r="I386" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J386" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K386" s="16"/>
@@ -10871,11 +10907,11 @@
       <c r="G387" s="14"/>
       <c r="H387" s="14"/>
       <c r="I387" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J387" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K387" s="16"/>
@@ -10893,11 +10929,11 @@
       <c r="G388" s="14"/>
       <c r="H388" s="14"/>
       <c r="I388" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J388" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K388" s="16"/>
@@ -10915,11 +10951,11 @@
       <c r="G389" s="14"/>
       <c r="H389" s="14"/>
       <c r="I389" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J389" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K389" s="16"/>
@@ -10937,11 +10973,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="16">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="18">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="17">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="19">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -10959,11 +10995,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -10981,11 +11017,11 @@
       <c r="G392" s="14"/>
       <c r="H392" s="14"/>
       <c r="I392" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J392" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K392" s="16"/>
@@ -11003,11 +11039,11 @@
       <c r="G393" s="14"/>
       <c r="H393" s="14"/>
       <c r="I393" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J393" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K393" s="16"/>
@@ -11025,11 +11061,11 @@
       <c r="G394" s="14"/>
       <c r="H394" s="14"/>
       <c r="I394" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J394" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K394" s="16"/>
@@ -11047,11 +11083,11 @@
       <c r="G395" s="14"/>
       <c r="H395" s="14"/>
       <c r="I395" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J395" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K395" s="16"/>
@@ -11069,11 +11105,11 @@
       <c r="G396" s="14"/>
       <c r="H396" s="14"/>
       <c r="I396" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J396" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K396" s="16"/>
@@ -11091,11 +11127,11 @@
       <c r="G397" s="14"/>
       <c r="H397" s="14"/>
       <c r="I397" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J397" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K397" s="16"/>
@@ -11113,11 +11149,11 @@
       <c r="G398" s="14"/>
       <c r="H398" s="14"/>
       <c r="I398" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J398" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K398" s="16"/>
@@ -11135,11 +11171,11 @@
       <c r="G399" s="14"/>
       <c r="H399" s="14"/>
       <c r="I399" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J399" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K399" s="16"/>
@@ -11157,11 +11193,11 @@
       <c r="G400" s="14"/>
       <c r="H400" s="14"/>
       <c r="I400" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J400" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K400" s="16"/>
@@ -11179,11 +11215,11 @@
       <c r="G401" s="14"/>
       <c r="H401" s="14"/>
       <c r="I401" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J401" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K401" s="16"/>

</xml_diff>

<commit_message>
File Updated On 16/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95F270BB-016F-4E77-AF19-6E199FBED1AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF80F2EF-E5A8-4264-A468-B5665CFA7383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="88">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -297,6 +297,9 @@
   <si>
     <t>3rd mid term exam</t>
   </si>
+  <si>
+    <t>4th mid term</t>
+  </si>
 </sst>
 </file>
 
@@ -520,19 +523,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3733,7 +3724,7 @@
         <v>740</v>
       </c>
       <c r="K62" s="16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L62" s="16" t="s">
         <v>71</v>
@@ -3779,7 +3770,7 @@
         <v>560</v>
       </c>
       <c r="K63" s="16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L63" s="16" t="s">
         <v>71</v>
@@ -3792,26 +3783,50 @@
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A64" s="13"/>
-      <c r="B64" s="14"/>
-      <c r="C64" s="14"/>
-      <c r="D64" s="14"/>
-      <c r="E64" s="14"/>
-      <c r="F64" s="14"/>
-      <c r="G64" s="14"/>
-      <c r="H64" s="14"/>
-      <c r="I64" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J64" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K64" s="16"/>
-      <c r="L64" s="16"/>
-      <c r="M64" s="16"/>
-      <c r="N64" s="17"/>
+      <c r="A64" s="13">
+        <v>46311</v>
+      </c>
+      <c r="B64" s="14">
+        <v>360</v>
+      </c>
+      <c r="C64" s="14">
+        <v>0</v>
+      </c>
+      <c r="D64" s="14">
+        <v>120</v>
+      </c>
+      <c r="E64" s="14">
+        <v>0</v>
+      </c>
+      <c r="F64" s="14">
+        <v>0</v>
+      </c>
+      <c r="G64" s="14">
+        <v>0</v>
+      </c>
+      <c r="H64" s="14">
+        <v>150</v>
+      </c>
+      <c r="I64" s="15">
+        <f t="shared" ref="I64" si="8">IF(SUM(B64:F64,H64)=0,"",SUM(B64:F64,H64))</f>
+        <v>630</v>
+      </c>
+      <c r="J64" s="15">
+        <f t="shared" ref="J64" si="9">IF(I64="","",1440-I64)</f>
+        <v>810</v>
+      </c>
+      <c r="K64" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L64" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="M64" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N64" s="17" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" s="13"/>
@@ -3933,11 +3948,11 @@
       <c r="G70" s="14"/>
       <c r="H70" s="14"/>
       <c r="I70" s="15" t="str">
-        <f t="shared" ref="I70:I133" si="8">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
+        <f t="shared" ref="I70:I133" si="10">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
         <v/>
       </c>
       <c r="J70" s="15" t="str">
-        <f t="shared" ref="J70:J133" si="9">IF(I70="","",1440-I70)</f>
+        <f t="shared" ref="J70:J133" si="11">IF(I70="","",1440-I70)</f>
         <v/>
       </c>
       <c r="K70" s="16"/>
@@ -3955,11 +3970,11 @@
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
       <c r="I71" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J71" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K71" s="16"/>
@@ -3977,11 +3992,11 @@
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
       <c r="I72" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J72" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K72" s="16"/>
@@ -3999,11 +4014,11 @@
       <c r="G73" s="14"/>
       <c r="H73" s="14"/>
       <c r="I73" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J73" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K73" s="16"/>
@@ -4021,11 +4036,11 @@
       <c r="G74" s="14"/>
       <c r="H74" s="14"/>
       <c r="I74" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J74" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K74" s="16"/>
@@ -4043,11 +4058,11 @@
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
       <c r="I75" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J75" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K75" s="16"/>
@@ -4065,11 +4080,11 @@
       <c r="G76" s="14"/>
       <c r="H76" s="14"/>
       <c r="I76" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J76" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K76" s="16"/>
@@ -4087,11 +4102,11 @@
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
       <c r="I77" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J77" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K77" s="16"/>
@@ -4109,11 +4124,11 @@
       <c r="G78" s="14"/>
       <c r="H78" s="14"/>
       <c r="I78" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J78" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K78" s="16"/>
@@ -4131,11 +4146,11 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J79" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K79" s="16"/>
@@ -4153,11 +4168,11 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J80" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K80" s="16"/>
@@ -4175,11 +4190,11 @@
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J81" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K81" s="16"/>
@@ -4197,11 +4212,11 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J82" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K82" s="16"/>
@@ -4219,11 +4234,11 @@
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
       <c r="I83" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J83" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K83" s="16"/>
@@ -4241,11 +4256,11 @@
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
       <c r="I84" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J84" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K84" s="16"/>
@@ -4263,11 +4278,11 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J85" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K85" s="16"/>
@@ -4285,11 +4300,11 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J86" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K86" s="16"/>
@@ -4307,11 +4322,11 @@
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
       <c r="I87" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J87" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K87" s="16"/>
@@ -4329,11 +4344,11 @@
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
       <c r="I88" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J88" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K88" s="16"/>
@@ -4351,11 +4366,11 @@
       <c r="G89" s="14"/>
       <c r="H89" s="14"/>
       <c r="I89" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J89" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K89" s="16"/>
@@ -4373,11 +4388,11 @@
       <c r="G90" s="14"/>
       <c r="H90" s="14"/>
       <c r="I90" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J90" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K90" s="16"/>
@@ -4395,11 +4410,11 @@
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
       <c r="I91" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J91" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K91" s="16"/>
@@ -4417,11 +4432,11 @@
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
       <c r="I92" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J92" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K92" s="16"/>
@@ -4439,11 +4454,11 @@
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J93" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K93" s="16"/>
@@ -4461,11 +4476,11 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J94" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K94" s="16"/>
@@ -4483,11 +4498,11 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J95" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K95" s="16"/>
@@ -4505,11 +4520,11 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J96" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K96" s="16"/>
@@ -4527,11 +4542,11 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J97" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K97" s="16"/>
@@ -4549,11 +4564,11 @@
       <c r="G98" s="14"/>
       <c r="H98" s="14"/>
       <c r="I98" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J98" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K98" s="16"/>
@@ -4571,11 +4586,11 @@
       <c r="G99" s="14"/>
       <c r="H99" s="14"/>
       <c r="I99" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J99" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K99" s="16"/>
@@ -4593,11 +4608,11 @@
       <c r="G100" s="14"/>
       <c r="H100" s="14"/>
       <c r="I100" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J100" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K100" s="16"/>
@@ -4615,11 +4630,11 @@
       <c r="G101" s="14"/>
       <c r="H101" s="14"/>
       <c r="I101" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J101" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K101" s="16"/>
@@ -4637,11 +4652,11 @@
       <c r="G102" s="14"/>
       <c r="H102" s="14"/>
       <c r="I102" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J102" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K102" s="16"/>
@@ -4659,11 +4674,11 @@
       <c r="G103" s="14"/>
       <c r="H103" s="14"/>
       <c r="I103" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J103" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K103" s="16"/>
@@ -4681,11 +4696,11 @@
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
       <c r="I104" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J104" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K104" s="16"/>
@@ -4703,11 +4718,11 @@
       <c r="G105" s="14"/>
       <c r="H105" s="14"/>
       <c r="I105" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J105" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K105" s="16"/>
@@ -4725,11 +4740,11 @@
       <c r="G106" s="14"/>
       <c r="H106" s="14"/>
       <c r="I106" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J106" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K106" s="16"/>
@@ -4747,11 +4762,11 @@
       <c r="G107" s="14"/>
       <c r="H107" s="14"/>
       <c r="I107" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J107" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K107" s="16"/>
@@ -4769,11 +4784,11 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J108" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K108" s="16"/>
@@ -4791,11 +4806,11 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J109" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K109" s="16"/>
@@ -4813,11 +4828,11 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J110" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K110" s="16"/>
@@ -4835,11 +4850,11 @@
       <c r="G111" s="14"/>
       <c r="H111" s="14"/>
       <c r="I111" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J111" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K111" s="16"/>
@@ -4857,11 +4872,11 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J112" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K112" s="16"/>
@@ -4879,11 +4894,11 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J113" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K113" s="16"/>
@@ -4901,11 +4916,11 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J114" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K114" s="16"/>
@@ -4923,11 +4938,11 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J115" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K115" s="16"/>
@@ -4945,11 +4960,11 @@
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
       <c r="I116" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J116" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K116" s="16"/>
@@ -4967,11 +4982,11 @@
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
       <c r="I117" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J117" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K117" s="16"/>
@@ -4989,11 +5004,11 @@
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
       <c r="I118" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J118" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K118" s="16"/>
@@ -5011,11 +5026,11 @@
       <c r="G119" s="14"/>
       <c r="H119" s="14"/>
       <c r="I119" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J119" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K119" s="16"/>
@@ -5033,11 +5048,11 @@
       <c r="G120" s="14"/>
       <c r="H120" s="14"/>
       <c r="I120" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J120" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K120" s="16"/>
@@ -5055,11 +5070,11 @@
       <c r="G121" s="14"/>
       <c r="H121" s="14"/>
       <c r="I121" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J121" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K121" s="16"/>
@@ -5077,11 +5092,11 @@
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
       <c r="I122" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J122" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K122" s="16"/>
@@ -5099,11 +5114,11 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J123" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K123" s="16"/>
@@ -5121,11 +5136,11 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J124" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K124" s="16"/>
@@ -5143,11 +5158,11 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J125" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K125" s="16"/>
@@ -5165,11 +5180,11 @@
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
       <c r="I126" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J126" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K126" s="16"/>
@@ -5187,11 +5202,11 @@
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J127" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K127" s="16"/>
@@ -5209,11 +5224,11 @@
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
       <c r="I128" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J128" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K128" s="16"/>
@@ -5231,11 +5246,11 @@
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
       <c r="I129" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J129" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K129" s="16"/>
@@ -5253,11 +5268,11 @@
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
       <c r="I130" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J130" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K130" s="16"/>
@@ -5275,11 +5290,11 @@
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
       <c r="I131" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J131" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K131" s="16"/>
@@ -5297,11 +5312,11 @@
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
       <c r="I132" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J132" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K132" s="16"/>
@@ -5319,11 +5334,11 @@
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
       <c r="I133" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J133" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K133" s="16"/>
@@ -5341,11 +5356,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="10">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" ref="I134:I197" si="12">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="11">IF(I134="","",1440-I134)</f>
+        <f t="shared" ref="J134:J197" si="13">IF(I134="","",1440-I134)</f>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -5363,11 +5378,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5385,11 +5400,11 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J136" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K136" s="16"/>
@@ -5407,11 +5422,11 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J137" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K137" s="16"/>
@@ -5429,11 +5444,11 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J138" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K138" s="16"/>
@@ -5451,11 +5466,11 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J139" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K139" s="16"/>
@@ -5473,11 +5488,11 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J140" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K140" s="16"/>
@@ -5495,11 +5510,11 @@
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J141" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K141" s="16"/>
@@ -5517,11 +5532,11 @@
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J142" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K142" s="16"/>
@@ -5539,11 +5554,11 @@
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J143" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K143" s="16"/>
@@ -5561,11 +5576,11 @@
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J144" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K144" s="16"/>
@@ -5583,11 +5598,11 @@
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J145" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K145" s="16"/>
@@ -5605,11 +5620,11 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J146" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K146" s="16"/>
@@ -5627,11 +5642,11 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J147" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K147" s="16"/>
@@ -5649,11 +5664,11 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J148" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K148" s="16"/>
@@ -5671,11 +5686,11 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J149" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K149" s="16"/>
@@ -5693,11 +5708,11 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J150" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K150" s="16"/>
@@ -5715,11 +5730,11 @@
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
       <c r="I151" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J151" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K151" s="16"/>
@@ -5737,11 +5752,11 @@
       <c r="G152" s="14"/>
       <c r="H152" s="14"/>
       <c r="I152" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J152" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K152" s="16"/>
@@ -5759,11 +5774,11 @@
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J153" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K153" s="16"/>
@@ -5781,11 +5796,11 @@
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J154" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K154" s="16"/>
@@ -5803,11 +5818,11 @@
       <c r="G155" s="14"/>
       <c r="H155" s="14"/>
       <c r="I155" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J155" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K155" s="16"/>
@@ -5825,11 +5840,11 @@
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
       <c r="I156" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J156" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K156" s="16"/>
@@ -5847,11 +5862,11 @@
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J157" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K157" s="16"/>
@@ -5869,11 +5884,11 @@
       <c r="G158" s="14"/>
       <c r="H158" s="14"/>
       <c r="I158" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J158" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K158" s="16"/>
@@ -5891,11 +5906,11 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J159" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K159" s="16"/>
@@ -5913,11 +5928,11 @@
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
       <c r="I160" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J160" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K160" s="16"/>
@@ -5935,11 +5950,11 @@
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
       <c r="I161" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J161" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K161" s="16"/>
@@ -5957,11 +5972,11 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J162" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K162" s="16"/>
@@ -5979,11 +5994,11 @@
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
       <c r="I163" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J163" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K163" s="16"/>
@@ -6001,11 +6016,11 @@
       <c r="G164" s="14"/>
       <c r="H164" s="14"/>
       <c r="I164" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J164" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K164" s="16"/>
@@ -6023,11 +6038,11 @@
       <c r="G165" s="14"/>
       <c r="H165" s="14"/>
       <c r="I165" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J165" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K165" s="16"/>
@@ -6045,11 +6060,11 @@
       <c r="G166" s="14"/>
       <c r="H166" s="14"/>
       <c r="I166" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J166" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K166" s="16"/>
@@ -6067,11 +6082,11 @@
       <c r="G167" s="14"/>
       <c r="H167" s="14"/>
       <c r="I167" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J167" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K167" s="16"/>
@@ -6089,11 +6104,11 @@
       <c r="G168" s="14"/>
       <c r="H168" s="14"/>
       <c r="I168" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J168" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K168" s="16"/>
@@ -6111,11 +6126,11 @@
       <c r="G169" s="14"/>
       <c r="H169" s="14"/>
       <c r="I169" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J169" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K169" s="16"/>
@@ -6133,11 +6148,11 @@
       <c r="G170" s="14"/>
       <c r="H170" s="14"/>
       <c r="I170" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J170" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K170" s="16"/>
@@ -6155,11 +6170,11 @@
       <c r="G171" s="14"/>
       <c r="H171" s="14"/>
       <c r="I171" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J171" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K171" s="16"/>
@@ -6177,11 +6192,11 @@
       <c r="G172" s="14"/>
       <c r="H172" s="14"/>
       <c r="I172" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J172" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K172" s="16"/>
@@ -6199,11 +6214,11 @@
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
       <c r="I173" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J173" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K173" s="16"/>
@@ -6221,11 +6236,11 @@
       <c r="G174" s="14"/>
       <c r="H174" s="14"/>
       <c r="I174" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J174" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K174" s="16"/>
@@ -6243,11 +6258,11 @@
       <c r="G175" s="14"/>
       <c r="H175" s="14"/>
       <c r="I175" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J175" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K175" s="16"/>
@@ -6265,11 +6280,11 @@
       <c r="G176" s="14"/>
       <c r="H176" s="14"/>
       <c r="I176" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J176" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K176" s="16"/>
@@ -6287,11 +6302,11 @@
       <c r="G177" s="14"/>
       <c r="H177" s="14"/>
       <c r="I177" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J177" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K177" s="16"/>
@@ -6309,11 +6324,11 @@
       <c r="G178" s="14"/>
       <c r="H178" s="14"/>
       <c r="I178" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J178" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K178" s="16"/>
@@ -6331,11 +6346,11 @@
       <c r="G179" s="14"/>
       <c r="H179" s="14"/>
       <c r="I179" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J179" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K179" s="16"/>
@@ -6353,11 +6368,11 @@
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
       <c r="I180" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J180" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K180" s="16"/>
@@ -6375,11 +6390,11 @@
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J181" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K181" s="16"/>
@@ -6397,11 +6412,11 @@
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J182" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K182" s="16"/>
@@ -6419,11 +6434,11 @@
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J183" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K183" s="16"/>
@@ -6441,11 +6456,11 @@
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
       <c r="I184" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J184" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K184" s="16"/>
@@ -6463,11 +6478,11 @@
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
       <c r="I185" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J185" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K185" s="16"/>
@@ -6485,11 +6500,11 @@
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J186" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K186" s="16"/>
@@ -6507,11 +6522,11 @@
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J187" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K187" s="16"/>
@@ -6529,11 +6544,11 @@
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
       <c r="I188" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J188" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K188" s="16"/>
@@ -6551,11 +6566,11 @@
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
       <c r="I189" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J189" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K189" s="16"/>
@@ -6573,11 +6588,11 @@
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J190" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K190" s="16"/>
@@ -6595,11 +6610,11 @@
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J191" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K191" s="16"/>
@@ -6617,11 +6632,11 @@
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J192" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K192" s="16"/>
@@ -6639,11 +6654,11 @@
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
       <c r="I193" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J193" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K193" s="16"/>
@@ -6661,11 +6676,11 @@
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
       <c r="I194" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J194" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K194" s="16"/>
@@ -6683,11 +6698,11 @@
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J195" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K195" s="16"/>
@@ -6705,11 +6720,11 @@
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J196" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K196" s="16"/>
@@ -6727,11 +6742,11 @@
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J197" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K197" s="16"/>
@@ -6749,11 +6764,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="12">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" ref="I198:I261" si="14">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="13">IF(I198="","",1440-I198)</f>
+        <f t="shared" ref="J198:J261" si="15">IF(I198="","",1440-I198)</f>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -6771,11 +6786,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -6793,11 +6808,11 @@
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J200" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K200" s="16"/>
@@ -6815,11 +6830,11 @@
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
       <c r="I201" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J201" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K201" s="16"/>
@@ -6837,11 +6852,11 @@
       <c r="G202" s="14"/>
       <c r="H202" s="14"/>
       <c r="I202" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J202" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K202" s="16"/>
@@ -6859,11 +6874,11 @@
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
       <c r="I203" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J203" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K203" s="16"/>
@@ -6881,11 +6896,11 @@
       <c r="G204" s="14"/>
       <c r="H204" s="14"/>
       <c r="I204" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J204" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K204" s="16"/>
@@ -6903,11 +6918,11 @@
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J205" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K205" s="16"/>
@@ -6925,11 +6940,11 @@
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J206" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K206" s="16"/>
@@ -6947,11 +6962,11 @@
       <c r="G207" s="14"/>
       <c r="H207" s="14"/>
       <c r="I207" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J207" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K207" s="16"/>
@@ -6969,11 +6984,11 @@
       <c r="G208" s="14"/>
       <c r="H208" s="14"/>
       <c r="I208" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J208" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K208" s="16"/>
@@ -6991,11 +7006,11 @@
       <c r="G209" s="14"/>
       <c r="H209" s="14"/>
       <c r="I209" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J209" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K209" s="16"/>
@@ -7013,11 +7028,11 @@
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J210" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K210" s="16"/>
@@ -7035,11 +7050,11 @@
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J211" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K211" s="16"/>
@@ -7057,11 +7072,11 @@
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J212" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K212" s="16"/>
@@ -7079,11 +7094,11 @@
       <c r="G213" s="14"/>
       <c r="H213" s="14"/>
       <c r="I213" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J213" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K213" s="16"/>
@@ -7101,11 +7116,11 @@
       <c r="G214" s="14"/>
       <c r="H214" s="14"/>
       <c r="I214" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J214" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K214" s="16"/>
@@ -7123,11 +7138,11 @@
       <c r="G215" s="14"/>
       <c r="H215" s="14"/>
       <c r="I215" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J215" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K215" s="16"/>
@@ -7145,11 +7160,11 @@
       <c r="G216" s="14"/>
       <c r="H216" s="14"/>
       <c r="I216" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J216" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K216" s="16"/>
@@ -7167,11 +7182,11 @@
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J217" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K217" s="16"/>
@@ -7189,11 +7204,11 @@
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J218" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K218" s="16"/>
@@ -7211,11 +7226,11 @@
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J219" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K219" s="16"/>
@@ -7233,11 +7248,11 @@
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J220" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K220" s="16"/>
@@ -7255,11 +7270,11 @@
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J221" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K221" s="16"/>
@@ -7277,11 +7292,11 @@
       <c r="G222" s="14"/>
       <c r="H222" s="14"/>
       <c r="I222" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J222" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K222" s="16"/>
@@ -7299,11 +7314,11 @@
       <c r="G223" s="14"/>
       <c r="H223" s="14"/>
       <c r="I223" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J223" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K223" s="16"/>
@@ -7321,11 +7336,11 @@
       <c r="G224" s="14"/>
       <c r="H224" s="14"/>
       <c r="I224" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J224" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K224" s="16"/>
@@ -7343,11 +7358,11 @@
       <c r="G225" s="14"/>
       <c r="H225" s="14"/>
       <c r="I225" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J225" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K225" s="16"/>
@@ -7365,11 +7380,11 @@
       <c r="G226" s="14"/>
       <c r="H226" s="14"/>
       <c r="I226" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J226" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K226" s="16"/>
@@ -7387,11 +7402,11 @@
       <c r="G227" s="14"/>
       <c r="H227" s="14"/>
       <c r="I227" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J227" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K227" s="16"/>
@@ -7409,11 +7424,11 @@
       <c r="G228" s="14"/>
       <c r="H228" s="14"/>
       <c r="I228" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J228" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K228" s="16"/>
@@ -7431,11 +7446,11 @@
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J229" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K229" s="16"/>
@@ -7453,11 +7468,11 @@
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J230" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K230" s="16"/>
@@ -7475,11 +7490,11 @@
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
       <c r="I231" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J231" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K231" s="16"/>
@@ -7497,11 +7512,11 @@
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
       <c r="I232" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J232" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K232" s="16"/>
@@ -7519,11 +7534,11 @@
       <c r="G233" s="14"/>
       <c r="H233" s="14"/>
       <c r="I233" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J233" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K233" s="16"/>
@@ -7541,11 +7556,11 @@
       <c r="G234" s="14"/>
       <c r="H234" s="14"/>
       <c r="I234" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J234" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K234" s="16"/>
@@ -7563,11 +7578,11 @@
       <c r="G235" s="14"/>
       <c r="H235" s="14"/>
       <c r="I235" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J235" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K235" s="16"/>
@@ -7585,11 +7600,11 @@
       <c r="G236" s="14"/>
       <c r="H236" s="14"/>
       <c r="I236" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J236" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K236" s="16"/>
@@ -7607,11 +7622,11 @@
       <c r="G237" s="14"/>
       <c r="H237" s="14"/>
       <c r="I237" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J237" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K237" s="16"/>
@@ -7629,11 +7644,11 @@
       <c r="G238" s="14"/>
       <c r="H238" s="14"/>
       <c r="I238" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J238" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K238" s="16"/>
@@ -7651,11 +7666,11 @@
       <c r="G239" s="14"/>
       <c r="H239" s="14"/>
       <c r="I239" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J239" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K239" s="16"/>
@@ -7673,11 +7688,11 @@
       <c r="G240" s="14"/>
       <c r="H240" s="14"/>
       <c r="I240" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J240" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K240" s="16"/>
@@ -7695,11 +7710,11 @@
       <c r="G241" s="14"/>
       <c r="H241" s="14"/>
       <c r="I241" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J241" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K241" s="16"/>
@@ -7717,11 +7732,11 @@
       <c r="G242" s="14"/>
       <c r="H242" s="14"/>
       <c r="I242" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J242" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K242" s="16"/>
@@ -7739,11 +7754,11 @@
       <c r="G243" s="14"/>
       <c r="H243" s="14"/>
       <c r="I243" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J243" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K243" s="16"/>
@@ -7761,11 +7776,11 @@
       <c r="G244" s="14"/>
       <c r="H244" s="14"/>
       <c r="I244" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J244" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K244" s="16"/>
@@ -7783,11 +7798,11 @@
       <c r="G245" s="14"/>
       <c r="H245" s="14"/>
       <c r="I245" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J245" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K245" s="16"/>
@@ -7805,11 +7820,11 @@
       <c r="G246" s="14"/>
       <c r="H246" s="14"/>
       <c r="I246" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J246" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K246" s="16"/>
@@ -7827,11 +7842,11 @@
       <c r="G247" s="14"/>
       <c r="H247" s="14"/>
       <c r="I247" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J247" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K247" s="16"/>
@@ -7849,11 +7864,11 @@
       <c r="G248" s="14"/>
       <c r="H248" s="14"/>
       <c r="I248" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J248" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K248" s="16"/>
@@ -7871,11 +7886,11 @@
       <c r="G249" s="14"/>
       <c r="H249" s="14"/>
       <c r="I249" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J249" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K249" s="16"/>
@@ -7893,11 +7908,11 @@
       <c r="G250" s="14"/>
       <c r="H250" s="14"/>
       <c r="I250" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J250" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K250" s="16"/>
@@ -7915,11 +7930,11 @@
       <c r="G251" s="14"/>
       <c r="H251" s="14"/>
       <c r="I251" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J251" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K251" s="16"/>
@@ -7937,11 +7952,11 @@
       <c r="G252" s="14"/>
       <c r="H252" s="14"/>
       <c r="I252" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J252" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K252" s="16"/>
@@ -7959,11 +7974,11 @@
       <c r="G253" s="14"/>
       <c r="H253" s="14"/>
       <c r="I253" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J253" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K253" s="16"/>
@@ -7981,11 +7996,11 @@
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
       <c r="I254" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J254" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K254" s="16"/>
@@ -8003,11 +8018,11 @@
       <c r="G255" s="14"/>
       <c r="H255" s="14"/>
       <c r="I255" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J255" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K255" s="16"/>
@@ -8025,11 +8040,11 @@
       <c r="G256" s="14"/>
       <c r="H256" s="14"/>
       <c r="I256" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J256" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K256" s="16"/>
@@ -8047,11 +8062,11 @@
       <c r="G257" s="14"/>
       <c r="H257" s="14"/>
       <c r="I257" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J257" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K257" s="16"/>
@@ -8069,11 +8084,11 @@
       <c r="G258" s="14"/>
       <c r="H258" s="14"/>
       <c r="I258" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J258" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K258" s="16"/>
@@ -8091,11 +8106,11 @@
       <c r="G259" s="14"/>
       <c r="H259" s="14"/>
       <c r="I259" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J259" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K259" s="16"/>
@@ -8113,11 +8128,11 @@
       <c r="G260" s="14"/>
       <c r="H260" s="14"/>
       <c r="I260" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J260" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K260" s="16"/>
@@ -8135,11 +8150,11 @@
       <c r="G261" s="14"/>
       <c r="H261" s="14"/>
       <c r="I261" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J261" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K261" s="16"/>
@@ -8157,11 +8172,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="14">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" ref="I262:I325" si="16">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="15">IF(I262="","",1440-I262)</f>
+        <f t="shared" ref="J262:J325" si="17">IF(I262="","",1440-I262)</f>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -8179,11 +8194,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8201,11 +8216,11 @@
       <c r="G264" s="14"/>
       <c r="H264" s="14"/>
       <c r="I264" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J264" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K264" s="16"/>
@@ -8223,11 +8238,11 @@
       <c r="G265" s="14"/>
       <c r="H265" s="14"/>
       <c r="I265" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J265" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K265" s="16"/>
@@ -8245,11 +8260,11 @@
       <c r="G266" s="14"/>
       <c r="H266" s="14"/>
       <c r="I266" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J266" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K266" s="16"/>
@@ -8267,11 +8282,11 @@
       <c r="G267" s="14"/>
       <c r="H267" s="14"/>
       <c r="I267" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J267" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K267" s="16"/>
@@ -8289,11 +8304,11 @@
       <c r="G268" s="14"/>
       <c r="H268" s="14"/>
       <c r="I268" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J268" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K268" s="16"/>
@@ -8311,11 +8326,11 @@
       <c r="G269" s="14"/>
       <c r="H269" s="14"/>
       <c r="I269" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J269" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K269" s="16"/>
@@ -8333,11 +8348,11 @@
       <c r="G270" s="14"/>
       <c r="H270" s="14"/>
       <c r="I270" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J270" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K270" s="16"/>
@@ -8355,11 +8370,11 @@
       <c r="G271" s="14"/>
       <c r="H271" s="14"/>
       <c r="I271" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J271" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K271" s="16"/>
@@ -8377,11 +8392,11 @@
       <c r="G272" s="14"/>
       <c r="H272" s="14"/>
       <c r="I272" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J272" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K272" s="16"/>
@@ -8399,11 +8414,11 @@
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
       <c r="I273" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J273" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K273" s="16"/>
@@ -8421,11 +8436,11 @@
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
       <c r="I274" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J274" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K274" s="16"/>
@@ -8443,11 +8458,11 @@
       <c r="G275" s="14"/>
       <c r="H275" s="14"/>
       <c r="I275" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J275" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K275" s="16"/>
@@ -8465,11 +8480,11 @@
       <c r="G276" s="14"/>
       <c r="H276" s="14"/>
       <c r="I276" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J276" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K276" s="16"/>
@@ -8487,11 +8502,11 @@
       <c r="G277" s="14"/>
       <c r="H277" s="14"/>
       <c r="I277" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J277" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K277" s="16"/>
@@ -8509,11 +8524,11 @@
       <c r="G278" s="14"/>
       <c r="H278" s="14"/>
       <c r="I278" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J278" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K278" s="16"/>
@@ -8531,11 +8546,11 @@
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
       <c r="I279" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J279" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K279" s="16"/>
@@ -8553,11 +8568,11 @@
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
       <c r="I280" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J280" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K280" s="16"/>
@@ -8575,11 +8590,11 @@
       <c r="G281" s="14"/>
       <c r="H281" s="14"/>
       <c r="I281" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J281" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K281" s="16"/>
@@ -8597,11 +8612,11 @@
       <c r="G282" s="14"/>
       <c r="H282" s="14"/>
       <c r="I282" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J282" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K282" s="16"/>
@@ -8619,11 +8634,11 @@
       <c r="G283" s="14"/>
       <c r="H283" s="14"/>
       <c r="I283" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J283" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K283" s="16"/>
@@ -8641,11 +8656,11 @@
       <c r="G284" s="14"/>
       <c r="H284" s="14"/>
       <c r="I284" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J284" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K284" s="16"/>
@@ -8663,11 +8678,11 @@
       <c r="G285" s="14"/>
       <c r="H285" s="14"/>
       <c r="I285" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J285" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K285" s="16"/>
@@ -8685,11 +8700,11 @@
       <c r="G286" s="14"/>
       <c r="H286" s="14"/>
       <c r="I286" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J286" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K286" s="16"/>
@@ -8707,11 +8722,11 @@
       <c r="G287" s="14"/>
       <c r="H287" s="14"/>
       <c r="I287" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J287" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K287" s="16"/>
@@ -8729,11 +8744,11 @@
       <c r="G288" s="14"/>
       <c r="H288" s="14"/>
       <c r="I288" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J288" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K288" s="16"/>
@@ -8751,11 +8766,11 @@
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
       <c r="I289" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J289" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K289" s="16"/>
@@ -8773,11 +8788,11 @@
       <c r="G290" s="14"/>
       <c r="H290" s="14"/>
       <c r="I290" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J290" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K290" s="16"/>
@@ -8795,11 +8810,11 @@
       <c r="G291" s="14"/>
       <c r="H291" s="14"/>
       <c r="I291" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J291" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K291" s="16"/>
@@ -8817,11 +8832,11 @@
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
       <c r="I292" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J292" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K292" s="16"/>
@@ -8839,11 +8854,11 @@
       <c r="G293" s="14"/>
       <c r="H293" s="14"/>
       <c r="I293" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J293" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K293" s="16"/>
@@ -8861,11 +8876,11 @@
       <c r="G294" s="14"/>
       <c r="H294" s="14"/>
       <c r="I294" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J294" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K294" s="16"/>
@@ -8883,11 +8898,11 @@
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
       <c r="I295" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J295" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K295" s="16"/>
@@ -8905,11 +8920,11 @@
       <c r="G296" s="14"/>
       <c r="H296" s="14"/>
       <c r="I296" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J296" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K296" s="16"/>
@@ -8927,11 +8942,11 @@
       <c r="G297" s="14"/>
       <c r="H297" s="14"/>
       <c r="I297" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J297" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K297" s="16"/>
@@ -8949,11 +8964,11 @@
       <c r="G298" s="14"/>
       <c r="H298" s="14"/>
       <c r="I298" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J298" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K298" s="16"/>
@@ -8971,11 +8986,11 @@
       <c r="G299" s="14"/>
       <c r="H299" s="14"/>
       <c r="I299" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J299" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K299" s="16"/>
@@ -8993,11 +9008,11 @@
       <c r="G300" s="14"/>
       <c r="H300" s="14"/>
       <c r="I300" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J300" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K300" s="16"/>
@@ -9015,11 +9030,11 @@
       <c r="G301" s="14"/>
       <c r="H301" s="14"/>
       <c r="I301" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J301" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K301" s="16"/>
@@ -9037,11 +9052,11 @@
       <c r="G302" s="14"/>
       <c r="H302" s="14"/>
       <c r="I302" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J302" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K302" s="16"/>
@@ -9059,11 +9074,11 @@
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
       <c r="I303" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J303" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K303" s="16"/>
@@ -9081,11 +9096,11 @@
       <c r="G304" s="14"/>
       <c r="H304" s="14"/>
       <c r="I304" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J304" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K304" s="16"/>
@@ -9103,11 +9118,11 @@
       <c r="G305" s="14"/>
       <c r="H305" s="14"/>
       <c r="I305" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J305" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K305" s="16"/>
@@ -9125,11 +9140,11 @@
       <c r="G306" s="14"/>
       <c r="H306" s="14"/>
       <c r="I306" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J306" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K306" s="16"/>
@@ -9147,11 +9162,11 @@
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
       <c r="I307" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J307" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K307" s="16"/>
@@ -9169,11 +9184,11 @@
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
       <c r="I308" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J308" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K308" s="16"/>
@@ -9191,11 +9206,11 @@
       <c r="G309" s="14"/>
       <c r="H309" s="14"/>
       <c r="I309" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J309" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K309" s="16"/>
@@ -9213,11 +9228,11 @@
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
       <c r="I310" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J310" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K310" s="16"/>
@@ -9235,11 +9250,11 @@
       <c r="G311" s="14"/>
       <c r="H311" s="14"/>
       <c r="I311" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J311" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K311" s="16"/>
@@ -9257,11 +9272,11 @@
       <c r="G312" s="14"/>
       <c r="H312" s="14"/>
       <c r="I312" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J312" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K312" s="16"/>
@@ -9279,11 +9294,11 @@
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
       <c r="I313" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J313" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K313" s="16"/>
@@ -9301,11 +9316,11 @@
       <c r="G314" s="14"/>
       <c r="H314" s="14"/>
       <c r="I314" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J314" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K314" s="16"/>
@@ -9323,11 +9338,11 @@
       <c r="G315" s="14"/>
       <c r="H315" s="14"/>
       <c r="I315" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J315" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K315" s="16"/>
@@ -9345,11 +9360,11 @@
       <c r="G316" s="14"/>
       <c r="H316" s="14"/>
       <c r="I316" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J316" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K316" s="16"/>
@@ -9367,11 +9382,11 @@
       <c r="G317" s="14"/>
       <c r="H317" s="14"/>
       <c r="I317" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J317" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K317" s="16"/>
@@ -9389,11 +9404,11 @@
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
       <c r="I318" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J318" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K318" s="16"/>
@@ -9411,11 +9426,11 @@
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
       <c r="I319" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J319" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K319" s="16"/>
@@ -9433,11 +9448,11 @@
       <c r="G320" s="14"/>
       <c r="H320" s="14"/>
       <c r="I320" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J320" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K320" s="16"/>
@@ -9455,11 +9470,11 @@
       <c r="G321" s="14"/>
       <c r="H321" s="14"/>
       <c r="I321" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J321" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K321" s="16"/>
@@ -9477,11 +9492,11 @@
       <c r="G322" s="14"/>
       <c r="H322" s="14"/>
       <c r="I322" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J322" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K322" s="16"/>
@@ -9499,11 +9514,11 @@
       <c r="G323" s="14"/>
       <c r="H323" s="14"/>
       <c r="I323" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J323" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K323" s="16"/>
@@ -9521,11 +9536,11 @@
       <c r="G324" s="14"/>
       <c r="H324" s="14"/>
       <c r="I324" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J324" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K324" s="16"/>
@@ -9543,11 +9558,11 @@
       <c r="G325" s="14"/>
       <c r="H325" s="14"/>
       <c r="I325" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J325" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K325" s="16"/>
@@ -9565,11 +9580,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="16">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" ref="I326:I389" si="18">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="17">IF(I326="","",1440-I326)</f>
+        <f t="shared" ref="J326:J389" si="19">IF(I326="","",1440-I326)</f>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -9587,11 +9602,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -9609,11 +9624,11 @@
       <c r="G328" s="14"/>
       <c r="H328" s="14"/>
       <c r="I328" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J328" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K328" s="16"/>
@@ -9631,11 +9646,11 @@
       <c r="G329" s="14"/>
       <c r="H329" s="14"/>
       <c r="I329" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J329" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K329" s="16"/>
@@ -9653,11 +9668,11 @@
       <c r="G330" s="14"/>
       <c r="H330" s="14"/>
       <c r="I330" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J330" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K330" s="16"/>
@@ -9675,11 +9690,11 @@
       <c r="G331" s="14"/>
       <c r="H331" s="14"/>
       <c r="I331" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J331" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K331" s="16"/>
@@ -9697,11 +9712,11 @@
       <c r="G332" s="14"/>
       <c r="H332" s="14"/>
       <c r="I332" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J332" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K332" s="16"/>
@@ -9719,11 +9734,11 @@
       <c r="G333" s="14"/>
       <c r="H333" s="14"/>
       <c r="I333" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J333" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K333" s="16"/>
@@ -9741,11 +9756,11 @@
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
       <c r="I334" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J334" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K334" s="16"/>
@@ -9763,11 +9778,11 @@
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
       <c r="I335" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J335" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K335" s="16"/>
@@ -9785,11 +9800,11 @@
       <c r="G336" s="14"/>
       <c r="H336" s="14"/>
       <c r="I336" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J336" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K336" s="16"/>
@@ -9807,11 +9822,11 @@
       <c r="G337" s="14"/>
       <c r="H337" s="14"/>
       <c r="I337" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J337" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K337" s="16"/>
@@ -9829,11 +9844,11 @@
       <c r="G338" s="14"/>
       <c r="H338" s="14"/>
       <c r="I338" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J338" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K338" s="16"/>
@@ -9851,11 +9866,11 @@
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
       <c r="I339" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J339" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K339" s="16"/>
@@ -9873,11 +9888,11 @@
       <c r="G340" s="14"/>
       <c r="H340" s="14"/>
       <c r="I340" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J340" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K340" s="16"/>
@@ -9895,11 +9910,11 @@
       <c r="G341" s="14"/>
       <c r="H341" s="14"/>
       <c r="I341" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J341" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K341" s="16"/>
@@ -9917,11 +9932,11 @@
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
       <c r="I342" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J342" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K342" s="16"/>
@@ -9939,11 +9954,11 @@
       <c r="G343" s="14"/>
       <c r="H343" s="14"/>
       <c r="I343" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J343" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K343" s="16"/>
@@ -9961,11 +9976,11 @@
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
       <c r="I344" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J344" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K344" s="16"/>
@@ -9983,11 +9998,11 @@
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
       <c r="I345" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J345" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K345" s="16"/>
@@ -10005,11 +10020,11 @@
       <c r="G346" s="14"/>
       <c r="H346" s="14"/>
       <c r="I346" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J346" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K346" s="16"/>
@@ -10027,11 +10042,11 @@
       <c r="G347" s="14"/>
       <c r="H347" s="14"/>
       <c r="I347" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J347" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K347" s="16"/>
@@ -10049,11 +10064,11 @@
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
       <c r="I348" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J348" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K348" s="16"/>
@@ -10071,11 +10086,11 @@
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
       <c r="I349" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J349" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K349" s="16"/>
@@ -10093,11 +10108,11 @@
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
       <c r="I350" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J350" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K350" s="16"/>
@@ -10115,11 +10130,11 @@
       <c r="G351" s="14"/>
       <c r="H351" s="14"/>
       <c r="I351" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J351" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K351" s="16"/>
@@ -10137,11 +10152,11 @@
       <c r="G352" s="14"/>
       <c r="H352" s="14"/>
       <c r="I352" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J352" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K352" s="16"/>
@@ -10159,11 +10174,11 @@
       <c r="G353" s="14"/>
       <c r="H353" s="14"/>
       <c r="I353" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J353" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K353" s="16"/>
@@ -10181,11 +10196,11 @@
       <c r="G354" s="14"/>
       <c r="H354" s="14"/>
       <c r="I354" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J354" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K354" s="16"/>
@@ -10203,11 +10218,11 @@
       <c r="G355" s="14"/>
       <c r="H355" s="14"/>
       <c r="I355" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J355" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K355" s="16"/>
@@ -10225,11 +10240,11 @@
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
       <c r="I356" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J356" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K356" s="16"/>
@@ -10247,11 +10262,11 @@
       <c r="G357" s="14"/>
       <c r="H357" s="14"/>
       <c r="I357" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J357" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K357" s="16"/>
@@ -10269,11 +10284,11 @@
       <c r="G358" s="14"/>
       <c r="H358" s="14"/>
       <c r="I358" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J358" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K358" s="16"/>
@@ -10291,11 +10306,11 @@
       <c r="G359" s="14"/>
       <c r="H359" s="14"/>
       <c r="I359" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J359" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K359" s="16"/>
@@ -10313,11 +10328,11 @@
       <c r="G360" s="14"/>
       <c r="H360" s="14"/>
       <c r="I360" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J360" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K360" s="16"/>
@@ -10335,11 +10350,11 @@
       <c r="G361" s="14"/>
       <c r="H361" s="14"/>
       <c r="I361" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J361" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K361" s="16"/>
@@ -10357,11 +10372,11 @@
       <c r="G362" s="14"/>
       <c r="H362" s="14"/>
       <c r="I362" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J362" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K362" s="16"/>
@@ -10379,11 +10394,11 @@
       <c r="G363" s="14"/>
       <c r="H363" s="14"/>
       <c r="I363" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J363" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K363" s="16"/>
@@ -10401,11 +10416,11 @@
       <c r="G364" s="14"/>
       <c r="H364" s="14"/>
       <c r="I364" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J364" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K364" s="16"/>
@@ -10423,11 +10438,11 @@
       <c r="G365" s="14"/>
       <c r="H365" s="14"/>
       <c r="I365" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J365" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K365" s="16"/>
@@ -10445,11 +10460,11 @@
       <c r="G366" s="14"/>
       <c r="H366" s="14"/>
       <c r="I366" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J366" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K366" s="16"/>
@@ -10467,11 +10482,11 @@
       <c r="G367" s="14"/>
       <c r="H367" s="14"/>
       <c r="I367" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J367" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K367" s="16"/>
@@ -10489,11 +10504,11 @@
       <c r="G368" s="14"/>
       <c r="H368" s="14"/>
       <c r="I368" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J368" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K368" s="16"/>
@@ -10511,11 +10526,11 @@
       <c r="G369" s="14"/>
       <c r="H369" s="14"/>
       <c r="I369" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J369" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K369" s="16"/>
@@ -10533,11 +10548,11 @@
       <c r="G370" s="14"/>
       <c r="H370" s="14"/>
       <c r="I370" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J370" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K370" s="16"/>
@@ -10555,11 +10570,11 @@
       <c r="G371" s="14"/>
       <c r="H371" s="14"/>
       <c r="I371" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J371" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K371" s="16"/>
@@ -10577,11 +10592,11 @@
       <c r="G372" s="14"/>
       <c r="H372" s="14"/>
       <c r="I372" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J372" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K372" s="16"/>
@@ -10599,11 +10614,11 @@
       <c r="G373" s="14"/>
       <c r="H373" s="14"/>
       <c r="I373" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J373" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K373" s="16"/>
@@ -10621,11 +10636,11 @@
       <c r="G374" s="14"/>
       <c r="H374" s="14"/>
       <c r="I374" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J374" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K374" s="16"/>
@@ -10643,11 +10658,11 @@
       <c r="G375" s="14"/>
       <c r="H375" s="14"/>
       <c r="I375" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J375" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K375" s="16"/>
@@ -10665,11 +10680,11 @@
       <c r="G376" s="14"/>
       <c r="H376" s="14"/>
       <c r="I376" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J376" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K376" s="16"/>
@@ -10687,11 +10702,11 @@
       <c r="G377" s="14"/>
       <c r="H377" s="14"/>
       <c r="I377" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J377" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K377" s="16"/>
@@ -10709,11 +10724,11 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K378" s="16"/>
@@ -10731,11 +10746,11 @@
       <c r="G379" s="14"/>
       <c r="H379" s="14"/>
       <c r="I379" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J379" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K379" s="16"/>
@@ -10753,11 +10768,11 @@
       <c r="G380" s="14"/>
       <c r="H380" s="14"/>
       <c r="I380" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J380" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K380" s="16"/>
@@ -10775,11 +10790,11 @@
       <c r="G381" s="14"/>
       <c r="H381" s="14"/>
       <c r="I381" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J381" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K381" s="16"/>
@@ -10797,11 +10812,11 @@
       <c r="G382" s="14"/>
       <c r="H382" s="14"/>
       <c r="I382" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J382" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K382" s="16"/>
@@ -10819,11 +10834,11 @@
       <c r="G383" s="14"/>
       <c r="H383" s="14"/>
       <c r="I383" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J383" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K383" s="16"/>
@@ -10841,11 +10856,11 @@
       <c r="G384" s="14"/>
       <c r="H384" s="14"/>
       <c r="I384" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J384" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K384" s="16"/>
@@ -10863,11 +10878,11 @@
       <c r="G385" s="14"/>
       <c r="H385" s="14"/>
       <c r="I385" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J385" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K385" s="16"/>
@@ -10885,11 +10900,11 @@
       <c r="G386" s="14"/>
       <c r="H386" s="14"/>
       <c r="I386" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J386" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K386" s="16"/>
@@ -10907,11 +10922,11 @@
       <c r="G387" s="14"/>
       <c r="H387" s="14"/>
       <c r="I387" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J387" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K387" s="16"/>
@@ -10929,11 +10944,11 @@
       <c r="G388" s="14"/>
       <c r="H388" s="14"/>
       <c r="I388" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J388" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K388" s="16"/>
@@ -10951,11 +10966,11 @@
       <c r="G389" s="14"/>
       <c r="H389" s="14"/>
       <c r="I389" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J389" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K389" s="16"/>
@@ -10973,11 +10988,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="18">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="20">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="19">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="21">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -10995,11 +11010,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -11017,11 +11032,11 @@
       <c r="G392" s="14"/>
       <c r="H392" s="14"/>
       <c r="I392" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J392" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K392" s="16"/>
@@ -11039,11 +11054,11 @@
       <c r="G393" s="14"/>
       <c r="H393" s="14"/>
       <c r="I393" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J393" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K393" s="16"/>
@@ -11061,11 +11076,11 @@
       <c r="G394" s="14"/>
       <c r="H394" s="14"/>
       <c r="I394" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J394" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K394" s="16"/>
@@ -11083,11 +11098,11 @@
       <c r="G395" s="14"/>
       <c r="H395" s="14"/>
       <c r="I395" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J395" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K395" s="16"/>
@@ -11105,11 +11120,11 @@
       <c r="G396" s="14"/>
       <c r="H396" s="14"/>
       <c r="I396" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J396" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K396" s="16"/>
@@ -11127,11 +11142,11 @@
       <c r="G397" s="14"/>
       <c r="H397" s="14"/>
       <c r="I397" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J397" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K397" s="16"/>
@@ -11149,11 +11164,11 @@
       <c r="G398" s="14"/>
       <c r="H398" s="14"/>
       <c r="I398" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J398" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K398" s="16"/>
@@ -11171,11 +11186,11 @@
       <c r="G399" s="14"/>
       <c r="H399" s="14"/>
       <c r="I399" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J399" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K399" s="16"/>
@@ -11193,11 +11208,11 @@
       <c r="G400" s="14"/>
       <c r="H400" s="14"/>
       <c r="I400" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J400" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K400" s="16"/>
@@ -11215,11 +11230,11 @@
       <c r="G401" s="14"/>
       <c r="H401" s="14"/>
       <c r="I401" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J401" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K401" s="16"/>

</xml_diff>

<commit_message>
File Updated On 17/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF80F2EF-E5A8-4264-A468-B5665CFA7383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A32E20D-8CC7-4525-9EF3-07996AF43BE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="612" yWindow="-108" windowWidth="22536" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="89">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -299,6 +299,9 @@
   </si>
   <si>
     <t>4th mid term</t>
+  </si>
+  <si>
+    <t>5th mid term</t>
   </si>
 </sst>
 </file>
@@ -3829,26 +3832,50 @@
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A65" s="13"/>
-      <c r="B65" s="14"/>
-      <c r="C65" s="14"/>
-      <c r="D65" s="14"/>
-      <c r="E65" s="14"/>
-      <c r="F65" s="14"/>
-      <c r="G65" s="14"/>
-      <c r="H65" s="14"/>
-      <c r="I65" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J65" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K65" s="16"/>
-      <c r="L65" s="16"/>
-      <c r="M65" s="16"/>
-      <c r="N65" s="17"/>
+      <c r="A65" s="13">
+        <v>46312</v>
+      </c>
+      <c r="B65" s="14">
+        <v>300</v>
+      </c>
+      <c r="C65" s="14">
+        <v>0</v>
+      </c>
+      <c r="D65" s="14">
+        <v>140</v>
+      </c>
+      <c r="E65" s="14">
+        <v>0</v>
+      </c>
+      <c r="F65" s="14">
+        <v>0</v>
+      </c>
+      <c r="G65" s="14">
+        <v>0</v>
+      </c>
+      <c r="H65" s="14">
+        <v>200</v>
+      </c>
+      <c r="I65" s="15">
+        <f t="shared" ref="I65" si="10">IF(SUM(B65:F65,H65)=0,"",SUM(B65:F65,H65))</f>
+        <v>640</v>
+      </c>
+      <c r="J65" s="15">
+        <f t="shared" ref="J65" si="11">IF(I65="","",1440-I65)</f>
+        <v>800</v>
+      </c>
+      <c r="K65" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L65" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M65" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N65" s="17" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" s="13"/>
@@ -3948,11 +3975,11 @@
       <c r="G70" s="14"/>
       <c r="H70" s="14"/>
       <c r="I70" s="15" t="str">
-        <f t="shared" ref="I70:I133" si="10">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
+        <f t="shared" ref="I70:I133" si="12">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
         <v/>
       </c>
       <c r="J70" s="15" t="str">
-        <f t="shared" ref="J70:J133" si="11">IF(I70="","",1440-I70)</f>
+        <f t="shared" ref="J70:J133" si="13">IF(I70="","",1440-I70)</f>
         <v/>
       </c>
       <c r="K70" s="16"/>
@@ -3970,11 +3997,11 @@
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
       <c r="I71" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J71" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K71" s="16"/>
@@ -3992,11 +4019,11 @@
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
       <c r="I72" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J72" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K72" s="16"/>
@@ -4014,11 +4041,11 @@
       <c r="G73" s="14"/>
       <c r="H73" s="14"/>
       <c r="I73" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J73" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K73" s="16"/>
@@ -4036,11 +4063,11 @@
       <c r="G74" s="14"/>
       <c r="H74" s="14"/>
       <c r="I74" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J74" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K74" s="16"/>
@@ -4058,11 +4085,11 @@
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
       <c r="I75" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J75" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K75" s="16"/>
@@ -4080,11 +4107,11 @@
       <c r="G76" s="14"/>
       <c r="H76" s="14"/>
       <c r="I76" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J76" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K76" s="16"/>
@@ -4102,11 +4129,11 @@
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
       <c r="I77" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J77" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K77" s="16"/>
@@ -4124,11 +4151,11 @@
       <c r="G78" s="14"/>
       <c r="H78" s="14"/>
       <c r="I78" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J78" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K78" s="16"/>
@@ -4146,11 +4173,11 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J79" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K79" s="16"/>
@@ -4168,11 +4195,11 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J80" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K80" s="16"/>
@@ -4190,11 +4217,11 @@
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J81" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K81" s="16"/>
@@ -4212,11 +4239,11 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J82" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K82" s="16"/>
@@ -4234,11 +4261,11 @@
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
       <c r="I83" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J83" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K83" s="16"/>
@@ -4256,11 +4283,11 @@
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
       <c r="I84" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J84" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K84" s="16"/>
@@ -4278,11 +4305,11 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J85" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K85" s="16"/>
@@ -4300,11 +4327,11 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J86" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K86" s="16"/>
@@ -4322,11 +4349,11 @@
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
       <c r="I87" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J87" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K87" s="16"/>
@@ -4344,11 +4371,11 @@
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
       <c r="I88" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J88" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K88" s="16"/>
@@ -4366,11 +4393,11 @@
       <c r="G89" s="14"/>
       <c r="H89" s="14"/>
       <c r="I89" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J89" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K89" s="16"/>
@@ -4388,11 +4415,11 @@
       <c r="G90" s="14"/>
       <c r="H90" s="14"/>
       <c r="I90" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J90" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K90" s="16"/>
@@ -4410,11 +4437,11 @@
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
       <c r="I91" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J91" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K91" s="16"/>
@@ -4432,11 +4459,11 @@
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
       <c r="I92" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J92" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K92" s="16"/>
@@ -4454,11 +4481,11 @@
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J93" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K93" s="16"/>
@@ -4476,11 +4503,11 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J94" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K94" s="16"/>
@@ -4498,11 +4525,11 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J95" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K95" s="16"/>
@@ -4520,11 +4547,11 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J96" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K96" s="16"/>
@@ -4542,11 +4569,11 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J97" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K97" s="16"/>
@@ -4564,11 +4591,11 @@
       <c r="G98" s="14"/>
       <c r="H98" s="14"/>
       <c r="I98" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J98" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K98" s="16"/>
@@ -4586,11 +4613,11 @@
       <c r="G99" s="14"/>
       <c r="H99" s="14"/>
       <c r="I99" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J99" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K99" s="16"/>
@@ -4608,11 +4635,11 @@
       <c r="G100" s="14"/>
       <c r="H100" s="14"/>
       <c r="I100" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J100" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K100" s="16"/>
@@ -4630,11 +4657,11 @@
       <c r="G101" s="14"/>
       <c r="H101" s="14"/>
       <c r="I101" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J101" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K101" s="16"/>
@@ -4652,11 +4679,11 @@
       <c r="G102" s="14"/>
       <c r="H102" s="14"/>
       <c r="I102" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J102" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K102" s="16"/>
@@ -4674,11 +4701,11 @@
       <c r="G103" s="14"/>
       <c r="H103" s="14"/>
       <c r="I103" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J103" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K103" s="16"/>
@@ -4696,11 +4723,11 @@
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
       <c r="I104" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J104" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K104" s="16"/>
@@ -4718,11 +4745,11 @@
       <c r="G105" s="14"/>
       <c r="H105" s="14"/>
       <c r="I105" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J105" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K105" s="16"/>
@@ -4740,11 +4767,11 @@
       <c r="G106" s="14"/>
       <c r="H106" s="14"/>
       <c r="I106" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J106" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K106" s="16"/>
@@ -4762,11 +4789,11 @@
       <c r="G107" s="14"/>
       <c r="H107" s="14"/>
       <c r="I107" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J107" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K107" s="16"/>
@@ -4784,11 +4811,11 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J108" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K108" s="16"/>
@@ -4806,11 +4833,11 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J109" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K109" s="16"/>
@@ -4828,11 +4855,11 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J110" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K110" s="16"/>
@@ -4850,11 +4877,11 @@
       <c r="G111" s="14"/>
       <c r="H111" s="14"/>
       <c r="I111" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J111" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K111" s="16"/>
@@ -4872,11 +4899,11 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J112" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K112" s="16"/>
@@ -4894,11 +4921,11 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J113" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K113" s="16"/>
@@ -4916,11 +4943,11 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J114" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K114" s="16"/>
@@ -4938,11 +4965,11 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J115" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K115" s="16"/>
@@ -4960,11 +4987,11 @@
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
       <c r="I116" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J116" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K116" s="16"/>
@@ -4982,11 +5009,11 @@
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
       <c r="I117" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J117" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K117" s="16"/>
@@ -5004,11 +5031,11 @@
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
       <c r="I118" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J118" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K118" s="16"/>
@@ -5026,11 +5053,11 @@
       <c r="G119" s="14"/>
       <c r="H119" s="14"/>
       <c r="I119" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J119" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K119" s="16"/>
@@ -5048,11 +5075,11 @@
       <c r="G120" s="14"/>
       <c r="H120" s="14"/>
       <c r="I120" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J120" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K120" s="16"/>
@@ -5070,11 +5097,11 @@
       <c r="G121" s="14"/>
       <c r="H121" s="14"/>
       <c r="I121" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J121" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K121" s="16"/>
@@ -5092,11 +5119,11 @@
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
       <c r="I122" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J122" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K122" s="16"/>
@@ -5114,11 +5141,11 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J123" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K123" s="16"/>
@@ -5136,11 +5163,11 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J124" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K124" s="16"/>
@@ -5158,11 +5185,11 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J125" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K125" s="16"/>
@@ -5180,11 +5207,11 @@
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
       <c r="I126" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J126" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K126" s="16"/>
@@ -5202,11 +5229,11 @@
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J127" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K127" s="16"/>
@@ -5224,11 +5251,11 @@
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
       <c r="I128" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J128" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K128" s="16"/>
@@ -5246,11 +5273,11 @@
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
       <c r="I129" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J129" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K129" s="16"/>
@@ -5268,11 +5295,11 @@
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
       <c r="I130" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J130" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K130" s="16"/>
@@ -5290,11 +5317,11 @@
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
       <c r="I131" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J131" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K131" s="16"/>
@@ -5312,11 +5339,11 @@
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
       <c r="I132" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J132" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K132" s="16"/>
@@ -5334,11 +5361,11 @@
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
       <c r="I133" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J133" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K133" s="16"/>
@@ -5356,11 +5383,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="12">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" ref="I134:I197" si="14">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="13">IF(I134="","",1440-I134)</f>
+        <f t="shared" ref="J134:J197" si="15">IF(I134="","",1440-I134)</f>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -5378,11 +5405,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5400,11 +5427,11 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J136" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K136" s="16"/>
@@ -5422,11 +5449,11 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J137" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K137" s="16"/>
@@ -5444,11 +5471,11 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J138" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K138" s="16"/>
@@ -5466,11 +5493,11 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J139" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K139" s="16"/>
@@ -5488,11 +5515,11 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J140" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K140" s="16"/>
@@ -5510,11 +5537,11 @@
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J141" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K141" s="16"/>
@@ -5532,11 +5559,11 @@
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J142" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K142" s="16"/>
@@ -5554,11 +5581,11 @@
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J143" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K143" s="16"/>
@@ -5576,11 +5603,11 @@
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J144" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K144" s="16"/>
@@ -5598,11 +5625,11 @@
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J145" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K145" s="16"/>
@@ -5620,11 +5647,11 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J146" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K146" s="16"/>
@@ -5642,11 +5669,11 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J147" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K147" s="16"/>
@@ -5664,11 +5691,11 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J148" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K148" s="16"/>
@@ -5686,11 +5713,11 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J149" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K149" s="16"/>
@@ -5708,11 +5735,11 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J150" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K150" s="16"/>
@@ -5730,11 +5757,11 @@
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
       <c r="I151" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J151" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K151" s="16"/>
@@ -5752,11 +5779,11 @@
       <c r="G152" s="14"/>
       <c r="H152" s="14"/>
       <c r="I152" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J152" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K152" s="16"/>
@@ -5774,11 +5801,11 @@
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J153" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K153" s="16"/>
@@ -5796,11 +5823,11 @@
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J154" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K154" s="16"/>
@@ -5818,11 +5845,11 @@
       <c r="G155" s="14"/>
       <c r="H155" s="14"/>
       <c r="I155" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J155" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K155" s="16"/>
@@ -5840,11 +5867,11 @@
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
       <c r="I156" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J156" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K156" s="16"/>
@@ -5862,11 +5889,11 @@
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J157" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K157" s="16"/>
@@ -5884,11 +5911,11 @@
       <c r="G158" s="14"/>
       <c r="H158" s="14"/>
       <c r="I158" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J158" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K158" s="16"/>
@@ -5906,11 +5933,11 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J159" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K159" s="16"/>
@@ -5928,11 +5955,11 @@
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
       <c r="I160" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J160" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K160" s="16"/>
@@ -5950,11 +5977,11 @@
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
       <c r="I161" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J161" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K161" s="16"/>
@@ -5972,11 +5999,11 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J162" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K162" s="16"/>
@@ -5994,11 +6021,11 @@
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
       <c r="I163" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J163" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K163" s="16"/>
@@ -6016,11 +6043,11 @@
       <c r="G164" s="14"/>
       <c r="H164" s="14"/>
       <c r="I164" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J164" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K164" s="16"/>
@@ -6038,11 +6065,11 @@
       <c r="G165" s="14"/>
       <c r="H165" s="14"/>
       <c r="I165" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J165" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K165" s="16"/>
@@ -6060,11 +6087,11 @@
       <c r="G166" s="14"/>
       <c r="H166" s="14"/>
       <c r="I166" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J166" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K166" s="16"/>
@@ -6082,11 +6109,11 @@
       <c r="G167" s="14"/>
       <c r="H167" s="14"/>
       <c r="I167" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J167" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K167" s="16"/>
@@ -6104,11 +6131,11 @@
       <c r="G168" s="14"/>
       <c r="H168" s="14"/>
       <c r="I168" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J168" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K168" s="16"/>
@@ -6126,11 +6153,11 @@
       <c r="G169" s="14"/>
       <c r="H169" s="14"/>
       <c r="I169" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J169" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K169" s="16"/>
@@ -6148,11 +6175,11 @@
       <c r="G170" s="14"/>
       <c r="H170" s="14"/>
       <c r="I170" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J170" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K170" s="16"/>
@@ -6170,11 +6197,11 @@
       <c r="G171" s="14"/>
       <c r="H171" s="14"/>
       <c r="I171" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J171" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K171" s="16"/>
@@ -6192,11 +6219,11 @@
       <c r="G172" s="14"/>
       <c r="H172" s="14"/>
       <c r="I172" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J172" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K172" s="16"/>
@@ -6214,11 +6241,11 @@
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
       <c r="I173" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J173" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K173" s="16"/>
@@ -6236,11 +6263,11 @@
       <c r="G174" s="14"/>
       <c r="H174" s="14"/>
       <c r="I174" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J174" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K174" s="16"/>
@@ -6258,11 +6285,11 @@
       <c r="G175" s="14"/>
       <c r="H175" s="14"/>
       <c r="I175" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J175" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K175" s="16"/>
@@ -6280,11 +6307,11 @@
       <c r="G176" s="14"/>
       <c r="H176" s="14"/>
       <c r="I176" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J176" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K176" s="16"/>
@@ -6302,11 +6329,11 @@
       <c r="G177" s="14"/>
       <c r="H177" s="14"/>
       <c r="I177" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J177" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K177" s="16"/>
@@ -6324,11 +6351,11 @@
       <c r="G178" s="14"/>
       <c r="H178" s="14"/>
       <c r="I178" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J178" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K178" s="16"/>
@@ -6346,11 +6373,11 @@
       <c r="G179" s="14"/>
       <c r="H179" s="14"/>
       <c r="I179" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J179" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K179" s="16"/>
@@ -6368,11 +6395,11 @@
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
       <c r="I180" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J180" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K180" s="16"/>
@@ -6390,11 +6417,11 @@
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J181" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K181" s="16"/>
@@ -6412,11 +6439,11 @@
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J182" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K182" s="16"/>
@@ -6434,11 +6461,11 @@
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J183" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K183" s="16"/>
@@ -6456,11 +6483,11 @@
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
       <c r="I184" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J184" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K184" s="16"/>
@@ -6478,11 +6505,11 @@
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
       <c r="I185" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J185" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K185" s="16"/>
@@ -6500,11 +6527,11 @@
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J186" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K186" s="16"/>
@@ -6522,11 +6549,11 @@
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J187" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K187" s="16"/>
@@ -6544,11 +6571,11 @@
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
       <c r="I188" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J188" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K188" s="16"/>
@@ -6566,11 +6593,11 @@
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
       <c r="I189" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J189" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K189" s="16"/>
@@ -6588,11 +6615,11 @@
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J190" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K190" s="16"/>
@@ -6610,11 +6637,11 @@
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J191" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K191" s="16"/>
@@ -6632,11 +6659,11 @@
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J192" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K192" s="16"/>
@@ -6654,11 +6681,11 @@
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
       <c r="I193" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J193" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K193" s="16"/>
@@ -6676,11 +6703,11 @@
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
       <c r="I194" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J194" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K194" s="16"/>
@@ -6698,11 +6725,11 @@
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J195" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K195" s="16"/>
@@ -6720,11 +6747,11 @@
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J196" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K196" s="16"/>
@@ -6742,11 +6769,11 @@
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J197" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K197" s="16"/>
@@ -6764,11 +6791,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="14">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" ref="I198:I261" si="16">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="15">IF(I198="","",1440-I198)</f>
+        <f t="shared" ref="J198:J261" si="17">IF(I198="","",1440-I198)</f>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -6786,11 +6813,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -6808,11 +6835,11 @@
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J200" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K200" s="16"/>
@@ -6830,11 +6857,11 @@
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
       <c r="I201" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J201" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K201" s="16"/>
@@ -6852,11 +6879,11 @@
       <c r="G202" s="14"/>
       <c r="H202" s="14"/>
       <c r="I202" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J202" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K202" s="16"/>
@@ -6874,11 +6901,11 @@
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
       <c r="I203" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J203" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K203" s="16"/>
@@ -6896,11 +6923,11 @@
       <c r="G204" s="14"/>
       <c r="H204" s="14"/>
       <c r="I204" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J204" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K204" s="16"/>
@@ -6918,11 +6945,11 @@
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J205" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K205" s="16"/>
@@ -6940,11 +6967,11 @@
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J206" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K206" s="16"/>
@@ -6962,11 +6989,11 @@
       <c r="G207" s="14"/>
       <c r="H207" s="14"/>
       <c r="I207" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J207" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K207" s="16"/>
@@ -6984,11 +7011,11 @@
       <c r="G208" s="14"/>
       <c r="H208" s="14"/>
       <c r="I208" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J208" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K208" s="16"/>
@@ -7006,11 +7033,11 @@
       <c r="G209" s="14"/>
       <c r="H209" s="14"/>
       <c r="I209" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J209" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K209" s="16"/>
@@ -7028,11 +7055,11 @@
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J210" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K210" s="16"/>
@@ -7050,11 +7077,11 @@
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J211" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K211" s="16"/>
@@ -7072,11 +7099,11 @@
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J212" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K212" s="16"/>
@@ -7094,11 +7121,11 @@
       <c r="G213" s="14"/>
       <c r="H213" s="14"/>
       <c r="I213" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J213" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K213" s="16"/>
@@ -7116,11 +7143,11 @@
       <c r="G214" s="14"/>
       <c r="H214" s="14"/>
       <c r="I214" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J214" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K214" s="16"/>
@@ -7138,11 +7165,11 @@
       <c r="G215" s="14"/>
       <c r="H215" s="14"/>
       <c r="I215" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J215" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K215" s="16"/>
@@ -7160,11 +7187,11 @@
       <c r="G216" s="14"/>
       <c r="H216" s="14"/>
       <c r="I216" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J216" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K216" s="16"/>
@@ -7182,11 +7209,11 @@
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J217" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K217" s="16"/>
@@ -7204,11 +7231,11 @@
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J218" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K218" s="16"/>
@@ -7226,11 +7253,11 @@
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J219" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K219" s="16"/>
@@ -7248,11 +7275,11 @@
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J220" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K220" s="16"/>
@@ -7270,11 +7297,11 @@
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J221" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K221" s="16"/>
@@ -7292,11 +7319,11 @@
       <c r="G222" s="14"/>
       <c r="H222" s="14"/>
       <c r="I222" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J222" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K222" s="16"/>
@@ -7314,11 +7341,11 @@
       <c r="G223" s="14"/>
       <c r="H223" s="14"/>
       <c r="I223" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J223" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K223" s="16"/>
@@ -7336,11 +7363,11 @@
       <c r="G224" s="14"/>
       <c r="H224" s="14"/>
       <c r="I224" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J224" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K224" s="16"/>
@@ -7358,11 +7385,11 @@
       <c r="G225" s="14"/>
       <c r="H225" s="14"/>
       <c r="I225" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J225" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K225" s="16"/>
@@ -7380,11 +7407,11 @@
       <c r="G226" s="14"/>
       <c r="H226" s="14"/>
       <c r="I226" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J226" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K226" s="16"/>
@@ -7402,11 +7429,11 @@
       <c r="G227" s="14"/>
       <c r="H227" s="14"/>
       <c r="I227" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J227" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K227" s="16"/>
@@ -7424,11 +7451,11 @@
       <c r="G228" s="14"/>
       <c r="H228" s="14"/>
       <c r="I228" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J228" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K228" s="16"/>
@@ -7446,11 +7473,11 @@
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J229" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K229" s="16"/>
@@ -7468,11 +7495,11 @@
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J230" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K230" s="16"/>
@@ -7490,11 +7517,11 @@
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
       <c r="I231" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J231" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K231" s="16"/>
@@ -7512,11 +7539,11 @@
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
       <c r="I232" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J232" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K232" s="16"/>
@@ -7534,11 +7561,11 @@
       <c r="G233" s="14"/>
       <c r="H233" s="14"/>
       <c r="I233" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J233" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K233" s="16"/>
@@ -7556,11 +7583,11 @@
       <c r="G234" s="14"/>
       <c r="H234" s="14"/>
       <c r="I234" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J234" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K234" s="16"/>
@@ -7578,11 +7605,11 @@
       <c r="G235" s="14"/>
       <c r="H235" s="14"/>
       <c r="I235" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J235" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K235" s="16"/>
@@ -7600,11 +7627,11 @@
       <c r="G236" s="14"/>
       <c r="H236" s="14"/>
       <c r="I236" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J236" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K236" s="16"/>
@@ -7622,11 +7649,11 @@
       <c r="G237" s="14"/>
       <c r="H237" s="14"/>
       <c r="I237" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J237" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K237" s="16"/>
@@ -7644,11 +7671,11 @@
       <c r="G238" s="14"/>
       <c r="H238" s="14"/>
       <c r="I238" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J238" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K238" s="16"/>
@@ -7666,11 +7693,11 @@
       <c r="G239" s="14"/>
       <c r="H239" s="14"/>
       <c r="I239" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J239" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K239" s="16"/>
@@ -7688,11 +7715,11 @@
       <c r="G240" s="14"/>
       <c r="H240" s="14"/>
       <c r="I240" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J240" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K240" s="16"/>
@@ -7710,11 +7737,11 @@
       <c r="G241" s="14"/>
       <c r="H241" s="14"/>
       <c r="I241" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J241" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K241" s="16"/>
@@ -7732,11 +7759,11 @@
       <c r="G242" s="14"/>
       <c r="H242" s="14"/>
       <c r="I242" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J242" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K242" s="16"/>
@@ -7754,11 +7781,11 @@
       <c r="G243" s="14"/>
       <c r="H243" s="14"/>
       <c r="I243" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J243" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K243" s="16"/>
@@ -7776,11 +7803,11 @@
       <c r="G244" s="14"/>
       <c r="H244" s="14"/>
       <c r="I244" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J244" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K244" s="16"/>
@@ -7798,11 +7825,11 @@
       <c r="G245" s="14"/>
       <c r="H245" s="14"/>
       <c r="I245" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J245" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K245" s="16"/>
@@ -7820,11 +7847,11 @@
       <c r="G246" s="14"/>
       <c r="H246" s="14"/>
       <c r="I246" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J246" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K246" s="16"/>
@@ -7842,11 +7869,11 @@
       <c r="G247" s="14"/>
       <c r="H247" s="14"/>
       <c r="I247" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J247" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K247" s="16"/>
@@ -7864,11 +7891,11 @@
       <c r="G248" s="14"/>
       <c r="H248" s="14"/>
       <c r="I248" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J248" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K248" s="16"/>
@@ -7886,11 +7913,11 @@
       <c r="G249" s="14"/>
       <c r="H249" s="14"/>
       <c r="I249" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J249" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K249" s="16"/>
@@ -7908,11 +7935,11 @@
       <c r="G250" s="14"/>
       <c r="H250" s="14"/>
       <c r="I250" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J250" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K250" s="16"/>
@@ -7930,11 +7957,11 @@
       <c r="G251" s="14"/>
       <c r="H251" s="14"/>
       <c r="I251" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J251" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K251" s="16"/>
@@ -7952,11 +7979,11 @@
       <c r="G252" s="14"/>
       <c r="H252" s="14"/>
       <c r="I252" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J252" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K252" s="16"/>
@@ -7974,11 +8001,11 @@
       <c r="G253" s="14"/>
       <c r="H253" s="14"/>
       <c r="I253" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J253" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K253" s="16"/>
@@ -7996,11 +8023,11 @@
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
       <c r="I254" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J254" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K254" s="16"/>
@@ -8018,11 +8045,11 @@
       <c r="G255" s="14"/>
       <c r="H255" s="14"/>
       <c r="I255" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J255" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K255" s="16"/>
@@ -8040,11 +8067,11 @@
       <c r="G256" s="14"/>
       <c r="H256" s="14"/>
       <c r="I256" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J256" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K256" s="16"/>
@@ -8062,11 +8089,11 @@
       <c r="G257" s="14"/>
       <c r="H257" s="14"/>
       <c r="I257" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J257" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K257" s="16"/>
@@ -8084,11 +8111,11 @@
       <c r="G258" s="14"/>
       <c r="H258" s="14"/>
       <c r="I258" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J258" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K258" s="16"/>
@@ -8106,11 +8133,11 @@
       <c r="G259" s="14"/>
       <c r="H259" s="14"/>
       <c r="I259" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J259" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K259" s="16"/>
@@ -8128,11 +8155,11 @@
       <c r="G260" s="14"/>
       <c r="H260" s="14"/>
       <c r="I260" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J260" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K260" s="16"/>
@@ -8150,11 +8177,11 @@
       <c r="G261" s="14"/>
       <c r="H261" s="14"/>
       <c r="I261" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J261" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K261" s="16"/>
@@ -8172,11 +8199,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="16">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" ref="I262:I325" si="18">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="17">IF(I262="","",1440-I262)</f>
+        <f t="shared" ref="J262:J325" si="19">IF(I262="","",1440-I262)</f>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -8194,11 +8221,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8216,11 +8243,11 @@
       <c r="G264" s="14"/>
       <c r="H264" s="14"/>
       <c r="I264" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J264" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K264" s="16"/>
@@ -8238,11 +8265,11 @@
       <c r="G265" s="14"/>
       <c r="H265" s="14"/>
       <c r="I265" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J265" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K265" s="16"/>
@@ -8260,11 +8287,11 @@
       <c r="G266" s="14"/>
       <c r="H266" s="14"/>
       <c r="I266" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J266" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K266" s="16"/>
@@ -8282,11 +8309,11 @@
       <c r="G267" s="14"/>
       <c r="H267" s="14"/>
       <c r="I267" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J267" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K267" s="16"/>
@@ -8304,11 +8331,11 @@
       <c r="G268" s="14"/>
       <c r="H268" s="14"/>
       <c r="I268" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J268" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K268" s="16"/>
@@ -8326,11 +8353,11 @@
       <c r="G269" s="14"/>
       <c r="H269" s="14"/>
       <c r="I269" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J269" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K269" s="16"/>
@@ -8348,11 +8375,11 @@
       <c r="G270" s="14"/>
       <c r="H270" s="14"/>
       <c r="I270" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J270" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K270" s="16"/>
@@ -8370,11 +8397,11 @@
       <c r="G271" s="14"/>
       <c r="H271" s="14"/>
       <c r="I271" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J271" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K271" s="16"/>
@@ -8392,11 +8419,11 @@
       <c r="G272" s="14"/>
       <c r="H272" s="14"/>
       <c r="I272" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J272" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K272" s="16"/>
@@ -8414,11 +8441,11 @@
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
       <c r="I273" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J273" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K273" s="16"/>
@@ -8436,11 +8463,11 @@
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
       <c r="I274" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J274" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K274" s="16"/>
@@ -8458,11 +8485,11 @@
       <c r="G275" s="14"/>
       <c r="H275" s="14"/>
       <c r="I275" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J275" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K275" s="16"/>
@@ -8480,11 +8507,11 @@
       <c r="G276" s="14"/>
       <c r="H276" s="14"/>
       <c r="I276" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J276" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K276" s="16"/>
@@ -8502,11 +8529,11 @@
       <c r="G277" s="14"/>
       <c r="H277" s="14"/>
       <c r="I277" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J277" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K277" s="16"/>
@@ -8524,11 +8551,11 @@
       <c r="G278" s="14"/>
       <c r="H278" s="14"/>
       <c r="I278" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J278" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K278" s="16"/>
@@ -8546,11 +8573,11 @@
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
       <c r="I279" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J279" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K279" s="16"/>
@@ -8568,11 +8595,11 @@
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
       <c r="I280" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J280" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K280" s="16"/>
@@ -8590,11 +8617,11 @@
       <c r="G281" s="14"/>
       <c r="H281" s="14"/>
       <c r="I281" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J281" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K281" s="16"/>
@@ -8612,11 +8639,11 @@
       <c r="G282" s="14"/>
       <c r="H282" s="14"/>
       <c r="I282" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J282" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K282" s="16"/>
@@ -8634,11 +8661,11 @@
       <c r="G283" s="14"/>
       <c r="H283" s="14"/>
       <c r="I283" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J283" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K283" s="16"/>
@@ -8656,11 +8683,11 @@
       <c r="G284" s="14"/>
       <c r="H284" s="14"/>
       <c r="I284" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J284" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K284" s="16"/>
@@ -8678,11 +8705,11 @@
       <c r="G285" s="14"/>
       <c r="H285" s="14"/>
       <c r="I285" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J285" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K285" s="16"/>
@@ -8700,11 +8727,11 @@
       <c r="G286" s="14"/>
       <c r="H286" s="14"/>
       <c r="I286" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J286" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K286" s="16"/>
@@ -8722,11 +8749,11 @@
       <c r="G287" s="14"/>
       <c r="H287" s="14"/>
       <c r="I287" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J287" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K287" s="16"/>
@@ -8744,11 +8771,11 @@
       <c r="G288" s="14"/>
       <c r="H288" s="14"/>
       <c r="I288" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J288" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K288" s="16"/>
@@ -8766,11 +8793,11 @@
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
       <c r="I289" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J289" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K289" s="16"/>
@@ -8788,11 +8815,11 @@
       <c r="G290" s="14"/>
       <c r="H290" s="14"/>
       <c r="I290" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J290" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K290" s="16"/>
@@ -8810,11 +8837,11 @@
       <c r="G291" s="14"/>
       <c r="H291" s="14"/>
       <c r="I291" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J291" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K291" s="16"/>
@@ -8832,11 +8859,11 @@
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
       <c r="I292" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J292" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K292" s="16"/>
@@ -8854,11 +8881,11 @@
       <c r="G293" s="14"/>
       <c r="H293" s="14"/>
       <c r="I293" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J293" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K293" s="16"/>
@@ -8876,11 +8903,11 @@
       <c r="G294" s="14"/>
       <c r="H294" s="14"/>
       <c r="I294" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J294" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K294" s="16"/>
@@ -8898,11 +8925,11 @@
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
       <c r="I295" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J295" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K295" s="16"/>
@@ -8920,11 +8947,11 @@
       <c r="G296" s="14"/>
       <c r="H296" s="14"/>
       <c r="I296" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J296" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K296" s="16"/>
@@ -8942,11 +8969,11 @@
       <c r="G297" s="14"/>
       <c r="H297" s="14"/>
       <c r="I297" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J297" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K297" s="16"/>
@@ -8964,11 +8991,11 @@
       <c r="G298" s="14"/>
       <c r="H298" s="14"/>
       <c r="I298" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J298" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K298" s="16"/>
@@ -8986,11 +9013,11 @@
       <c r="G299" s="14"/>
       <c r="H299" s="14"/>
       <c r="I299" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J299" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K299" s="16"/>
@@ -9008,11 +9035,11 @@
       <c r="G300" s="14"/>
       <c r="H300" s="14"/>
       <c r="I300" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J300" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K300" s="16"/>
@@ -9030,11 +9057,11 @@
       <c r="G301" s="14"/>
       <c r="H301" s="14"/>
       <c r="I301" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J301" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K301" s="16"/>
@@ -9052,11 +9079,11 @@
       <c r="G302" s="14"/>
       <c r="H302" s="14"/>
       <c r="I302" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J302" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K302" s="16"/>
@@ -9074,11 +9101,11 @@
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
       <c r="I303" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J303" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K303" s="16"/>
@@ -9096,11 +9123,11 @@
       <c r="G304" s="14"/>
       <c r="H304" s="14"/>
       <c r="I304" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J304" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K304" s="16"/>
@@ -9118,11 +9145,11 @@
       <c r="G305" s="14"/>
       <c r="H305" s="14"/>
       <c r="I305" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J305" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K305" s="16"/>
@@ -9140,11 +9167,11 @@
       <c r="G306" s="14"/>
       <c r="H306" s="14"/>
       <c r="I306" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J306" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K306" s="16"/>
@@ -9162,11 +9189,11 @@
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
       <c r="I307" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J307" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K307" s="16"/>
@@ -9184,11 +9211,11 @@
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
       <c r="I308" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J308" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K308" s="16"/>
@@ -9206,11 +9233,11 @@
       <c r="G309" s="14"/>
       <c r="H309" s="14"/>
       <c r="I309" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J309" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K309" s="16"/>
@@ -9228,11 +9255,11 @@
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
       <c r="I310" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J310" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K310" s="16"/>
@@ -9250,11 +9277,11 @@
       <c r="G311" s="14"/>
       <c r="H311" s="14"/>
       <c r="I311" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J311" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K311" s="16"/>
@@ -9272,11 +9299,11 @@
       <c r="G312" s="14"/>
       <c r="H312" s="14"/>
       <c r="I312" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J312" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K312" s="16"/>
@@ -9294,11 +9321,11 @@
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
       <c r="I313" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J313" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K313" s="16"/>
@@ -9316,11 +9343,11 @@
       <c r="G314" s="14"/>
       <c r="H314" s="14"/>
       <c r="I314" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J314" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K314" s="16"/>
@@ -9338,11 +9365,11 @@
       <c r="G315" s="14"/>
       <c r="H315" s="14"/>
       <c r="I315" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J315" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K315" s="16"/>
@@ -9360,11 +9387,11 @@
       <c r="G316" s="14"/>
       <c r="H316" s="14"/>
       <c r="I316" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J316" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K316" s="16"/>
@@ -9382,11 +9409,11 @@
       <c r="G317" s="14"/>
       <c r="H317" s="14"/>
       <c r="I317" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J317" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K317" s="16"/>
@@ -9404,11 +9431,11 @@
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
       <c r="I318" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J318" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K318" s="16"/>
@@ -9426,11 +9453,11 @@
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
       <c r="I319" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J319" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K319" s="16"/>
@@ -9448,11 +9475,11 @@
       <c r="G320" s="14"/>
       <c r="H320" s="14"/>
       <c r="I320" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J320" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K320" s="16"/>
@@ -9470,11 +9497,11 @@
       <c r="G321" s="14"/>
       <c r="H321" s="14"/>
       <c r="I321" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J321" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K321" s="16"/>
@@ -9492,11 +9519,11 @@
       <c r="G322" s="14"/>
       <c r="H322" s="14"/>
       <c r="I322" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J322" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K322" s="16"/>
@@ -9514,11 +9541,11 @@
       <c r="G323" s="14"/>
       <c r="H323" s="14"/>
       <c r="I323" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J323" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K323" s="16"/>
@@ -9536,11 +9563,11 @@
       <c r="G324" s="14"/>
       <c r="H324" s="14"/>
       <c r="I324" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J324" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K324" s="16"/>
@@ -9558,11 +9585,11 @@
       <c r="G325" s="14"/>
       <c r="H325" s="14"/>
       <c r="I325" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J325" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K325" s="16"/>
@@ -9580,11 +9607,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="18">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" ref="I326:I389" si="20">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="19">IF(I326="","",1440-I326)</f>
+        <f t="shared" ref="J326:J389" si="21">IF(I326="","",1440-I326)</f>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -9602,11 +9629,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -9624,11 +9651,11 @@
       <c r="G328" s="14"/>
       <c r="H328" s="14"/>
       <c r="I328" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J328" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K328" s="16"/>
@@ -9646,11 +9673,11 @@
       <c r="G329" s="14"/>
       <c r="H329" s="14"/>
       <c r="I329" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J329" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K329" s="16"/>
@@ -9668,11 +9695,11 @@
       <c r="G330" s="14"/>
       <c r="H330" s="14"/>
       <c r="I330" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J330" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K330" s="16"/>
@@ -9690,11 +9717,11 @@
       <c r="G331" s="14"/>
       <c r="H331" s="14"/>
       <c r="I331" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J331" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K331" s="16"/>
@@ -9712,11 +9739,11 @@
       <c r="G332" s="14"/>
       <c r="H332" s="14"/>
       <c r="I332" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J332" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K332" s="16"/>
@@ -9734,11 +9761,11 @@
       <c r="G333" s="14"/>
       <c r="H333" s="14"/>
       <c r="I333" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J333" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K333" s="16"/>
@@ -9756,11 +9783,11 @@
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
       <c r="I334" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J334" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K334" s="16"/>
@@ -9778,11 +9805,11 @@
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
       <c r="I335" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J335" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K335" s="16"/>
@@ -9800,11 +9827,11 @@
       <c r="G336" s="14"/>
       <c r="H336" s="14"/>
       <c r="I336" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J336" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K336" s="16"/>
@@ -9822,11 +9849,11 @@
       <c r="G337" s="14"/>
       <c r="H337" s="14"/>
       <c r="I337" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J337" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K337" s="16"/>
@@ -9844,11 +9871,11 @@
       <c r="G338" s="14"/>
       <c r="H338" s="14"/>
       <c r="I338" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J338" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K338" s="16"/>
@@ -9866,11 +9893,11 @@
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
       <c r="I339" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J339" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K339" s="16"/>
@@ -9888,11 +9915,11 @@
       <c r="G340" s="14"/>
       <c r="H340" s="14"/>
       <c r="I340" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J340" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K340" s="16"/>
@@ -9910,11 +9937,11 @@
       <c r="G341" s="14"/>
       <c r="H341" s="14"/>
       <c r="I341" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J341" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K341" s="16"/>
@@ -9932,11 +9959,11 @@
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
       <c r="I342" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J342" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K342" s="16"/>
@@ -9954,11 +9981,11 @@
       <c r="G343" s="14"/>
       <c r="H343" s="14"/>
       <c r="I343" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J343" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K343" s="16"/>
@@ -9976,11 +10003,11 @@
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
       <c r="I344" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J344" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K344" s="16"/>
@@ -9998,11 +10025,11 @@
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
       <c r="I345" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J345" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K345" s="16"/>
@@ -10020,11 +10047,11 @@
       <c r="G346" s="14"/>
       <c r="H346" s="14"/>
       <c r="I346" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J346" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K346" s="16"/>
@@ -10042,11 +10069,11 @@
       <c r="G347" s="14"/>
       <c r="H347" s="14"/>
       <c r="I347" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J347" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K347" s="16"/>
@@ -10064,11 +10091,11 @@
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
       <c r="I348" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J348" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K348" s="16"/>
@@ -10086,11 +10113,11 @@
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
       <c r="I349" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J349" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K349" s="16"/>
@@ -10108,11 +10135,11 @@
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
       <c r="I350" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J350" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K350" s="16"/>
@@ -10130,11 +10157,11 @@
       <c r="G351" s="14"/>
       <c r="H351" s="14"/>
       <c r="I351" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J351" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K351" s="16"/>
@@ -10152,11 +10179,11 @@
       <c r="G352" s="14"/>
       <c r="H352" s="14"/>
       <c r="I352" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J352" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K352" s="16"/>
@@ -10174,11 +10201,11 @@
       <c r="G353" s="14"/>
       <c r="H353" s="14"/>
       <c r="I353" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J353" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K353" s="16"/>
@@ -10196,11 +10223,11 @@
       <c r="G354" s="14"/>
       <c r="H354" s="14"/>
       <c r="I354" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J354" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K354" s="16"/>
@@ -10218,11 +10245,11 @@
       <c r="G355" s="14"/>
       <c r="H355" s="14"/>
       <c r="I355" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J355" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K355" s="16"/>
@@ -10240,11 +10267,11 @@
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
       <c r="I356" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J356" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K356" s="16"/>
@@ -10262,11 +10289,11 @@
       <c r="G357" s="14"/>
       <c r="H357" s="14"/>
       <c r="I357" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J357" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K357" s="16"/>
@@ -10284,11 +10311,11 @@
       <c r="G358" s="14"/>
       <c r="H358" s="14"/>
       <c r="I358" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J358" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K358" s="16"/>
@@ -10306,11 +10333,11 @@
       <c r="G359" s="14"/>
       <c r="H359" s="14"/>
       <c r="I359" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J359" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K359" s="16"/>
@@ -10328,11 +10355,11 @@
       <c r="G360" s="14"/>
       <c r="H360" s="14"/>
       <c r="I360" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J360" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K360" s="16"/>
@@ -10350,11 +10377,11 @@
       <c r="G361" s="14"/>
       <c r="H361" s="14"/>
       <c r="I361" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J361" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K361" s="16"/>
@@ -10372,11 +10399,11 @@
       <c r="G362" s="14"/>
       <c r="H362" s="14"/>
       <c r="I362" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J362" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K362" s="16"/>
@@ -10394,11 +10421,11 @@
       <c r="G363" s="14"/>
       <c r="H363" s="14"/>
       <c r="I363" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J363" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K363" s="16"/>
@@ -10416,11 +10443,11 @@
       <c r="G364" s="14"/>
       <c r="H364" s="14"/>
       <c r="I364" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J364" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K364" s="16"/>
@@ -10438,11 +10465,11 @@
       <c r="G365" s="14"/>
       <c r="H365" s="14"/>
       <c r="I365" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J365" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K365" s="16"/>
@@ -10460,11 +10487,11 @@
       <c r="G366" s="14"/>
       <c r="H366" s="14"/>
       <c r="I366" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J366" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K366" s="16"/>
@@ -10482,11 +10509,11 @@
       <c r="G367" s="14"/>
       <c r="H367" s="14"/>
       <c r="I367" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J367" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K367" s="16"/>
@@ -10504,11 +10531,11 @@
       <c r="G368" s="14"/>
       <c r="H368" s="14"/>
       <c r="I368" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J368" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K368" s="16"/>
@@ -10526,11 +10553,11 @@
       <c r="G369" s="14"/>
       <c r="H369" s="14"/>
       <c r="I369" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J369" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K369" s="16"/>
@@ -10548,11 +10575,11 @@
       <c r="G370" s="14"/>
       <c r="H370" s="14"/>
       <c r="I370" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J370" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K370" s="16"/>
@@ -10570,11 +10597,11 @@
       <c r="G371" s="14"/>
       <c r="H371" s="14"/>
       <c r="I371" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J371" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K371" s="16"/>
@@ -10592,11 +10619,11 @@
       <c r="G372" s="14"/>
       <c r="H372" s="14"/>
       <c r="I372" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J372" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K372" s="16"/>
@@ -10614,11 +10641,11 @@
       <c r="G373" s="14"/>
       <c r="H373" s="14"/>
       <c r="I373" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J373" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K373" s="16"/>
@@ -10636,11 +10663,11 @@
       <c r="G374" s="14"/>
       <c r="H374" s="14"/>
       <c r="I374" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J374" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K374" s="16"/>
@@ -10658,11 +10685,11 @@
       <c r="G375" s="14"/>
       <c r="H375" s="14"/>
       <c r="I375" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J375" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K375" s="16"/>
@@ -10680,11 +10707,11 @@
       <c r="G376" s="14"/>
       <c r="H376" s="14"/>
       <c r="I376" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J376" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K376" s="16"/>
@@ -10702,11 +10729,11 @@
       <c r="G377" s="14"/>
       <c r="H377" s="14"/>
       <c r="I377" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J377" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K377" s="16"/>
@@ -10724,11 +10751,11 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K378" s="16"/>
@@ -10746,11 +10773,11 @@
       <c r="G379" s="14"/>
       <c r="H379" s="14"/>
       <c r="I379" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J379" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K379" s="16"/>
@@ -10768,11 +10795,11 @@
       <c r="G380" s="14"/>
       <c r="H380" s="14"/>
       <c r="I380" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J380" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K380" s="16"/>
@@ -10790,11 +10817,11 @@
       <c r="G381" s="14"/>
       <c r="H381" s="14"/>
       <c r="I381" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J381" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K381" s="16"/>
@@ -10812,11 +10839,11 @@
       <c r="G382" s="14"/>
       <c r="H382" s="14"/>
       <c r="I382" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J382" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K382" s="16"/>
@@ -10834,11 +10861,11 @@
       <c r="G383" s="14"/>
       <c r="H383" s="14"/>
       <c r="I383" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J383" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K383" s="16"/>
@@ -10856,11 +10883,11 @@
       <c r="G384" s="14"/>
       <c r="H384" s="14"/>
       <c r="I384" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J384" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K384" s="16"/>
@@ -10878,11 +10905,11 @@
       <c r="G385" s="14"/>
       <c r="H385" s="14"/>
       <c r="I385" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J385" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K385" s="16"/>
@@ -10900,11 +10927,11 @@
       <c r="G386" s="14"/>
       <c r="H386" s="14"/>
       <c r="I386" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J386" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K386" s="16"/>
@@ -10922,11 +10949,11 @@
       <c r="G387" s="14"/>
       <c r="H387" s="14"/>
       <c r="I387" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J387" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K387" s="16"/>
@@ -10944,11 +10971,11 @@
       <c r="G388" s="14"/>
       <c r="H388" s="14"/>
       <c r="I388" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J388" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K388" s="16"/>
@@ -10966,11 +10993,11 @@
       <c r="G389" s="14"/>
       <c r="H389" s="14"/>
       <c r="I389" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J389" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K389" s="16"/>
@@ -10988,11 +11015,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="20">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="22">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="21">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="23">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -11010,11 +11037,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -11032,11 +11059,11 @@
       <c r="G392" s="14"/>
       <c r="H392" s="14"/>
       <c r="I392" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J392" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K392" s="16"/>
@@ -11054,11 +11081,11 @@
       <c r="G393" s="14"/>
       <c r="H393" s="14"/>
       <c r="I393" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J393" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K393" s="16"/>
@@ -11076,11 +11103,11 @@
       <c r="G394" s="14"/>
       <c r="H394" s="14"/>
       <c r="I394" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J394" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K394" s="16"/>
@@ -11098,11 +11125,11 @@
       <c r="G395" s="14"/>
       <c r="H395" s="14"/>
       <c r="I395" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J395" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K395" s="16"/>
@@ -11120,11 +11147,11 @@
       <c r="G396" s="14"/>
       <c r="H396" s="14"/>
       <c r="I396" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J396" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K396" s="16"/>
@@ -11142,11 +11169,11 @@
       <c r="G397" s="14"/>
       <c r="H397" s="14"/>
       <c r="I397" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J397" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K397" s="16"/>
@@ -11164,11 +11191,11 @@
       <c r="G398" s="14"/>
       <c r="H398" s="14"/>
       <c r="I398" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J398" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K398" s="16"/>
@@ -11186,11 +11213,11 @@
       <c r="G399" s="14"/>
       <c r="H399" s="14"/>
       <c r="I399" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J399" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K399" s="16"/>
@@ -11208,11 +11235,11 @@
       <c r="G400" s="14"/>
       <c r="H400" s="14"/>
       <c r="I400" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J400" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K400" s="16"/>
@@ -11230,11 +11257,11 @@
       <c r="G401" s="14"/>
       <c r="H401" s="14"/>
       <c r="I401" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J401" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K401" s="16"/>

</xml_diff>

<commit_message>
File Updated On 18/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A32E20D-8CC7-4525-9EF3-07996AF43BE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20EED29D-D852-45C1-A4D5-883EAE5151FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="612" yWindow="-108" windowWidth="22536" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -302,6 +302,9 @@
   </si>
   <si>
     <t>5th mid term</t>
+  </si>
+  <si>
+    <t>s</t>
   </si>
 </sst>
 </file>
@@ -3878,26 +3881,50 @@
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A66" s="13"/>
-      <c r="B66" s="14"/>
-      <c r="C66" s="14"/>
-      <c r="D66" s="14"/>
-      <c r="E66" s="14"/>
-      <c r="F66" s="14"/>
-      <c r="G66" s="14"/>
-      <c r="H66" s="14"/>
-      <c r="I66" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J66" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K66" s="16"/>
-      <c r="L66" s="16"/>
-      <c r="M66" s="16"/>
-      <c r="N66" s="17"/>
+      <c r="A66" s="13">
+        <v>46313</v>
+      </c>
+      <c r="B66" s="14">
+        <v>480</v>
+      </c>
+      <c r="C66" s="14">
+        <v>0</v>
+      </c>
+      <c r="D66" s="14">
+        <v>100</v>
+      </c>
+      <c r="E66" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="F66" s="14">
+        <v>0</v>
+      </c>
+      <c r="G66" s="14">
+        <v>0</v>
+      </c>
+      <c r="H66" s="14">
+        <v>200</v>
+      </c>
+      <c r="I66" s="15">
+        <f t="shared" ref="I66" si="12">IF(SUM(B66:F66,H66)=0,"",SUM(B66:F66,H66))</f>
+        <v>780</v>
+      </c>
+      <c r="J66" s="15">
+        <f t="shared" ref="J66" si="13">IF(I66="","",1440-I66)</f>
+        <v>660</v>
+      </c>
+      <c r="K66" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L66" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M66" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N66" s="17" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" s="13"/>
@@ -3975,11 +4002,11 @@
       <c r="G70" s="14"/>
       <c r="H70" s="14"/>
       <c r="I70" s="15" t="str">
-        <f t="shared" ref="I70:I133" si="12">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
+        <f t="shared" ref="I70:I133" si="14">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
         <v/>
       </c>
       <c r="J70" s="15" t="str">
-        <f t="shared" ref="J70:J133" si="13">IF(I70="","",1440-I70)</f>
+        <f t="shared" ref="J70:J133" si="15">IF(I70="","",1440-I70)</f>
         <v/>
       </c>
       <c r="K70" s="16"/>
@@ -3997,11 +4024,11 @@
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
       <c r="I71" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J71" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K71" s="16"/>
@@ -4019,11 +4046,11 @@
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
       <c r="I72" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J72" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K72" s="16"/>
@@ -4041,11 +4068,11 @@
       <c r="G73" s="14"/>
       <c r="H73" s="14"/>
       <c r="I73" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J73" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K73" s="16"/>
@@ -4063,11 +4090,11 @@
       <c r="G74" s="14"/>
       <c r="H74" s="14"/>
       <c r="I74" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J74" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K74" s="16"/>
@@ -4085,11 +4112,11 @@
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
       <c r="I75" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J75" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K75" s="16"/>
@@ -4107,11 +4134,11 @@
       <c r="G76" s="14"/>
       <c r="H76" s="14"/>
       <c r="I76" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J76" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K76" s="16"/>
@@ -4129,11 +4156,11 @@
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
       <c r="I77" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J77" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K77" s="16"/>
@@ -4151,11 +4178,11 @@
       <c r="G78" s="14"/>
       <c r="H78" s="14"/>
       <c r="I78" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J78" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K78" s="16"/>
@@ -4173,11 +4200,11 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J79" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K79" s="16"/>
@@ -4195,11 +4222,11 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J80" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K80" s="16"/>
@@ -4217,11 +4244,11 @@
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J81" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K81" s="16"/>
@@ -4239,11 +4266,11 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J82" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K82" s="16"/>
@@ -4261,11 +4288,11 @@
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
       <c r="I83" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J83" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K83" s="16"/>
@@ -4283,11 +4310,11 @@
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
       <c r="I84" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J84" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K84" s="16"/>
@@ -4305,11 +4332,11 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J85" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K85" s="16"/>
@@ -4327,11 +4354,11 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J86" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K86" s="16"/>
@@ -4349,11 +4376,11 @@
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
       <c r="I87" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J87" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K87" s="16"/>
@@ -4371,11 +4398,11 @@
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
       <c r="I88" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J88" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K88" s="16"/>
@@ -4393,11 +4420,11 @@
       <c r="G89" s="14"/>
       <c r="H89" s="14"/>
       <c r="I89" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J89" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K89" s="16"/>
@@ -4415,11 +4442,11 @@
       <c r="G90" s="14"/>
       <c r="H90" s="14"/>
       <c r="I90" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J90" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K90" s="16"/>
@@ -4437,11 +4464,11 @@
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
       <c r="I91" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J91" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K91" s="16"/>
@@ -4459,11 +4486,11 @@
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
       <c r="I92" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J92" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K92" s="16"/>
@@ -4481,11 +4508,11 @@
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J93" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K93" s="16"/>
@@ -4503,11 +4530,11 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J94" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K94" s="16"/>
@@ -4525,11 +4552,11 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J95" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K95" s="16"/>
@@ -4547,11 +4574,11 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J96" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K96" s="16"/>
@@ -4569,11 +4596,11 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J97" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K97" s="16"/>
@@ -4591,11 +4618,11 @@
       <c r="G98" s="14"/>
       <c r="H98" s="14"/>
       <c r="I98" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J98" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K98" s="16"/>
@@ -4613,11 +4640,11 @@
       <c r="G99" s="14"/>
       <c r="H99" s="14"/>
       <c r="I99" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J99" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K99" s="16"/>
@@ -4635,11 +4662,11 @@
       <c r="G100" s="14"/>
       <c r="H100" s="14"/>
       <c r="I100" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J100" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K100" s="16"/>
@@ -4657,11 +4684,11 @@
       <c r="G101" s="14"/>
       <c r="H101" s="14"/>
       <c r="I101" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J101" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K101" s="16"/>
@@ -4679,11 +4706,11 @@
       <c r="G102" s="14"/>
       <c r="H102" s="14"/>
       <c r="I102" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J102" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K102" s="16"/>
@@ -4701,11 +4728,11 @@
       <c r="G103" s="14"/>
       <c r="H103" s="14"/>
       <c r="I103" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J103" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K103" s="16"/>
@@ -4723,11 +4750,11 @@
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
       <c r="I104" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J104" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K104" s="16"/>
@@ -4745,11 +4772,11 @@
       <c r="G105" s="14"/>
       <c r="H105" s="14"/>
       <c r="I105" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J105" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K105" s="16"/>
@@ -4767,11 +4794,11 @@
       <c r="G106" s="14"/>
       <c r="H106" s="14"/>
       <c r="I106" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J106" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K106" s="16"/>
@@ -4789,11 +4816,11 @@
       <c r="G107" s="14"/>
       <c r="H107" s="14"/>
       <c r="I107" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J107" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K107" s="16"/>
@@ -4811,11 +4838,11 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J108" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K108" s="16"/>
@@ -4833,11 +4860,11 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J109" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K109" s="16"/>
@@ -4855,11 +4882,11 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J110" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K110" s="16"/>
@@ -4877,11 +4904,11 @@
       <c r="G111" s="14"/>
       <c r="H111" s="14"/>
       <c r="I111" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J111" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K111" s="16"/>
@@ -4899,11 +4926,11 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J112" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K112" s="16"/>
@@ -4921,11 +4948,11 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J113" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K113" s="16"/>
@@ -4943,11 +4970,11 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J114" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K114" s="16"/>
@@ -4965,11 +4992,11 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J115" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K115" s="16"/>
@@ -4987,11 +5014,11 @@
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
       <c r="I116" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J116" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K116" s="16"/>
@@ -5009,11 +5036,11 @@
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
       <c r="I117" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J117" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K117" s="16"/>
@@ -5031,11 +5058,11 @@
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
       <c r="I118" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J118" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K118" s="16"/>
@@ -5053,11 +5080,11 @@
       <c r="G119" s="14"/>
       <c r="H119" s="14"/>
       <c r="I119" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J119" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K119" s="16"/>
@@ -5075,11 +5102,11 @@
       <c r="G120" s="14"/>
       <c r="H120" s="14"/>
       <c r="I120" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J120" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K120" s="16"/>
@@ -5097,11 +5124,11 @@
       <c r="G121" s="14"/>
       <c r="H121" s="14"/>
       <c r="I121" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J121" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K121" s="16"/>
@@ -5119,11 +5146,11 @@
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
       <c r="I122" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J122" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K122" s="16"/>
@@ -5141,11 +5168,11 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J123" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K123" s="16"/>
@@ -5163,11 +5190,11 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J124" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K124" s="16"/>
@@ -5185,11 +5212,11 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J125" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K125" s="16"/>
@@ -5207,11 +5234,11 @@
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
       <c r="I126" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J126" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K126" s="16"/>
@@ -5229,11 +5256,11 @@
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J127" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K127" s="16"/>
@@ -5251,11 +5278,11 @@
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
       <c r="I128" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J128" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K128" s="16"/>
@@ -5273,11 +5300,11 @@
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
       <c r="I129" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J129" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K129" s="16"/>
@@ -5295,11 +5322,11 @@
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
       <c r="I130" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J130" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K130" s="16"/>
@@ -5317,11 +5344,11 @@
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
       <c r="I131" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J131" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K131" s="16"/>
@@ -5339,11 +5366,11 @@
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
       <c r="I132" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J132" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K132" s="16"/>
@@ -5361,11 +5388,11 @@
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
       <c r="I133" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J133" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K133" s="16"/>
@@ -5383,11 +5410,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="14">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" ref="I134:I197" si="16">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="15">IF(I134="","",1440-I134)</f>
+        <f t="shared" ref="J134:J197" si="17">IF(I134="","",1440-I134)</f>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -5405,11 +5432,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5427,11 +5454,11 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J136" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K136" s="16"/>
@@ -5449,11 +5476,11 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J137" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K137" s="16"/>
@@ -5471,11 +5498,11 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J138" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K138" s="16"/>
@@ -5493,11 +5520,11 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J139" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K139" s="16"/>
@@ -5515,11 +5542,11 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J140" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K140" s="16"/>
@@ -5537,11 +5564,11 @@
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J141" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K141" s="16"/>
@@ -5559,11 +5586,11 @@
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J142" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K142" s="16"/>
@@ -5581,11 +5608,11 @@
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J143" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K143" s="16"/>
@@ -5603,11 +5630,11 @@
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J144" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K144" s="16"/>
@@ -5625,11 +5652,11 @@
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J145" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K145" s="16"/>
@@ -5647,11 +5674,11 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J146" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K146" s="16"/>
@@ -5669,11 +5696,11 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J147" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K147" s="16"/>
@@ -5691,11 +5718,11 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J148" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K148" s="16"/>
@@ -5713,11 +5740,11 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J149" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K149" s="16"/>
@@ -5735,11 +5762,11 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J150" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K150" s="16"/>
@@ -5757,11 +5784,11 @@
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
       <c r="I151" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J151" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K151" s="16"/>
@@ -5779,11 +5806,11 @@
       <c r="G152" s="14"/>
       <c r="H152" s="14"/>
       <c r="I152" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J152" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K152" s="16"/>
@@ -5801,11 +5828,11 @@
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J153" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K153" s="16"/>
@@ -5823,11 +5850,11 @@
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J154" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K154" s="16"/>
@@ -5845,11 +5872,11 @@
       <c r="G155" s="14"/>
       <c r="H155" s="14"/>
       <c r="I155" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J155" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K155" s="16"/>
@@ -5867,11 +5894,11 @@
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
       <c r="I156" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J156" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K156" s="16"/>
@@ -5889,11 +5916,11 @@
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J157" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K157" s="16"/>
@@ -5911,11 +5938,11 @@
       <c r="G158" s="14"/>
       <c r="H158" s="14"/>
       <c r="I158" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J158" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K158" s="16"/>
@@ -5933,11 +5960,11 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J159" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K159" s="16"/>
@@ -5955,11 +5982,11 @@
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
       <c r="I160" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J160" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K160" s="16"/>
@@ -5977,11 +6004,11 @@
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
       <c r="I161" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J161" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K161" s="16"/>
@@ -5999,11 +6026,11 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J162" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K162" s="16"/>
@@ -6021,11 +6048,11 @@
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
       <c r="I163" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J163" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K163" s="16"/>
@@ -6043,11 +6070,11 @@
       <c r="G164" s="14"/>
       <c r="H164" s="14"/>
       <c r="I164" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J164" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K164" s="16"/>
@@ -6065,11 +6092,11 @@
       <c r="G165" s="14"/>
       <c r="H165" s="14"/>
       <c r="I165" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J165" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K165" s="16"/>
@@ -6087,11 +6114,11 @@
       <c r="G166" s="14"/>
       <c r="H166" s="14"/>
       <c r="I166" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J166" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K166" s="16"/>
@@ -6109,11 +6136,11 @@
       <c r="G167" s="14"/>
       <c r="H167" s="14"/>
       <c r="I167" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J167" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K167" s="16"/>
@@ -6131,11 +6158,11 @@
       <c r="G168" s="14"/>
       <c r="H168" s="14"/>
       <c r="I168" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J168" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K168" s="16"/>
@@ -6153,11 +6180,11 @@
       <c r="G169" s="14"/>
       <c r="H169" s="14"/>
       <c r="I169" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J169" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K169" s="16"/>
@@ -6175,11 +6202,11 @@
       <c r="G170" s="14"/>
       <c r="H170" s="14"/>
       <c r="I170" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J170" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K170" s="16"/>
@@ -6197,11 +6224,11 @@
       <c r="G171" s="14"/>
       <c r="H171" s="14"/>
       <c r="I171" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J171" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K171" s="16"/>
@@ -6219,11 +6246,11 @@
       <c r="G172" s="14"/>
       <c r="H172" s="14"/>
       <c r="I172" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J172" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K172" s="16"/>
@@ -6241,11 +6268,11 @@
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
       <c r="I173" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J173" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K173" s="16"/>
@@ -6263,11 +6290,11 @@
       <c r="G174" s="14"/>
       <c r="H174" s="14"/>
       <c r="I174" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J174" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K174" s="16"/>
@@ -6285,11 +6312,11 @@
       <c r="G175" s="14"/>
       <c r="H175" s="14"/>
       <c r="I175" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J175" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K175" s="16"/>
@@ -6307,11 +6334,11 @@
       <c r="G176" s="14"/>
       <c r="H176" s="14"/>
       <c r="I176" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J176" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K176" s="16"/>
@@ -6329,11 +6356,11 @@
       <c r="G177" s="14"/>
       <c r="H177" s="14"/>
       <c r="I177" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J177" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K177" s="16"/>
@@ -6351,11 +6378,11 @@
       <c r="G178" s="14"/>
       <c r="H178" s="14"/>
       <c r="I178" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J178" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K178" s="16"/>
@@ -6373,11 +6400,11 @@
       <c r="G179" s="14"/>
       <c r="H179" s="14"/>
       <c r="I179" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J179" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K179" s="16"/>
@@ -6395,11 +6422,11 @@
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
       <c r="I180" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J180" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K180" s="16"/>
@@ -6417,11 +6444,11 @@
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J181" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K181" s="16"/>
@@ -6439,11 +6466,11 @@
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J182" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K182" s="16"/>
@@ -6461,11 +6488,11 @@
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J183" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K183" s="16"/>
@@ -6483,11 +6510,11 @@
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
       <c r="I184" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J184" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K184" s="16"/>
@@ -6505,11 +6532,11 @@
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
       <c r="I185" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J185" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K185" s="16"/>
@@ -6527,11 +6554,11 @@
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J186" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K186" s="16"/>
@@ -6549,11 +6576,11 @@
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J187" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K187" s="16"/>
@@ -6571,11 +6598,11 @@
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
       <c r="I188" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J188" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K188" s="16"/>
@@ -6593,11 +6620,11 @@
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
       <c r="I189" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J189" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K189" s="16"/>
@@ -6615,11 +6642,11 @@
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J190" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K190" s="16"/>
@@ -6637,11 +6664,11 @@
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J191" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K191" s="16"/>
@@ -6659,11 +6686,11 @@
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J192" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K192" s="16"/>
@@ -6681,11 +6708,11 @@
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
       <c r="I193" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J193" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K193" s="16"/>
@@ -6703,11 +6730,11 @@
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
       <c r="I194" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J194" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K194" s="16"/>
@@ -6725,11 +6752,11 @@
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J195" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K195" s="16"/>
@@ -6747,11 +6774,11 @@
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J196" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K196" s="16"/>
@@ -6769,11 +6796,11 @@
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J197" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K197" s="16"/>
@@ -6791,11 +6818,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="16">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" ref="I198:I261" si="18">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="17">IF(I198="","",1440-I198)</f>
+        <f t="shared" ref="J198:J261" si="19">IF(I198="","",1440-I198)</f>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -6813,11 +6840,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -6835,11 +6862,11 @@
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J200" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K200" s="16"/>
@@ -6857,11 +6884,11 @@
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
       <c r="I201" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J201" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K201" s="16"/>
@@ -6879,11 +6906,11 @@
       <c r="G202" s="14"/>
       <c r="H202" s="14"/>
       <c r="I202" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J202" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K202" s="16"/>
@@ -6901,11 +6928,11 @@
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
       <c r="I203" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J203" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K203" s="16"/>
@@ -6923,11 +6950,11 @@
       <c r="G204" s="14"/>
       <c r="H204" s="14"/>
       <c r="I204" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J204" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K204" s="16"/>
@@ -6945,11 +6972,11 @@
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J205" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K205" s="16"/>
@@ -6967,11 +6994,11 @@
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J206" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K206" s="16"/>
@@ -6989,11 +7016,11 @@
       <c r="G207" s="14"/>
       <c r="H207" s="14"/>
       <c r="I207" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J207" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K207" s="16"/>
@@ -7011,11 +7038,11 @@
       <c r="G208" s="14"/>
       <c r="H208" s="14"/>
       <c r="I208" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J208" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K208" s="16"/>
@@ -7033,11 +7060,11 @@
       <c r="G209" s="14"/>
       <c r="H209" s="14"/>
       <c r="I209" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J209" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K209" s="16"/>
@@ -7055,11 +7082,11 @@
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J210" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K210" s="16"/>
@@ -7077,11 +7104,11 @@
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J211" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K211" s="16"/>
@@ -7099,11 +7126,11 @@
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J212" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K212" s="16"/>
@@ -7121,11 +7148,11 @@
       <c r="G213" s="14"/>
       <c r="H213" s="14"/>
       <c r="I213" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J213" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K213" s="16"/>
@@ -7143,11 +7170,11 @@
       <c r="G214" s="14"/>
       <c r="H214" s="14"/>
       <c r="I214" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J214" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K214" s="16"/>
@@ -7165,11 +7192,11 @@
       <c r="G215" s="14"/>
       <c r="H215" s="14"/>
       <c r="I215" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J215" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K215" s="16"/>
@@ -7187,11 +7214,11 @@
       <c r="G216" s="14"/>
       <c r="H216" s="14"/>
       <c r="I216" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J216" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K216" s="16"/>
@@ -7209,11 +7236,11 @@
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J217" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K217" s="16"/>
@@ -7231,11 +7258,11 @@
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J218" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K218" s="16"/>
@@ -7253,11 +7280,11 @@
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J219" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K219" s="16"/>
@@ -7275,11 +7302,11 @@
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J220" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K220" s="16"/>
@@ -7297,11 +7324,11 @@
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J221" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K221" s="16"/>
@@ -7319,11 +7346,11 @@
       <c r="G222" s="14"/>
       <c r="H222" s="14"/>
       <c r="I222" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J222" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K222" s="16"/>
@@ -7341,11 +7368,11 @@
       <c r="G223" s="14"/>
       <c r="H223" s="14"/>
       <c r="I223" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J223" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K223" s="16"/>
@@ -7363,11 +7390,11 @@
       <c r="G224" s="14"/>
       <c r="H224" s="14"/>
       <c r="I224" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J224" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K224" s="16"/>
@@ -7385,11 +7412,11 @@
       <c r="G225" s="14"/>
       <c r="H225" s="14"/>
       <c r="I225" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J225" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K225" s="16"/>
@@ -7407,11 +7434,11 @@
       <c r="G226" s="14"/>
       <c r="H226" s="14"/>
       <c r="I226" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J226" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K226" s="16"/>
@@ -7429,11 +7456,11 @@
       <c r="G227" s="14"/>
       <c r="H227" s="14"/>
       <c r="I227" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J227" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K227" s="16"/>
@@ -7451,11 +7478,11 @@
       <c r="G228" s="14"/>
       <c r="H228" s="14"/>
       <c r="I228" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J228" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K228" s="16"/>
@@ -7473,11 +7500,11 @@
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J229" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K229" s="16"/>
@@ -7495,11 +7522,11 @@
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J230" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K230" s="16"/>
@@ -7517,11 +7544,11 @@
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
       <c r="I231" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J231" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K231" s="16"/>
@@ -7539,11 +7566,11 @@
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
       <c r="I232" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J232" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K232" s="16"/>
@@ -7561,11 +7588,11 @@
       <c r="G233" s="14"/>
       <c r="H233" s="14"/>
       <c r="I233" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J233" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K233" s="16"/>
@@ -7583,11 +7610,11 @@
       <c r="G234" s="14"/>
       <c r="H234" s="14"/>
       <c r="I234" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J234" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K234" s="16"/>
@@ -7605,11 +7632,11 @@
       <c r="G235" s="14"/>
       <c r="H235" s="14"/>
       <c r="I235" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J235" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K235" s="16"/>
@@ -7627,11 +7654,11 @@
       <c r="G236" s="14"/>
       <c r="H236" s="14"/>
       <c r="I236" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J236" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K236" s="16"/>
@@ -7649,11 +7676,11 @@
       <c r="G237" s="14"/>
       <c r="H237" s="14"/>
       <c r="I237" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J237" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K237" s="16"/>
@@ -7671,11 +7698,11 @@
       <c r="G238" s="14"/>
       <c r="H238" s="14"/>
       <c r="I238" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J238" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K238" s="16"/>
@@ -7693,11 +7720,11 @@
       <c r="G239" s="14"/>
       <c r="H239" s="14"/>
       <c r="I239" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J239" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K239" s="16"/>
@@ -7715,11 +7742,11 @@
       <c r="G240" s="14"/>
       <c r="H240" s="14"/>
       <c r="I240" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J240" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K240" s="16"/>
@@ -7737,11 +7764,11 @@
       <c r="G241" s="14"/>
       <c r="H241" s="14"/>
       <c r="I241" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J241" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K241" s="16"/>
@@ -7759,11 +7786,11 @@
       <c r="G242" s="14"/>
       <c r="H242" s="14"/>
       <c r="I242" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J242" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K242" s="16"/>
@@ -7781,11 +7808,11 @@
       <c r="G243" s="14"/>
       <c r="H243" s="14"/>
       <c r="I243" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J243" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K243" s="16"/>
@@ -7803,11 +7830,11 @@
       <c r="G244" s="14"/>
       <c r="H244" s="14"/>
       <c r="I244" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J244" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K244" s="16"/>
@@ -7825,11 +7852,11 @@
       <c r="G245" s="14"/>
       <c r="H245" s="14"/>
       <c r="I245" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J245" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K245" s="16"/>
@@ -7847,11 +7874,11 @@
       <c r="G246" s="14"/>
       <c r="H246" s="14"/>
       <c r="I246" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J246" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K246" s="16"/>
@@ -7869,11 +7896,11 @@
       <c r="G247" s="14"/>
       <c r="H247" s="14"/>
       <c r="I247" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J247" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K247" s="16"/>
@@ -7891,11 +7918,11 @@
       <c r="G248" s="14"/>
       <c r="H248" s="14"/>
       <c r="I248" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J248" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K248" s="16"/>
@@ -7913,11 +7940,11 @@
       <c r="G249" s="14"/>
       <c r="H249" s="14"/>
       <c r="I249" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J249" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K249" s="16"/>
@@ -7935,11 +7962,11 @@
       <c r="G250" s="14"/>
       <c r="H250" s="14"/>
       <c r="I250" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J250" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K250" s="16"/>
@@ -7957,11 +7984,11 @@
       <c r="G251" s="14"/>
       <c r="H251" s="14"/>
       <c r="I251" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J251" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K251" s="16"/>
@@ -7979,11 +8006,11 @@
       <c r="G252" s="14"/>
       <c r="H252" s="14"/>
       <c r="I252" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J252" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K252" s="16"/>
@@ -8001,11 +8028,11 @@
       <c r="G253" s="14"/>
       <c r="H253" s="14"/>
       <c r="I253" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J253" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K253" s="16"/>
@@ -8023,11 +8050,11 @@
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
       <c r="I254" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J254" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K254" s="16"/>
@@ -8045,11 +8072,11 @@
       <c r="G255" s="14"/>
       <c r="H255" s="14"/>
       <c r="I255" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J255" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K255" s="16"/>
@@ -8067,11 +8094,11 @@
       <c r="G256" s="14"/>
       <c r="H256" s="14"/>
       <c r="I256" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J256" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K256" s="16"/>
@@ -8089,11 +8116,11 @@
       <c r="G257" s="14"/>
       <c r="H257" s="14"/>
       <c r="I257" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J257" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K257" s="16"/>
@@ -8111,11 +8138,11 @@
       <c r="G258" s="14"/>
       <c r="H258" s="14"/>
       <c r="I258" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J258" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K258" s="16"/>
@@ -8133,11 +8160,11 @@
       <c r="G259" s="14"/>
       <c r="H259" s="14"/>
       <c r="I259" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J259" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K259" s="16"/>
@@ -8155,11 +8182,11 @@
       <c r="G260" s="14"/>
       <c r="H260" s="14"/>
       <c r="I260" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J260" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K260" s="16"/>
@@ -8177,11 +8204,11 @@
       <c r="G261" s="14"/>
       <c r="H261" s="14"/>
       <c r="I261" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J261" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K261" s="16"/>
@@ -8199,11 +8226,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="18">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" ref="I262:I325" si="20">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="19">IF(I262="","",1440-I262)</f>
+        <f t="shared" ref="J262:J325" si="21">IF(I262="","",1440-I262)</f>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -8221,11 +8248,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8243,11 +8270,11 @@
       <c r="G264" s="14"/>
       <c r="H264" s="14"/>
       <c r="I264" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J264" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K264" s="16"/>
@@ -8265,11 +8292,11 @@
       <c r="G265" s="14"/>
       <c r="H265" s="14"/>
       <c r="I265" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J265" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K265" s="16"/>
@@ -8287,11 +8314,11 @@
       <c r="G266" s="14"/>
       <c r="H266" s="14"/>
       <c r="I266" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J266" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K266" s="16"/>
@@ -8309,11 +8336,11 @@
       <c r="G267" s="14"/>
       <c r="H267" s="14"/>
       <c r="I267" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J267" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K267" s="16"/>
@@ -8331,11 +8358,11 @@
       <c r="G268" s="14"/>
       <c r="H268" s="14"/>
       <c r="I268" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J268" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K268" s="16"/>
@@ -8353,11 +8380,11 @@
       <c r="G269" s="14"/>
       <c r="H269" s="14"/>
       <c r="I269" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J269" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K269" s="16"/>
@@ -8375,11 +8402,11 @@
       <c r="G270" s="14"/>
       <c r="H270" s="14"/>
       <c r="I270" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J270" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K270" s="16"/>
@@ -8397,11 +8424,11 @@
       <c r="G271" s="14"/>
       <c r="H271" s="14"/>
       <c r="I271" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J271" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K271" s="16"/>
@@ -8419,11 +8446,11 @@
       <c r="G272" s="14"/>
       <c r="H272" s="14"/>
       <c r="I272" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J272" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K272" s="16"/>
@@ -8441,11 +8468,11 @@
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
       <c r="I273" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J273" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K273" s="16"/>
@@ -8463,11 +8490,11 @@
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
       <c r="I274" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J274" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K274" s="16"/>
@@ -8485,11 +8512,11 @@
       <c r="G275" s="14"/>
       <c r="H275" s="14"/>
       <c r="I275" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J275" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K275" s="16"/>
@@ -8507,11 +8534,11 @@
       <c r="G276" s="14"/>
       <c r="H276" s="14"/>
       <c r="I276" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J276" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K276" s="16"/>
@@ -8529,11 +8556,11 @@
       <c r="G277" s="14"/>
       <c r="H277" s="14"/>
       <c r="I277" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J277" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K277" s="16"/>
@@ -8551,11 +8578,11 @@
       <c r="G278" s="14"/>
       <c r="H278" s="14"/>
       <c r="I278" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J278" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K278" s="16"/>
@@ -8573,11 +8600,11 @@
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
       <c r="I279" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J279" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K279" s="16"/>
@@ -8595,11 +8622,11 @@
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
       <c r="I280" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J280" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K280" s="16"/>
@@ -8617,11 +8644,11 @@
       <c r="G281" s="14"/>
       <c r="H281" s="14"/>
       <c r="I281" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J281" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K281" s="16"/>
@@ -8639,11 +8666,11 @@
       <c r="G282" s="14"/>
       <c r="H282" s="14"/>
       <c r="I282" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J282" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K282" s="16"/>
@@ -8661,11 +8688,11 @@
       <c r="G283" s="14"/>
       <c r="H283" s="14"/>
       <c r="I283" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J283" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K283" s="16"/>
@@ -8683,11 +8710,11 @@
       <c r="G284" s="14"/>
       <c r="H284" s="14"/>
       <c r="I284" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J284" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K284" s="16"/>
@@ -8705,11 +8732,11 @@
       <c r="G285" s="14"/>
       <c r="H285" s="14"/>
       <c r="I285" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J285" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K285" s="16"/>
@@ -8727,11 +8754,11 @@
       <c r="G286" s="14"/>
       <c r="H286" s="14"/>
       <c r="I286" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J286" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K286" s="16"/>
@@ -8749,11 +8776,11 @@
       <c r="G287" s="14"/>
       <c r="H287" s="14"/>
       <c r="I287" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J287" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K287" s="16"/>
@@ -8771,11 +8798,11 @@
       <c r="G288" s="14"/>
       <c r="H288" s="14"/>
       <c r="I288" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J288" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K288" s="16"/>
@@ -8793,11 +8820,11 @@
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
       <c r="I289" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J289" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K289" s="16"/>
@@ -8815,11 +8842,11 @@
       <c r="G290" s="14"/>
       <c r="H290" s="14"/>
       <c r="I290" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J290" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K290" s="16"/>
@@ -8837,11 +8864,11 @@
       <c r="G291" s="14"/>
       <c r="H291" s="14"/>
       <c r="I291" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J291" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K291" s="16"/>
@@ -8859,11 +8886,11 @@
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
       <c r="I292" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J292" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K292" s="16"/>
@@ -8881,11 +8908,11 @@
       <c r="G293" s="14"/>
       <c r="H293" s="14"/>
       <c r="I293" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J293" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K293" s="16"/>
@@ -8903,11 +8930,11 @@
       <c r="G294" s="14"/>
       <c r="H294" s="14"/>
       <c r="I294" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J294" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K294" s="16"/>
@@ -8925,11 +8952,11 @@
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
       <c r="I295" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J295" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K295" s="16"/>
@@ -8947,11 +8974,11 @@
       <c r="G296" s="14"/>
       <c r="H296" s="14"/>
       <c r="I296" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J296" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K296" s="16"/>
@@ -8969,11 +8996,11 @@
       <c r="G297" s="14"/>
       <c r="H297" s="14"/>
       <c r="I297" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J297" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K297" s="16"/>
@@ -8991,11 +9018,11 @@
       <c r="G298" s="14"/>
       <c r="H298" s="14"/>
       <c r="I298" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J298" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K298" s="16"/>
@@ -9013,11 +9040,11 @@
       <c r="G299" s="14"/>
       <c r="H299" s="14"/>
       <c r="I299" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J299" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K299" s="16"/>
@@ -9035,11 +9062,11 @@
       <c r="G300" s="14"/>
       <c r="H300" s="14"/>
       <c r="I300" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J300" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K300" s="16"/>
@@ -9057,11 +9084,11 @@
       <c r="G301" s="14"/>
       <c r="H301" s="14"/>
       <c r="I301" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J301" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K301" s="16"/>
@@ -9079,11 +9106,11 @@
       <c r="G302" s="14"/>
       <c r="H302" s="14"/>
       <c r="I302" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J302" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K302" s="16"/>
@@ -9101,11 +9128,11 @@
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
       <c r="I303" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J303" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K303" s="16"/>
@@ -9123,11 +9150,11 @@
       <c r="G304" s="14"/>
       <c r="H304" s="14"/>
       <c r="I304" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J304" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K304" s="16"/>
@@ -9145,11 +9172,11 @@
       <c r="G305" s="14"/>
       <c r="H305" s="14"/>
       <c r="I305" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J305" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K305" s="16"/>
@@ -9167,11 +9194,11 @@
       <c r="G306" s="14"/>
       <c r="H306" s="14"/>
       <c r="I306" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J306" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K306" s="16"/>
@@ -9189,11 +9216,11 @@
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
       <c r="I307" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J307" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K307" s="16"/>
@@ -9211,11 +9238,11 @@
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
       <c r="I308" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J308" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K308" s="16"/>
@@ -9233,11 +9260,11 @@
       <c r="G309" s="14"/>
       <c r="H309" s="14"/>
       <c r="I309" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J309" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K309" s="16"/>
@@ -9255,11 +9282,11 @@
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
       <c r="I310" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J310" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K310" s="16"/>
@@ -9277,11 +9304,11 @@
       <c r="G311" s="14"/>
       <c r="H311" s="14"/>
       <c r="I311" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J311" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K311" s="16"/>
@@ -9299,11 +9326,11 @@
       <c r="G312" s="14"/>
       <c r="H312" s="14"/>
       <c r="I312" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J312" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K312" s="16"/>
@@ -9321,11 +9348,11 @@
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
       <c r="I313" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J313" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K313" s="16"/>
@@ -9343,11 +9370,11 @@
       <c r="G314" s="14"/>
       <c r="H314" s="14"/>
       <c r="I314" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J314" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K314" s="16"/>
@@ -9365,11 +9392,11 @@
       <c r="G315" s="14"/>
       <c r="H315" s="14"/>
       <c r="I315" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J315" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K315" s="16"/>
@@ -9387,11 +9414,11 @@
       <c r="G316" s="14"/>
       <c r="H316" s="14"/>
       <c r="I316" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J316" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K316" s="16"/>
@@ -9409,11 +9436,11 @@
       <c r="G317" s="14"/>
       <c r="H317" s="14"/>
       <c r="I317" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J317" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K317" s="16"/>
@@ -9431,11 +9458,11 @@
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
       <c r="I318" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J318" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K318" s="16"/>
@@ -9453,11 +9480,11 @@
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
       <c r="I319" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J319" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K319" s="16"/>
@@ -9475,11 +9502,11 @@
       <c r="G320" s="14"/>
       <c r="H320" s="14"/>
       <c r="I320" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J320" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K320" s="16"/>
@@ -9497,11 +9524,11 @@
       <c r="G321" s="14"/>
       <c r="H321" s="14"/>
       <c r="I321" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J321" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K321" s="16"/>
@@ -9519,11 +9546,11 @@
       <c r="G322" s="14"/>
       <c r="H322" s="14"/>
       <c r="I322" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J322" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K322" s="16"/>
@@ -9541,11 +9568,11 @@
       <c r="G323" s="14"/>
       <c r="H323" s="14"/>
       <c r="I323" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J323" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K323" s="16"/>
@@ -9563,11 +9590,11 @@
       <c r="G324" s="14"/>
       <c r="H324" s="14"/>
       <c r="I324" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J324" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K324" s="16"/>
@@ -9585,11 +9612,11 @@
       <c r="G325" s="14"/>
       <c r="H325" s="14"/>
       <c r="I325" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J325" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K325" s="16"/>
@@ -9607,11 +9634,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="20">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" ref="I326:I389" si="22">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="21">IF(I326="","",1440-I326)</f>
+        <f t="shared" ref="J326:J389" si="23">IF(I326="","",1440-I326)</f>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -9629,11 +9656,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -9651,11 +9678,11 @@
       <c r="G328" s="14"/>
       <c r="H328" s="14"/>
       <c r="I328" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J328" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K328" s="16"/>
@@ -9673,11 +9700,11 @@
       <c r="G329" s="14"/>
       <c r="H329" s="14"/>
       <c r="I329" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J329" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K329" s="16"/>
@@ -9695,11 +9722,11 @@
       <c r="G330" s="14"/>
       <c r="H330" s="14"/>
       <c r="I330" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J330" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K330" s="16"/>
@@ -9717,11 +9744,11 @@
       <c r="G331" s="14"/>
       <c r="H331" s="14"/>
       <c r="I331" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J331" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K331" s="16"/>
@@ -9739,11 +9766,11 @@
       <c r="G332" s="14"/>
       <c r="H332" s="14"/>
       <c r="I332" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J332" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K332" s="16"/>
@@ -9761,11 +9788,11 @@
       <c r="G333" s="14"/>
       <c r="H333" s="14"/>
       <c r="I333" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J333" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K333" s="16"/>
@@ -9783,11 +9810,11 @@
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
       <c r="I334" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J334" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K334" s="16"/>
@@ -9805,11 +9832,11 @@
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
       <c r="I335" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J335" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K335" s="16"/>
@@ -9827,11 +9854,11 @@
       <c r="G336" s="14"/>
       <c r="H336" s="14"/>
       <c r="I336" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J336" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K336" s="16"/>
@@ -9849,11 +9876,11 @@
       <c r="G337" s="14"/>
       <c r="H337" s="14"/>
       <c r="I337" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J337" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K337" s="16"/>
@@ -9871,11 +9898,11 @@
       <c r="G338" s="14"/>
       <c r="H338" s="14"/>
       <c r="I338" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J338" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K338" s="16"/>
@@ -9893,11 +9920,11 @@
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
       <c r="I339" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J339" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K339" s="16"/>
@@ -9915,11 +9942,11 @@
       <c r="G340" s="14"/>
       <c r="H340" s="14"/>
       <c r="I340" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J340" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K340" s="16"/>
@@ -9937,11 +9964,11 @@
       <c r="G341" s="14"/>
       <c r="H341" s="14"/>
       <c r="I341" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J341" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K341" s="16"/>
@@ -9959,11 +9986,11 @@
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
       <c r="I342" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J342" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K342" s="16"/>
@@ -9981,11 +10008,11 @@
       <c r="G343" s="14"/>
       <c r="H343" s="14"/>
       <c r="I343" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J343" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K343" s="16"/>
@@ -10003,11 +10030,11 @@
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
       <c r="I344" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J344" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K344" s="16"/>
@@ -10025,11 +10052,11 @@
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
       <c r="I345" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J345" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K345" s="16"/>
@@ -10047,11 +10074,11 @@
       <c r="G346" s="14"/>
       <c r="H346" s="14"/>
       <c r="I346" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J346" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K346" s="16"/>
@@ -10069,11 +10096,11 @@
       <c r="G347" s="14"/>
       <c r="H347" s="14"/>
       <c r="I347" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J347" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K347" s="16"/>
@@ -10091,11 +10118,11 @@
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
       <c r="I348" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J348" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K348" s="16"/>
@@ -10113,11 +10140,11 @@
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
       <c r="I349" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J349" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K349" s="16"/>
@@ -10135,11 +10162,11 @@
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
       <c r="I350" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J350" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K350" s="16"/>
@@ -10157,11 +10184,11 @@
       <c r="G351" s="14"/>
       <c r="H351" s="14"/>
       <c r="I351" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J351" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K351" s="16"/>
@@ -10179,11 +10206,11 @@
       <c r="G352" s="14"/>
       <c r="H352" s="14"/>
       <c r="I352" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J352" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K352" s="16"/>
@@ -10201,11 +10228,11 @@
       <c r="G353" s="14"/>
       <c r="H353" s="14"/>
       <c r="I353" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J353" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K353" s="16"/>
@@ -10223,11 +10250,11 @@
       <c r="G354" s="14"/>
       <c r="H354" s="14"/>
       <c r="I354" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J354" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K354" s="16"/>
@@ -10245,11 +10272,11 @@
       <c r="G355" s="14"/>
       <c r="H355" s="14"/>
       <c r="I355" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J355" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K355" s="16"/>
@@ -10267,11 +10294,11 @@
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
       <c r="I356" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J356" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K356" s="16"/>
@@ -10289,11 +10316,11 @@
       <c r="G357" s="14"/>
       <c r="H357" s="14"/>
       <c r="I357" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J357" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K357" s="16"/>
@@ -10311,11 +10338,11 @@
       <c r="G358" s="14"/>
       <c r="H358" s="14"/>
       <c r="I358" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J358" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K358" s="16"/>
@@ -10333,11 +10360,11 @@
       <c r="G359" s="14"/>
       <c r="H359" s="14"/>
       <c r="I359" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J359" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K359" s="16"/>
@@ -10355,11 +10382,11 @@
       <c r="G360" s="14"/>
       <c r="H360" s="14"/>
       <c r="I360" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J360" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K360" s="16"/>
@@ -10377,11 +10404,11 @@
       <c r="G361" s="14"/>
       <c r="H361" s="14"/>
       <c r="I361" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J361" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K361" s="16"/>
@@ -10399,11 +10426,11 @@
       <c r="G362" s="14"/>
       <c r="H362" s="14"/>
       <c r="I362" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J362" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K362" s="16"/>
@@ -10421,11 +10448,11 @@
       <c r="G363" s="14"/>
       <c r="H363" s="14"/>
       <c r="I363" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J363" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K363" s="16"/>
@@ -10443,11 +10470,11 @@
       <c r="G364" s="14"/>
       <c r="H364" s="14"/>
       <c r="I364" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J364" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K364" s="16"/>
@@ -10465,11 +10492,11 @@
       <c r="G365" s="14"/>
       <c r="H365" s="14"/>
       <c r="I365" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J365" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K365" s="16"/>
@@ -10487,11 +10514,11 @@
       <c r="G366" s="14"/>
       <c r="H366" s="14"/>
       <c r="I366" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J366" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K366" s="16"/>
@@ -10509,11 +10536,11 @@
       <c r="G367" s="14"/>
       <c r="H367" s="14"/>
       <c r="I367" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J367" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K367" s="16"/>
@@ -10531,11 +10558,11 @@
       <c r="G368" s="14"/>
       <c r="H368" s="14"/>
       <c r="I368" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J368" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K368" s="16"/>
@@ -10553,11 +10580,11 @@
       <c r="G369" s="14"/>
       <c r="H369" s="14"/>
       <c r="I369" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J369" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K369" s="16"/>
@@ -10575,11 +10602,11 @@
       <c r="G370" s="14"/>
       <c r="H370" s="14"/>
       <c r="I370" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J370" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K370" s="16"/>
@@ -10597,11 +10624,11 @@
       <c r="G371" s="14"/>
       <c r="H371" s="14"/>
       <c r="I371" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J371" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K371" s="16"/>
@@ -10619,11 +10646,11 @@
       <c r="G372" s="14"/>
       <c r="H372" s="14"/>
       <c r="I372" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J372" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K372" s="16"/>
@@ -10641,11 +10668,11 @@
       <c r="G373" s="14"/>
       <c r="H373" s="14"/>
       <c r="I373" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J373" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K373" s="16"/>
@@ -10663,11 +10690,11 @@
       <c r="G374" s="14"/>
       <c r="H374" s="14"/>
       <c r="I374" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J374" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K374" s="16"/>
@@ -10685,11 +10712,11 @@
       <c r="G375" s="14"/>
       <c r="H375" s="14"/>
       <c r="I375" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J375" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K375" s="16"/>
@@ -10707,11 +10734,11 @@
       <c r="G376" s="14"/>
       <c r="H376" s="14"/>
       <c r="I376" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J376" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K376" s="16"/>
@@ -10729,11 +10756,11 @@
       <c r="G377" s="14"/>
       <c r="H377" s="14"/>
       <c r="I377" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J377" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K377" s="16"/>
@@ -10751,11 +10778,11 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K378" s="16"/>
@@ -10773,11 +10800,11 @@
       <c r="G379" s="14"/>
       <c r="H379" s="14"/>
       <c r="I379" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J379" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K379" s="16"/>
@@ -10795,11 +10822,11 @@
       <c r="G380" s="14"/>
       <c r="H380" s="14"/>
       <c r="I380" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J380" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K380" s="16"/>
@@ -10817,11 +10844,11 @@
       <c r="G381" s="14"/>
       <c r="H381" s="14"/>
       <c r="I381" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J381" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K381" s="16"/>
@@ -10839,11 +10866,11 @@
       <c r="G382" s="14"/>
       <c r="H382" s="14"/>
       <c r="I382" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J382" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K382" s="16"/>
@@ -10861,11 +10888,11 @@
       <c r="G383" s="14"/>
       <c r="H383" s="14"/>
       <c r="I383" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J383" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K383" s="16"/>
@@ -10883,11 +10910,11 @@
       <c r="G384" s="14"/>
       <c r="H384" s="14"/>
       <c r="I384" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J384" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K384" s="16"/>
@@ -10905,11 +10932,11 @@
       <c r="G385" s="14"/>
       <c r="H385" s="14"/>
       <c r="I385" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J385" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K385" s="16"/>
@@ -10927,11 +10954,11 @@
       <c r="G386" s="14"/>
       <c r="H386" s="14"/>
       <c r="I386" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J386" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K386" s="16"/>
@@ -10949,11 +10976,11 @@
       <c r="G387" s="14"/>
       <c r="H387" s="14"/>
       <c r="I387" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J387" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K387" s="16"/>
@@ -10971,11 +10998,11 @@
       <c r="G388" s="14"/>
       <c r="H388" s="14"/>
       <c r="I388" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J388" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K388" s="16"/>
@@ -10993,11 +11020,11 @@
       <c r="G389" s="14"/>
       <c r="H389" s="14"/>
       <c r="I389" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J389" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K389" s="16"/>
@@ -11015,11 +11042,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="22">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="24">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="23">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="25">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -11037,11 +11064,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -11059,11 +11086,11 @@
       <c r="G392" s="14"/>
       <c r="H392" s="14"/>
       <c r="I392" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J392" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K392" s="16"/>
@@ -11081,11 +11108,11 @@
       <c r="G393" s="14"/>
       <c r="H393" s="14"/>
       <c r="I393" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J393" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K393" s="16"/>
@@ -11103,11 +11130,11 @@
       <c r="G394" s="14"/>
       <c r="H394" s="14"/>
       <c r="I394" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J394" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K394" s="16"/>
@@ -11125,11 +11152,11 @@
       <c r="G395" s="14"/>
       <c r="H395" s="14"/>
       <c r="I395" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J395" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K395" s="16"/>
@@ -11147,11 +11174,11 @@
       <c r="G396" s="14"/>
       <c r="H396" s="14"/>
       <c r="I396" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J396" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K396" s="16"/>
@@ -11169,11 +11196,11 @@
       <c r="G397" s="14"/>
       <c r="H397" s="14"/>
       <c r="I397" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J397" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K397" s="16"/>
@@ -11191,11 +11218,11 @@
       <c r="G398" s="14"/>
       <c r="H398" s="14"/>
       <c r="I398" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J398" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K398" s="16"/>
@@ -11213,11 +11240,11 @@
       <c r="G399" s="14"/>
       <c r="H399" s="14"/>
       <c r="I399" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J399" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K399" s="16"/>
@@ -11235,11 +11262,11 @@
       <c r="G400" s="14"/>
       <c r="H400" s="14"/>
       <c r="I400" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J400" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K400" s="16"/>
@@ -11257,11 +11284,11 @@
       <c r="G401" s="14"/>
       <c r="H401" s="14"/>
       <c r="I401" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J401" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K401" s="16"/>

</xml_diff>

<commit_message>
File Updated On 19/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20EED29D-D852-45C1-A4D5-883EAE5151FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FCEC20-4567-4288-981C-5073C6364B96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="612" yWindow="-108" windowWidth="22536" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -304,7 +304,7 @@
     <t>5th mid term</t>
   </si>
   <si>
-    <t>s</t>
+    <t>Classes started from today after mid terms</t>
   </si>
 </sst>
 </file>
@@ -3893,8 +3893,8 @@
       <c r="D66" s="14">
         <v>100</v>
       </c>
-      <c r="E66" s="14" t="s">
-        <v>89</v>
+      <c r="E66" s="14">
+        <v>0</v>
       </c>
       <c r="F66" s="14">
         <v>0</v>
@@ -3926,27 +3926,51 @@
         <v>82</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A67" s="13"/>
-      <c r="B67" s="14"/>
-      <c r="C67" s="14"/>
-      <c r="D67" s="14"/>
-      <c r="E67" s="14"/>
-      <c r="F67" s="14"/>
-      <c r="G67" s="14"/>
-      <c r="H67" s="14"/>
-      <c r="I67" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J67" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K67" s="16"/>
-      <c r="L67" s="16"/>
-      <c r="M67" s="16"/>
-      <c r="N67" s="17"/>
+    <row r="67" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A67" s="13">
+        <v>46314</v>
+      </c>
+      <c r="B67" s="14">
+        <v>420</v>
+      </c>
+      <c r="C67" s="14">
+        <v>0</v>
+      </c>
+      <c r="D67" s="14">
+        <v>150</v>
+      </c>
+      <c r="E67" s="14">
+        <v>0</v>
+      </c>
+      <c r="F67" s="14">
+        <v>0</v>
+      </c>
+      <c r="G67" s="14">
+        <v>0</v>
+      </c>
+      <c r="H67" s="14">
+        <v>120</v>
+      </c>
+      <c r="I67" s="15">
+        <f t="shared" ref="I67" si="14">IF(SUM(B67:F67,H67)=0,"",SUM(B67:F67,H67))</f>
+        <v>690</v>
+      </c>
+      <c r="J67" s="15">
+        <f t="shared" ref="J67" si="15">IF(I67="","",1440-I67)</f>
+        <v>750</v>
+      </c>
+      <c r="K67" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L67" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M67" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N67" s="17" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" s="13"/>
@@ -4002,11 +4026,11 @@
       <c r="G70" s="14"/>
       <c r="H70" s="14"/>
       <c r="I70" s="15" t="str">
-        <f t="shared" ref="I70:I133" si="14">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
+        <f t="shared" ref="I70:I133" si="16">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
         <v/>
       </c>
       <c r="J70" s="15" t="str">
-        <f t="shared" ref="J70:J133" si="15">IF(I70="","",1440-I70)</f>
+        <f t="shared" ref="J70:J133" si="17">IF(I70="","",1440-I70)</f>
         <v/>
       </c>
       <c r="K70" s="16"/>
@@ -4024,11 +4048,11 @@
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
       <c r="I71" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J71" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K71" s="16"/>
@@ -4046,11 +4070,11 @@
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
       <c r="I72" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J72" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K72" s="16"/>
@@ -4068,11 +4092,11 @@
       <c r="G73" s="14"/>
       <c r="H73" s="14"/>
       <c r="I73" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J73" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K73" s="16"/>
@@ -4090,11 +4114,11 @@
       <c r="G74" s="14"/>
       <c r="H74" s="14"/>
       <c r="I74" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J74" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K74" s="16"/>
@@ -4112,11 +4136,11 @@
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
       <c r="I75" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J75" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K75" s="16"/>
@@ -4134,11 +4158,11 @@
       <c r="G76" s="14"/>
       <c r="H76" s="14"/>
       <c r="I76" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J76" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K76" s="16"/>
@@ -4156,11 +4180,11 @@
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
       <c r="I77" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J77" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K77" s="16"/>
@@ -4178,11 +4202,11 @@
       <c r="G78" s="14"/>
       <c r="H78" s="14"/>
       <c r="I78" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J78" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K78" s="16"/>
@@ -4200,11 +4224,11 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J79" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K79" s="16"/>
@@ -4222,11 +4246,11 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J80" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K80" s="16"/>
@@ -4244,11 +4268,11 @@
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J81" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K81" s="16"/>
@@ -4266,11 +4290,11 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J82" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K82" s="16"/>
@@ -4288,11 +4312,11 @@
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
       <c r="I83" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J83" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K83" s="16"/>
@@ -4310,11 +4334,11 @@
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
       <c r="I84" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J84" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K84" s="16"/>
@@ -4332,11 +4356,11 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J85" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K85" s="16"/>
@@ -4354,11 +4378,11 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J86" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K86" s="16"/>
@@ -4376,11 +4400,11 @@
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
       <c r="I87" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J87" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K87" s="16"/>
@@ -4398,11 +4422,11 @@
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
       <c r="I88" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J88" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K88" s="16"/>
@@ -4420,11 +4444,11 @@
       <c r="G89" s="14"/>
       <c r="H89" s="14"/>
       <c r="I89" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J89" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K89" s="16"/>
@@ -4442,11 +4466,11 @@
       <c r="G90" s="14"/>
       <c r="H90" s="14"/>
       <c r="I90" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J90" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K90" s="16"/>
@@ -4464,11 +4488,11 @@
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
       <c r="I91" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J91" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K91" s="16"/>
@@ -4486,11 +4510,11 @@
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
       <c r="I92" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J92" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K92" s="16"/>
@@ -4508,11 +4532,11 @@
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J93" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K93" s="16"/>
@@ -4530,11 +4554,11 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J94" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K94" s="16"/>
@@ -4552,11 +4576,11 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J95" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K95" s="16"/>
@@ -4574,11 +4598,11 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J96" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K96" s="16"/>
@@ -4596,11 +4620,11 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J97" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K97" s="16"/>
@@ -4618,11 +4642,11 @@
       <c r="G98" s="14"/>
       <c r="H98" s="14"/>
       <c r="I98" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J98" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K98" s="16"/>
@@ -4640,11 +4664,11 @@
       <c r="G99" s="14"/>
       <c r="H99" s="14"/>
       <c r="I99" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J99" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K99" s="16"/>
@@ -4662,11 +4686,11 @@
       <c r="G100" s="14"/>
       <c r="H100" s="14"/>
       <c r="I100" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J100" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K100" s="16"/>
@@ -4684,11 +4708,11 @@
       <c r="G101" s="14"/>
       <c r="H101" s="14"/>
       <c r="I101" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J101" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K101" s="16"/>
@@ -4706,11 +4730,11 @@
       <c r="G102" s="14"/>
       <c r="H102" s="14"/>
       <c r="I102" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J102" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K102" s="16"/>
@@ -4728,11 +4752,11 @@
       <c r="G103" s="14"/>
       <c r="H103" s="14"/>
       <c r="I103" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J103" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K103" s="16"/>
@@ -4750,11 +4774,11 @@
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
       <c r="I104" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J104" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K104" s="16"/>
@@ -4772,11 +4796,11 @@
       <c r="G105" s="14"/>
       <c r="H105" s="14"/>
       <c r="I105" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J105" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K105" s="16"/>
@@ -4794,11 +4818,11 @@
       <c r="G106" s="14"/>
       <c r="H106" s="14"/>
       <c r="I106" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J106" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K106" s="16"/>
@@ -4816,11 +4840,11 @@
       <c r="G107" s="14"/>
       <c r="H107" s="14"/>
       <c r="I107" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J107" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K107" s="16"/>
@@ -4838,11 +4862,11 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J108" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K108" s="16"/>
@@ -4860,11 +4884,11 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J109" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K109" s="16"/>
@@ -4882,11 +4906,11 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J110" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K110" s="16"/>
@@ -4904,11 +4928,11 @@
       <c r="G111" s="14"/>
       <c r="H111" s="14"/>
       <c r="I111" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J111" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K111" s="16"/>
@@ -4926,11 +4950,11 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J112" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K112" s="16"/>
@@ -4948,11 +4972,11 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J113" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K113" s="16"/>
@@ -4970,11 +4994,11 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J114" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K114" s="16"/>
@@ -4992,11 +5016,11 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J115" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K115" s="16"/>
@@ -5014,11 +5038,11 @@
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
       <c r="I116" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J116" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K116" s="16"/>
@@ -5036,11 +5060,11 @@
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
       <c r="I117" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J117" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K117" s="16"/>
@@ -5058,11 +5082,11 @@
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
       <c r="I118" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J118" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K118" s="16"/>
@@ -5080,11 +5104,11 @@
       <c r="G119" s="14"/>
       <c r="H119" s="14"/>
       <c r="I119" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J119" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K119" s="16"/>
@@ -5102,11 +5126,11 @@
       <c r="G120" s="14"/>
       <c r="H120" s="14"/>
       <c r="I120" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J120" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K120" s="16"/>
@@ -5124,11 +5148,11 @@
       <c r="G121" s="14"/>
       <c r="H121" s="14"/>
       <c r="I121" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J121" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K121" s="16"/>
@@ -5146,11 +5170,11 @@
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
       <c r="I122" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J122" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K122" s="16"/>
@@ -5168,11 +5192,11 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J123" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K123" s="16"/>
@@ -5190,11 +5214,11 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J124" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K124" s="16"/>
@@ -5212,11 +5236,11 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J125" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K125" s="16"/>
@@ -5234,11 +5258,11 @@
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
       <c r="I126" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J126" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K126" s="16"/>
@@ -5256,11 +5280,11 @@
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J127" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K127" s="16"/>
@@ -5278,11 +5302,11 @@
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
       <c r="I128" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J128" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K128" s="16"/>
@@ -5300,11 +5324,11 @@
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
       <c r="I129" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J129" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K129" s="16"/>
@@ -5322,11 +5346,11 @@
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
       <c r="I130" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J130" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K130" s="16"/>
@@ -5344,11 +5368,11 @@
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
       <c r="I131" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J131" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K131" s="16"/>
@@ -5366,11 +5390,11 @@
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
       <c r="I132" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J132" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K132" s="16"/>
@@ -5388,11 +5412,11 @@
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
       <c r="I133" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J133" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K133" s="16"/>
@@ -5410,11 +5434,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="16">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" ref="I134:I197" si="18">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="17">IF(I134="","",1440-I134)</f>
+        <f t="shared" ref="J134:J197" si="19">IF(I134="","",1440-I134)</f>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -5432,11 +5456,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5454,11 +5478,11 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J136" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K136" s="16"/>
@@ -5476,11 +5500,11 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J137" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K137" s="16"/>
@@ -5498,11 +5522,11 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J138" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K138" s="16"/>
@@ -5520,11 +5544,11 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J139" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K139" s="16"/>
@@ -5542,11 +5566,11 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J140" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K140" s="16"/>
@@ -5564,11 +5588,11 @@
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J141" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K141" s="16"/>
@@ -5586,11 +5610,11 @@
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J142" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K142" s="16"/>
@@ -5608,11 +5632,11 @@
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J143" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K143" s="16"/>
@@ -5630,11 +5654,11 @@
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J144" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K144" s="16"/>
@@ -5652,11 +5676,11 @@
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J145" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K145" s="16"/>
@@ -5674,11 +5698,11 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J146" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K146" s="16"/>
@@ -5696,11 +5720,11 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J147" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K147" s="16"/>
@@ -5718,11 +5742,11 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J148" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K148" s="16"/>
@@ -5740,11 +5764,11 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J149" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K149" s="16"/>
@@ -5762,11 +5786,11 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J150" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K150" s="16"/>
@@ -5784,11 +5808,11 @@
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
       <c r="I151" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J151" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K151" s="16"/>
@@ -5806,11 +5830,11 @@
       <c r="G152" s="14"/>
       <c r="H152" s="14"/>
       <c r="I152" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J152" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K152" s="16"/>
@@ -5828,11 +5852,11 @@
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J153" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K153" s="16"/>
@@ -5850,11 +5874,11 @@
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J154" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K154" s="16"/>
@@ -5872,11 +5896,11 @@
       <c r="G155" s="14"/>
       <c r="H155" s="14"/>
       <c r="I155" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J155" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K155" s="16"/>
@@ -5894,11 +5918,11 @@
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
       <c r="I156" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J156" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K156" s="16"/>
@@ -5916,11 +5940,11 @@
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J157" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K157" s="16"/>
@@ -5938,11 +5962,11 @@
       <c r="G158" s="14"/>
       <c r="H158" s="14"/>
       <c r="I158" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J158" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K158" s="16"/>
@@ -5960,11 +5984,11 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J159" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K159" s="16"/>
@@ -5982,11 +6006,11 @@
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
       <c r="I160" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J160" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K160" s="16"/>
@@ -6004,11 +6028,11 @@
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
       <c r="I161" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J161" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K161" s="16"/>
@@ -6026,11 +6050,11 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J162" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K162" s="16"/>
@@ -6048,11 +6072,11 @@
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
       <c r="I163" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J163" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K163" s="16"/>
@@ -6070,11 +6094,11 @@
       <c r="G164" s="14"/>
       <c r="H164" s="14"/>
       <c r="I164" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J164" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K164" s="16"/>
@@ -6092,11 +6116,11 @@
       <c r="G165" s="14"/>
       <c r="H165" s="14"/>
       <c r="I165" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J165" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K165" s="16"/>
@@ -6114,11 +6138,11 @@
       <c r="G166" s="14"/>
       <c r="H166" s="14"/>
       <c r="I166" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J166" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K166" s="16"/>
@@ -6136,11 +6160,11 @@
       <c r="G167" s="14"/>
       <c r="H167" s="14"/>
       <c r="I167" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J167" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K167" s="16"/>
@@ -6158,11 +6182,11 @@
       <c r="G168" s="14"/>
       <c r="H168" s="14"/>
       <c r="I168" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J168" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K168" s="16"/>
@@ -6180,11 +6204,11 @@
       <c r="G169" s="14"/>
       <c r="H169" s="14"/>
       <c r="I169" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J169" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K169" s="16"/>
@@ -6202,11 +6226,11 @@
       <c r="G170" s="14"/>
       <c r="H170" s="14"/>
       <c r="I170" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J170" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K170" s="16"/>
@@ -6224,11 +6248,11 @@
       <c r="G171" s="14"/>
       <c r="H171" s="14"/>
       <c r="I171" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J171" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K171" s="16"/>
@@ -6246,11 +6270,11 @@
       <c r="G172" s="14"/>
       <c r="H172" s="14"/>
       <c r="I172" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J172" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K172" s="16"/>
@@ -6268,11 +6292,11 @@
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
       <c r="I173" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J173" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K173" s="16"/>
@@ -6290,11 +6314,11 @@
       <c r="G174" s="14"/>
       <c r="H174" s="14"/>
       <c r="I174" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J174" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K174" s="16"/>
@@ -6312,11 +6336,11 @@
       <c r="G175" s="14"/>
       <c r="H175" s="14"/>
       <c r="I175" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J175" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K175" s="16"/>
@@ -6334,11 +6358,11 @@
       <c r="G176" s="14"/>
       <c r="H176" s="14"/>
       <c r="I176" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J176" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K176" s="16"/>
@@ -6356,11 +6380,11 @@
       <c r="G177" s="14"/>
       <c r="H177" s="14"/>
       <c r="I177" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J177" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K177" s="16"/>
@@ -6378,11 +6402,11 @@
       <c r="G178" s="14"/>
       <c r="H178" s="14"/>
       <c r="I178" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J178" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K178" s="16"/>
@@ -6400,11 +6424,11 @@
       <c r="G179" s="14"/>
       <c r="H179" s="14"/>
       <c r="I179" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J179" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K179" s="16"/>
@@ -6422,11 +6446,11 @@
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
       <c r="I180" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J180" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K180" s="16"/>
@@ -6444,11 +6468,11 @@
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J181" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K181" s="16"/>
@@ -6466,11 +6490,11 @@
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J182" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K182" s="16"/>
@@ -6488,11 +6512,11 @@
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J183" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K183" s="16"/>
@@ -6510,11 +6534,11 @@
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
       <c r="I184" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J184" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K184" s="16"/>
@@ -6532,11 +6556,11 @@
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
       <c r="I185" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J185" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K185" s="16"/>
@@ -6554,11 +6578,11 @@
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J186" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K186" s="16"/>
@@ -6576,11 +6600,11 @@
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J187" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K187" s="16"/>
@@ -6598,11 +6622,11 @@
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
       <c r="I188" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J188" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K188" s="16"/>
@@ -6620,11 +6644,11 @@
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
       <c r="I189" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J189" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K189" s="16"/>
@@ -6642,11 +6666,11 @@
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J190" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K190" s="16"/>
@@ -6664,11 +6688,11 @@
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J191" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K191" s="16"/>
@@ -6686,11 +6710,11 @@
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J192" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K192" s="16"/>
@@ -6708,11 +6732,11 @@
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
       <c r="I193" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J193" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K193" s="16"/>
@@ -6730,11 +6754,11 @@
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
       <c r="I194" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J194" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K194" s="16"/>
@@ -6752,11 +6776,11 @@
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J195" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K195" s="16"/>
@@ -6774,11 +6798,11 @@
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J196" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K196" s="16"/>
@@ -6796,11 +6820,11 @@
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J197" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K197" s="16"/>
@@ -6818,11 +6842,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="18">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" ref="I198:I261" si="20">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="19">IF(I198="","",1440-I198)</f>
+        <f t="shared" ref="J198:J261" si="21">IF(I198="","",1440-I198)</f>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -6840,11 +6864,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -6862,11 +6886,11 @@
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J200" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K200" s="16"/>
@@ -6884,11 +6908,11 @@
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
       <c r="I201" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J201" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K201" s="16"/>
@@ -6906,11 +6930,11 @@
       <c r="G202" s="14"/>
       <c r="H202" s="14"/>
       <c r="I202" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J202" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K202" s="16"/>
@@ -6928,11 +6952,11 @@
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
       <c r="I203" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J203" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K203" s="16"/>
@@ -6950,11 +6974,11 @@
       <c r="G204" s="14"/>
       <c r="H204" s="14"/>
       <c r="I204" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J204" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K204" s="16"/>
@@ -6972,11 +6996,11 @@
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J205" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K205" s="16"/>
@@ -6994,11 +7018,11 @@
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J206" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K206" s="16"/>
@@ -7016,11 +7040,11 @@
       <c r="G207" s="14"/>
       <c r="H207" s="14"/>
       <c r="I207" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J207" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K207" s="16"/>
@@ -7038,11 +7062,11 @@
       <c r="G208" s="14"/>
       <c r="H208" s="14"/>
       <c r="I208" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J208" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K208" s="16"/>
@@ -7060,11 +7084,11 @@
       <c r="G209" s="14"/>
       <c r="H209" s="14"/>
       <c r="I209" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J209" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K209" s="16"/>
@@ -7082,11 +7106,11 @@
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J210" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K210" s="16"/>
@@ -7104,11 +7128,11 @@
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J211" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K211" s="16"/>
@@ -7126,11 +7150,11 @@
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J212" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K212" s="16"/>
@@ -7148,11 +7172,11 @@
       <c r="G213" s="14"/>
       <c r="H213" s="14"/>
       <c r="I213" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J213" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K213" s="16"/>
@@ -7170,11 +7194,11 @@
       <c r="G214" s="14"/>
       <c r="H214" s="14"/>
       <c r="I214" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J214" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K214" s="16"/>
@@ -7192,11 +7216,11 @@
       <c r="G215" s="14"/>
       <c r="H215" s="14"/>
       <c r="I215" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J215" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K215" s="16"/>
@@ -7214,11 +7238,11 @@
       <c r="G216" s="14"/>
       <c r="H216" s="14"/>
       <c r="I216" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J216" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K216" s="16"/>
@@ -7236,11 +7260,11 @@
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J217" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K217" s="16"/>
@@ -7258,11 +7282,11 @@
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J218" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K218" s="16"/>
@@ -7280,11 +7304,11 @@
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J219" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K219" s="16"/>
@@ -7302,11 +7326,11 @@
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J220" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K220" s="16"/>
@@ -7324,11 +7348,11 @@
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J221" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K221" s="16"/>
@@ -7346,11 +7370,11 @@
       <c r="G222" s="14"/>
       <c r="H222" s="14"/>
       <c r="I222" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J222" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K222" s="16"/>
@@ -7368,11 +7392,11 @@
       <c r="G223" s="14"/>
       <c r="H223" s="14"/>
       <c r="I223" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J223" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K223" s="16"/>
@@ -7390,11 +7414,11 @@
       <c r="G224" s="14"/>
       <c r="H224" s="14"/>
       <c r="I224" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J224" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K224" s="16"/>
@@ -7412,11 +7436,11 @@
       <c r="G225" s="14"/>
       <c r="H225" s="14"/>
       <c r="I225" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J225" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K225" s="16"/>
@@ -7434,11 +7458,11 @@
       <c r="G226" s="14"/>
       <c r="H226" s="14"/>
       <c r="I226" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J226" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K226" s="16"/>
@@ -7456,11 +7480,11 @@
       <c r="G227" s="14"/>
       <c r="H227" s="14"/>
       <c r="I227" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J227" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K227" s="16"/>
@@ -7478,11 +7502,11 @@
       <c r="G228" s="14"/>
       <c r="H228" s="14"/>
       <c r="I228" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J228" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K228" s="16"/>
@@ -7500,11 +7524,11 @@
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J229" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K229" s="16"/>
@@ -7522,11 +7546,11 @@
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J230" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K230" s="16"/>
@@ -7544,11 +7568,11 @@
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
       <c r="I231" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J231" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K231" s="16"/>
@@ -7566,11 +7590,11 @@
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
       <c r="I232" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J232" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K232" s="16"/>
@@ -7588,11 +7612,11 @@
       <c r="G233" s="14"/>
       <c r="H233" s="14"/>
       <c r="I233" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J233" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K233" s="16"/>
@@ -7610,11 +7634,11 @@
       <c r="G234" s="14"/>
       <c r="H234" s="14"/>
       <c r="I234" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J234" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K234" s="16"/>
@@ -7632,11 +7656,11 @@
       <c r="G235" s="14"/>
       <c r="H235" s="14"/>
       <c r="I235" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J235" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K235" s="16"/>
@@ -7654,11 +7678,11 @@
       <c r="G236" s="14"/>
       <c r="H236" s="14"/>
       <c r="I236" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J236" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K236" s="16"/>
@@ -7676,11 +7700,11 @@
       <c r="G237" s="14"/>
       <c r="H237" s="14"/>
       <c r="I237" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J237" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K237" s="16"/>
@@ -7698,11 +7722,11 @@
       <c r="G238" s="14"/>
       <c r="H238" s="14"/>
       <c r="I238" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J238" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K238" s="16"/>
@@ -7720,11 +7744,11 @@
       <c r="G239" s="14"/>
       <c r="H239" s="14"/>
       <c r="I239" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J239" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K239" s="16"/>
@@ -7742,11 +7766,11 @@
       <c r="G240" s="14"/>
       <c r="H240" s="14"/>
       <c r="I240" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J240" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K240" s="16"/>
@@ -7764,11 +7788,11 @@
       <c r="G241" s="14"/>
       <c r="H241" s="14"/>
       <c r="I241" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J241" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K241" s="16"/>
@@ -7786,11 +7810,11 @@
       <c r="G242" s="14"/>
       <c r="H242" s="14"/>
       <c r="I242" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J242" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K242" s="16"/>
@@ -7808,11 +7832,11 @@
       <c r="G243" s="14"/>
       <c r="H243" s="14"/>
       <c r="I243" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J243" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K243" s="16"/>
@@ -7830,11 +7854,11 @@
       <c r="G244" s="14"/>
       <c r="H244" s="14"/>
       <c r="I244" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J244" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K244" s="16"/>
@@ -7852,11 +7876,11 @@
       <c r="G245" s="14"/>
       <c r="H245" s="14"/>
       <c r="I245" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J245" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K245" s="16"/>
@@ -7874,11 +7898,11 @@
       <c r="G246" s="14"/>
       <c r="H246" s="14"/>
       <c r="I246" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J246" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K246" s="16"/>
@@ -7896,11 +7920,11 @@
       <c r="G247" s="14"/>
       <c r="H247" s="14"/>
       <c r="I247" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J247" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K247" s="16"/>
@@ -7918,11 +7942,11 @@
       <c r="G248" s="14"/>
       <c r="H248" s="14"/>
       <c r="I248" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J248" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K248" s="16"/>
@@ -7940,11 +7964,11 @@
       <c r="G249" s="14"/>
       <c r="H249" s="14"/>
       <c r="I249" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J249" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K249" s="16"/>
@@ -7962,11 +7986,11 @@
       <c r="G250" s="14"/>
       <c r="H250" s="14"/>
       <c r="I250" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J250" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K250" s="16"/>
@@ -7984,11 +8008,11 @@
       <c r="G251" s="14"/>
       <c r="H251" s="14"/>
       <c r="I251" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J251" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K251" s="16"/>
@@ -8006,11 +8030,11 @@
       <c r="G252" s="14"/>
       <c r="H252" s="14"/>
       <c r="I252" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J252" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K252" s="16"/>
@@ -8028,11 +8052,11 @@
       <c r="G253" s="14"/>
       <c r="H253" s="14"/>
       <c r="I253" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J253" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K253" s="16"/>
@@ -8050,11 +8074,11 @@
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
       <c r="I254" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J254" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K254" s="16"/>
@@ -8072,11 +8096,11 @@
       <c r="G255" s="14"/>
       <c r="H255" s="14"/>
       <c r="I255" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J255" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K255" s="16"/>
@@ -8094,11 +8118,11 @@
       <c r="G256" s="14"/>
       <c r="H256" s="14"/>
       <c r="I256" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J256" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K256" s="16"/>
@@ -8116,11 +8140,11 @@
       <c r="G257" s="14"/>
       <c r="H257" s="14"/>
       <c r="I257" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J257" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K257" s="16"/>
@@ -8138,11 +8162,11 @@
       <c r="G258" s="14"/>
       <c r="H258" s="14"/>
       <c r="I258" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J258" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K258" s="16"/>
@@ -8160,11 +8184,11 @@
       <c r="G259" s="14"/>
       <c r="H259" s="14"/>
       <c r="I259" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J259" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K259" s="16"/>
@@ -8182,11 +8206,11 @@
       <c r="G260" s="14"/>
       <c r="H260" s="14"/>
       <c r="I260" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J260" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K260" s="16"/>
@@ -8204,11 +8228,11 @@
       <c r="G261" s="14"/>
       <c r="H261" s="14"/>
       <c r="I261" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J261" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K261" s="16"/>
@@ -8226,11 +8250,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="20">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" ref="I262:I325" si="22">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="21">IF(I262="","",1440-I262)</f>
+        <f t="shared" ref="J262:J325" si="23">IF(I262="","",1440-I262)</f>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -8248,11 +8272,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8270,11 +8294,11 @@
       <c r="G264" s="14"/>
       <c r="H264" s="14"/>
       <c r="I264" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J264" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K264" s="16"/>
@@ -8292,11 +8316,11 @@
       <c r="G265" s="14"/>
       <c r="H265" s="14"/>
       <c r="I265" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J265" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K265" s="16"/>
@@ -8314,11 +8338,11 @@
       <c r="G266" s="14"/>
       <c r="H266" s="14"/>
       <c r="I266" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J266" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K266" s="16"/>
@@ -8336,11 +8360,11 @@
       <c r="G267" s="14"/>
       <c r="H267" s="14"/>
       <c r="I267" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J267" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K267" s="16"/>
@@ -8358,11 +8382,11 @@
       <c r="G268" s="14"/>
       <c r="H268" s="14"/>
       <c r="I268" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J268" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K268" s="16"/>
@@ -8380,11 +8404,11 @@
       <c r="G269" s="14"/>
       <c r="H269" s="14"/>
       <c r="I269" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J269" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K269" s="16"/>
@@ -8402,11 +8426,11 @@
       <c r="G270" s="14"/>
       <c r="H270" s="14"/>
       <c r="I270" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J270" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K270" s="16"/>
@@ -8424,11 +8448,11 @@
       <c r="G271" s="14"/>
       <c r="H271" s="14"/>
       <c r="I271" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J271" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K271" s="16"/>
@@ -8446,11 +8470,11 @@
       <c r="G272" s="14"/>
       <c r="H272" s="14"/>
       <c r="I272" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J272" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K272" s="16"/>
@@ -8468,11 +8492,11 @@
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
       <c r="I273" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J273" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K273" s="16"/>
@@ -8490,11 +8514,11 @@
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
       <c r="I274" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J274" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K274" s="16"/>
@@ -8512,11 +8536,11 @@
       <c r="G275" s="14"/>
       <c r="H275" s="14"/>
       <c r="I275" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J275" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K275" s="16"/>
@@ -8534,11 +8558,11 @@
       <c r="G276" s="14"/>
       <c r="H276" s="14"/>
       <c r="I276" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J276" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K276" s="16"/>
@@ -8556,11 +8580,11 @@
       <c r="G277" s="14"/>
       <c r="H277" s="14"/>
       <c r="I277" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J277" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K277" s="16"/>
@@ -8578,11 +8602,11 @@
       <c r="G278" s="14"/>
       <c r="H278" s="14"/>
       <c r="I278" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J278" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K278" s="16"/>
@@ -8600,11 +8624,11 @@
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
       <c r="I279" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J279" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K279" s="16"/>
@@ -8622,11 +8646,11 @@
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
       <c r="I280" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J280" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K280" s="16"/>
@@ -8644,11 +8668,11 @@
       <c r="G281" s="14"/>
       <c r="H281" s="14"/>
       <c r="I281" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J281" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K281" s="16"/>
@@ -8666,11 +8690,11 @@
       <c r="G282" s="14"/>
       <c r="H282" s="14"/>
       <c r="I282" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J282" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K282" s="16"/>
@@ -8688,11 +8712,11 @@
       <c r="G283" s="14"/>
       <c r="H283" s="14"/>
       <c r="I283" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J283" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K283" s="16"/>
@@ -8710,11 +8734,11 @@
       <c r="G284" s="14"/>
       <c r="H284" s="14"/>
       <c r="I284" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J284" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K284" s="16"/>
@@ -8732,11 +8756,11 @@
       <c r="G285" s="14"/>
       <c r="H285" s="14"/>
       <c r="I285" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J285" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K285" s="16"/>
@@ -8754,11 +8778,11 @@
       <c r="G286" s="14"/>
       <c r="H286" s="14"/>
       <c r="I286" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J286" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K286" s="16"/>
@@ -8776,11 +8800,11 @@
       <c r="G287" s="14"/>
       <c r="H287" s="14"/>
       <c r="I287" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J287" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K287" s="16"/>
@@ -8798,11 +8822,11 @@
       <c r="G288" s="14"/>
       <c r="H288" s="14"/>
       <c r="I288" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J288" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K288" s="16"/>
@@ -8820,11 +8844,11 @@
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
       <c r="I289" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J289" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K289" s="16"/>
@@ -8842,11 +8866,11 @@
       <c r="G290" s="14"/>
       <c r="H290" s="14"/>
       <c r="I290" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J290" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K290" s="16"/>
@@ -8864,11 +8888,11 @@
       <c r="G291" s="14"/>
       <c r="H291" s="14"/>
       <c r="I291" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J291" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K291" s="16"/>
@@ -8886,11 +8910,11 @@
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
       <c r="I292" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J292" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K292" s="16"/>
@@ -8908,11 +8932,11 @@
       <c r="G293" s="14"/>
       <c r="H293" s="14"/>
       <c r="I293" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J293" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K293" s="16"/>
@@ -8930,11 +8954,11 @@
       <c r="G294" s="14"/>
       <c r="H294" s="14"/>
       <c r="I294" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J294" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K294" s="16"/>
@@ -8952,11 +8976,11 @@
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
       <c r="I295" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J295" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K295" s="16"/>
@@ -8974,11 +8998,11 @@
       <c r="G296" s="14"/>
       <c r="H296" s="14"/>
       <c r="I296" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J296" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K296" s="16"/>
@@ -8996,11 +9020,11 @@
       <c r="G297" s="14"/>
       <c r="H297" s="14"/>
       <c r="I297" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J297" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K297" s="16"/>
@@ -9018,11 +9042,11 @@
       <c r="G298" s="14"/>
       <c r="H298" s="14"/>
       <c r="I298" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J298" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K298" s="16"/>
@@ -9040,11 +9064,11 @@
       <c r="G299" s="14"/>
       <c r="H299" s="14"/>
       <c r="I299" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J299" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K299" s="16"/>
@@ -9062,11 +9086,11 @@
       <c r="G300" s="14"/>
       <c r="H300" s="14"/>
       <c r="I300" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J300" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K300" s="16"/>
@@ -9084,11 +9108,11 @@
       <c r="G301" s="14"/>
       <c r="H301" s="14"/>
       <c r="I301" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J301" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K301" s="16"/>
@@ -9106,11 +9130,11 @@
       <c r="G302" s="14"/>
       <c r="H302" s="14"/>
       <c r="I302" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J302" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K302" s="16"/>
@@ -9128,11 +9152,11 @@
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
       <c r="I303" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J303" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K303" s="16"/>
@@ -9150,11 +9174,11 @@
       <c r="G304" s="14"/>
       <c r="H304" s="14"/>
       <c r="I304" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J304" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K304" s="16"/>
@@ -9172,11 +9196,11 @@
       <c r="G305" s="14"/>
       <c r="H305" s="14"/>
       <c r="I305" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J305" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K305" s="16"/>
@@ -9194,11 +9218,11 @@
       <c r="G306" s="14"/>
       <c r="H306" s="14"/>
       <c r="I306" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J306" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K306" s="16"/>
@@ -9216,11 +9240,11 @@
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
       <c r="I307" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J307" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K307" s="16"/>
@@ -9238,11 +9262,11 @@
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
       <c r="I308" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J308" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K308" s="16"/>
@@ -9260,11 +9284,11 @@
       <c r="G309" s="14"/>
       <c r="H309" s="14"/>
       <c r="I309" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J309" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K309" s="16"/>
@@ -9282,11 +9306,11 @@
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
       <c r="I310" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J310" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K310" s="16"/>
@@ -9304,11 +9328,11 @@
       <c r="G311" s="14"/>
       <c r="H311" s="14"/>
       <c r="I311" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J311" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K311" s="16"/>
@@ -9326,11 +9350,11 @@
       <c r="G312" s="14"/>
       <c r="H312" s="14"/>
       <c r="I312" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J312" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K312" s="16"/>
@@ -9348,11 +9372,11 @@
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
       <c r="I313" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J313" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K313" s="16"/>
@@ -9370,11 +9394,11 @@
       <c r="G314" s="14"/>
       <c r="H314" s="14"/>
       <c r="I314" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J314" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K314" s="16"/>
@@ -9392,11 +9416,11 @@
       <c r="G315" s="14"/>
       <c r="H315" s="14"/>
       <c r="I315" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J315" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K315" s="16"/>
@@ -9414,11 +9438,11 @@
       <c r="G316" s="14"/>
       <c r="H316" s="14"/>
       <c r="I316" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J316" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K316" s="16"/>
@@ -9436,11 +9460,11 @@
       <c r="G317" s="14"/>
       <c r="H317" s="14"/>
       <c r="I317" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J317" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K317" s="16"/>
@@ -9458,11 +9482,11 @@
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
       <c r="I318" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J318" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K318" s="16"/>
@@ -9480,11 +9504,11 @@
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
       <c r="I319" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J319" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K319" s="16"/>
@@ -9502,11 +9526,11 @@
       <c r="G320" s="14"/>
       <c r="H320" s="14"/>
       <c r="I320" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J320" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K320" s="16"/>
@@ -9524,11 +9548,11 @@
       <c r="G321" s="14"/>
       <c r="H321" s="14"/>
       <c r="I321" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J321" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K321" s="16"/>
@@ -9546,11 +9570,11 @@
       <c r="G322" s="14"/>
       <c r="H322" s="14"/>
       <c r="I322" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J322" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K322" s="16"/>
@@ -9568,11 +9592,11 @@
       <c r="G323" s="14"/>
       <c r="H323" s="14"/>
       <c r="I323" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J323" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K323" s="16"/>
@@ -9590,11 +9614,11 @@
       <c r="G324" s="14"/>
       <c r="H324" s="14"/>
       <c r="I324" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J324" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K324" s="16"/>
@@ -9612,11 +9636,11 @@
       <c r="G325" s="14"/>
       <c r="H325" s="14"/>
       <c r="I325" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J325" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K325" s="16"/>
@@ -9634,11 +9658,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="22">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" ref="I326:I389" si="24">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="23">IF(I326="","",1440-I326)</f>
+        <f t="shared" ref="J326:J389" si="25">IF(I326="","",1440-I326)</f>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -9656,11 +9680,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -9678,11 +9702,11 @@
       <c r="G328" s="14"/>
       <c r="H328" s="14"/>
       <c r="I328" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J328" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K328" s="16"/>
@@ -9700,11 +9724,11 @@
       <c r="G329" s="14"/>
       <c r="H329" s="14"/>
       <c r="I329" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J329" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K329" s="16"/>
@@ -9722,11 +9746,11 @@
       <c r="G330" s="14"/>
       <c r="H330" s="14"/>
       <c r="I330" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J330" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K330" s="16"/>
@@ -9744,11 +9768,11 @@
       <c r="G331" s="14"/>
       <c r="H331" s="14"/>
       <c r="I331" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J331" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K331" s="16"/>
@@ -9766,11 +9790,11 @@
       <c r="G332" s="14"/>
       <c r="H332" s="14"/>
       <c r="I332" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J332" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K332" s="16"/>
@@ -9788,11 +9812,11 @@
       <c r="G333" s="14"/>
       <c r="H333" s="14"/>
       <c r="I333" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J333" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K333" s="16"/>
@@ -9810,11 +9834,11 @@
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
       <c r="I334" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J334" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K334" s="16"/>
@@ -9832,11 +9856,11 @@
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
       <c r="I335" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J335" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K335" s="16"/>
@@ -9854,11 +9878,11 @@
       <c r="G336" s="14"/>
       <c r="H336" s="14"/>
       <c r="I336" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J336" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K336" s="16"/>
@@ -9876,11 +9900,11 @@
       <c r="G337" s="14"/>
       <c r="H337" s="14"/>
       <c r="I337" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J337" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K337" s="16"/>
@@ -9898,11 +9922,11 @@
       <c r="G338" s="14"/>
       <c r="H338" s="14"/>
       <c r="I338" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J338" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K338" s="16"/>
@@ -9920,11 +9944,11 @@
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
       <c r="I339" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J339" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K339" s="16"/>
@@ -9942,11 +9966,11 @@
       <c r="G340" s="14"/>
       <c r="H340" s="14"/>
       <c r="I340" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J340" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K340" s="16"/>
@@ -9964,11 +9988,11 @@
       <c r="G341" s="14"/>
       <c r="H341" s="14"/>
       <c r="I341" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J341" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K341" s="16"/>
@@ -9986,11 +10010,11 @@
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
       <c r="I342" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J342" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K342" s="16"/>
@@ -10008,11 +10032,11 @@
       <c r="G343" s="14"/>
       <c r="H343" s="14"/>
       <c r="I343" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J343" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K343" s="16"/>
@@ -10030,11 +10054,11 @@
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
       <c r="I344" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J344" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K344" s="16"/>
@@ -10052,11 +10076,11 @@
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
       <c r="I345" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J345" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K345" s="16"/>
@@ -10074,11 +10098,11 @@
       <c r="G346" s="14"/>
       <c r="H346" s="14"/>
       <c r="I346" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J346" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K346" s="16"/>
@@ -10096,11 +10120,11 @@
       <c r="G347" s="14"/>
       <c r="H347" s="14"/>
       <c r="I347" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J347" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K347" s="16"/>
@@ -10118,11 +10142,11 @@
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
       <c r="I348" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J348" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K348" s="16"/>
@@ -10140,11 +10164,11 @@
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
       <c r="I349" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J349" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K349" s="16"/>
@@ -10162,11 +10186,11 @@
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
       <c r="I350" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J350" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K350" s="16"/>
@@ -10184,11 +10208,11 @@
       <c r="G351" s="14"/>
       <c r="H351" s="14"/>
       <c r="I351" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J351" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K351" s="16"/>
@@ -10206,11 +10230,11 @@
       <c r="G352" s="14"/>
       <c r="H352" s="14"/>
       <c r="I352" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J352" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K352" s="16"/>
@@ -10228,11 +10252,11 @@
       <c r="G353" s="14"/>
       <c r="H353" s="14"/>
       <c r="I353" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J353" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K353" s="16"/>
@@ -10250,11 +10274,11 @@
       <c r="G354" s="14"/>
       <c r="H354" s="14"/>
       <c r="I354" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J354" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K354" s="16"/>
@@ -10272,11 +10296,11 @@
       <c r="G355" s="14"/>
       <c r="H355" s="14"/>
       <c r="I355" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J355" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K355" s="16"/>
@@ -10294,11 +10318,11 @@
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
       <c r="I356" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J356" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K356" s="16"/>
@@ -10316,11 +10340,11 @@
       <c r="G357" s="14"/>
       <c r="H357" s="14"/>
       <c r="I357" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J357" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K357" s="16"/>
@@ -10338,11 +10362,11 @@
       <c r="G358" s="14"/>
       <c r="H358" s="14"/>
       <c r="I358" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J358" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K358" s="16"/>
@@ -10360,11 +10384,11 @@
       <c r="G359" s="14"/>
       <c r="H359" s="14"/>
       <c r="I359" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J359" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K359" s="16"/>
@@ -10382,11 +10406,11 @@
       <c r="G360" s="14"/>
       <c r="H360" s="14"/>
       <c r="I360" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J360" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K360" s="16"/>
@@ -10404,11 +10428,11 @@
       <c r="G361" s="14"/>
       <c r="H361" s="14"/>
       <c r="I361" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J361" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K361" s="16"/>
@@ -10426,11 +10450,11 @@
       <c r="G362" s="14"/>
       <c r="H362" s="14"/>
       <c r="I362" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J362" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K362" s="16"/>
@@ -10448,11 +10472,11 @@
       <c r="G363" s="14"/>
       <c r="H363" s="14"/>
       <c r="I363" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J363" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K363" s="16"/>
@@ -10470,11 +10494,11 @@
       <c r="G364" s="14"/>
       <c r="H364" s="14"/>
       <c r="I364" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J364" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K364" s="16"/>
@@ -10492,11 +10516,11 @@
       <c r="G365" s="14"/>
       <c r="H365" s="14"/>
       <c r="I365" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J365" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K365" s="16"/>
@@ -10514,11 +10538,11 @@
       <c r="G366" s="14"/>
       <c r="H366" s="14"/>
       <c r="I366" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J366" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K366" s="16"/>
@@ -10536,11 +10560,11 @@
       <c r="G367" s="14"/>
       <c r="H367" s="14"/>
       <c r="I367" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J367" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K367" s="16"/>
@@ -10558,11 +10582,11 @@
       <c r="G368" s="14"/>
       <c r="H368" s="14"/>
       <c r="I368" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J368" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K368" s="16"/>
@@ -10580,11 +10604,11 @@
       <c r="G369" s="14"/>
       <c r="H369" s="14"/>
       <c r="I369" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J369" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K369" s="16"/>
@@ -10602,11 +10626,11 @@
       <c r="G370" s="14"/>
       <c r="H370" s="14"/>
       <c r="I370" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J370" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K370" s="16"/>
@@ -10624,11 +10648,11 @@
       <c r="G371" s="14"/>
       <c r="H371" s="14"/>
       <c r="I371" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J371" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K371" s="16"/>
@@ -10646,11 +10670,11 @@
       <c r="G372" s="14"/>
       <c r="H372" s="14"/>
       <c r="I372" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J372" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K372" s="16"/>
@@ -10668,11 +10692,11 @@
       <c r="G373" s="14"/>
       <c r="H373" s="14"/>
       <c r="I373" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J373" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K373" s="16"/>
@@ -10690,11 +10714,11 @@
       <c r="G374" s="14"/>
       <c r="H374" s="14"/>
       <c r="I374" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J374" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K374" s="16"/>
@@ -10712,11 +10736,11 @@
       <c r="G375" s="14"/>
       <c r="H375" s="14"/>
       <c r="I375" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J375" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K375" s="16"/>
@@ -10734,11 +10758,11 @@
       <c r="G376" s="14"/>
       <c r="H376" s="14"/>
       <c r="I376" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J376" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K376" s="16"/>
@@ -10756,11 +10780,11 @@
       <c r="G377" s="14"/>
       <c r="H377" s="14"/>
       <c r="I377" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J377" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K377" s="16"/>
@@ -10778,11 +10802,11 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K378" s="16"/>
@@ -10800,11 +10824,11 @@
       <c r="G379" s="14"/>
       <c r="H379" s="14"/>
       <c r="I379" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J379" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K379" s="16"/>
@@ -10822,11 +10846,11 @@
       <c r="G380" s="14"/>
       <c r="H380" s="14"/>
       <c r="I380" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J380" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K380" s="16"/>
@@ -10844,11 +10868,11 @@
       <c r="G381" s="14"/>
       <c r="H381" s="14"/>
       <c r="I381" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J381" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K381" s="16"/>
@@ -10866,11 +10890,11 @@
       <c r="G382" s="14"/>
       <c r="H382" s="14"/>
       <c r="I382" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J382" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K382" s="16"/>
@@ -10888,11 +10912,11 @@
       <c r="G383" s="14"/>
       <c r="H383" s="14"/>
       <c r="I383" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J383" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K383" s="16"/>
@@ -10910,11 +10934,11 @@
       <c r="G384" s="14"/>
       <c r="H384" s="14"/>
       <c r="I384" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J384" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K384" s="16"/>
@@ -10932,11 +10956,11 @@
       <c r="G385" s="14"/>
       <c r="H385" s="14"/>
       <c r="I385" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J385" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K385" s="16"/>
@@ -10954,11 +10978,11 @@
       <c r="G386" s="14"/>
       <c r="H386" s="14"/>
       <c r="I386" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J386" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K386" s="16"/>
@@ -10976,11 +11000,11 @@
       <c r="G387" s="14"/>
       <c r="H387" s="14"/>
       <c r="I387" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J387" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K387" s="16"/>
@@ -10998,11 +11022,11 @@
       <c r="G388" s="14"/>
       <c r="H388" s="14"/>
       <c r="I388" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J388" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K388" s="16"/>
@@ -11020,11 +11044,11 @@
       <c r="G389" s="14"/>
       <c r="H389" s="14"/>
       <c r="I389" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J389" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K389" s="16"/>
@@ -11042,11 +11066,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="24">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="26">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="25">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="27">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -11064,11 +11088,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -11086,11 +11110,11 @@
       <c r="G392" s="14"/>
       <c r="H392" s="14"/>
       <c r="I392" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J392" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K392" s="16"/>
@@ -11108,11 +11132,11 @@
       <c r="G393" s="14"/>
       <c r="H393" s="14"/>
       <c r="I393" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J393" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K393" s="16"/>
@@ -11130,11 +11154,11 @@
       <c r="G394" s="14"/>
       <c r="H394" s="14"/>
       <c r="I394" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J394" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K394" s="16"/>
@@ -11152,11 +11176,11 @@
       <c r="G395" s="14"/>
       <c r="H395" s="14"/>
       <c r="I395" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J395" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K395" s="16"/>
@@ -11174,11 +11198,11 @@
       <c r="G396" s="14"/>
       <c r="H396" s="14"/>
       <c r="I396" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J396" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K396" s="16"/>
@@ -11196,11 +11220,11 @@
       <c r="G397" s="14"/>
       <c r="H397" s="14"/>
       <c r="I397" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J397" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K397" s="16"/>
@@ -11218,11 +11242,11 @@
       <c r="G398" s="14"/>
       <c r="H398" s="14"/>
       <c r="I398" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J398" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K398" s="16"/>
@@ -11240,11 +11264,11 @@
       <c r="G399" s="14"/>
       <c r="H399" s="14"/>
       <c r="I399" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J399" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K399" s="16"/>
@@ -11262,11 +11286,11 @@
       <c r="G400" s="14"/>
       <c r="H400" s="14"/>
       <c r="I400" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J400" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K400" s="16"/>
@@ -11284,11 +11308,11 @@
       <c r="G401" s="14"/>
       <c r="H401" s="14"/>
       <c r="I401" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J401" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K401" s="16"/>

</xml_diff>

<commit_message>
File Updated On 20/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FCEC20-4567-4288-981C-5073C6364B96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3242867D-B5AA-419A-97D2-434941DE538E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="612" yWindow="-108" windowWidth="22536" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="91">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -305,6 +305,9 @@
   </si>
   <si>
     <t>Classes started from today after mid terms</t>
+  </si>
+  <si>
+    <t>Practiced analytic skills questions</t>
   </si>
 </sst>
 </file>
@@ -3972,27 +3975,51 @@
         <v>89</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A68" s="13"/>
-      <c r="B68" s="14"/>
-      <c r="C68" s="14"/>
-      <c r="D68" s="14"/>
-      <c r="E68" s="14"/>
-      <c r="F68" s="14"/>
-      <c r="G68" s="14"/>
-      <c r="H68" s="14"/>
-      <c r="I68" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J68" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K68" s="16"/>
-      <c r="L68" s="16"/>
-      <c r="M68" s="16"/>
-      <c r="N68" s="17"/>
+    <row r="68" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A68" s="13">
+        <v>46315</v>
+      </c>
+      <c r="B68" s="14">
+        <v>420</v>
+      </c>
+      <c r="C68" s="14">
+        <v>0</v>
+      </c>
+      <c r="D68" s="14">
+        <v>120</v>
+      </c>
+      <c r="E68" s="14">
+        <v>0</v>
+      </c>
+      <c r="F68" s="14">
+        <v>0</v>
+      </c>
+      <c r="G68" s="14">
+        <v>0</v>
+      </c>
+      <c r="H68" s="14">
+        <v>170</v>
+      </c>
+      <c r="I68" s="15">
+        <f t="shared" ref="I68" si="16">IF(SUM(B68:F68,H68)=0,"",SUM(B68:F68,H68))</f>
+        <v>710</v>
+      </c>
+      <c r="J68" s="15">
+        <f t="shared" ref="J68" si="17">IF(I68="","",1440-I68)</f>
+        <v>730</v>
+      </c>
+      <c r="K68" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L68" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M68" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N68" s="17" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69" s="13"/>
@@ -4026,11 +4053,11 @@
       <c r="G70" s="14"/>
       <c r="H70" s="14"/>
       <c r="I70" s="15" t="str">
-        <f t="shared" ref="I70:I133" si="16">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
+        <f t="shared" ref="I70:I133" si="18">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
         <v/>
       </c>
       <c r="J70" s="15" t="str">
-        <f t="shared" ref="J70:J133" si="17">IF(I70="","",1440-I70)</f>
+        <f t="shared" ref="J70:J133" si="19">IF(I70="","",1440-I70)</f>
         <v/>
       </c>
       <c r="K70" s="16"/>
@@ -4048,11 +4075,11 @@
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
       <c r="I71" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J71" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K71" s="16"/>
@@ -4070,11 +4097,11 @@
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
       <c r="I72" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J72" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K72" s="16"/>
@@ -4092,11 +4119,11 @@
       <c r="G73" s="14"/>
       <c r="H73" s="14"/>
       <c r="I73" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J73" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K73" s="16"/>
@@ -4114,11 +4141,11 @@
       <c r="G74" s="14"/>
       <c r="H74" s="14"/>
       <c r="I74" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J74" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K74" s="16"/>
@@ -4136,11 +4163,11 @@
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
       <c r="I75" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J75" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K75" s="16"/>
@@ -4158,11 +4185,11 @@
       <c r="G76" s="14"/>
       <c r="H76" s="14"/>
       <c r="I76" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J76" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K76" s="16"/>
@@ -4180,11 +4207,11 @@
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
       <c r="I77" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J77" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K77" s="16"/>
@@ -4202,11 +4229,11 @@
       <c r="G78" s="14"/>
       <c r="H78" s="14"/>
       <c r="I78" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J78" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K78" s="16"/>
@@ -4224,11 +4251,11 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J79" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K79" s="16"/>
@@ -4246,11 +4273,11 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J80" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K80" s="16"/>
@@ -4268,11 +4295,11 @@
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J81" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K81" s="16"/>
@@ -4290,11 +4317,11 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J82" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K82" s="16"/>
@@ -4312,11 +4339,11 @@
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
       <c r="I83" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J83" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K83" s="16"/>
@@ -4334,11 +4361,11 @@
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
       <c r="I84" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J84" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K84" s="16"/>
@@ -4356,11 +4383,11 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J85" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K85" s="16"/>
@@ -4378,11 +4405,11 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J86" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K86" s="16"/>
@@ -4400,11 +4427,11 @@
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
       <c r="I87" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J87" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K87" s="16"/>
@@ -4422,11 +4449,11 @@
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
       <c r="I88" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J88" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K88" s="16"/>
@@ -4444,11 +4471,11 @@
       <c r="G89" s="14"/>
       <c r="H89" s="14"/>
       <c r="I89" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J89" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K89" s="16"/>
@@ -4466,11 +4493,11 @@
       <c r="G90" s="14"/>
       <c r="H90" s="14"/>
       <c r="I90" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J90" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K90" s="16"/>
@@ -4488,11 +4515,11 @@
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
       <c r="I91" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J91" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K91" s="16"/>
@@ -4510,11 +4537,11 @@
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
       <c r="I92" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J92" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K92" s="16"/>
@@ -4532,11 +4559,11 @@
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J93" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K93" s="16"/>
@@ -4554,11 +4581,11 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J94" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K94" s="16"/>
@@ -4576,11 +4603,11 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J95" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K95" s="16"/>
@@ -4598,11 +4625,11 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J96" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K96" s="16"/>
@@ -4620,11 +4647,11 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J97" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K97" s="16"/>
@@ -4642,11 +4669,11 @@
       <c r="G98" s="14"/>
       <c r="H98" s="14"/>
       <c r="I98" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J98" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K98" s="16"/>
@@ -4664,11 +4691,11 @@
       <c r="G99" s="14"/>
       <c r="H99" s="14"/>
       <c r="I99" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J99" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K99" s="16"/>
@@ -4686,11 +4713,11 @@
       <c r="G100" s="14"/>
       <c r="H100" s="14"/>
       <c r="I100" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J100" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K100" s="16"/>
@@ -4708,11 +4735,11 @@
       <c r="G101" s="14"/>
       <c r="H101" s="14"/>
       <c r="I101" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J101" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K101" s="16"/>
@@ -4730,11 +4757,11 @@
       <c r="G102" s="14"/>
       <c r="H102" s="14"/>
       <c r="I102" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J102" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K102" s="16"/>
@@ -4752,11 +4779,11 @@
       <c r="G103" s="14"/>
       <c r="H103" s="14"/>
       <c r="I103" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J103" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K103" s="16"/>
@@ -4774,11 +4801,11 @@
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
       <c r="I104" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J104" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K104" s="16"/>
@@ -4796,11 +4823,11 @@
       <c r="G105" s="14"/>
       <c r="H105" s="14"/>
       <c r="I105" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J105" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K105" s="16"/>
@@ -4818,11 +4845,11 @@
       <c r="G106" s="14"/>
       <c r="H106" s="14"/>
       <c r="I106" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J106" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K106" s="16"/>
@@ -4840,11 +4867,11 @@
       <c r="G107" s="14"/>
       <c r="H107" s="14"/>
       <c r="I107" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J107" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K107" s="16"/>
@@ -4862,11 +4889,11 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J108" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K108" s="16"/>
@@ -4884,11 +4911,11 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J109" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K109" s="16"/>
@@ -4906,11 +4933,11 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J110" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K110" s="16"/>
@@ -4928,11 +4955,11 @@
       <c r="G111" s="14"/>
       <c r="H111" s="14"/>
       <c r="I111" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J111" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K111" s="16"/>
@@ -4950,11 +4977,11 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J112" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K112" s="16"/>
@@ -4972,11 +4999,11 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J113" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K113" s="16"/>
@@ -4994,11 +5021,11 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J114" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K114" s="16"/>
@@ -5016,11 +5043,11 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J115" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K115" s="16"/>
@@ -5038,11 +5065,11 @@
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
       <c r="I116" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J116" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K116" s="16"/>
@@ -5060,11 +5087,11 @@
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
       <c r="I117" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J117" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K117" s="16"/>
@@ -5082,11 +5109,11 @@
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
       <c r="I118" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J118" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K118" s="16"/>
@@ -5104,11 +5131,11 @@
       <c r="G119" s="14"/>
       <c r="H119" s="14"/>
       <c r="I119" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J119" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K119" s="16"/>
@@ -5126,11 +5153,11 @@
       <c r="G120" s="14"/>
       <c r="H120" s="14"/>
       <c r="I120" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J120" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K120" s="16"/>
@@ -5148,11 +5175,11 @@
       <c r="G121" s="14"/>
       <c r="H121" s="14"/>
       <c r="I121" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J121" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K121" s="16"/>
@@ -5170,11 +5197,11 @@
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
       <c r="I122" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J122" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K122" s="16"/>
@@ -5192,11 +5219,11 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J123" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K123" s="16"/>
@@ -5214,11 +5241,11 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J124" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K124" s="16"/>
@@ -5236,11 +5263,11 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J125" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K125" s="16"/>
@@ -5258,11 +5285,11 @@
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
       <c r="I126" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J126" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K126" s="16"/>
@@ -5280,11 +5307,11 @@
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J127" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K127" s="16"/>
@@ -5302,11 +5329,11 @@
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
       <c r="I128" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J128" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K128" s="16"/>
@@ -5324,11 +5351,11 @@
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
       <c r="I129" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J129" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K129" s="16"/>
@@ -5346,11 +5373,11 @@
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
       <c r="I130" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J130" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K130" s="16"/>
@@ -5368,11 +5395,11 @@
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
       <c r="I131" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J131" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K131" s="16"/>
@@ -5390,11 +5417,11 @@
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
       <c r="I132" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J132" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K132" s="16"/>
@@ -5412,11 +5439,11 @@
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
       <c r="I133" s="15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="J133" s="15" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="K133" s="16"/>
@@ -5434,11 +5461,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="18">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" ref="I134:I197" si="20">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="19">IF(I134="","",1440-I134)</f>
+        <f t="shared" ref="J134:J197" si="21">IF(I134="","",1440-I134)</f>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -5456,11 +5483,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5478,11 +5505,11 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J136" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K136" s="16"/>
@@ -5500,11 +5527,11 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J137" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K137" s="16"/>
@@ -5522,11 +5549,11 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J138" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K138" s="16"/>
@@ -5544,11 +5571,11 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J139" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K139" s="16"/>
@@ -5566,11 +5593,11 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J140" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K140" s="16"/>
@@ -5588,11 +5615,11 @@
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J141" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K141" s="16"/>
@@ -5610,11 +5637,11 @@
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J142" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K142" s="16"/>
@@ -5632,11 +5659,11 @@
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J143" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K143" s="16"/>
@@ -5654,11 +5681,11 @@
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J144" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K144" s="16"/>
@@ -5676,11 +5703,11 @@
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J145" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K145" s="16"/>
@@ -5698,11 +5725,11 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J146" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K146" s="16"/>
@@ -5720,11 +5747,11 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J147" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K147" s="16"/>
@@ -5742,11 +5769,11 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J148" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K148" s="16"/>
@@ -5764,11 +5791,11 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J149" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K149" s="16"/>
@@ -5786,11 +5813,11 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J150" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K150" s="16"/>
@@ -5808,11 +5835,11 @@
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
       <c r="I151" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J151" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K151" s="16"/>
@@ -5830,11 +5857,11 @@
       <c r="G152" s="14"/>
       <c r="H152" s="14"/>
       <c r="I152" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J152" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K152" s="16"/>
@@ -5852,11 +5879,11 @@
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J153" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K153" s="16"/>
@@ -5874,11 +5901,11 @@
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J154" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K154" s="16"/>
@@ -5896,11 +5923,11 @@
       <c r="G155" s="14"/>
       <c r="H155" s="14"/>
       <c r="I155" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J155" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K155" s="16"/>
@@ -5918,11 +5945,11 @@
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
       <c r="I156" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J156" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K156" s="16"/>
@@ -5940,11 +5967,11 @@
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J157" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K157" s="16"/>
@@ -5962,11 +5989,11 @@
       <c r="G158" s="14"/>
       <c r="H158" s="14"/>
       <c r="I158" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J158" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K158" s="16"/>
@@ -5984,11 +6011,11 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J159" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K159" s="16"/>
@@ -6006,11 +6033,11 @@
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
       <c r="I160" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J160" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K160" s="16"/>
@@ -6028,11 +6055,11 @@
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
       <c r="I161" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J161" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K161" s="16"/>
@@ -6050,11 +6077,11 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J162" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K162" s="16"/>
@@ -6072,11 +6099,11 @@
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
       <c r="I163" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J163" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K163" s="16"/>
@@ -6094,11 +6121,11 @@
       <c r="G164" s="14"/>
       <c r="H164" s="14"/>
       <c r="I164" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J164" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K164" s="16"/>
@@ -6116,11 +6143,11 @@
       <c r="G165" s="14"/>
       <c r="H165" s="14"/>
       <c r="I165" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J165" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K165" s="16"/>
@@ -6138,11 +6165,11 @@
       <c r="G166" s="14"/>
       <c r="H166" s="14"/>
       <c r="I166" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J166" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K166" s="16"/>
@@ -6160,11 +6187,11 @@
       <c r="G167" s="14"/>
       <c r="H167" s="14"/>
       <c r="I167" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J167" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K167" s="16"/>
@@ -6182,11 +6209,11 @@
       <c r="G168" s="14"/>
       <c r="H168" s="14"/>
       <c r="I168" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J168" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K168" s="16"/>
@@ -6204,11 +6231,11 @@
       <c r="G169" s="14"/>
       <c r="H169" s="14"/>
       <c r="I169" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J169" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K169" s="16"/>
@@ -6226,11 +6253,11 @@
       <c r="G170" s="14"/>
       <c r="H170" s="14"/>
       <c r="I170" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J170" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K170" s="16"/>
@@ -6248,11 +6275,11 @@
       <c r="G171" s="14"/>
       <c r="H171" s="14"/>
       <c r="I171" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J171" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K171" s="16"/>
@@ -6270,11 +6297,11 @@
       <c r="G172" s="14"/>
       <c r="H172" s="14"/>
       <c r="I172" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J172" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K172" s="16"/>
@@ -6292,11 +6319,11 @@
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
       <c r="I173" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J173" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K173" s="16"/>
@@ -6314,11 +6341,11 @@
       <c r="G174" s="14"/>
       <c r="H174" s="14"/>
       <c r="I174" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J174" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K174" s="16"/>
@@ -6336,11 +6363,11 @@
       <c r="G175" s="14"/>
       <c r="H175" s="14"/>
       <c r="I175" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J175" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K175" s="16"/>
@@ -6358,11 +6385,11 @@
       <c r="G176" s="14"/>
       <c r="H176" s="14"/>
       <c r="I176" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J176" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K176" s="16"/>
@@ -6380,11 +6407,11 @@
       <c r="G177" s="14"/>
       <c r="H177" s="14"/>
       <c r="I177" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J177" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K177" s="16"/>
@@ -6402,11 +6429,11 @@
       <c r="G178" s="14"/>
       <c r="H178" s="14"/>
       <c r="I178" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J178" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K178" s="16"/>
@@ -6424,11 +6451,11 @@
       <c r="G179" s="14"/>
       <c r="H179" s="14"/>
       <c r="I179" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J179" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K179" s="16"/>
@@ -6446,11 +6473,11 @@
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
       <c r="I180" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J180" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K180" s="16"/>
@@ -6468,11 +6495,11 @@
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J181" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K181" s="16"/>
@@ -6490,11 +6517,11 @@
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J182" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K182" s="16"/>
@@ -6512,11 +6539,11 @@
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J183" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K183" s="16"/>
@@ -6534,11 +6561,11 @@
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
       <c r="I184" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J184" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K184" s="16"/>
@@ -6556,11 +6583,11 @@
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
       <c r="I185" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J185" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K185" s="16"/>
@@ -6578,11 +6605,11 @@
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J186" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K186" s="16"/>
@@ -6600,11 +6627,11 @@
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J187" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K187" s="16"/>
@@ -6622,11 +6649,11 @@
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
       <c r="I188" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J188" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K188" s="16"/>
@@ -6644,11 +6671,11 @@
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
       <c r="I189" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J189" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K189" s="16"/>
@@ -6666,11 +6693,11 @@
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J190" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K190" s="16"/>
@@ -6688,11 +6715,11 @@
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J191" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K191" s="16"/>
@@ -6710,11 +6737,11 @@
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J192" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K192" s="16"/>
@@ -6732,11 +6759,11 @@
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
       <c r="I193" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J193" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K193" s="16"/>
@@ -6754,11 +6781,11 @@
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
       <c r="I194" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J194" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K194" s="16"/>
@@ -6776,11 +6803,11 @@
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J195" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K195" s="16"/>
@@ -6798,11 +6825,11 @@
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J196" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K196" s="16"/>
@@ -6820,11 +6847,11 @@
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J197" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K197" s="16"/>
@@ -6842,11 +6869,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="20">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" ref="I198:I261" si="22">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="21">IF(I198="","",1440-I198)</f>
+        <f t="shared" ref="J198:J261" si="23">IF(I198="","",1440-I198)</f>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -6864,11 +6891,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -6886,11 +6913,11 @@
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J200" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K200" s="16"/>
@@ -6908,11 +6935,11 @@
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
       <c r="I201" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J201" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K201" s="16"/>
@@ -6930,11 +6957,11 @@
       <c r="G202" s="14"/>
       <c r="H202" s="14"/>
       <c r="I202" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J202" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K202" s="16"/>
@@ -6952,11 +6979,11 @@
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
       <c r="I203" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J203" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K203" s="16"/>
@@ -6974,11 +7001,11 @@
       <c r="G204" s="14"/>
       <c r="H204" s="14"/>
       <c r="I204" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J204" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K204" s="16"/>
@@ -6996,11 +7023,11 @@
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J205" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K205" s="16"/>
@@ -7018,11 +7045,11 @@
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J206" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K206" s="16"/>
@@ -7040,11 +7067,11 @@
       <c r="G207" s="14"/>
       <c r="H207" s="14"/>
       <c r="I207" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J207" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K207" s="16"/>
@@ -7062,11 +7089,11 @@
       <c r="G208" s="14"/>
       <c r="H208" s="14"/>
       <c r="I208" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J208" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K208" s="16"/>
@@ -7084,11 +7111,11 @@
       <c r="G209" s="14"/>
       <c r="H209" s="14"/>
       <c r="I209" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J209" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K209" s="16"/>
@@ -7106,11 +7133,11 @@
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J210" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K210" s="16"/>
@@ -7128,11 +7155,11 @@
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J211" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K211" s="16"/>
@@ -7150,11 +7177,11 @@
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J212" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K212" s="16"/>
@@ -7172,11 +7199,11 @@
       <c r="G213" s="14"/>
       <c r="H213" s="14"/>
       <c r="I213" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J213" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K213" s="16"/>
@@ -7194,11 +7221,11 @@
       <c r="G214" s="14"/>
       <c r="H214" s="14"/>
       <c r="I214" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J214" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K214" s="16"/>
@@ -7216,11 +7243,11 @@
       <c r="G215" s="14"/>
       <c r="H215" s="14"/>
       <c r="I215" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J215" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K215" s="16"/>
@@ -7238,11 +7265,11 @@
       <c r="G216" s="14"/>
       <c r="H216" s="14"/>
       <c r="I216" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J216" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K216" s="16"/>
@@ -7260,11 +7287,11 @@
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J217" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K217" s="16"/>
@@ -7282,11 +7309,11 @@
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J218" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K218" s="16"/>
@@ -7304,11 +7331,11 @@
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J219" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K219" s="16"/>
@@ -7326,11 +7353,11 @@
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J220" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K220" s="16"/>
@@ -7348,11 +7375,11 @@
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J221" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K221" s="16"/>
@@ -7370,11 +7397,11 @@
       <c r="G222" s="14"/>
       <c r="H222" s="14"/>
       <c r="I222" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J222" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K222" s="16"/>
@@ -7392,11 +7419,11 @@
       <c r="G223" s="14"/>
       <c r="H223" s="14"/>
       <c r="I223" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J223" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K223" s="16"/>
@@ -7414,11 +7441,11 @@
       <c r="G224" s="14"/>
       <c r="H224" s="14"/>
       <c r="I224" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J224" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K224" s="16"/>
@@ -7436,11 +7463,11 @@
       <c r="G225" s="14"/>
       <c r="H225" s="14"/>
       <c r="I225" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J225" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K225" s="16"/>
@@ -7458,11 +7485,11 @@
       <c r="G226" s="14"/>
       <c r="H226" s="14"/>
       <c r="I226" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J226" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K226" s="16"/>
@@ -7480,11 +7507,11 @@
       <c r="G227" s="14"/>
       <c r="H227" s="14"/>
       <c r="I227" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J227" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K227" s="16"/>
@@ -7502,11 +7529,11 @@
       <c r="G228" s="14"/>
       <c r="H228" s="14"/>
       <c r="I228" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J228" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K228" s="16"/>
@@ -7524,11 +7551,11 @@
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J229" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K229" s="16"/>
@@ -7546,11 +7573,11 @@
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J230" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K230" s="16"/>
@@ -7568,11 +7595,11 @@
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
       <c r="I231" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J231" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K231" s="16"/>
@@ -7590,11 +7617,11 @@
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
       <c r="I232" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J232" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K232" s="16"/>
@@ -7612,11 +7639,11 @@
       <c r="G233" s="14"/>
       <c r="H233" s="14"/>
       <c r="I233" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J233" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K233" s="16"/>
@@ -7634,11 +7661,11 @@
       <c r="G234" s="14"/>
       <c r="H234" s="14"/>
       <c r="I234" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J234" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K234" s="16"/>
@@ -7656,11 +7683,11 @@
       <c r="G235" s="14"/>
       <c r="H235" s="14"/>
       <c r="I235" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J235" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K235" s="16"/>
@@ -7678,11 +7705,11 @@
       <c r="G236" s="14"/>
       <c r="H236" s="14"/>
       <c r="I236" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J236" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K236" s="16"/>
@@ -7700,11 +7727,11 @@
       <c r="G237" s="14"/>
       <c r="H237" s="14"/>
       <c r="I237" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J237" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K237" s="16"/>
@@ -7722,11 +7749,11 @@
       <c r="G238" s="14"/>
       <c r="H238" s="14"/>
       <c r="I238" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J238" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K238" s="16"/>
@@ -7744,11 +7771,11 @@
       <c r="G239" s="14"/>
       <c r="H239" s="14"/>
       <c r="I239" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J239" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K239" s="16"/>
@@ -7766,11 +7793,11 @@
       <c r="G240" s="14"/>
       <c r="H240" s="14"/>
       <c r="I240" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J240" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K240" s="16"/>
@@ -7788,11 +7815,11 @@
       <c r="G241" s="14"/>
       <c r="H241" s="14"/>
       <c r="I241" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J241" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K241" s="16"/>
@@ -7810,11 +7837,11 @@
       <c r="G242" s="14"/>
       <c r="H242" s="14"/>
       <c r="I242" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J242" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K242" s="16"/>
@@ -7832,11 +7859,11 @@
       <c r="G243" s="14"/>
       <c r="H243" s="14"/>
       <c r="I243" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J243" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K243" s="16"/>
@@ -7854,11 +7881,11 @@
       <c r="G244" s="14"/>
       <c r="H244" s="14"/>
       <c r="I244" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J244" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K244" s="16"/>
@@ -7876,11 +7903,11 @@
       <c r="G245" s="14"/>
       <c r="H245" s="14"/>
       <c r="I245" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J245" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K245" s="16"/>
@@ -7898,11 +7925,11 @@
       <c r="G246" s="14"/>
       <c r="H246" s="14"/>
       <c r="I246" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J246" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K246" s="16"/>
@@ -7920,11 +7947,11 @@
       <c r="G247" s="14"/>
       <c r="H247" s="14"/>
       <c r="I247" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J247" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K247" s="16"/>
@@ -7942,11 +7969,11 @@
       <c r="G248" s="14"/>
       <c r="H248" s="14"/>
       <c r="I248" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J248" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K248" s="16"/>
@@ -7964,11 +7991,11 @@
       <c r="G249" s="14"/>
       <c r="H249" s="14"/>
       <c r="I249" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J249" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K249" s="16"/>
@@ -7986,11 +8013,11 @@
       <c r="G250" s="14"/>
       <c r="H250" s="14"/>
       <c r="I250" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J250" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K250" s="16"/>
@@ -8008,11 +8035,11 @@
       <c r="G251" s="14"/>
       <c r="H251" s="14"/>
       <c r="I251" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J251" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K251" s="16"/>
@@ -8030,11 +8057,11 @@
       <c r="G252" s="14"/>
       <c r="H252" s="14"/>
       <c r="I252" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J252" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K252" s="16"/>
@@ -8052,11 +8079,11 @@
       <c r="G253" s="14"/>
       <c r="H253" s="14"/>
       <c r="I253" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J253" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K253" s="16"/>
@@ -8074,11 +8101,11 @@
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
       <c r="I254" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J254" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K254" s="16"/>
@@ -8096,11 +8123,11 @@
       <c r="G255" s="14"/>
       <c r="H255" s="14"/>
       <c r="I255" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J255" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K255" s="16"/>
@@ -8118,11 +8145,11 @@
       <c r="G256" s="14"/>
       <c r="H256" s="14"/>
       <c r="I256" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J256" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K256" s="16"/>
@@ -8140,11 +8167,11 @@
       <c r="G257" s="14"/>
       <c r="H257" s="14"/>
       <c r="I257" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J257" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K257" s="16"/>
@@ -8162,11 +8189,11 @@
       <c r="G258" s="14"/>
       <c r="H258" s="14"/>
       <c r="I258" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J258" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K258" s="16"/>
@@ -8184,11 +8211,11 @@
       <c r="G259" s="14"/>
       <c r="H259" s="14"/>
       <c r="I259" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J259" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K259" s="16"/>
@@ -8206,11 +8233,11 @@
       <c r="G260" s="14"/>
       <c r="H260" s="14"/>
       <c r="I260" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J260" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K260" s="16"/>
@@ -8228,11 +8255,11 @@
       <c r="G261" s="14"/>
       <c r="H261" s="14"/>
       <c r="I261" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J261" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K261" s="16"/>
@@ -8250,11 +8277,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="22">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" ref="I262:I325" si="24">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="23">IF(I262="","",1440-I262)</f>
+        <f t="shared" ref="J262:J325" si="25">IF(I262="","",1440-I262)</f>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -8272,11 +8299,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8294,11 +8321,11 @@
       <c r="G264" s="14"/>
       <c r="H264" s="14"/>
       <c r="I264" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J264" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K264" s="16"/>
@@ -8316,11 +8343,11 @@
       <c r="G265" s="14"/>
       <c r="H265" s="14"/>
       <c r="I265" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J265" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K265" s="16"/>
@@ -8338,11 +8365,11 @@
       <c r="G266" s="14"/>
       <c r="H266" s="14"/>
       <c r="I266" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J266" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K266" s="16"/>
@@ -8360,11 +8387,11 @@
       <c r="G267" s="14"/>
       <c r="H267" s="14"/>
       <c r="I267" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J267" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K267" s="16"/>
@@ -8382,11 +8409,11 @@
       <c r="G268" s="14"/>
       <c r="H268" s="14"/>
       <c r="I268" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J268" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K268" s="16"/>
@@ -8404,11 +8431,11 @@
       <c r="G269" s="14"/>
       <c r="H269" s="14"/>
       <c r="I269" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J269" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K269" s="16"/>
@@ -8426,11 +8453,11 @@
       <c r="G270" s="14"/>
       <c r="H270" s="14"/>
       <c r="I270" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J270" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K270" s="16"/>
@@ -8448,11 +8475,11 @@
       <c r="G271" s="14"/>
       <c r="H271" s="14"/>
       <c r="I271" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J271" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K271" s="16"/>
@@ -8470,11 +8497,11 @@
       <c r="G272" s="14"/>
       <c r="H272" s="14"/>
       <c r="I272" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J272" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K272" s="16"/>
@@ -8492,11 +8519,11 @@
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
       <c r="I273" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J273" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K273" s="16"/>
@@ -8514,11 +8541,11 @@
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
       <c r="I274" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J274" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K274" s="16"/>
@@ -8536,11 +8563,11 @@
       <c r="G275" s="14"/>
       <c r="H275" s="14"/>
       <c r="I275" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J275" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K275" s="16"/>
@@ -8558,11 +8585,11 @@
       <c r="G276" s="14"/>
       <c r="H276" s="14"/>
       <c r="I276" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J276" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K276" s="16"/>
@@ -8580,11 +8607,11 @@
       <c r="G277" s="14"/>
       <c r="H277" s="14"/>
       <c r="I277" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J277" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K277" s="16"/>
@@ -8602,11 +8629,11 @@
       <c r="G278" s="14"/>
       <c r="H278" s="14"/>
       <c r="I278" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J278" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K278" s="16"/>
@@ -8624,11 +8651,11 @@
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
       <c r="I279" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J279" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K279" s="16"/>
@@ -8646,11 +8673,11 @@
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
       <c r="I280" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J280" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K280" s="16"/>
@@ -8668,11 +8695,11 @@
       <c r="G281" s="14"/>
       <c r="H281" s="14"/>
       <c r="I281" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J281" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K281" s="16"/>
@@ -8690,11 +8717,11 @@
       <c r="G282" s="14"/>
       <c r="H282" s="14"/>
       <c r="I282" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J282" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K282" s="16"/>
@@ -8712,11 +8739,11 @@
       <c r="G283" s="14"/>
       <c r="H283" s="14"/>
       <c r="I283" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J283" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K283" s="16"/>
@@ -8734,11 +8761,11 @@
       <c r="G284" s="14"/>
       <c r="H284" s="14"/>
       <c r="I284" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J284" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K284" s="16"/>
@@ -8756,11 +8783,11 @@
       <c r="G285" s="14"/>
       <c r="H285" s="14"/>
       <c r="I285" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J285" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K285" s="16"/>
@@ -8778,11 +8805,11 @@
       <c r="G286" s="14"/>
       <c r="H286" s="14"/>
       <c r="I286" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J286" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K286" s="16"/>
@@ -8800,11 +8827,11 @@
       <c r="G287" s="14"/>
       <c r="H287" s="14"/>
       <c r="I287" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J287" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K287" s="16"/>
@@ -8822,11 +8849,11 @@
       <c r="G288" s="14"/>
       <c r="H288" s="14"/>
       <c r="I288" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J288" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K288" s="16"/>
@@ -8844,11 +8871,11 @@
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
       <c r="I289" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J289" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K289" s="16"/>
@@ -8866,11 +8893,11 @@
       <c r="G290" s="14"/>
       <c r="H290" s="14"/>
       <c r="I290" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J290" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K290" s="16"/>
@@ -8888,11 +8915,11 @@
       <c r="G291" s="14"/>
       <c r="H291" s="14"/>
       <c r="I291" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J291" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K291" s="16"/>
@@ -8910,11 +8937,11 @@
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
       <c r="I292" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J292" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K292" s="16"/>
@@ -8932,11 +8959,11 @@
       <c r="G293" s="14"/>
       <c r="H293" s="14"/>
       <c r="I293" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J293" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K293" s="16"/>
@@ -8954,11 +8981,11 @@
       <c r="G294" s="14"/>
       <c r="H294" s="14"/>
       <c r="I294" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J294" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K294" s="16"/>
@@ -8976,11 +9003,11 @@
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
       <c r="I295" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J295" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K295" s="16"/>
@@ -8998,11 +9025,11 @@
       <c r="G296" s="14"/>
       <c r="H296" s="14"/>
       <c r="I296" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J296" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K296" s="16"/>
@@ -9020,11 +9047,11 @@
       <c r="G297" s="14"/>
       <c r="H297" s="14"/>
       <c r="I297" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J297" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K297" s="16"/>
@@ -9042,11 +9069,11 @@
       <c r="G298" s="14"/>
       <c r="H298" s="14"/>
       <c r="I298" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J298" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K298" s="16"/>
@@ -9064,11 +9091,11 @@
       <c r="G299" s="14"/>
       <c r="H299" s="14"/>
       <c r="I299" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J299" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K299" s="16"/>
@@ -9086,11 +9113,11 @@
       <c r="G300" s="14"/>
       <c r="H300" s="14"/>
       <c r="I300" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J300" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K300" s="16"/>
@@ -9108,11 +9135,11 @@
       <c r="G301" s="14"/>
       <c r="H301" s="14"/>
       <c r="I301" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J301" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K301" s="16"/>
@@ -9130,11 +9157,11 @@
       <c r="G302" s="14"/>
       <c r="H302" s="14"/>
       <c r="I302" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J302" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K302" s="16"/>
@@ -9152,11 +9179,11 @@
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
       <c r="I303" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J303" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K303" s="16"/>
@@ -9174,11 +9201,11 @@
       <c r="G304" s="14"/>
       <c r="H304" s="14"/>
       <c r="I304" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J304" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K304" s="16"/>
@@ -9196,11 +9223,11 @@
       <c r="G305" s="14"/>
       <c r="H305" s="14"/>
       <c r="I305" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J305" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K305" s="16"/>
@@ -9218,11 +9245,11 @@
       <c r="G306" s="14"/>
       <c r="H306" s="14"/>
       <c r="I306" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J306" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K306" s="16"/>
@@ -9240,11 +9267,11 @@
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
       <c r="I307" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J307" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K307" s="16"/>
@@ -9262,11 +9289,11 @@
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
       <c r="I308" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J308" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K308" s="16"/>
@@ -9284,11 +9311,11 @@
       <c r="G309" s="14"/>
       <c r="H309" s="14"/>
       <c r="I309" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J309" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K309" s="16"/>
@@ -9306,11 +9333,11 @@
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
       <c r="I310" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J310" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K310" s="16"/>
@@ -9328,11 +9355,11 @@
       <c r="G311" s="14"/>
       <c r="H311" s="14"/>
       <c r="I311" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J311" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K311" s="16"/>
@@ -9350,11 +9377,11 @@
       <c r="G312" s="14"/>
       <c r="H312" s="14"/>
       <c r="I312" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J312" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K312" s="16"/>
@@ -9372,11 +9399,11 @@
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
       <c r="I313" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J313" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K313" s="16"/>
@@ -9394,11 +9421,11 @@
       <c r="G314" s="14"/>
       <c r="H314" s="14"/>
       <c r="I314" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J314" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K314" s="16"/>
@@ -9416,11 +9443,11 @@
       <c r="G315" s="14"/>
       <c r="H315" s="14"/>
       <c r="I315" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J315" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K315" s="16"/>
@@ -9438,11 +9465,11 @@
       <c r="G316" s="14"/>
       <c r="H316" s="14"/>
       <c r="I316" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J316" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K316" s="16"/>
@@ -9460,11 +9487,11 @@
       <c r="G317" s="14"/>
       <c r="H317" s="14"/>
       <c r="I317" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J317" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K317" s="16"/>
@@ -9482,11 +9509,11 @@
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
       <c r="I318" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J318" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K318" s="16"/>
@@ -9504,11 +9531,11 @@
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
       <c r="I319" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J319" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K319" s="16"/>
@@ -9526,11 +9553,11 @@
       <c r="G320" s="14"/>
       <c r="H320" s="14"/>
       <c r="I320" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J320" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K320" s="16"/>
@@ -9548,11 +9575,11 @@
       <c r="G321" s="14"/>
       <c r="H321" s="14"/>
       <c r="I321" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J321" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K321" s="16"/>
@@ -9570,11 +9597,11 @@
       <c r="G322" s="14"/>
       <c r="H322" s="14"/>
       <c r="I322" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J322" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K322" s="16"/>
@@ -9592,11 +9619,11 @@
       <c r="G323" s="14"/>
       <c r="H323" s="14"/>
       <c r="I323" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J323" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K323" s="16"/>
@@ -9614,11 +9641,11 @@
       <c r="G324" s="14"/>
       <c r="H324" s="14"/>
       <c r="I324" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J324" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K324" s="16"/>
@@ -9636,11 +9663,11 @@
       <c r="G325" s="14"/>
       <c r="H325" s="14"/>
       <c r="I325" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J325" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K325" s="16"/>
@@ -9658,11 +9685,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="24">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" ref="I326:I389" si="26">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="25">IF(I326="","",1440-I326)</f>
+        <f t="shared" ref="J326:J389" si="27">IF(I326="","",1440-I326)</f>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -9680,11 +9707,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -9702,11 +9729,11 @@
       <c r="G328" s="14"/>
       <c r="H328" s="14"/>
       <c r="I328" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J328" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K328" s="16"/>
@@ -9724,11 +9751,11 @@
       <c r="G329" s="14"/>
       <c r="H329" s="14"/>
       <c r="I329" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J329" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K329" s="16"/>
@@ -9746,11 +9773,11 @@
       <c r="G330" s="14"/>
       <c r="H330" s="14"/>
       <c r="I330" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J330" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K330" s="16"/>
@@ -9768,11 +9795,11 @@
       <c r="G331" s="14"/>
       <c r="H331" s="14"/>
       <c r="I331" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J331" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K331" s="16"/>
@@ -9790,11 +9817,11 @@
       <c r="G332" s="14"/>
       <c r="H332" s="14"/>
       <c r="I332" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J332" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K332" s="16"/>
@@ -9812,11 +9839,11 @@
       <c r="G333" s="14"/>
       <c r="H333" s="14"/>
       <c r="I333" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J333" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K333" s="16"/>
@@ -9834,11 +9861,11 @@
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
       <c r="I334" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J334" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K334" s="16"/>
@@ -9856,11 +9883,11 @@
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
       <c r="I335" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J335" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K335" s="16"/>
@@ -9878,11 +9905,11 @@
       <c r="G336" s="14"/>
       <c r="H336" s="14"/>
       <c r="I336" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J336" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K336" s="16"/>
@@ -9900,11 +9927,11 @@
       <c r="G337" s="14"/>
       <c r="H337" s="14"/>
       <c r="I337" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J337" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K337" s="16"/>
@@ -9922,11 +9949,11 @@
       <c r="G338" s="14"/>
       <c r="H338" s="14"/>
       <c r="I338" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J338" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K338" s="16"/>
@@ -9944,11 +9971,11 @@
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
       <c r="I339" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J339" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K339" s="16"/>
@@ -9966,11 +9993,11 @@
       <c r="G340" s="14"/>
       <c r="H340" s="14"/>
       <c r="I340" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J340" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K340" s="16"/>
@@ -9988,11 +10015,11 @@
       <c r="G341" s="14"/>
       <c r="H341" s="14"/>
       <c r="I341" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J341" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K341" s="16"/>
@@ -10010,11 +10037,11 @@
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
       <c r="I342" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J342" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K342" s="16"/>
@@ -10032,11 +10059,11 @@
       <c r="G343" s="14"/>
       <c r="H343" s="14"/>
       <c r="I343" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J343" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K343" s="16"/>
@@ -10054,11 +10081,11 @@
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
       <c r="I344" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J344" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K344" s="16"/>
@@ -10076,11 +10103,11 @@
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
       <c r="I345" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J345" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K345" s="16"/>
@@ -10098,11 +10125,11 @@
       <c r="G346" s="14"/>
       <c r="H346" s="14"/>
       <c r="I346" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J346" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K346" s="16"/>
@@ -10120,11 +10147,11 @@
       <c r="G347" s="14"/>
       <c r="H347" s="14"/>
       <c r="I347" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J347" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K347" s="16"/>
@@ -10142,11 +10169,11 @@
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
       <c r="I348" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J348" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K348" s="16"/>
@@ -10164,11 +10191,11 @@
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
       <c r="I349" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J349" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K349" s="16"/>
@@ -10186,11 +10213,11 @@
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
       <c r="I350" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J350" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K350" s="16"/>
@@ -10208,11 +10235,11 @@
       <c r="G351" s="14"/>
       <c r="H351" s="14"/>
       <c r="I351" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J351" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K351" s="16"/>
@@ -10230,11 +10257,11 @@
       <c r="G352" s="14"/>
       <c r="H352" s="14"/>
       <c r="I352" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J352" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K352" s="16"/>
@@ -10252,11 +10279,11 @@
       <c r="G353" s="14"/>
       <c r="H353" s="14"/>
       <c r="I353" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J353" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K353" s="16"/>
@@ -10274,11 +10301,11 @@
       <c r="G354" s="14"/>
       <c r="H354" s="14"/>
       <c r="I354" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J354" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K354" s="16"/>
@@ -10296,11 +10323,11 @@
       <c r="G355" s="14"/>
       <c r="H355" s="14"/>
       <c r="I355" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J355" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K355" s="16"/>
@@ -10318,11 +10345,11 @@
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
       <c r="I356" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J356" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K356" s="16"/>
@@ -10340,11 +10367,11 @@
       <c r="G357" s="14"/>
       <c r="H357" s="14"/>
       <c r="I357" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J357" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K357" s="16"/>
@@ -10362,11 +10389,11 @@
       <c r="G358" s="14"/>
       <c r="H358" s="14"/>
       <c r="I358" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J358" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K358" s="16"/>
@@ -10384,11 +10411,11 @@
       <c r="G359" s="14"/>
       <c r="H359" s="14"/>
       <c r="I359" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J359" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K359" s="16"/>
@@ -10406,11 +10433,11 @@
       <c r="G360" s="14"/>
       <c r="H360" s="14"/>
       <c r="I360" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J360" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K360" s="16"/>
@@ -10428,11 +10455,11 @@
       <c r="G361" s="14"/>
       <c r="H361" s="14"/>
       <c r="I361" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J361" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K361" s="16"/>
@@ -10450,11 +10477,11 @@
       <c r="G362" s="14"/>
       <c r="H362" s="14"/>
       <c r="I362" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J362" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K362" s="16"/>
@@ -10472,11 +10499,11 @@
       <c r="G363" s="14"/>
       <c r="H363" s="14"/>
       <c r="I363" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J363" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K363" s="16"/>
@@ -10494,11 +10521,11 @@
       <c r="G364" s="14"/>
       <c r="H364" s="14"/>
       <c r="I364" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J364" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K364" s="16"/>
@@ -10516,11 +10543,11 @@
       <c r="G365" s="14"/>
       <c r="H365" s="14"/>
       <c r="I365" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J365" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K365" s="16"/>
@@ -10538,11 +10565,11 @@
       <c r="G366" s="14"/>
       <c r="H366" s="14"/>
       <c r="I366" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J366" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K366" s="16"/>
@@ -10560,11 +10587,11 @@
       <c r="G367" s="14"/>
       <c r="H367" s="14"/>
       <c r="I367" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J367" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K367" s="16"/>
@@ -10582,11 +10609,11 @@
       <c r="G368" s="14"/>
       <c r="H368" s="14"/>
       <c r="I368" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J368" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K368" s="16"/>
@@ -10604,11 +10631,11 @@
       <c r="G369" s="14"/>
       <c r="H369" s="14"/>
       <c r="I369" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J369" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K369" s="16"/>
@@ -10626,11 +10653,11 @@
       <c r="G370" s="14"/>
       <c r="H370" s="14"/>
       <c r="I370" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J370" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K370" s="16"/>
@@ -10648,11 +10675,11 @@
       <c r="G371" s="14"/>
       <c r="H371" s="14"/>
       <c r="I371" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J371" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K371" s="16"/>
@@ -10670,11 +10697,11 @@
       <c r="G372" s="14"/>
       <c r="H372" s="14"/>
       <c r="I372" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J372" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K372" s="16"/>
@@ -10692,11 +10719,11 @@
       <c r="G373" s="14"/>
       <c r="H373" s="14"/>
       <c r="I373" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J373" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K373" s="16"/>
@@ -10714,11 +10741,11 @@
       <c r="G374" s="14"/>
       <c r="H374" s="14"/>
       <c r="I374" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J374" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K374" s="16"/>
@@ -10736,11 +10763,11 @@
       <c r="G375" s="14"/>
       <c r="H375" s="14"/>
       <c r="I375" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J375" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K375" s="16"/>
@@ -10758,11 +10785,11 @@
       <c r="G376" s="14"/>
       <c r="H376" s="14"/>
       <c r="I376" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J376" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K376" s="16"/>
@@ -10780,11 +10807,11 @@
       <c r="G377" s="14"/>
       <c r="H377" s="14"/>
       <c r="I377" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J377" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K377" s="16"/>
@@ -10802,11 +10829,11 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K378" s="16"/>
@@ -10824,11 +10851,11 @@
       <c r="G379" s="14"/>
       <c r="H379" s="14"/>
       <c r="I379" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J379" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K379" s="16"/>
@@ -10846,11 +10873,11 @@
       <c r="G380" s="14"/>
       <c r="H380" s="14"/>
       <c r="I380" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J380" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K380" s="16"/>
@@ -10868,11 +10895,11 @@
       <c r="G381" s="14"/>
       <c r="H381" s="14"/>
       <c r="I381" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J381" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K381" s="16"/>
@@ -10890,11 +10917,11 @@
       <c r="G382" s="14"/>
       <c r="H382" s="14"/>
       <c r="I382" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J382" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K382" s="16"/>
@@ -10912,11 +10939,11 @@
       <c r="G383" s="14"/>
       <c r="H383" s="14"/>
       <c r="I383" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J383" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K383" s="16"/>
@@ -10934,11 +10961,11 @@
       <c r="G384" s="14"/>
       <c r="H384" s="14"/>
       <c r="I384" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J384" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K384" s="16"/>
@@ -10956,11 +10983,11 @@
       <c r="G385" s="14"/>
       <c r="H385" s="14"/>
       <c r="I385" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J385" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K385" s="16"/>
@@ -10978,11 +11005,11 @@
       <c r="G386" s="14"/>
       <c r="H386" s="14"/>
       <c r="I386" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J386" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K386" s="16"/>
@@ -11000,11 +11027,11 @@
       <c r="G387" s="14"/>
       <c r="H387" s="14"/>
       <c r="I387" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J387" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K387" s="16"/>
@@ -11022,11 +11049,11 @@
       <c r="G388" s="14"/>
       <c r="H388" s="14"/>
       <c r="I388" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J388" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K388" s="16"/>
@@ -11044,11 +11071,11 @@
       <c r="G389" s="14"/>
       <c r="H389" s="14"/>
       <c r="I389" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J389" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K389" s="16"/>
@@ -11066,11 +11093,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="26">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="28">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="27">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="29">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -11088,11 +11115,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -11110,11 +11137,11 @@
       <c r="G392" s="14"/>
       <c r="H392" s="14"/>
       <c r="I392" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J392" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K392" s="16"/>
@@ -11132,11 +11159,11 @@
       <c r="G393" s="14"/>
       <c r="H393" s="14"/>
       <c r="I393" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J393" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K393" s="16"/>
@@ -11154,11 +11181,11 @@
       <c r="G394" s="14"/>
       <c r="H394" s="14"/>
       <c r="I394" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J394" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K394" s="16"/>
@@ -11176,11 +11203,11 @@
       <c r="G395" s="14"/>
       <c r="H395" s="14"/>
       <c r="I395" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J395" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K395" s="16"/>
@@ -11198,11 +11225,11 @@
       <c r="G396" s="14"/>
       <c r="H396" s="14"/>
       <c r="I396" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J396" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K396" s="16"/>
@@ -11220,11 +11247,11 @@
       <c r="G397" s="14"/>
       <c r="H397" s="14"/>
       <c r="I397" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J397" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K397" s="16"/>
@@ -11242,11 +11269,11 @@
       <c r="G398" s="14"/>
       <c r="H398" s="14"/>
       <c r="I398" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J398" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K398" s="16"/>
@@ -11264,11 +11291,11 @@
       <c r="G399" s="14"/>
       <c r="H399" s="14"/>
       <c r="I399" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J399" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K399" s="16"/>
@@ -11286,11 +11313,11 @@
       <c r="G400" s="14"/>
       <c r="H400" s="14"/>
       <c r="I400" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J400" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K400" s="16"/>
@@ -11308,11 +11335,11 @@
       <c r="G401" s="14"/>
       <c r="H401" s="14"/>
       <c r="I401" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J401" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K401" s="16"/>

</xml_diff>

<commit_message>
File Uploaded On 21/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3242867D-B5AA-419A-97D2-434941DE538E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{864E045D-DA0E-4C1D-B48A-49240020AC42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="612" yWindow="-108" windowWidth="22536" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="92">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -308,6 +308,9 @@
   </si>
   <si>
     <t>Practiced analytic skills questions</t>
+  </si>
+  <si>
+    <t>Tired because of classes</t>
   </si>
 </sst>
 </file>
@@ -3946,21 +3949,21 @@
         <v>0</v>
       </c>
       <c r="F67" s="14">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="G67" s="14">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H67" s="14">
         <v>120</v>
       </c>
       <c r="I67" s="15">
         <f t="shared" ref="I67" si="14">IF(SUM(B67:F67,H67)=0,"",SUM(B67:F67,H67))</f>
-        <v>690</v>
+        <v>940</v>
       </c>
       <c r="J67" s="15">
         <f t="shared" ref="J67" si="15">IF(I67="","",1440-I67)</f>
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="K67" s="16" t="s">
         <v>67</v>
@@ -4022,26 +4025,50 @@
       </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A69" s="13"/>
-      <c r="B69" s="14"/>
-      <c r="C69" s="14"/>
-      <c r="D69" s="14"/>
-      <c r="E69" s="14"/>
-      <c r="F69" s="14"/>
-      <c r="G69" s="14"/>
-      <c r="H69" s="14"/>
-      <c r="I69" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J69" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K69" s="16"/>
-      <c r="L69" s="16"/>
-      <c r="M69" s="16"/>
-      <c r="N69" s="17"/>
+      <c r="A69" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B69" s="14">
+        <v>420</v>
+      </c>
+      <c r="C69" s="14">
+        <v>0</v>
+      </c>
+      <c r="D69" s="14">
+        <v>60</v>
+      </c>
+      <c r="E69" s="14">
+        <v>200</v>
+      </c>
+      <c r="F69" s="14">
+        <v>300</v>
+      </c>
+      <c r="G69" s="14">
+        <v>6</v>
+      </c>
+      <c r="H69" s="14">
+        <v>170</v>
+      </c>
+      <c r="I69" s="15">
+        <f t="shared" ref="I69" si="18">IF(SUM(B69:F69,H69)=0,"",SUM(B69:F69,H69))</f>
+        <v>1150</v>
+      </c>
+      <c r="J69" s="15">
+        <f t="shared" ref="J69" si="19">IF(I69="","",1440-I69)</f>
+        <v>290</v>
+      </c>
+      <c r="K69" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L69" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M69" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N69" s="17" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70" s="13"/>
@@ -4053,11 +4080,11 @@
       <c r="G70" s="14"/>
       <c r="H70" s="14"/>
       <c r="I70" s="15" t="str">
-        <f t="shared" ref="I70:I133" si="18">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
+        <f t="shared" ref="I70:I133" si="20">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
         <v/>
       </c>
       <c r="J70" s="15" t="str">
-        <f t="shared" ref="J70:J133" si="19">IF(I70="","",1440-I70)</f>
+        <f t="shared" ref="J70:J133" si="21">IF(I70="","",1440-I70)</f>
         <v/>
       </c>
       <c r="K70" s="16"/>
@@ -4075,11 +4102,11 @@
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
       <c r="I71" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J71" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K71" s="16"/>
@@ -4097,11 +4124,11 @@
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
       <c r="I72" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J72" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K72" s="16"/>
@@ -4119,11 +4146,11 @@
       <c r="G73" s="14"/>
       <c r="H73" s="14"/>
       <c r="I73" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J73" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K73" s="16"/>
@@ -4141,11 +4168,11 @@
       <c r="G74" s="14"/>
       <c r="H74" s="14"/>
       <c r="I74" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J74" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K74" s="16"/>
@@ -4163,11 +4190,11 @@
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
       <c r="I75" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J75" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K75" s="16"/>
@@ -4185,11 +4212,11 @@
       <c r="G76" s="14"/>
       <c r="H76" s="14"/>
       <c r="I76" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J76" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K76" s="16"/>
@@ -4207,11 +4234,11 @@
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
       <c r="I77" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J77" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K77" s="16"/>
@@ -4229,11 +4256,11 @@
       <c r="G78" s="14"/>
       <c r="H78" s="14"/>
       <c r="I78" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J78" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K78" s="16"/>
@@ -4251,11 +4278,11 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J79" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K79" s="16"/>
@@ -4273,11 +4300,11 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J80" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K80" s="16"/>
@@ -4295,11 +4322,11 @@
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J81" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K81" s="16"/>
@@ -4317,11 +4344,11 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J82" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K82" s="16"/>
@@ -4339,11 +4366,11 @@
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
       <c r="I83" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J83" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K83" s="16"/>
@@ -4361,11 +4388,11 @@
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
       <c r="I84" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J84" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K84" s="16"/>
@@ -4383,11 +4410,11 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J85" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K85" s="16"/>
@@ -4405,11 +4432,11 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J86" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K86" s="16"/>
@@ -4427,11 +4454,11 @@
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
       <c r="I87" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J87" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K87" s="16"/>
@@ -4449,11 +4476,11 @@
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
       <c r="I88" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J88" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K88" s="16"/>
@@ -4471,11 +4498,11 @@
       <c r="G89" s="14"/>
       <c r="H89" s="14"/>
       <c r="I89" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J89" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K89" s="16"/>
@@ -4493,11 +4520,11 @@
       <c r="G90" s="14"/>
       <c r="H90" s="14"/>
       <c r="I90" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J90" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K90" s="16"/>
@@ -4515,11 +4542,11 @@
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
       <c r="I91" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J91" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K91" s="16"/>
@@ -4537,11 +4564,11 @@
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
       <c r="I92" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J92" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K92" s="16"/>
@@ -4559,11 +4586,11 @@
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J93" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K93" s="16"/>
@@ -4581,11 +4608,11 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J94" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K94" s="16"/>
@@ -4603,11 +4630,11 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J95" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K95" s="16"/>
@@ -4625,11 +4652,11 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J96" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K96" s="16"/>
@@ -4647,11 +4674,11 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J97" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K97" s="16"/>
@@ -4669,11 +4696,11 @@
       <c r="G98" s="14"/>
       <c r="H98" s="14"/>
       <c r="I98" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J98" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K98" s="16"/>
@@ -4691,11 +4718,11 @@
       <c r="G99" s="14"/>
       <c r="H99" s="14"/>
       <c r="I99" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J99" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K99" s="16"/>
@@ -4713,11 +4740,11 @@
       <c r="G100" s="14"/>
       <c r="H100" s="14"/>
       <c r="I100" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J100" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K100" s="16"/>
@@ -4735,11 +4762,11 @@
       <c r="G101" s="14"/>
       <c r="H101" s="14"/>
       <c r="I101" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J101" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K101" s="16"/>
@@ -4757,11 +4784,11 @@
       <c r="G102" s="14"/>
       <c r="H102" s="14"/>
       <c r="I102" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J102" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K102" s="16"/>
@@ -4779,11 +4806,11 @@
       <c r="G103" s="14"/>
       <c r="H103" s="14"/>
       <c r="I103" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J103" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K103" s="16"/>
@@ -4801,11 +4828,11 @@
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
       <c r="I104" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J104" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K104" s="16"/>
@@ -4823,11 +4850,11 @@
       <c r="G105" s="14"/>
       <c r="H105" s="14"/>
       <c r="I105" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J105" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K105" s="16"/>
@@ -4845,11 +4872,11 @@
       <c r="G106" s="14"/>
       <c r="H106" s="14"/>
       <c r="I106" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J106" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K106" s="16"/>
@@ -4867,11 +4894,11 @@
       <c r="G107" s="14"/>
       <c r="H107" s="14"/>
       <c r="I107" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J107" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K107" s="16"/>
@@ -4889,11 +4916,11 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J108" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K108" s="16"/>
@@ -4911,11 +4938,11 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J109" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K109" s="16"/>
@@ -4933,11 +4960,11 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J110" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K110" s="16"/>
@@ -4955,11 +4982,11 @@
       <c r="G111" s="14"/>
       <c r="H111" s="14"/>
       <c r="I111" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J111" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K111" s="16"/>
@@ -4977,11 +5004,11 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J112" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K112" s="16"/>
@@ -4999,11 +5026,11 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J113" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K113" s="16"/>
@@ -5021,11 +5048,11 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J114" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K114" s="16"/>
@@ -5043,11 +5070,11 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J115" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K115" s="16"/>
@@ -5065,11 +5092,11 @@
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
       <c r="I116" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J116" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K116" s="16"/>
@@ -5087,11 +5114,11 @@
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
       <c r="I117" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J117" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K117" s="16"/>
@@ -5109,11 +5136,11 @@
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
       <c r="I118" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J118" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K118" s="16"/>
@@ -5131,11 +5158,11 @@
       <c r="G119" s="14"/>
       <c r="H119" s="14"/>
       <c r="I119" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J119" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K119" s="16"/>
@@ -5153,11 +5180,11 @@
       <c r="G120" s="14"/>
       <c r="H120" s="14"/>
       <c r="I120" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J120" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K120" s="16"/>
@@ -5175,11 +5202,11 @@
       <c r="G121" s="14"/>
       <c r="H121" s="14"/>
       <c r="I121" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J121" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K121" s="16"/>
@@ -5197,11 +5224,11 @@
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
       <c r="I122" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J122" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K122" s="16"/>
@@ -5219,11 +5246,11 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J123" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K123" s="16"/>
@@ -5241,11 +5268,11 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J124" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K124" s="16"/>
@@ -5263,11 +5290,11 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J125" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K125" s="16"/>
@@ -5285,11 +5312,11 @@
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
       <c r="I126" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J126" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K126" s="16"/>
@@ -5307,11 +5334,11 @@
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J127" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K127" s="16"/>
@@ -5329,11 +5356,11 @@
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
       <c r="I128" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J128" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K128" s="16"/>
@@ -5351,11 +5378,11 @@
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
       <c r="I129" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J129" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K129" s="16"/>
@@ -5373,11 +5400,11 @@
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
       <c r="I130" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J130" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K130" s="16"/>
@@ -5395,11 +5422,11 @@
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
       <c r="I131" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J131" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K131" s="16"/>
@@ -5417,11 +5444,11 @@
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
       <c r="I132" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J132" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K132" s="16"/>
@@ -5439,11 +5466,11 @@
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
       <c r="I133" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="J133" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="K133" s="16"/>
@@ -5461,11 +5488,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="20">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" ref="I134:I197" si="22">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="21">IF(I134="","",1440-I134)</f>
+        <f t="shared" ref="J134:J197" si="23">IF(I134="","",1440-I134)</f>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -5483,11 +5510,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5505,11 +5532,11 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J136" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K136" s="16"/>
@@ -5527,11 +5554,11 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J137" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K137" s="16"/>
@@ -5549,11 +5576,11 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J138" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K138" s="16"/>
@@ -5571,11 +5598,11 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J139" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K139" s="16"/>
@@ -5593,11 +5620,11 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J140" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K140" s="16"/>
@@ -5615,11 +5642,11 @@
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J141" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K141" s="16"/>
@@ -5637,11 +5664,11 @@
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J142" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K142" s="16"/>
@@ -5659,11 +5686,11 @@
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J143" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K143" s="16"/>
@@ -5681,11 +5708,11 @@
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J144" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K144" s="16"/>
@@ -5703,11 +5730,11 @@
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J145" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K145" s="16"/>
@@ -5725,11 +5752,11 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J146" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K146" s="16"/>
@@ -5747,11 +5774,11 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J147" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K147" s="16"/>
@@ -5769,11 +5796,11 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J148" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K148" s="16"/>
@@ -5791,11 +5818,11 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J149" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K149" s="16"/>
@@ -5813,11 +5840,11 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J150" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K150" s="16"/>
@@ -5835,11 +5862,11 @@
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
       <c r="I151" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J151" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K151" s="16"/>
@@ -5857,11 +5884,11 @@
       <c r="G152" s="14"/>
       <c r="H152" s="14"/>
       <c r="I152" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J152" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K152" s="16"/>
@@ -5879,11 +5906,11 @@
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J153" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K153" s="16"/>
@@ -5901,11 +5928,11 @@
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J154" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K154" s="16"/>
@@ -5923,11 +5950,11 @@
       <c r="G155" s="14"/>
       <c r="H155" s="14"/>
       <c r="I155" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J155" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K155" s="16"/>
@@ -5945,11 +5972,11 @@
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
       <c r="I156" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J156" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K156" s="16"/>
@@ -5967,11 +5994,11 @@
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J157" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K157" s="16"/>
@@ -5989,11 +6016,11 @@
       <c r="G158" s="14"/>
       <c r="H158" s="14"/>
       <c r="I158" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J158" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K158" s="16"/>
@@ -6011,11 +6038,11 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J159" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K159" s="16"/>
@@ -6033,11 +6060,11 @@
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
       <c r="I160" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J160" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K160" s="16"/>
@@ -6055,11 +6082,11 @@
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
       <c r="I161" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J161" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K161" s="16"/>
@@ -6077,11 +6104,11 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J162" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K162" s="16"/>
@@ -6099,11 +6126,11 @@
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
       <c r="I163" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J163" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K163" s="16"/>
@@ -6121,11 +6148,11 @@
       <c r="G164" s="14"/>
       <c r="H164" s="14"/>
       <c r="I164" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J164" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K164" s="16"/>
@@ -6143,11 +6170,11 @@
       <c r="G165" s="14"/>
       <c r="H165" s="14"/>
       <c r="I165" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J165" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K165" s="16"/>
@@ -6165,11 +6192,11 @@
       <c r="G166" s="14"/>
       <c r="H166" s="14"/>
       <c r="I166" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J166" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K166" s="16"/>
@@ -6187,11 +6214,11 @@
       <c r="G167" s="14"/>
       <c r="H167" s="14"/>
       <c r="I167" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J167" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K167" s="16"/>
@@ -6209,11 +6236,11 @@
       <c r="G168" s="14"/>
       <c r="H168" s="14"/>
       <c r="I168" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J168" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K168" s="16"/>
@@ -6231,11 +6258,11 @@
       <c r="G169" s="14"/>
       <c r="H169" s="14"/>
       <c r="I169" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J169" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K169" s="16"/>
@@ -6253,11 +6280,11 @@
       <c r="G170" s="14"/>
       <c r="H170" s="14"/>
       <c r="I170" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J170" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K170" s="16"/>
@@ -6275,11 +6302,11 @@
       <c r="G171" s="14"/>
       <c r="H171" s="14"/>
       <c r="I171" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J171" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K171" s="16"/>
@@ -6297,11 +6324,11 @@
       <c r="G172" s="14"/>
       <c r="H172" s="14"/>
       <c r="I172" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J172" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K172" s="16"/>
@@ -6319,11 +6346,11 @@
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
       <c r="I173" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J173" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K173" s="16"/>
@@ -6341,11 +6368,11 @@
       <c r="G174" s="14"/>
       <c r="H174" s="14"/>
       <c r="I174" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J174" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K174" s="16"/>
@@ -6363,11 +6390,11 @@
       <c r="G175" s="14"/>
       <c r="H175" s="14"/>
       <c r="I175" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J175" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K175" s="16"/>
@@ -6385,11 +6412,11 @@
       <c r="G176" s="14"/>
       <c r="H176" s="14"/>
       <c r="I176" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J176" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K176" s="16"/>
@@ -6407,11 +6434,11 @@
       <c r="G177" s="14"/>
       <c r="H177" s="14"/>
       <c r="I177" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J177" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K177" s="16"/>
@@ -6429,11 +6456,11 @@
       <c r="G178" s="14"/>
       <c r="H178" s="14"/>
       <c r="I178" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J178" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K178" s="16"/>
@@ -6451,11 +6478,11 @@
       <c r="G179" s="14"/>
       <c r="H179" s="14"/>
       <c r="I179" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J179" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K179" s="16"/>
@@ -6473,11 +6500,11 @@
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
       <c r="I180" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J180" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K180" s="16"/>
@@ -6495,11 +6522,11 @@
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J181" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K181" s="16"/>
@@ -6517,11 +6544,11 @@
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J182" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K182" s="16"/>
@@ -6539,11 +6566,11 @@
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J183" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K183" s="16"/>
@@ -6561,11 +6588,11 @@
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
       <c r="I184" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J184" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K184" s="16"/>
@@ -6583,11 +6610,11 @@
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
       <c r="I185" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J185" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K185" s="16"/>
@@ -6605,11 +6632,11 @@
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J186" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K186" s="16"/>
@@ -6627,11 +6654,11 @@
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J187" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K187" s="16"/>
@@ -6649,11 +6676,11 @@
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
       <c r="I188" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J188" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K188" s="16"/>
@@ -6671,11 +6698,11 @@
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
       <c r="I189" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J189" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K189" s="16"/>
@@ -6693,11 +6720,11 @@
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J190" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K190" s="16"/>
@@ -6715,11 +6742,11 @@
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J191" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K191" s="16"/>
@@ -6737,11 +6764,11 @@
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J192" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K192" s="16"/>
@@ -6759,11 +6786,11 @@
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
       <c r="I193" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J193" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K193" s="16"/>
@@ -6781,11 +6808,11 @@
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
       <c r="I194" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J194" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K194" s="16"/>
@@ -6803,11 +6830,11 @@
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J195" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K195" s="16"/>
@@ -6825,11 +6852,11 @@
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J196" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K196" s="16"/>
@@ -6847,11 +6874,11 @@
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J197" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K197" s="16"/>
@@ -6869,11 +6896,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="22">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" ref="I198:I261" si="24">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="23">IF(I198="","",1440-I198)</f>
+        <f t="shared" ref="J198:J261" si="25">IF(I198="","",1440-I198)</f>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -6891,11 +6918,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -6913,11 +6940,11 @@
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J200" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K200" s="16"/>
@@ -6935,11 +6962,11 @@
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
       <c r="I201" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J201" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K201" s="16"/>
@@ -6957,11 +6984,11 @@
       <c r="G202" s="14"/>
       <c r="H202" s="14"/>
       <c r="I202" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J202" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K202" s="16"/>
@@ -6979,11 +7006,11 @@
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
       <c r="I203" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J203" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K203" s="16"/>
@@ -7001,11 +7028,11 @@
       <c r="G204" s="14"/>
       <c r="H204" s="14"/>
       <c r="I204" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J204" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K204" s="16"/>
@@ -7023,11 +7050,11 @@
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J205" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K205" s="16"/>
@@ -7045,11 +7072,11 @@
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J206" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K206" s="16"/>
@@ -7067,11 +7094,11 @@
       <c r="G207" s="14"/>
       <c r="H207" s="14"/>
       <c r="I207" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J207" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K207" s="16"/>
@@ -7089,11 +7116,11 @@
       <c r="G208" s="14"/>
       <c r="H208" s="14"/>
       <c r="I208" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J208" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K208" s="16"/>
@@ -7111,11 +7138,11 @@
       <c r="G209" s="14"/>
       <c r="H209" s="14"/>
       <c r="I209" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J209" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K209" s="16"/>
@@ -7133,11 +7160,11 @@
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J210" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K210" s="16"/>
@@ -7155,11 +7182,11 @@
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J211" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K211" s="16"/>
@@ -7177,11 +7204,11 @@
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J212" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K212" s="16"/>
@@ -7199,11 +7226,11 @@
       <c r="G213" s="14"/>
       <c r="H213" s="14"/>
       <c r="I213" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J213" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K213" s="16"/>
@@ -7221,11 +7248,11 @@
       <c r="G214" s="14"/>
       <c r="H214" s="14"/>
       <c r="I214" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J214" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K214" s="16"/>
@@ -7243,11 +7270,11 @@
       <c r="G215" s="14"/>
       <c r="H215" s="14"/>
       <c r="I215" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J215" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K215" s="16"/>
@@ -7265,11 +7292,11 @@
       <c r="G216" s="14"/>
       <c r="H216" s="14"/>
       <c r="I216" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J216" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K216" s="16"/>
@@ -7287,11 +7314,11 @@
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J217" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K217" s="16"/>
@@ -7309,11 +7336,11 @@
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J218" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K218" s="16"/>
@@ -7331,11 +7358,11 @@
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J219" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K219" s="16"/>
@@ -7353,11 +7380,11 @@
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J220" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K220" s="16"/>
@@ -7375,11 +7402,11 @@
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J221" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K221" s="16"/>
@@ -7397,11 +7424,11 @@
       <c r="G222" s="14"/>
       <c r="H222" s="14"/>
       <c r="I222" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J222" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K222" s="16"/>
@@ -7419,11 +7446,11 @@
       <c r="G223" s="14"/>
       <c r="H223" s="14"/>
       <c r="I223" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J223" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K223" s="16"/>
@@ -7441,11 +7468,11 @@
       <c r="G224" s="14"/>
       <c r="H224" s="14"/>
       <c r="I224" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J224" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K224" s="16"/>
@@ -7463,11 +7490,11 @@
       <c r="G225" s="14"/>
       <c r="H225" s="14"/>
       <c r="I225" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J225" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K225" s="16"/>
@@ -7485,11 +7512,11 @@
       <c r="G226" s="14"/>
       <c r="H226" s="14"/>
       <c r="I226" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J226" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K226" s="16"/>
@@ -7507,11 +7534,11 @@
       <c r="G227" s="14"/>
       <c r="H227" s="14"/>
       <c r="I227" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J227" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K227" s="16"/>
@@ -7529,11 +7556,11 @@
       <c r="G228" s="14"/>
       <c r="H228" s="14"/>
       <c r="I228" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J228" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K228" s="16"/>
@@ -7551,11 +7578,11 @@
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J229" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K229" s="16"/>
@@ -7573,11 +7600,11 @@
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J230" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K230" s="16"/>
@@ -7595,11 +7622,11 @@
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
       <c r="I231" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J231" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K231" s="16"/>
@@ -7617,11 +7644,11 @@
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
       <c r="I232" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J232" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K232" s="16"/>
@@ -7639,11 +7666,11 @@
       <c r="G233" s="14"/>
       <c r="H233" s="14"/>
       <c r="I233" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J233" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K233" s="16"/>
@@ -7661,11 +7688,11 @@
       <c r="G234" s="14"/>
       <c r="H234" s="14"/>
       <c r="I234" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J234" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K234" s="16"/>
@@ -7683,11 +7710,11 @@
       <c r="G235" s="14"/>
       <c r="H235" s="14"/>
       <c r="I235" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J235" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K235" s="16"/>
@@ -7705,11 +7732,11 @@
       <c r="G236" s="14"/>
       <c r="H236" s="14"/>
       <c r="I236" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J236" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K236" s="16"/>
@@ -7727,11 +7754,11 @@
       <c r="G237" s="14"/>
       <c r="H237" s="14"/>
       <c r="I237" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J237" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K237" s="16"/>
@@ -7749,11 +7776,11 @@
       <c r="G238" s="14"/>
       <c r="H238" s="14"/>
       <c r="I238" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J238" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K238" s="16"/>
@@ -7771,11 +7798,11 @@
       <c r="G239" s="14"/>
       <c r="H239" s="14"/>
       <c r="I239" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J239" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K239" s="16"/>
@@ -7793,11 +7820,11 @@
       <c r="G240" s="14"/>
       <c r="H240" s="14"/>
       <c r="I240" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J240" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K240" s="16"/>
@@ -7815,11 +7842,11 @@
       <c r="G241" s="14"/>
       <c r="H241" s="14"/>
       <c r="I241" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J241" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K241" s="16"/>
@@ -7837,11 +7864,11 @@
       <c r="G242" s="14"/>
       <c r="H242" s="14"/>
       <c r="I242" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J242" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K242" s="16"/>
@@ -7859,11 +7886,11 @@
       <c r="G243" s="14"/>
       <c r="H243" s="14"/>
       <c r="I243" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J243" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K243" s="16"/>
@@ -7881,11 +7908,11 @@
       <c r="G244" s="14"/>
       <c r="H244" s="14"/>
       <c r="I244" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J244" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K244" s="16"/>
@@ -7903,11 +7930,11 @@
       <c r="G245" s="14"/>
       <c r="H245" s="14"/>
       <c r="I245" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J245" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K245" s="16"/>
@@ -7925,11 +7952,11 @@
       <c r="G246" s="14"/>
       <c r="H246" s="14"/>
       <c r="I246" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J246" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K246" s="16"/>
@@ -7947,11 +7974,11 @@
       <c r="G247" s="14"/>
       <c r="H247" s="14"/>
       <c r="I247" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J247" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K247" s="16"/>
@@ -7969,11 +7996,11 @@
       <c r="G248" s="14"/>
       <c r="H248" s="14"/>
       <c r="I248" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J248" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K248" s="16"/>
@@ -7991,11 +8018,11 @@
       <c r="G249" s="14"/>
       <c r="H249" s="14"/>
       <c r="I249" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J249" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K249" s="16"/>
@@ -8013,11 +8040,11 @@
       <c r="G250" s="14"/>
       <c r="H250" s="14"/>
       <c r="I250" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J250" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K250" s="16"/>
@@ -8035,11 +8062,11 @@
       <c r="G251" s="14"/>
       <c r="H251" s="14"/>
       <c r="I251" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J251" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K251" s="16"/>
@@ -8057,11 +8084,11 @@
       <c r="G252" s="14"/>
       <c r="H252" s="14"/>
       <c r="I252" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J252" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K252" s="16"/>
@@ -8079,11 +8106,11 @@
       <c r="G253" s="14"/>
       <c r="H253" s="14"/>
       <c r="I253" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J253" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K253" s="16"/>
@@ -8101,11 +8128,11 @@
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
       <c r="I254" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J254" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K254" s="16"/>
@@ -8123,11 +8150,11 @@
       <c r="G255" s="14"/>
       <c r="H255" s="14"/>
       <c r="I255" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J255" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K255" s="16"/>
@@ -8145,11 +8172,11 @@
       <c r="G256" s="14"/>
       <c r="H256" s="14"/>
       <c r="I256" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J256" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K256" s="16"/>
@@ -8167,11 +8194,11 @@
       <c r="G257" s="14"/>
       <c r="H257" s="14"/>
       <c r="I257" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J257" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K257" s="16"/>
@@ -8189,11 +8216,11 @@
       <c r="G258" s="14"/>
       <c r="H258" s="14"/>
       <c r="I258" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J258" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K258" s="16"/>
@@ -8211,11 +8238,11 @@
       <c r="G259" s="14"/>
       <c r="H259" s="14"/>
       <c r="I259" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J259" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K259" s="16"/>
@@ -8233,11 +8260,11 @@
       <c r="G260" s="14"/>
       <c r="H260" s="14"/>
       <c r="I260" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J260" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K260" s="16"/>
@@ -8255,11 +8282,11 @@
       <c r="G261" s="14"/>
       <c r="H261" s="14"/>
       <c r="I261" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J261" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K261" s="16"/>
@@ -8277,11 +8304,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="24">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" ref="I262:I325" si="26">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="25">IF(I262="","",1440-I262)</f>
+        <f t="shared" ref="J262:J325" si="27">IF(I262="","",1440-I262)</f>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -8299,11 +8326,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8321,11 +8348,11 @@
       <c r="G264" s="14"/>
       <c r="H264" s="14"/>
       <c r="I264" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J264" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K264" s="16"/>
@@ -8343,11 +8370,11 @@
       <c r="G265" s="14"/>
       <c r="H265" s="14"/>
       <c r="I265" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J265" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K265" s="16"/>
@@ -8365,11 +8392,11 @@
       <c r="G266" s="14"/>
       <c r="H266" s="14"/>
       <c r="I266" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J266" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K266" s="16"/>
@@ -8387,11 +8414,11 @@
       <c r="G267" s="14"/>
       <c r="H267" s="14"/>
       <c r="I267" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J267" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K267" s="16"/>
@@ -8409,11 +8436,11 @@
       <c r="G268" s="14"/>
       <c r="H268" s="14"/>
       <c r="I268" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J268" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K268" s="16"/>
@@ -8431,11 +8458,11 @@
       <c r="G269" s="14"/>
       <c r="H269" s="14"/>
       <c r="I269" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J269" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K269" s="16"/>
@@ -8453,11 +8480,11 @@
       <c r="G270" s="14"/>
       <c r="H270" s="14"/>
       <c r="I270" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J270" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K270" s="16"/>
@@ -8475,11 +8502,11 @@
       <c r="G271" s="14"/>
       <c r="H271" s="14"/>
       <c r="I271" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J271" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K271" s="16"/>
@@ -8497,11 +8524,11 @@
       <c r="G272" s="14"/>
       <c r="H272" s="14"/>
       <c r="I272" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J272" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K272" s="16"/>
@@ -8519,11 +8546,11 @@
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
       <c r="I273" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J273" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K273" s="16"/>
@@ -8541,11 +8568,11 @@
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
       <c r="I274" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J274" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K274" s="16"/>
@@ -8563,11 +8590,11 @@
       <c r="G275" s="14"/>
       <c r="H275" s="14"/>
       <c r="I275" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J275" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K275" s="16"/>
@@ -8585,11 +8612,11 @@
       <c r="G276" s="14"/>
       <c r="H276" s="14"/>
       <c r="I276" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J276" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K276" s="16"/>
@@ -8607,11 +8634,11 @@
       <c r="G277" s="14"/>
       <c r="H277" s="14"/>
       <c r="I277" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J277" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K277" s="16"/>
@@ -8629,11 +8656,11 @@
       <c r="G278" s="14"/>
       <c r="H278" s="14"/>
       <c r="I278" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J278" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K278" s="16"/>
@@ -8651,11 +8678,11 @@
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
       <c r="I279" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J279" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K279" s="16"/>
@@ -8673,11 +8700,11 @@
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
       <c r="I280" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J280" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K280" s="16"/>
@@ -8695,11 +8722,11 @@
       <c r="G281" s="14"/>
       <c r="H281" s="14"/>
       <c r="I281" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J281" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K281" s="16"/>
@@ -8717,11 +8744,11 @@
       <c r="G282" s="14"/>
       <c r="H282" s="14"/>
       <c r="I282" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J282" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K282" s="16"/>
@@ -8739,11 +8766,11 @@
       <c r="G283" s="14"/>
       <c r="H283" s="14"/>
       <c r="I283" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J283" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K283" s="16"/>
@@ -8761,11 +8788,11 @@
       <c r="G284" s="14"/>
       <c r="H284" s="14"/>
       <c r="I284" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J284" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K284" s="16"/>
@@ -8783,11 +8810,11 @@
       <c r="G285" s="14"/>
       <c r="H285" s="14"/>
       <c r="I285" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J285" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K285" s="16"/>
@@ -8805,11 +8832,11 @@
       <c r="G286" s="14"/>
       <c r="H286" s="14"/>
       <c r="I286" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J286" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K286" s="16"/>
@@ -8827,11 +8854,11 @@
       <c r="G287" s="14"/>
       <c r="H287" s="14"/>
       <c r="I287" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J287" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K287" s="16"/>
@@ -8849,11 +8876,11 @@
       <c r="G288" s="14"/>
       <c r="H288" s="14"/>
       <c r="I288" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J288" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K288" s="16"/>
@@ -8871,11 +8898,11 @@
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
       <c r="I289" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J289" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K289" s="16"/>
@@ -8893,11 +8920,11 @@
       <c r="G290" s="14"/>
       <c r="H290" s="14"/>
       <c r="I290" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J290" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K290" s="16"/>
@@ -8915,11 +8942,11 @@
       <c r="G291" s="14"/>
       <c r="H291" s="14"/>
       <c r="I291" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J291" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K291" s="16"/>
@@ -8937,11 +8964,11 @@
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
       <c r="I292" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J292" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K292" s="16"/>
@@ -8959,11 +8986,11 @@
       <c r="G293" s="14"/>
       <c r="H293" s="14"/>
       <c r="I293" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J293" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K293" s="16"/>
@@ -8981,11 +9008,11 @@
       <c r="G294" s="14"/>
       <c r="H294" s="14"/>
       <c r="I294" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J294" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K294" s="16"/>
@@ -9003,11 +9030,11 @@
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
       <c r="I295" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J295" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K295" s="16"/>
@@ -9025,11 +9052,11 @@
       <c r="G296" s="14"/>
       <c r="H296" s="14"/>
       <c r="I296" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J296" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K296" s="16"/>
@@ -9047,11 +9074,11 @@
       <c r="G297" s="14"/>
       <c r="H297" s="14"/>
       <c r="I297" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J297" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K297" s="16"/>
@@ -9069,11 +9096,11 @@
       <c r="G298" s="14"/>
       <c r="H298" s="14"/>
       <c r="I298" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J298" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K298" s="16"/>
@@ -9091,11 +9118,11 @@
       <c r="G299" s="14"/>
       <c r="H299" s="14"/>
       <c r="I299" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J299" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K299" s="16"/>
@@ -9113,11 +9140,11 @@
       <c r="G300" s="14"/>
       <c r="H300" s="14"/>
       <c r="I300" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J300" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K300" s="16"/>
@@ -9135,11 +9162,11 @@
       <c r="G301" s="14"/>
       <c r="H301" s="14"/>
       <c r="I301" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J301" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K301" s="16"/>
@@ -9157,11 +9184,11 @@
       <c r="G302" s="14"/>
       <c r="H302" s="14"/>
       <c r="I302" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J302" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K302" s="16"/>
@@ -9179,11 +9206,11 @@
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
       <c r="I303" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J303" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K303" s="16"/>
@@ -9201,11 +9228,11 @@
       <c r="G304" s="14"/>
       <c r="H304" s="14"/>
       <c r="I304" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J304" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K304" s="16"/>
@@ -9223,11 +9250,11 @@
       <c r="G305" s="14"/>
       <c r="H305" s="14"/>
       <c r="I305" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J305" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K305" s="16"/>
@@ -9245,11 +9272,11 @@
       <c r="G306" s="14"/>
       <c r="H306" s="14"/>
       <c r="I306" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J306" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K306" s="16"/>
@@ -9267,11 +9294,11 @@
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
       <c r="I307" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J307" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K307" s="16"/>
@@ -9289,11 +9316,11 @@
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
       <c r="I308" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J308" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K308" s="16"/>
@@ -9311,11 +9338,11 @@
       <c r="G309" s="14"/>
       <c r="H309" s="14"/>
       <c r="I309" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J309" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K309" s="16"/>
@@ -9333,11 +9360,11 @@
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
       <c r="I310" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J310" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K310" s="16"/>
@@ -9355,11 +9382,11 @@
       <c r="G311" s="14"/>
       <c r="H311" s="14"/>
       <c r="I311" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J311" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K311" s="16"/>
@@ -9377,11 +9404,11 @@
       <c r="G312" s="14"/>
       <c r="H312" s="14"/>
       <c r="I312" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J312" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K312" s="16"/>
@@ -9399,11 +9426,11 @@
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
       <c r="I313" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J313" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K313" s="16"/>
@@ -9421,11 +9448,11 @@
       <c r="G314" s="14"/>
       <c r="H314" s="14"/>
       <c r="I314" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J314" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K314" s="16"/>
@@ -9443,11 +9470,11 @@
       <c r="G315" s="14"/>
       <c r="H315" s="14"/>
       <c r="I315" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J315" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K315" s="16"/>
@@ -9465,11 +9492,11 @@
       <c r="G316" s="14"/>
       <c r="H316" s="14"/>
       <c r="I316" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J316" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K316" s="16"/>
@@ -9487,11 +9514,11 @@
       <c r="G317" s="14"/>
       <c r="H317" s="14"/>
       <c r="I317" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J317" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K317" s="16"/>
@@ -9509,11 +9536,11 @@
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
       <c r="I318" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J318" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K318" s="16"/>
@@ -9531,11 +9558,11 @@
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
       <c r="I319" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J319" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K319" s="16"/>
@@ -9553,11 +9580,11 @@
       <c r="G320" s="14"/>
       <c r="H320" s="14"/>
       <c r="I320" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J320" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K320" s="16"/>
@@ -9575,11 +9602,11 @@
       <c r="G321" s="14"/>
       <c r="H321" s="14"/>
       <c r="I321" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J321" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K321" s="16"/>
@@ -9597,11 +9624,11 @@
       <c r="G322" s="14"/>
       <c r="H322" s="14"/>
       <c r="I322" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J322" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K322" s="16"/>
@@ -9619,11 +9646,11 @@
       <c r="G323" s="14"/>
       <c r="H323" s="14"/>
       <c r="I323" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J323" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K323" s="16"/>
@@ -9641,11 +9668,11 @@
       <c r="G324" s="14"/>
       <c r="H324" s="14"/>
       <c r="I324" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J324" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K324" s="16"/>
@@ -9663,11 +9690,11 @@
       <c r="G325" s="14"/>
       <c r="H325" s="14"/>
       <c r="I325" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J325" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K325" s="16"/>
@@ -9685,11 +9712,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="26">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" ref="I326:I389" si="28">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="27">IF(I326="","",1440-I326)</f>
+        <f t="shared" ref="J326:J389" si="29">IF(I326="","",1440-I326)</f>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -9707,11 +9734,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -9729,11 +9756,11 @@
       <c r="G328" s="14"/>
       <c r="H328" s="14"/>
       <c r="I328" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J328" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K328" s="16"/>
@@ -9751,11 +9778,11 @@
       <c r="G329" s="14"/>
       <c r="H329" s="14"/>
       <c r="I329" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J329" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K329" s="16"/>
@@ -9773,11 +9800,11 @@
       <c r="G330" s="14"/>
       <c r="H330" s="14"/>
       <c r="I330" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J330" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K330" s="16"/>
@@ -9795,11 +9822,11 @@
       <c r="G331" s="14"/>
       <c r="H331" s="14"/>
       <c r="I331" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J331" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K331" s="16"/>
@@ -9817,11 +9844,11 @@
       <c r="G332" s="14"/>
       <c r="H332" s="14"/>
       <c r="I332" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J332" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K332" s="16"/>
@@ -9839,11 +9866,11 @@
       <c r="G333" s="14"/>
       <c r="H333" s="14"/>
       <c r="I333" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J333" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K333" s="16"/>
@@ -9861,11 +9888,11 @@
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
       <c r="I334" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J334" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K334" s="16"/>
@@ -9883,11 +9910,11 @@
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
       <c r="I335" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J335" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K335" s="16"/>
@@ -9905,11 +9932,11 @@
       <c r="G336" s="14"/>
       <c r="H336" s="14"/>
       <c r="I336" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J336" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K336" s="16"/>
@@ -9927,11 +9954,11 @@
       <c r="G337" s="14"/>
       <c r="H337" s="14"/>
       <c r="I337" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J337" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K337" s="16"/>
@@ -9949,11 +9976,11 @@
       <c r="G338" s="14"/>
       <c r="H338" s="14"/>
       <c r="I338" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J338" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K338" s="16"/>
@@ -9971,11 +9998,11 @@
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
       <c r="I339" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J339" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K339" s="16"/>
@@ -9993,11 +10020,11 @@
       <c r="G340" s="14"/>
       <c r="H340" s="14"/>
       <c r="I340" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J340" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K340" s="16"/>
@@ -10015,11 +10042,11 @@
       <c r="G341" s="14"/>
       <c r="H341" s="14"/>
       <c r="I341" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J341" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K341" s="16"/>
@@ -10037,11 +10064,11 @@
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
       <c r="I342" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J342" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K342" s="16"/>
@@ -10059,11 +10086,11 @@
       <c r="G343" s="14"/>
       <c r="H343" s="14"/>
       <c r="I343" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J343" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K343" s="16"/>
@@ -10081,11 +10108,11 @@
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
       <c r="I344" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J344" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K344" s="16"/>
@@ -10103,11 +10130,11 @@
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
       <c r="I345" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J345" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K345" s="16"/>
@@ -10125,11 +10152,11 @@
       <c r="G346" s="14"/>
       <c r="H346" s="14"/>
       <c r="I346" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J346" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K346" s="16"/>
@@ -10147,11 +10174,11 @@
       <c r="G347" s="14"/>
       <c r="H347" s="14"/>
       <c r="I347" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J347" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K347" s="16"/>
@@ -10169,11 +10196,11 @@
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
       <c r="I348" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J348" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K348" s="16"/>
@@ -10191,11 +10218,11 @@
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
       <c r="I349" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J349" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K349" s="16"/>
@@ -10213,11 +10240,11 @@
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
       <c r="I350" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J350" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K350" s="16"/>
@@ -10235,11 +10262,11 @@
       <c r="G351" s="14"/>
       <c r="H351" s="14"/>
       <c r="I351" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J351" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K351" s="16"/>
@@ -10257,11 +10284,11 @@
       <c r="G352" s="14"/>
       <c r="H352" s="14"/>
       <c r="I352" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J352" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K352" s="16"/>
@@ -10279,11 +10306,11 @@
       <c r="G353" s="14"/>
       <c r="H353" s="14"/>
       <c r="I353" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J353" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K353" s="16"/>
@@ -10301,11 +10328,11 @@
       <c r="G354" s="14"/>
       <c r="H354" s="14"/>
       <c r="I354" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J354" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K354" s="16"/>
@@ -10323,11 +10350,11 @@
       <c r="G355" s="14"/>
       <c r="H355" s="14"/>
       <c r="I355" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J355" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K355" s="16"/>
@@ -10345,11 +10372,11 @@
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
       <c r="I356" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J356" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K356" s="16"/>
@@ -10367,11 +10394,11 @@
       <c r="G357" s="14"/>
       <c r="H357" s="14"/>
       <c r="I357" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J357" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K357" s="16"/>
@@ -10389,11 +10416,11 @@
       <c r="G358" s="14"/>
       <c r="H358" s="14"/>
       <c r="I358" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J358" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K358" s="16"/>
@@ -10411,11 +10438,11 @@
       <c r="G359" s="14"/>
       <c r="H359" s="14"/>
       <c r="I359" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J359" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K359" s="16"/>
@@ -10433,11 +10460,11 @@
       <c r="G360" s="14"/>
       <c r="H360" s="14"/>
       <c r="I360" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J360" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K360" s="16"/>
@@ -10455,11 +10482,11 @@
       <c r="G361" s="14"/>
       <c r="H361" s="14"/>
       <c r="I361" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J361" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K361" s="16"/>
@@ -10477,11 +10504,11 @@
       <c r="G362" s="14"/>
       <c r="H362" s="14"/>
       <c r="I362" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J362" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K362" s="16"/>
@@ -10499,11 +10526,11 @@
       <c r="G363" s="14"/>
       <c r="H363" s="14"/>
       <c r="I363" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J363" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K363" s="16"/>
@@ -10521,11 +10548,11 @@
       <c r="G364" s="14"/>
       <c r="H364" s="14"/>
       <c r="I364" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J364" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K364" s="16"/>
@@ -10543,11 +10570,11 @@
       <c r="G365" s="14"/>
       <c r="H365" s="14"/>
       <c r="I365" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J365" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K365" s="16"/>
@@ -10565,11 +10592,11 @@
       <c r="G366" s="14"/>
       <c r="H366" s="14"/>
       <c r="I366" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J366" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K366" s="16"/>
@@ -10587,11 +10614,11 @@
       <c r="G367" s="14"/>
       <c r="H367" s="14"/>
       <c r="I367" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J367" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K367" s="16"/>
@@ -10609,11 +10636,11 @@
       <c r="G368" s="14"/>
       <c r="H368" s="14"/>
       <c r="I368" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J368" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K368" s="16"/>
@@ -10631,11 +10658,11 @@
       <c r="G369" s="14"/>
       <c r="H369" s="14"/>
       <c r="I369" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J369" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K369" s="16"/>
@@ -10653,11 +10680,11 @@
       <c r="G370" s="14"/>
       <c r="H370" s="14"/>
       <c r="I370" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J370" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K370" s="16"/>
@@ -10675,11 +10702,11 @@
       <c r="G371" s="14"/>
       <c r="H371" s="14"/>
       <c r="I371" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J371" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K371" s="16"/>
@@ -10697,11 +10724,11 @@
       <c r="G372" s="14"/>
       <c r="H372" s="14"/>
       <c r="I372" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J372" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K372" s="16"/>
@@ -10719,11 +10746,11 @@
       <c r="G373" s="14"/>
       <c r="H373" s="14"/>
       <c r="I373" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J373" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K373" s="16"/>
@@ -10741,11 +10768,11 @@
       <c r="G374" s="14"/>
       <c r="H374" s="14"/>
       <c r="I374" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J374" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K374" s="16"/>
@@ -10763,11 +10790,11 @@
       <c r="G375" s="14"/>
       <c r="H375" s="14"/>
       <c r="I375" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J375" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K375" s="16"/>
@@ -10785,11 +10812,11 @@
       <c r="G376" s="14"/>
       <c r="H376" s="14"/>
       <c r="I376" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J376" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K376" s="16"/>
@@ -10807,11 +10834,11 @@
       <c r="G377" s="14"/>
       <c r="H377" s="14"/>
       <c r="I377" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J377" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K377" s="16"/>
@@ -10829,11 +10856,11 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K378" s="16"/>
@@ -10851,11 +10878,11 @@
       <c r="G379" s="14"/>
       <c r="H379" s="14"/>
       <c r="I379" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J379" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K379" s="16"/>
@@ -10873,11 +10900,11 @@
       <c r="G380" s="14"/>
       <c r="H380" s="14"/>
       <c r="I380" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J380" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K380" s="16"/>
@@ -10895,11 +10922,11 @@
       <c r="G381" s="14"/>
       <c r="H381" s="14"/>
       <c r="I381" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J381" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K381" s="16"/>
@@ -10917,11 +10944,11 @@
       <c r="G382" s="14"/>
       <c r="H382" s="14"/>
       <c r="I382" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J382" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K382" s="16"/>
@@ -10939,11 +10966,11 @@
       <c r="G383" s="14"/>
       <c r="H383" s="14"/>
       <c r="I383" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J383" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K383" s="16"/>
@@ -10961,11 +10988,11 @@
       <c r="G384" s="14"/>
       <c r="H384" s="14"/>
       <c r="I384" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J384" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K384" s="16"/>
@@ -10983,11 +11010,11 @@
       <c r="G385" s="14"/>
       <c r="H385" s="14"/>
       <c r="I385" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J385" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K385" s="16"/>
@@ -11005,11 +11032,11 @@
       <c r="G386" s="14"/>
       <c r="H386" s="14"/>
       <c r="I386" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J386" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K386" s="16"/>
@@ -11027,11 +11054,11 @@
       <c r="G387" s="14"/>
       <c r="H387" s="14"/>
       <c r="I387" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J387" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K387" s="16"/>
@@ -11049,11 +11076,11 @@
       <c r="G388" s="14"/>
       <c r="H388" s="14"/>
       <c r="I388" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J388" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K388" s="16"/>
@@ -11071,11 +11098,11 @@
       <c r="G389" s="14"/>
       <c r="H389" s="14"/>
       <c r="I389" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J389" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K389" s="16"/>
@@ -11093,11 +11120,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="28">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="30">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="29">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="31">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -11115,11 +11142,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -11137,11 +11164,11 @@
       <c r="G392" s="14"/>
       <c r="H392" s="14"/>
       <c r="I392" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J392" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K392" s="16"/>
@@ -11159,11 +11186,11 @@
       <c r="G393" s="14"/>
       <c r="H393" s="14"/>
       <c r="I393" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J393" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K393" s="16"/>
@@ -11181,11 +11208,11 @@
       <c r="G394" s="14"/>
       <c r="H394" s="14"/>
       <c r="I394" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J394" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K394" s="16"/>
@@ -11203,11 +11230,11 @@
       <c r="G395" s="14"/>
       <c r="H395" s="14"/>
       <c r="I395" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J395" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K395" s="16"/>
@@ -11225,11 +11252,11 @@
       <c r="G396" s="14"/>
       <c r="H396" s="14"/>
       <c r="I396" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J396" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K396" s="16"/>
@@ -11247,11 +11274,11 @@
       <c r="G397" s="14"/>
       <c r="H397" s="14"/>
       <c r="I397" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J397" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K397" s="16"/>
@@ -11269,11 +11296,11 @@
       <c r="G398" s="14"/>
       <c r="H398" s="14"/>
       <c r="I398" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J398" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K398" s="16"/>
@@ -11291,11 +11318,11 @@
       <c r="G399" s="14"/>
       <c r="H399" s="14"/>
       <c r="I399" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J399" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K399" s="16"/>
@@ -11313,11 +11340,11 @@
       <c r="G400" s="14"/>
       <c r="H400" s="14"/>
       <c r="I400" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J400" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K400" s="16"/>
@@ -11335,11 +11362,11 @@
       <c r="G401" s="14"/>
       <c r="H401" s="14"/>
       <c r="I401" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J401" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K401" s="16"/>

</xml_diff>

<commit_message>
File Updated On 22/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{864E045D-DA0E-4C1D-B48A-49240020AC42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2AF8E4D-CF94-4DD1-9D46-949D51706584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="612" yWindow="-108" windowWidth="22536" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="93">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -311,6 +311,9 @@
   </si>
   <si>
     <t>Tired because of classes</t>
+  </si>
+  <si>
+    <t>Only 2 classes were there today</t>
   </si>
 </sst>
 </file>
@@ -1198,11 +1201,11 @@
         <v>120</v>
       </c>
       <c r="I7" s="15">
-        <f t="shared" ref="I7:I69" si="0">IF(SUM(B7:F7,H7)=0,"",SUM(B7:F7,H7))</f>
+        <f t="shared" ref="I7:I61" si="0">IF(SUM(B7:F7,H7)=0,"",SUM(B7:F7,H7))</f>
         <v>830</v>
       </c>
       <c r="J7" s="15">
-        <f t="shared" ref="J7:J69" si="1">IF(I7="","",1440-I7)</f>
+        <f t="shared" ref="J7:J61" si="1">IF(I7="","",1440-I7)</f>
         <v>610</v>
       </c>
       <c r="K7" s="16" t="s">
@@ -4071,26 +4074,50 @@
       </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A70" s="13"/>
-      <c r="B70" s="14"/>
-      <c r="C70" s="14"/>
-      <c r="D70" s="14"/>
-      <c r="E70" s="14"/>
-      <c r="F70" s="14"/>
-      <c r="G70" s="14"/>
-      <c r="H70" s="14"/>
-      <c r="I70" s="15" t="str">
-        <f t="shared" ref="I70:I133" si="20">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
-        <v/>
-      </c>
-      <c r="J70" s="15" t="str">
-        <f t="shared" ref="J70:J133" si="21">IF(I70="","",1440-I70)</f>
-        <v/>
-      </c>
-      <c r="K70" s="16"/>
-      <c r="L70" s="16"/>
-      <c r="M70" s="16"/>
-      <c r="N70" s="17"/>
+      <c r="A70" s="13">
+        <v>46317</v>
+      </c>
+      <c r="B70" s="14">
+        <v>420</v>
+      </c>
+      <c r="C70" s="14">
+        <v>0</v>
+      </c>
+      <c r="D70" s="14">
+        <v>0</v>
+      </c>
+      <c r="E70" s="14">
+        <v>120</v>
+      </c>
+      <c r="F70" s="14">
+        <v>150</v>
+      </c>
+      <c r="G70" s="14">
+        <v>2</v>
+      </c>
+      <c r="H70" s="14">
+        <v>150</v>
+      </c>
+      <c r="I70" s="15">
+        <f t="shared" ref="I70" si="20">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
+        <v>840</v>
+      </c>
+      <c r="J70" s="15">
+        <f t="shared" ref="J70" si="21">IF(I70="","",1440-I70)</f>
+        <v>600</v>
+      </c>
+      <c r="K70" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L70" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M70" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N70" s="17" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71" s="13"/>
@@ -4102,11 +4129,11 @@
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
       <c r="I71" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" ref="I70:I133" si="22">IF(SUM(B71:F71,H71)=0,"",SUM(B71:F71,H71))</f>
         <v/>
       </c>
       <c r="J71" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" ref="J70:J133" si="23">IF(I71="","",1440-I71)</f>
         <v/>
       </c>
       <c r="K71" s="16"/>
@@ -4124,11 +4151,11 @@
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
       <c r="I72" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J72" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K72" s="16"/>
@@ -4146,11 +4173,11 @@
       <c r="G73" s="14"/>
       <c r="H73" s="14"/>
       <c r="I73" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J73" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K73" s="16"/>
@@ -4168,11 +4195,11 @@
       <c r="G74" s="14"/>
       <c r="H74" s="14"/>
       <c r="I74" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J74" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K74" s="16"/>
@@ -4190,11 +4217,11 @@
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
       <c r="I75" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J75" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K75" s="16"/>
@@ -4212,11 +4239,11 @@
       <c r="G76" s="14"/>
       <c r="H76" s="14"/>
       <c r="I76" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J76" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K76" s="16"/>
@@ -4234,11 +4261,11 @@
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
       <c r="I77" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J77" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K77" s="16"/>
@@ -4256,11 +4283,11 @@
       <c r="G78" s="14"/>
       <c r="H78" s="14"/>
       <c r="I78" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J78" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K78" s="16"/>
@@ -4278,11 +4305,11 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J79" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K79" s="16"/>
@@ -4300,11 +4327,11 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J80" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K80" s="16"/>
@@ -4322,11 +4349,11 @@
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J81" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K81" s="16"/>
@@ -4344,11 +4371,11 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J82" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K82" s="16"/>
@@ -4366,11 +4393,11 @@
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
       <c r="I83" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J83" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K83" s="16"/>
@@ -4388,11 +4415,11 @@
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
       <c r="I84" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J84" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K84" s="16"/>
@@ -4410,11 +4437,11 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J85" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K85" s="16"/>
@@ -4432,11 +4459,11 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J86" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K86" s="16"/>
@@ -4454,11 +4481,11 @@
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
       <c r="I87" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J87" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K87" s="16"/>
@@ -4476,11 +4503,11 @@
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
       <c r="I88" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J88" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K88" s="16"/>
@@ -4498,11 +4525,11 @@
       <c r="G89" s="14"/>
       <c r="H89" s="14"/>
       <c r="I89" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J89" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K89" s="16"/>
@@ -4520,11 +4547,11 @@
       <c r="G90" s="14"/>
       <c r="H90" s="14"/>
       <c r="I90" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J90" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K90" s="16"/>
@@ -4542,11 +4569,11 @@
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
       <c r="I91" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J91" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K91" s="16"/>
@@ -4564,11 +4591,11 @@
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
       <c r="I92" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J92" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K92" s="16"/>
@@ -4586,11 +4613,11 @@
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J93" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K93" s="16"/>
@@ -4608,11 +4635,11 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J94" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K94" s="16"/>
@@ -4630,11 +4657,11 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J95" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K95" s="16"/>
@@ -4652,11 +4679,11 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J96" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K96" s="16"/>
@@ -4674,11 +4701,11 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J97" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K97" s="16"/>
@@ -4696,11 +4723,11 @@
       <c r="G98" s="14"/>
       <c r="H98" s="14"/>
       <c r="I98" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J98" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K98" s="16"/>
@@ -4718,11 +4745,11 @@
       <c r="G99" s="14"/>
       <c r="H99" s="14"/>
       <c r="I99" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J99" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K99" s="16"/>
@@ -4740,11 +4767,11 @@
       <c r="G100" s="14"/>
       <c r="H100" s="14"/>
       <c r="I100" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J100" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K100" s="16"/>
@@ -4762,11 +4789,11 @@
       <c r="G101" s="14"/>
       <c r="H101" s="14"/>
       <c r="I101" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J101" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K101" s="16"/>
@@ -4784,11 +4811,11 @@
       <c r="G102" s="14"/>
       <c r="H102" s="14"/>
       <c r="I102" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J102" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K102" s="16"/>
@@ -4806,11 +4833,11 @@
       <c r="G103" s="14"/>
       <c r="H103" s="14"/>
       <c r="I103" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J103" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K103" s="16"/>
@@ -4828,11 +4855,11 @@
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
       <c r="I104" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J104" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K104" s="16"/>
@@ -4850,11 +4877,11 @@
       <c r="G105" s="14"/>
       <c r="H105" s="14"/>
       <c r="I105" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J105" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K105" s="16"/>
@@ -4872,11 +4899,11 @@
       <c r="G106" s="14"/>
       <c r="H106" s="14"/>
       <c r="I106" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J106" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K106" s="16"/>
@@ -4894,11 +4921,11 @@
       <c r="G107" s="14"/>
       <c r="H107" s="14"/>
       <c r="I107" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J107" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K107" s="16"/>
@@ -4916,11 +4943,11 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J108" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K108" s="16"/>
@@ -4938,11 +4965,11 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J109" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K109" s="16"/>
@@ -4960,11 +4987,11 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J110" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K110" s="16"/>
@@ -4982,11 +5009,11 @@
       <c r="G111" s="14"/>
       <c r="H111" s="14"/>
       <c r="I111" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J111" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K111" s="16"/>
@@ -5004,11 +5031,11 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J112" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K112" s="16"/>
@@ -5026,11 +5053,11 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J113" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K113" s="16"/>
@@ -5048,11 +5075,11 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J114" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K114" s="16"/>
@@ -5070,11 +5097,11 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J115" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K115" s="16"/>
@@ -5092,11 +5119,11 @@
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
       <c r="I116" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J116" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K116" s="16"/>
@@ -5114,11 +5141,11 @@
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
       <c r="I117" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J117" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K117" s="16"/>
@@ -5136,11 +5163,11 @@
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
       <c r="I118" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J118" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K118" s="16"/>
@@ -5158,11 +5185,11 @@
       <c r="G119" s="14"/>
       <c r="H119" s="14"/>
       <c r="I119" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J119" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K119" s="16"/>
@@ -5180,11 +5207,11 @@
       <c r="G120" s="14"/>
       <c r="H120" s="14"/>
       <c r="I120" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J120" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K120" s="16"/>
@@ -5202,11 +5229,11 @@
       <c r="G121" s="14"/>
       <c r="H121" s="14"/>
       <c r="I121" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J121" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K121" s="16"/>
@@ -5224,11 +5251,11 @@
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
       <c r="I122" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J122" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K122" s="16"/>
@@ -5246,11 +5273,11 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J123" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K123" s="16"/>
@@ -5268,11 +5295,11 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J124" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K124" s="16"/>
@@ -5290,11 +5317,11 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J125" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K125" s="16"/>
@@ -5312,11 +5339,11 @@
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
       <c r="I126" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J126" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K126" s="16"/>
@@ -5334,11 +5361,11 @@
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J127" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K127" s="16"/>
@@ -5356,11 +5383,11 @@
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
       <c r="I128" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J128" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K128" s="16"/>
@@ -5378,11 +5405,11 @@
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
       <c r="I129" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J129" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K129" s="16"/>
@@ -5400,11 +5427,11 @@
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
       <c r="I130" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J130" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K130" s="16"/>
@@ -5422,11 +5449,11 @@
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
       <c r="I131" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J131" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K131" s="16"/>
@@ -5444,11 +5471,11 @@
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
       <c r="I132" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J132" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K132" s="16"/>
@@ -5466,11 +5493,11 @@
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
       <c r="I133" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="J133" s="15" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="K133" s="16"/>
@@ -5488,11 +5515,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="22">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" ref="I134:I197" si="24">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="23">IF(I134="","",1440-I134)</f>
+        <f t="shared" ref="J134:J197" si="25">IF(I134="","",1440-I134)</f>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -5510,11 +5537,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5532,11 +5559,11 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J136" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K136" s="16"/>
@@ -5554,11 +5581,11 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J137" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K137" s="16"/>
@@ -5576,11 +5603,11 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J138" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K138" s="16"/>
@@ -5598,11 +5625,11 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J139" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K139" s="16"/>
@@ -5620,11 +5647,11 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J140" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K140" s="16"/>
@@ -5642,11 +5669,11 @@
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J141" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K141" s="16"/>
@@ -5664,11 +5691,11 @@
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J142" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K142" s="16"/>
@@ -5686,11 +5713,11 @@
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J143" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K143" s="16"/>
@@ -5708,11 +5735,11 @@
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J144" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K144" s="16"/>
@@ -5730,11 +5757,11 @@
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J145" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K145" s="16"/>
@@ -5752,11 +5779,11 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J146" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K146" s="16"/>
@@ -5774,11 +5801,11 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J147" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K147" s="16"/>
@@ -5796,11 +5823,11 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J148" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K148" s="16"/>
@@ -5818,11 +5845,11 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J149" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K149" s="16"/>
@@ -5840,11 +5867,11 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J150" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K150" s="16"/>
@@ -5862,11 +5889,11 @@
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
       <c r="I151" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J151" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K151" s="16"/>
@@ -5884,11 +5911,11 @@
       <c r="G152" s="14"/>
       <c r="H152" s="14"/>
       <c r="I152" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J152" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K152" s="16"/>
@@ -5906,11 +5933,11 @@
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J153" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K153" s="16"/>
@@ -5928,11 +5955,11 @@
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J154" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K154" s="16"/>
@@ -5950,11 +5977,11 @@
       <c r="G155" s="14"/>
       <c r="H155" s="14"/>
       <c r="I155" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J155" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K155" s="16"/>
@@ -5972,11 +5999,11 @@
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
       <c r="I156" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J156" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K156" s="16"/>
@@ -5994,11 +6021,11 @@
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J157" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K157" s="16"/>
@@ -6016,11 +6043,11 @@
       <c r="G158" s="14"/>
       <c r="H158" s="14"/>
       <c r="I158" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J158" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K158" s="16"/>
@@ -6038,11 +6065,11 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J159" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K159" s="16"/>
@@ -6060,11 +6087,11 @@
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
       <c r="I160" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J160" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K160" s="16"/>
@@ -6082,11 +6109,11 @@
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
       <c r="I161" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J161" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K161" s="16"/>
@@ -6104,11 +6131,11 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J162" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K162" s="16"/>
@@ -6126,11 +6153,11 @@
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
       <c r="I163" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J163" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K163" s="16"/>
@@ -6148,11 +6175,11 @@
       <c r="G164" s="14"/>
       <c r="H164" s="14"/>
       <c r="I164" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J164" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K164" s="16"/>
@@ -6170,11 +6197,11 @@
       <c r="G165" s="14"/>
       <c r="H165" s="14"/>
       <c r="I165" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J165" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K165" s="16"/>
@@ -6192,11 +6219,11 @@
       <c r="G166" s="14"/>
       <c r="H166" s="14"/>
       <c r="I166" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J166" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K166" s="16"/>
@@ -6214,11 +6241,11 @@
       <c r="G167" s="14"/>
       <c r="H167" s="14"/>
       <c r="I167" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J167" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K167" s="16"/>
@@ -6236,11 +6263,11 @@
       <c r="G168" s="14"/>
       <c r="H168" s="14"/>
       <c r="I168" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J168" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K168" s="16"/>
@@ -6258,11 +6285,11 @@
       <c r="G169" s="14"/>
       <c r="H169" s="14"/>
       <c r="I169" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J169" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K169" s="16"/>
@@ -6280,11 +6307,11 @@
       <c r="G170" s="14"/>
       <c r="H170" s="14"/>
       <c r="I170" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J170" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K170" s="16"/>
@@ -6302,11 +6329,11 @@
       <c r="G171" s="14"/>
       <c r="H171" s="14"/>
       <c r="I171" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J171" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K171" s="16"/>
@@ -6324,11 +6351,11 @@
       <c r="G172" s="14"/>
       <c r="H172" s="14"/>
       <c r="I172" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J172" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K172" s="16"/>
@@ -6346,11 +6373,11 @@
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
       <c r="I173" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J173" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K173" s="16"/>
@@ -6368,11 +6395,11 @@
       <c r="G174" s="14"/>
       <c r="H174" s="14"/>
       <c r="I174" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J174" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K174" s="16"/>
@@ -6390,11 +6417,11 @@
       <c r="G175" s="14"/>
       <c r="H175" s="14"/>
       <c r="I175" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J175" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K175" s="16"/>
@@ -6412,11 +6439,11 @@
       <c r="G176" s="14"/>
       <c r="H176" s="14"/>
       <c r="I176" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J176" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K176" s="16"/>
@@ -6434,11 +6461,11 @@
       <c r="G177" s="14"/>
       <c r="H177" s="14"/>
       <c r="I177" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J177" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K177" s="16"/>
@@ -6456,11 +6483,11 @@
       <c r="G178" s="14"/>
       <c r="H178" s="14"/>
       <c r="I178" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J178" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K178" s="16"/>
@@ -6478,11 +6505,11 @@
       <c r="G179" s="14"/>
       <c r="H179" s="14"/>
       <c r="I179" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J179" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K179" s="16"/>
@@ -6500,11 +6527,11 @@
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
       <c r="I180" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J180" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K180" s="16"/>
@@ -6522,11 +6549,11 @@
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J181" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K181" s="16"/>
@@ -6544,11 +6571,11 @@
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J182" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K182" s="16"/>
@@ -6566,11 +6593,11 @@
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J183" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K183" s="16"/>
@@ -6588,11 +6615,11 @@
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
       <c r="I184" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J184" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K184" s="16"/>
@@ -6610,11 +6637,11 @@
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
       <c r="I185" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J185" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K185" s="16"/>
@@ -6632,11 +6659,11 @@
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J186" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K186" s="16"/>
@@ -6654,11 +6681,11 @@
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J187" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K187" s="16"/>
@@ -6676,11 +6703,11 @@
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
       <c r="I188" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J188" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K188" s="16"/>
@@ -6698,11 +6725,11 @@
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
       <c r="I189" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J189" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K189" s="16"/>
@@ -6720,11 +6747,11 @@
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J190" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K190" s="16"/>
@@ -6742,11 +6769,11 @@
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J191" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K191" s="16"/>
@@ -6764,11 +6791,11 @@
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J192" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K192" s="16"/>
@@ -6786,11 +6813,11 @@
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
       <c r="I193" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J193" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K193" s="16"/>
@@ -6808,11 +6835,11 @@
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
       <c r="I194" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J194" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K194" s="16"/>
@@ -6830,11 +6857,11 @@
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J195" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K195" s="16"/>
@@ -6852,11 +6879,11 @@
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J196" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K196" s="16"/>
@@ -6874,11 +6901,11 @@
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J197" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K197" s="16"/>
@@ -6896,11 +6923,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="24">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" ref="I198:I261" si="26">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="25">IF(I198="","",1440-I198)</f>
+        <f t="shared" ref="J198:J261" si="27">IF(I198="","",1440-I198)</f>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -6918,11 +6945,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -6940,11 +6967,11 @@
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J200" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K200" s="16"/>
@@ -6962,11 +6989,11 @@
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
       <c r="I201" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J201" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K201" s="16"/>
@@ -6984,11 +7011,11 @@
       <c r="G202" s="14"/>
       <c r="H202" s="14"/>
       <c r="I202" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J202" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K202" s="16"/>
@@ -7006,11 +7033,11 @@
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
       <c r="I203" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J203" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K203" s="16"/>
@@ -7028,11 +7055,11 @@
       <c r="G204" s="14"/>
       <c r="H204" s="14"/>
       <c r="I204" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J204" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K204" s="16"/>
@@ -7050,11 +7077,11 @@
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J205" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K205" s="16"/>
@@ -7072,11 +7099,11 @@
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J206" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K206" s="16"/>
@@ -7094,11 +7121,11 @@
       <c r="G207" s="14"/>
       <c r="H207" s="14"/>
       <c r="I207" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J207" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K207" s="16"/>
@@ -7116,11 +7143,11 @@
       <c r="G208" s="14"/>
       <c r="H208" s="14"/>
       <c r="I208" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J208" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K208" s="16"/>
@@ -7138,11 +7165,11 @@
       <c r="G209" s="14"/>
       <c r="H209" s="14"/>
       <c r="I209" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J209" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K209" s="16"/>
@@ -7160,11 +7187,11 @@
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J210" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K210" s="16"/>
@@ -7182,11 +7209,11 @@
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J211" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K211" s="16"/>
@@ -7204,11 +7231,11 @@
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J212" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K212" s="16"/>
@@ -7226,11 +7253,11 @@
       <c r="G213" s="14"/>
       <c r="H213" s="14"/>
       <c r="I213" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J213" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K213" s="16"/>
@@ -7248,11 +7275,11 @@
       <c r="G214" s="14"/>
       <c r="H214" s="14"/>
       <c r="I214" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J214" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K214" s="16"/>
@@ -7270,11 +7297,11 @@
       <c r="G215" s="14"/>
       <c r="H215" s="14"/>
       <c r="I215" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J215" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K215" s="16"/>
@@ -7292,11 +7319,11 @@
       <c r="G216" s="14"/>
       <c r="H216" s="14"/>
       <c r="I216" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J216" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K216" s="16"/>
@@ -7314,11 +7341,11 @@
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J217" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K217" s="16"/>
@@ -7336,11 +7363,11 @@
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J218" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K218" s="16"/>
@@ -7358,11 +7385,11 @@
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J219" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K219" s="16"/>
@@ -7380,11 +7407,11 @@
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J220" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K220" s="16"/>
@@ -7402,11 +7429,11 @@
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J221" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K221" s="16"/>
@@ -7424,11 +7451,11 @@
       <c r="G222" s="14"/>
       <c r="H222" s="14"/>
       <c r="I222" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J222" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K222" s="16"/>
@@ -7446,11 +7473,11 @@
       <c r="G223" s="14"/>
       <c r="H223" s="14"/>
       <c r="I223" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J223" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K223" s="16"/>
@@ -7468,11 +7495,11 @@
       <c r="G224" s="14"/>
       <c r="H224" s="14"/>
       <c r="I224" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J224" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K224" s="16"/>
@@ -7490,11 +7517,11 @@
       <c r="G225" s="14"/>
       <c r="H225" s="14"/>
       <c r="I225" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J225" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K225" s="16"/>
@@ -7512,11 +7539,11 @@
       <c r="G226" s="14"/>
       <c r="H226" s="14"/>
       <c r="I226" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J226" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K226" s="16"/>
@@ -7534,11 +7561,11 @@
       <c r="G227" s="14"/>
       <c r="H227" s="14"/>
       <c r="I227" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J227" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K227" s="16"/>
@@ -7556,11 +7583,11 @@
       <c r="G228" s="14"/>
       <c r="H228" s="14"/>
       <c r="I228" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J228" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K228" s="16"/>
@@ -7578,11 +7605,11 @@
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J229" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K229" s="16"/>
@@ -7600,11 +7627,11 @@
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J230" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K230" s="16"/>
@@ -7622,11 +7649,11 @@
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
       <c r="I231" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J231" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K231" s="16"/>
@@ -7644,11 +7671,11 @@
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
       <c r="I232" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J232" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K232" s="16"/>
@@ -7666,11 +7693,11 @@
       <c r="G233" s="14"/>
       <c r="H233" s="14"/>
       <c r="I233" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J233" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K233" s="16"/>
@@ -7688,11 +7715,11 @@
       <c r="G234" s="14"/>
       <c r="H234" s="14"/>
       <c r="I234" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J234" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K234" s="16"/>
@@ -7710,11 +7737,11 @@
       <c r="G235" s="14"/>
       <c r="H235" s="14"/>
       <c r="I235" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J235" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K235" s="16"/>
@@ -7732,11 +7759,11 @@
       <c r="G236" s="14"/>
       <c r="H236" s="14"/>
       <c r="I236" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J236" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K236" s="16"/>
@@ -7754,11 +7781,11 @@
       <c r="G237" s="14"/>
       <c r="H237" s="14"/>
       <c r="I237" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J237" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K237" s="16"/>
@@ -7776,11 +7803,11 @@
       <c r="G238" s="14"/>
       <c r="H238" s="14"/>
       <c r="I238" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J238" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K238" s="16"/>
@@ -7798,11 +7825,11 @@
       <c r="G239" s="14"/>
       <c r="H239" s="14"/>
       <c r="I239" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J239" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K239" s="16"/>
@@ -7820,11 +7847,11 @@
       <c r="G240" s="14"/>
       <c r="H240" s="14"/>
       <c r="I240" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J240" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K240" s="16"/>
@@ -7842,11 +7869,11 @@
       <c r="G241" s="14"/>
       <c r="H241" s="14"/>
       <c r="I241" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J241" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K241" s="16"/>
@@ -7864,11 +7891,11 @@
       <c r="G242" s="14"/>
       <c r="H242" s="14"/>
       <c r="I242" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J242" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K242" s="16"/>
@@ -7886,11 +7913,11 @@
       <c r="G243" s="14"/>
       <c r="H243" s="14"/>
       <c r="I243" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J243" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K243" s="16"/>
@@ -7908,11 +7935,11 @@
       <c r="G244" s="14"/>
       <c r="H244" s="14"/>
       <c r="I244" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J244" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K244" s="16"/>
@@ -7930,11 +7957,11 @@
       <c r="G245" s="14"/>
       <c r="H245" s="14"/>
       <c r="I245" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J245" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K245" s="16"/>
@@ -7952,11 +7979,11 @@
       <c r="G246" s="14"/>
       <c r="H246" s="14"/>
       <c r="I246" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J246" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K246" s="16"/>
@@ -7974,11 +8001,11 @@
       <c r="G247" s="14"/>
       <c r="H247" s="14"/>
       <c r="I247" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J247" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K247" s="16"/>
@@ -7996,11 +8023,11 @@
       <c r="G248" s="14"/>
       <c r="H248" s="14"/>
       <c r="I248" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J248" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K248" s="16"/>
@@ -8018,11 +8045,11 @@
       <c r="G249" s="14"/>
       <c r="H249" s="14"/>
       <c r="I249" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J249" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K249" s="16"/>
@@ -8040,11 +8067,11 @@
       <c r="G250" s="14"/>
       <c r="H250" s="14"/>
       <c r="I250" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J250" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K250" s="16"/>
@@ -8062,11 +8089,11 @@
       <c r="G251" s="14"/>
       <c r="H251" s="14"/>
       <c r="I251" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J251" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K251" s="16"/>
@@ -8084,11 +8111,11 @@
       <c r="G252" s="14"/>
       <c r="H252" s="14"/>
       <c r="I252" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J252" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K252" s="16"/>
@@ -8106,11 +8133,11 @@
       <c r="G253" s="14"/>
       <c r="H253" s="14"/>
       <c r="I253" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J253" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K253" s="16"/>
@@ -8128,11 +8155,11 @@
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
       <c r="I254" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J254" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K254" s="16"/>
@@ -8150,11 +8177,11 @@
       <c r="G255" s="14"/>
       <c r="H255" s="14"/>
       <c r="I255" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J255" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K255" s="16"/>
@@ -8172,11 +8199,11 @@
       <c r="G256" s="14"/>
       <c r="H256" s="14"/>
       <c r="I256" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J256" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K256" s="16"/>
@@ -8194,11 +8221,11 @@
       <c r="G257" s="14"/>
       <c r="H257" s="14"/>
       <c r="I257" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J257" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K257" s="16"/>
@@ -8216,11 +8243,11 @@
       <c r="G258" s="14"/>
       <c r="H258" s="14"/>
       <c r="I258" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J258" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K258" s="16"/>
@@ -8238,11 +8265,11 @@
       <c r="G259" s="14"/>
       <c r="H259" s="14"/>
       <c r="I259" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J259" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K259" s="16"/>
@@ -8260,11 +8287,11 @@
       <c r="G260" s="14"/>
       <c r="H260" s="14"/>
       <c r="I260" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J260" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K260" s="16"/>
@@ -8282,11 +8309,11 @@
       <c r="G261" s="14"/>
       <c r="H261" s="14"/>
       <c r="I261" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J261" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K261" s="16"/>
@@ -8304,11 +8331,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="26">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" ref="I262:I325" si="28">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="27">IF(I262="","",1440-I262)</f>
+        <f t="shared" ref="J262:J325" si="29">IF(I262="","",1440-I262)</f>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -8326,11 +8353,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8348,11 +8375,11 @@
       <c r="G264" s="14"/>
       <c r="H264" s="14"/>
       <c r="I264" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J264" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K264" s="16"/>
@@ -8370,11 +8397,11 @@
       <c r="G265" s="14"/>
       <c r="H265" s="14"/>
       <c r="I265" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J265" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K265" s="16"/>
@@ -8392,11 +8419,11 @@
       <c r="G266" s="14"/>
       <c r="H266" s="14"/>
       <c r="I266" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J266" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K266" s="16"/>
@@ -8414,11 +8441,11 @@
       <c r="G267" s="14"/>
       <c r="H267" s="14"/>
       <c r="I267" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J267" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K267" s="16"/>
@@ -8436,11 +8463,11 @@
       <c r="G268" s="14"/>
       <c r="H268" s="14"/>
       <c r="I268" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J268" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K268" s="16"/>
@@ -8458,11 +8485,11 @@
       <c r="G269" s="14"/>
       <c r="H269" s="14"/>
       <c r="I269" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J269" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K269" s="16"/>
@@ -8480,11 +8507,11 @@
       <c r="G270" s="14"/>
       <c r="H270" s="14"/>
       <c r="I270" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J270" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K270" s="16"/>
@@ -8502,11 +8529,11 @@
       <c r="G271" s="14"/>
       <c r="H271" s="14"/>
       <c r="I271" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J271" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K271" s="16"/>
@@ -8524,11 +8551,11 @@
       <c r="G272" s="14"/>
       <c r="H272" s="14"/>
       <c r="I272" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J272" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K272" s="16"/>
@@ -8546,11 +8573,11 @@
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
       <c r="I273" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J273" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K273" s="16"/>
@@ -8568,11 +8595,11 @@
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
       <c r="I274" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J274" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K274" s="16"/>
@@ -8590,11 +8617,11 @@
       <c r="G275" s="14"/>
       <c r="H275" s="14"/>
       <c r="I275" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J275" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K275" s="16"/>
@@ -8612,11 +8639,11 @@
       <c r="G276" s="14"/>
       <c r="H276" s="14"/>
       <c r="I276" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J276" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K276" s="16"/>
@@ -8634,11 +8661,11 @@
       <c r="G277" s="14"/>
       <c r="H277" s="14"/>
       <c r="I277" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J277" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K277" s="16"/>
@@ -8656,11 +8683,11 @@
       <c r="G278" s="14"/>
       <c r="H278" s="14"/>
       <c r="I278" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J278" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K278" s="16"/>
@@ -8678,11 +8705,11 @@
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
       <c r="I279" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J279" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K279" s="16"/>
@@ -8700,11 +8727,11 @@
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
       <c r="I280" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J280" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K280" s="16"/>
@@ -8722,11 +8749,11 @@
       <c r="G281" s="14"/>
       <c r="H281" s="14"/>
       <c r="I281" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J281" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K281" s="16"/>
@@ -8744,11 +8771,11 @@
       <c r="G282" s="14"/>
       <c r="H282" s="14"/>
       <c r="I282" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J282" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K282" s="16"/>
@@ -8766,11 +8793,11 @@
       <c r="G283" s="14"/>
       <c r="H283" s="14"/>
       <c r="I283" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J283" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K283" s="16"/>
@@ -8788,11 +8815,11 @@
       <c r="G284" s="14"/>
       <c r="H284" s="14"/>
       <c r="I284" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J284" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K284" s="16"/>
@@ -8810,11 +8837,11 @@
       <c r="G285" s="14"/>
       <c r="H285" s="14"/>
       <c r="I285" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J285" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K285" s="16"/>
@@ -8832,11 +8859,11 @@
       <c r="G286" s="14"/>
       <c r="H286" s="14"/>
       <c r="I286" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J286" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K286" s="16"/>
@@ -8854,11 +8881,11 @@
       <c r="G287" s="14"/>
       <c r="H287" s="14"/>
       <c r="I287" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J287" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K287" s="16"/>
@@ -8876,11 +8903,11 @@
       <c r="G288" s="14"/>
       <c r="H288" s="14"/>
       <c r="I288" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J288" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K288" s="16"/>
@@ -8898,11 +8925,11 @@
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
       <c r="I289" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J289" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K289" s="16"/>
@@ -8920,11 +8947,11 @@
       <c r="G290" s="14"/>
       <c r="H290" s="14"/>
       <c r="I290" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J290" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K290" s="16"/>
@@ -8942,11 +8969,11 @@
       <c r="G291" s="14"/>
       <c r="H291" s="14"/>
       <c r="I291" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J291" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K291" s="16"/>
@@ -8964,11 +8991,11 @@
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
       <c r="I292" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J292" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K292" s="16"/>
@@ -8986,11 +9013,11 @@
       <c r="G293" s="14"/>
       <c r="H293" s="14"/>
       <c r="I293" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J293" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K293" s="16"/>
@@ -9008,11 +9035,11 @@
       <c r="G294" s="14"/>
       <c r="H294" s="14"/>
       <c r="I294" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J294" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K294" s="16"/>
@@ -9030,11 +9057,11 @@
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
       <c r="I295" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J295" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K295" s="16"/>
@@ -9052,11 +9079,11 @@
       <c r="G296" s="14"/>
       <c r="H296" s="14"/>
       <c r="I296" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J296" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K296" s="16"/>
@@ -9074,11 +9101,11 @@
       <c r="G297" s="14"/>
       <c r="H297" s="14"/>
       <c r="I297" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J297" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K297" s="16"/>
@@ -9096,11 +9123,11 @@
       <c r="G298" s="14"/>
       <c r="H298" s="14"/>
       <c r="I298" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J298" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K298" s="16"/>
@@ -9118,11 +9145,11 @@
       <c r="G299" s="14"/>
       <c r="H299" s="14"/>
       <c r="I299" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J299" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K299" s="16"/>
@@ -9140,11 +9167,11 @@
       <c r="G300" s="14"/>
       <c r="H300" s="14"/>
       <c r="I300" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J300" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K300" s="16"/>
@@ -9162,11 +9189,11 @@
       <c r="G301" s="14"/>
       <c r="H301" s="14"/>
       <c r="I301" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J301" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K301" s="16"/>
@@ -9184,11 +9211,11 @@
       <c r="G302" s="14"/>
       <c r="H302" s="14"/>
       <c r="I302" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J302" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K302" s="16"/>
@@ -9206,11 +9233,11 @@
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
       <c r="I303" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J303" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K303" s="16"/>
@@ -9228,11 +9255,11 @@
       <c r="G304" s="14"/>
       <c r="H304" s="14"/>
       <c r="I304" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J304" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K304" s="16"/>
@@ -9250,11 +9277,11 @@
       <c r="G305" s="14"/>
       <c r="H305" s="14"/>
       <c r="I305" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J305" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K305" s="16"/>
@@ -9272,11 +9299,11 @@
       <c r="G306" s="14"/>
       <c r="H306" s="14"/>
       <c r="I306" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J306" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K306" s="16"/>
@@ -9294,11 +9321,11 @@
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
       <c r="I307" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J307" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K307" s="16"/>
@@ -9316,11 +9343,11 @@
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
       <c r="I308" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J308" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K308" s="16"/>
@@ -9338,11 +9365,11 @@
       <c r="G309" s="14"/>
       <c r="H309" s="14"/>
       <c r="I309" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J309" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K309" s="16"/>
@@ -9360,11 +9387,11 @@
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
       <c r="I310" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J310" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K310" s="16"/>
@@ -9382,11 +9409,11 @@
       <c r="G311" s="14"/>
       <c r="H311" s="14"/>
       <c r="I311" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J311" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K311" s="16"/>
@@ -9404,11 +9431,11 @@
       <c r="G312" s="14"/>
       <c r="H312" s="14"/>
       <c r="I312" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J312" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K312" s="16"/>
@@ -9426,11 +9453,11 @@
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
       <c r="I313" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J313" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K313" s="16"/>
@@ -9448,11 +9475,11 @@
       <c r="G314" s="14"/>
       <c r="H314" s="14"/>
       <c r="I314" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J314" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K314" s="16"/>
@@ -9470,11 +9497,11 @@
       <c r="G315" s="14"/>
       <c r="H315" s="14"/>
       <c r="I315" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J315" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K315" s="16"/>
@@ -9492,11 +9519,11 @@
       <c r="G316" s="14"/>
       <c r="H316" s="14"/>
       <c r="I316" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J316" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K316" s="16"/>
@@ -9514,11 +9541,11 @@
       <c r="G317" s="14"/>
       <c r="H317" s="14"/>
       <c r="I317" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J317" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K317" s="16"/>
@@ -9536,11 +9563,11 @@
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
       <c r="I318" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J318" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K318" s="16"/>
@@ -9558,11 +9585,11 @@
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
       <c r="I319" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J319" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K319" s="16"/>
@@ -9580,11 +9607,11 @@
       <c r="G320" s="14"/>
       <c r="H320" s="14"/>
       <c r="I320" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J320" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K320" s="16"/>
@@ -9602,11 +9629,11 @@
       <c r="G321" s="14"/>
       <c r="H321" s="14"/>
       <c r="I321" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J321" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K321" s="16"/>
@@ -9624,11 +9651,11 @@
       <c r="G322" s="14"/>
       <c r="H322" s="14"/>
       <c r="I322" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J322" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K322" s="16"/>
@@ -9646,11 +9673,11 @@
       <c r="G323" s="14"/>
       <c r="H323" s="14"/>
       <c r="I323" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J323" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K323" s="16"/>
@@ -9668,11 +9695,11 @@
       <c r="G324" s="14"/>
       <c r="H324" s="14"/>
       <c r="I324" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J324" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K324" s="16"/>
@@ -9690,11 +9717,11 @@
       <c r="G325" s="14"/>
       <c r="H325" s="14"/>
       <c r="I325" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J325" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K325" s="16"/>
@@ -9712,11 +9739,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="28">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" ref="I326:I389" si="30">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="29">IF(I326="","",1440-I326)</f>
+        <f t="shared" ref="J326:J389" si="31">IF(I326="","",1440-I326)</f>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -9734,11 +9761,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -9756,11 +9783,11 @@
       <c r="G328" s="14"/>
       <c r="H328" s="14"/>
       <c r="I328" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J328" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K328" s="16"/>
@@ -9778,11 +9805,11 @@
       <c r="G329" s="14"/>
       <c r="H329" s="14"/>
       <c r="I329" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J329" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K329" s="16"/>
@@ -9800,11 +9827,11 @@
       <c r="G330" s="14"/>
       <c r="H330" s="14"/>
       <c r="I330" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J330" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K330" s="16"/>
@@ -9822,11 +9849,11 @@
       <c r="G331" s="14"/>
       <c r="H331" s="14"/>
       <c r="I331" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J331" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K331" s="16"/>
@@ -9844,11 +9871,11 @@
       <c r="G332" s="14"/>
       <c r="H332" s="14"/>
       <c r="I332" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J332" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K332" s="16"/>
@@ -9866,11 +9893,11 @@
       <c r="G333" s="14"/>
       <c r="H333" s="14"/>
       <c r="I333" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J333" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K333" s="16"/>
@@ -9888,11 +9915,11 @@
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
       <c r="I334" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J334" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K334" s="16"/>
@@ -9910,11 +9937,11 @@
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
       <c r="I335" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J335" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K335" s="16"/>
@@ -9932,11 +9959,11 @@
       <c r="G336" s="14"/>
       <c r="H336" s="14"/>
       <c r="I336" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J336" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K336" s="16"/>
@@ -9954,11 +9981,11 @@
       <c r="G337" s="14"/>
       <c r="H337" s="14"/>
       <c r="I337" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J337" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K337" s="16"/>
@@ -9976,11 +10003,11 @@
       <c r="G338" s="14"/>
       <c r="H338" s="14"/>
       <c r="I338" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J338" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K338" s="16"/>
@@ -9998,11 +10025,11 @@
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
       <c r="I339" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J339" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K339" s="16"/>
@@ -10020,11 +10047,11 @@
       <c r="G340" s="14"/>
       <c r="H340" s="14"/>
       <c r="I340" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J340" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K340" s="16"/>
@@ -10042,11 +10069,11 @@
       <c r="G341" s="14"/>
       <c r="H341" s="14"/>
       <c r="I341" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J341" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K341" s="16"/>
@@ -10064,11 +10091,11 @@
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
       <c r="I342" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J342" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K342" s="16"/>
@@ -10086,11 +10113,11 @@
       <c r="G343" s="14"/>
       <c r="H343" s="14"/>
       <c r="I343" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J343" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K343" s="16"/>
@@ -10108,11 +10135,11 @@
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
       <c r="I344" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J344" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K344" s="16"/>
@@ -10130,11 +10157,11 @@
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
       <c r="I345" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J345" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K345" s="16"/>
@@ -10152,11 +10179,11 @@
       <c r="G346" s="14"/>
       <c r="H346" s="14"/>
       <c r="I346" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J346" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K346" s="16"/>
@@ -10174,11 +10201,11 @@
       <c r="G347" s="14"/>
       <c r="H347" s="14"/>
       <c r="I347" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J347" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K347" s="16"/>
@@ -10196,11 +10223,11 @@
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
       <c r="I348" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J348" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K348" s="16"/>
@@ -10218,11 +10245,11 @@
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
       <c r="I349" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J349" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K349" s="16"/>
@@ -10240,11 +10267,11 @@
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
       <c r="I350" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J350" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K350" s="16"/>
@@ -10262,11 +10289,11 @@
       <c r="G351" s="14"/>
       <c r="H351" s="14"/>
       <c r="I351" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J351" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K351" s="16"/>
@@ -10284,11 +10311,11 @@
       <c r="G352" s="14"/>
       <c r="H352" s="14"/>
       <c r="I352" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J352" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K352" s="16"/>
@@ -10306,11 +10333,11 @@
       <c r="G353" s="14"/>
       <c r="H353" s="14"/>
       <c r="I353" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J353" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K353" s="16"/>
@@ -10328,11 +10355,11 @@
       <c r="G354" s="14"/>
       <c r="H354" s="14"/>
       <c r="I354" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J354" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K354" s="16"/>
@@ -10350,11 +10377,11 @@
       <c r="G355" s="14"/>
       <c r="H355" s="14"/>
       <c r="I355" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J355" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K355" s="16"/>
@@ -10372,11 +10399,11 @@
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
       <c r="I356" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J356" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K356" s="16"/>
@@ -10394,11 +10421,11 @@
       <c r="G357" s="14"/>
       <c r="H357" s="14"/>
       <c r="I357" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J357" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K357" s="16"/>
@@ -10416,11 +10443,11 @@
       <c r="G358" s="14"/>
       <c r="H358" s="14"/>
       <c r="I358" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J358" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K358" s="16"/>
@@ -10438,11 +10465,11 @@
       <c r="G359" s="14"/>
       <c r="H359" s="14"/>
       <c r="I359" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J359" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K359" s="16"/>
@@ -10460,11 +10487,11 @@
       <c r="G360" s="14"/>
       <c r="H360" s="14"/>
       <c r="I360" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J360" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K360" s="16"/>
@@ -10482,11 +10509,11 @@
       <c r="G361" s="14"/>
       <c r="H361" s="14"/>
       <c r="I361" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J361" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K361" s="16"/>
@@ -10504,11 +10531,11 @@
       <c r="G362" s="14"/>
       <c r="H362" s="14"/>
       <c r="I362" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J362" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K362" s="16"/>
@@ -10526,11 +10553,11 @@
       <c r="G363" s="14"/>
       <c r="H363" s="14"/>
       <c r="I363" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J363" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K363" s="16"/>
@@ -10548,11 +10575,11 @@
       <c r="G364" s="14"/>
       <c r="H364" s="14"/>
       <c r="I364" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J364" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K364" s="16"/>
@@ -10570,11 +10597,11 @@
       <c r="G365" s="14"/>
       <c r="H365" s="14"/>
       <c r="I365" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J365" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K365" s="16"/>
@@ -10592,11 +10619,11 @@
       <c r="G366" s="14"/>
       <c r="H366" s="14"/>
       <c r="I366" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J366" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K366" s="16"/>
@@ -10614,11 +10641,11 @@
       <c r="G367" s="14"/>
       <c r="H367" s="14"/>
       <c r="I367" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J367" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K367" s="16"/>
@@ -10636,11 +10663,11 @@
       <c r="G368" s="14"/>
       <c r="H368" s="14"/>
       <c r="I368" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J368" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K368" s="16"/>
@@ -10658,11 +10685,11 @@
       <c r="G369" s="14"/>
       <c r="H369" s="14"/>
       <c r="I369" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J369" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K369" s="16"/>
@@ -10680,11 +10707,11 @@
       <c r="G370" s="14"/>
       <c r="H370" s="14"/>
       <c r="I370" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J370" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K370" s="16"/>
@@ -10702,11 +10729,11 @@
       <c r="G371" s="14"/>
       <c r="H371" s="14"/>
       <c r="I371" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J371" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K371" s="16"/>
@@ -10724,11 +10751,11 @@
       <c r="G372" s="14"/>
       <c r="H372" s="14"/>
       <c r="I372" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J372" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K372" s="16"/>
@@ -10746,11 +10773,11 @@
       <c r="G373" s="14"/>
       <c r="H373" s="14"/>
       <c r="I373" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J373" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K373" s="16"/>
@@ -10768,11 +10795,11 @@
       <c r="G374" s="14"/>
       <c r="H374" s="14"/>
       <c r="I374" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J374" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K374" s="16"/>
@@ -10790,11 +10817,11 @@
       <c r="G375" s="14"/>
       <c r="H375" s="14"/>
       <c r="I375" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J375" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K375" s="16"/>
@@ -10812,11 +10839,11 @@
       <c r="G376" s="14"/>
       <c r="H376" s="14"/>
       <c r="I376" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J376" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K376" s="16"/>
@@ -10834,11 +10861,11 @@
       <c r="G377" s="14"/>
       <c r="H377" s="14"/>
       <c r="I377" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J377" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K377" s="16"/>
@@ -10856,11 +10883,11 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K378" s="16"/>
@@ -10878,11 +10905,11 @@
       <c r="G379" s="14"/>
       <c r="H379" s="14"/>
       <c r="I379" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J379" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K379" s="16"/>
@@ -10900,11 +10927,11 @@
       <c r="G380" s="14"/>
       <c r="H380" s="14"/>
       <c r="I380" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J380" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K380" s="16"/>
@@ -10922,11 +10949,11 @@
       <c r="G381" s="14"/>
       <c r="H381" s="14"/>
       <c r="I381" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J381" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K381" s="16"/>
@@ -10944,11 +10971,11 @@
       <c r="G382" s="14"/>
       <c r="H382" s="14"/>
       <c r="I382" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J382" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K382" s="16"/>
@@ -10966,11 +10993,11 @@
       <c r="G383" s="14"/>
       <c r="H383" s="14"/>
       <c r="I383" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J383" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K383" s="16"/>
@@ -10988,11 +11015,11 @@
       <c r="G384" s="14"/>
       <c r="H384" s="14"/>
       <c r="I384" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J384" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K384" s="16"/>
@@ -11010,11 +11037,11 @@
       <c r="G385" s="14"/>
       <c r="H385" s="14"/>
       <c r="I385" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J385" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K385" s="16"/>
@@ -11032,11 +11059,11 @@
       <c r="G386" s="14"/>
       <c r="H386" s="14"/>
       <c r="I386" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J386" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K386" s="16"/>
@@ -11054,11 +11081,11 @@
       <c r="G387" s="14"/>
       <c r="H387" s="14"/>
       <c r="I387" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J387" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K387" s="16"/>
@@ -11076,11 +11103,11 @@
       <c r="G388" s="14"/>
       <c r="H388" s="14"/>
       <c r="I388" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J388" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K388" s="16"/>
@@ -11098,11 +11125,11 @@
       <c r="G389" s="14"/>
       <c r="H389" s="14"/>
       <c r="I389" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J389" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K389" s="16"/>
@@ -11120,11 +11147,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="30">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="32">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="31">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="33">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -11142,11 +11169,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -11164,11 +11191,11 @@
       <c r="G392" s="14"/>
       <c r="H392" s="14"/>
       <c r="I392" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J392" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K392" s="16"/>
@@ -11186,11 +11213,11 @@
       <c r="G393" s="14"/>
       <c r="H393" s="14"/>
       <c r="I393" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J393" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K393" s="16"/>
@@ -11208,11 +11235,11 @@
       <c r="G394" s="14"/>
       <c r="H394" s="14"/>
       <c r="I394" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J394" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K394" s="16"/>
@@ -11230,11 +11257,11 @@
       <c r="G395" s="14"/>
       <c r="H395" s="14"/>
       <c r="I395" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J395" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K395" s="16"/>
@@ -11252,11 +11279,11 @@
       <c r="G396" s="14"/>
       <c r="H396" s="14"/>
       <c r="I396" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J396" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K396" s="16"/>
@@ -11274,11 +11301,11 @@
       <c r="G397" s="14"/>
       <c r="H397" s="14"/>
       <c r="I397" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J397" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K397" s="16"/>
@@ -11296,11 +11323,11 @@
       <c r="G398" s="14"/>
       <c r="H398" s="14"/>
       <c r="I398" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J398" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K398" s="16"/>
@@ -11318,11 +11345,11 @@
       <c r="G399" s="14"/>
       <c r="H399" s="14"/>
       <c r="I399" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J399" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K399" s="16"/>
@@ -11340,11 +11367,11 @@
       <c r="G400" s="14"/>
       <c r="H400" s="14"/>
       <c r="I400" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J400" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K400" s="16"/>
@@ -11362,11 +11389,11 @@
       <c r="G401" s="14"/>
       <c r="H401" s="14"/>
       <c r="I401" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J401" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K401" s="16"/>

</xml_diff>

<commit_message>
File Updated On 23/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2AF8E4D-CF94-4DD1-9D46-949D51706584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A0AAD3F-634D-448C-A7C3-5D99A5BB58F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="612" yWindow="-108" windowWidth="22536" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="94">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -314,6 +314,9 @@
   </si>
   <si>
     <t>Only 2 classes were there today</t>
+  </si>
+  <si>
+    <t>Feeling low</t>
   </si>
 </sst>
 </file>
@@ -4120,26 +4123,50 @@
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A71" s="13"/>
-      <c r="B71" s="14"/>
-      <c r="C71" s="14"/>
-      <c r="D71" s="14"/>
-      <c r="E71" s="14"/>
-      <c r="F71" s="14"/>
-      <c r="G71" s="14"/>
-      <c r="H71" s="14"/>
-      <c r="I71" s="15" t="str">
-        <f t="shared" ref="I70:I133" si="22">IF(SUM(B71:F71,H71)=0,"",SUM(B71:F71,H71))</f>
-        <v/>
-      </c>
-      <c r="J71" s="15" t="str">
-        <f t="shared" ref="J70:J133" si="23">IF(I71="","",1440-I71)</f>
-        <v/>
-      </c>
-      <c r="K71" s="16"/>
-      <c r="L71" s="16"/>
-      <c r="M71" s="16"/>
-      <c r="N71" s="17"/>
+      <c r="A71" s="13">
+        <v>46318</v>
+      </c>
+      <c r="B71" s="14">
+        <v>420</v>
+      </c>
+      <c r="C71" s="14">
+        <v>0</v>
+      </c>
+      <c r="D71" s="14">
+        <v>50</v>
+      </c>
+      <c r="E71" s="14">
+        <v>60</v>
+      </c>
+      <c r="F71" s="14">
+        <v>200</v>
+      </c>
+      <c r="G71" s="14">
+        <v>3</v>
+      </c>
+      <c r="H71" s="14">
+        <v>40</v>
+      </c>
+      <c r="I71" s="15">
+        <f t="shared" ref="I71" si="22">IF(SUM(B71:F71,H71)=0,"",SUM(B71:F71,H71))</f>
+        <v>770</v>
+      </c>
+      <c r="J71" s="15">
+        <f t="shared" ref="J71" si="23">IF(I71="","",1440-I71)</f>
+        <v>670</v>
+      </c>
+      <c r="K71" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L71" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M71" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N71" s="17" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" s="13"/>
@@ -4151,11 +4178,11 @@
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
       <c r="I72" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" ref="I71:I133" si="24">IF(SUM(B72:F72,H72)=0,"",SUM(B72:F72,H72))</f>
         <v/>
       </c>
       <c r="J72" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" ref="J71:J133" si="25">IF(I72="","",1440-I72)</f>
         <v/>
       </c>
       <c r="K72" s="16"/>
@@ -4173,11 +4200,11 @@
       <c r="G73" s="14"/>
       <c r="H73" s="14"/>
       <c r="I73" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J73" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K73" s="16"/>
@@ -4195,11 +4222,11 @@
       <c r="G74" s="14"/>
       <c r="H74" s="14"/>
       <c r="I74" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J74" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K74" s="16"/>
@@ -4217,11 +4244,11 @@
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
       <c r="I75" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J75" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K75" s="16"/>
@@ -4239,11 +4266,11 @@
       <c r="G76" s="14"/>
       <c r="H76" s="14"/>
       <c r="I76" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J76" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K76" s="16"/>
@@ -4261,11 +4288,11 @@
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
       <c r="I77" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J77" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K77" s="16"/>
@@ -4283,11 +4310,11 @@
       <c r="G78" s="14"/>
       <c r="H78" s="14"/>
       <c r="I78" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J78" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K78" s="16"/>
@@ -4305,11 +4332,11 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J79" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K79" s="16"/>
@@ -4327,11 +4354,11 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J80" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K80" s="16"/>
@@ -4349,11 +4376,11 @@
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J81" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K81" s="16"/>
@@ -4371,11 +4398,11 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J82" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K82" s="16"/>
@@ -4393,11 +4420,11 @@
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
       <c r="I83" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J83" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K83" s="16"/>
@@ -4415,11 +4442,11 @@
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
       <c r="I84" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J84" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K84" s="16"/>
@@ -4437,11 +4464,11 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J85" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K85" s="16"/>
@@ -4459,11 +4486,11 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J86" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K86" s="16"/>
@@ -4481,11 +4508,11 @@
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
       <c r="I87" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J87" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K87" s="16"/>
@@ -4503,11 +4530,11 @@
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
       <c r="I88" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J88" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K88" s="16"/>
@@ -4525,11 +4552,11 @@
       <c r="G89" s="14"/>
       <c r="H89" s="14"/>
       <c r="I89" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J89" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K89" s="16"/>
@@ -4547,11 +4574,11 @@
       <c r="G90" s="14"/>
       <c r="H90" s="14"/>
       <c r="I90" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J90" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K90" s="16"/>
@@ -4569,11 +4596,11 @@
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
       <c r="I91" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J91" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K91" s="16"/>
@@ -4591,11 +4618,11 @@
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
       <c r="I92" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J92" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K92" s="16"/>
@@ -4613,11 +4640,11 @@
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J93" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K93" s="16"/>
@@ -4635,11 +4662,11 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J94" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K94" s="16"/>
@@ -4657,11 +4684,11 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J95" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K95" s="16"/>
@@ -4679,11 +4706,11 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J96" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K96" s="16"/>
@@ -4701,11 +4728,11 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J97" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K97" s="16"/>
@@ -4723,11 +4750,11 @@
       <c r="G98" s="14"/>
       <c r="H98" s="14"/>
       <c r="I98" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J98" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K98" s="16"/>
@@ -4745,11 +4772,11 @@
       <c r="G99" s="14"/>
       <c r="H99" s="14"/>
       <c r="I99" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J99" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K99" s="16"/>
@@ -4767,11 +4794,11 @@
       <c r="G100" s="14"/>
       <c r="H100" s="14"/>
       <c r="I100" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J100" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K100" s="16"/>
@@ -4789,11 +4816,11 @@
       <c r="G101" s="14"/>
       <c r="H101" s="14"/>
       <c r="I101" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J101" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K101" s="16"/>
@@ -4811,11 +4838,11 @@
       <c r="G102" s="14"/>
       <c r="H102" s="14"/>
       <c r="I102" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J102" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K102" s="16"/>
@@ -4833,11 +4860,11 @@
       <c r="G103" s="14"/>
       <c r="H103" s="14"/>
       <c r="I103" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J103" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K103" s="16"/>
@@ -4855,11 +4882,11 @@
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
       <c r="I104" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J104" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K104" s="16"/>
@@ -4877,11 +4904,11 @@
       <c r="G105" s="14"/>
       <c r="H105" s="14"/>
       <c r="I105" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J105" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K105" s="16"/>
@@ -4899,11 +4926,11 @@
       <c r="G106" s="14"/>
       <c r="H106" s="14"/>
       <c r="I106" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J106" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K106" s="16"/>
@@ -4921,11 +4948,11 @@
       <c r="G107" s="14"/>
       <c r="H107" s="14"/>
       <c r="I107" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J107" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K107" s="16"/>
@@ -4943,11 +4970,11 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J108" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K108" s="16"/>
@@ -4965,11 +4992,11 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J109" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K109" s="16"/>
@@ -4987,11 +5014,11 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J110" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K110" s="16"/>
@@ -5009,11 +5036,11 @@
       <c r="G111" s="14"/>
       <c r="H111" s="14"/>
       <c r="I111" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J111" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K111" s="16"/>
@@ -5031,11 +5058,11 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J112" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K112" s="16"/>
@@ -5053,11 +5080,11 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J113" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K113" s="16"/>
@@ -5075,11 +5102,11 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J114" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K114" s="16"/>
@@ -5097,11 +5124,11 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J115" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K115" s="16"/>
@@ -5119,11 +5146,11 @@
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
       <c r="I116" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J116" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K116" s="16"/>
@@ -5141,11 +5168,11 @@
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
       <c r="I117" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J117" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K117" s="16"/>
@@ -5163,11 +5190,11 @@
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
       <c r="I118" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J118" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K118" s="16"/>
@@ -5185,11 +5212,11 @@
       <c r="G119" s="14"/>
       <c r="H119" s="14"/>
       <c r="I119" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J119" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K119" s="16"/>
@@ -5207,11 +5234,11 @@
       <c r="G120" s="14"/>
       <c r="H120" s="14"/>
       <c r="I120" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J120" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K120" s="16"/>
@@ -5229,11 +5256,11 @@
       <c r="G121" s="14"/>
       <c r="H121" s="14"/>
       <c r="I121" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J121" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K121" s="16"/>
@@ -5251,11 +5278,11 @@
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
       <c r="I122" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J122" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K122" s="16"/>
@@ -5273,11 +5300,11 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J123" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K123" s="16"/>
@@ -5295,11 +5322,11 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J124" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K124" s="16"/>
@@ -5317,11 +5344,11 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J125" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K125" s="16"/>
@@ -5339,11 +5366,11 @@
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
       <c r="I126" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J126" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K126" s="16"/>
@@ -5361,11 +5388,11 @@
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J127" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K127" s="16"/>
@@ -5383,11 +5410,11 @@
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
       <c r="I128" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J128" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K128" s="16"/>
@@ -5405,11 +5432,11 @@
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
       <c r="I129" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J129" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K129" s="16"/>
@@ -5427,11 +5454,11 @@
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
       <c r="I130" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J130" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K130" s="16"/>
@@ -5449,11 +5476,11 @@
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
       <c r="I131" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J131" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K131" s="16"/>
@@ -5471,11 +5498,11 @@
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
       <c r="I132" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J132" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K132" s="16"/>
@@ -5493,11 +5520,11 @@
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
       <c r="I133" s="15" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="J133" s="15" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="K133" s="16"/>
@@ -5515,11 +5542,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="24">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" ref="I134:I197" si="26">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="25">IF(I134="","",1440-I134)</f>
+        <f t="shared" ref="J134:J197" si="27">IF(I134="","",1440-I134)</f>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -5537,11 +5564,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5559,11 +5586,11 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J136" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K136" s="16"/>
@@ -5581,11 +5608,11 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J137" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K137" s="16"/>
@@ -5603,11 +5630,11 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J138" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K138" s="16"/>
@@ -5625,11 +5652,11 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J139" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K139" s="16"/>
@@ -5647,11 +5674,11 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J140" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K140" s="16"/>
@@ -5669,11 +5696,11 @@
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J141" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K141" s="16"/>
@@ -5691,11 +5718,11 @@
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J142" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K142" s="16"/>
@@ -5713,11 +5740,11 @@
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J143" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K143" s="16"/>
@@ -5735,11 +5762,11 @@
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J144" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K144" s="16"/>
@@ -5757,11 +5784,11 @@
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J145" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K145" s="16"/>
@@ -5779,11 +5806,11 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J146" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K146" s="16"/>
@@ -5801,11 +5828,11 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J147" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K147" s="16"/>
@@ -5823,11 +5850,11 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J148" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K148" s="16"/>
@@ -5845,11 +5872,11 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J149" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K149" s="16"/>
@@ -5867,11 +5894,11 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J150" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K150" s="16"/>
@@ -5889,11 +5916,11 @@
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
       <c r="I151" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J151" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K151" s="16"/>
@@ -5911,11 +5938,11 @@
       <c r="G152" s="14"/>
       <c r="H152" s="14"/>
       <c r="I152" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J152" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K152" s="16"/>
@@ -5933,11 +5960,11 @@
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J153" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K153" s="16"/>
@@ -5955,11 +5982,11 @@
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J154" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K154" s="16"/>
@@ -5977,11 +6004,11 @@
       <c r="G155" s="14"/>
       <c r="H155" s="14"/>
       <c r="I155" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J155" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K155" s="16"/>
@@ -5999,11 +6026,11 @@
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
       <c r="I156" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J156" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K156" s="16"/>
@@ -6021,11 +6048,11 @@
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J157" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K157" s="16"/>
@@ -6043,11 +6070,11 @@
       <c r="G158" s="14"/>
       <c r="H158" s="14"/>
       <c r="I158" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J158" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K158" s="16"/>
@@ -6065,11 +6092,11 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J159" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K159" s="16"/>
@@ -6087,11 +6114,11 @@
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
       <c r="I160" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J160" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K160" s="16"/>
@@ -6109,11 +6136,11 @@
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
       <c r="I161" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J161" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K161" s="16"/>
@@ -6131,11 +6158,11 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J162" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K162" s="16"/>
@@ -6153,11 +6180,11 @@
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
       <c r="I163" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J163" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K163" s="16"/>
@@ -6175,11 +6202,11 @@
       <c r="G164" s="14"/>
       <c r="H164" s="14"/>
       <c r="I164" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J164" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K164" s="16"/>
@@ -6197,11 +6224,11 @@
       <c r="G165" s="14"/>
       <c r="H165" s="14"/>
       <c r="I165" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J165" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K165" s="16"/>
@@ -6219,11 +6246,11 @@
       <c r="G166" s="14"/>
       <c r="H166" s="14"/>
       <c r="I166" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J166" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K166" s="16"/>
@@ -6241,11 +6268,11 @@
       <c r="G167" s="14"/>
       <c r="H167" s="14"/>
       <c r="I167" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J167" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K167" s="16"/>
@@ -6263,11 +6290,11 @@
       <c r="G168" s="14"/>
       <c r="H168" s="14"/>
       <c r="I168" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J168" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K168" s="16"/>
@@ -6285,11 +6312,11 @@
       <c r="G169" s="14"/>
       <c r="H169" s="14"/>
       <c r="I169" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J169" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K169" s="16"/>
@@ -6307,11 +6334,11 @@
       <c r="G170" s="14"/>
       <c r="H170" s="14"/>
       <c r="I170" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J170" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K170" s="16"/>
@@ -6329,11 +6356,11 @@
       <c r="G171" s="14"/>
       <c r="H171" s="14"/>
       <c r="I171" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J171" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K171" s="16"/>
@@ -6351,11 +6378,11 @@
       <c r="G172" s="14"/>
       <c r="H172" s="14"/>
       <c r="I172" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J172" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K172" s="16"/>
@@ -6373,11 +6400,11 @@
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
       <c r="I173" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J173" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K173" s="16"/>
@@ -6395,11 +6422,11 @@
       <c r="G174" s="14"/>
       <c r="H174" s="14"/>
       <c r="I174" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J174" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K174" s="16"/>
@@ -6417,11 +6444,11 @@
       <c r="G175" s="14"/>
       <c r="H175" s="14"/>
       <c r="I175" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J175" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K175" s="16"/>
@@ -6439,11 +6466,11 @@
       <c r="G176" s="14"/>
       <c r="H176" s="14"/>
       <c r="I176" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J176" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K176" s="16"/>
@@ -6461,11 +6488,11 @@
       <c r="G177" s="14"/>
       <c r="H177" s="14"/>
       <c r="I177" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J177" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K177" s="16"/>
@@ -6483,11 +6510,11 @@
       <c r="G178" s="14"/>
       <c r="H178" s="14"/>
       <c r="I178" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J178" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K178" s="16"/>
@@ -6505,11 +6532,11 @@
       <c r="G179" s="14"/>
       <c r="H179" s="14"/>
       <c r="I179" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J179" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K179" s="16"/>
@@ -6527,11 +6554,11 @@
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
       <c r="I180" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J180" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K180" s="16"/>
@@ -6549,11 +6576,11 @@
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J181" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K181" s="16"/>
@@ -6571,11 +6598,11 @@
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J182" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K182" s="16"/>
@@ -6593,11 +6620,11 @@
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J183" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K183" s="16"/>
@@ -6615,11 +6642,11 @@
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
       <c r="I184" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J184" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K184" s="16"/>
@@ -6637,11 +6664,11 @@
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
       <c r="I185" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J185" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K185" s="16"/>
@@ -6659,11 +6686,11 @@
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J186" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K186" s="16"/>
@@ -6681,11 +6708,11 @@
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J187" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K187" s="16"/>
@@ -6703,11 +6730,11 @@
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
       <c r="I188" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J188" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K188" s="16"/>
@@ -6725,11 +6752,11 @@
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
       <c r="I189" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J189" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K189" s="16"/>
@@ -6747,11 +6774,11 @@
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J190" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K190" s="16"/>
@@ -6769,11 +6796,11 @@
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J191" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K191" s="16"/>
@@ -6791,11 +6818,11 @@
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J192" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K192" s="16"/>
@@ -6813,11 +6840,11 @@
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
       <c r="I193" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J193" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K193" s="16"/>
@@ -6835,11 +6862,11 @@
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
       <c r="I194" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J194" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K194" s="16"/>
@@ -6857,11 +6884,11 @@
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J195" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K195" s="16"/>
@@ -6879,11 +6906,11 @@
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J196" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K196" s="16"/>
@@ -6901,11 +6928,11 @@
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="J197" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="K197" s="16"/>
@@ -6923,11 +6950,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="26">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" ref="I198:I261" si="28">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="27">IF(I198="","",1440-I198)</f>
+        <f t="shared" ref="J198:J261" si="29">IF(I198="","",1440-I198)</f>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -6945,11 +6972,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -6967,11 +6994,11 @@
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J200" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K200" s="16"/>
@@ -6989,11 +7016,11 @@
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
       <c r="I201" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J201" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K201" s="16"/>
@@ -7011,11 +7038,11 @@
       <c r="G202" s="14"/>
       <c r="H202" s="14"/>
       <c r="I202" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J202" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K202" s="16"/>
@@ -7033,11 +7060,11 @@
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
       <c r="I203" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J203" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K203" s="16"/>
@@ -7055,11 +7082,11 @@
       <c r="G204" s="14"/>
       <c r="H204" s="14"/>
       <c r="I204" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J204" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K204" s="16"/>
@@ -7077,11 +7104,11 @@
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J205" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K205" s="16"/>
@@ -7099,11 +7126,11 @@
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J206" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K206" s="16"/>
@@ -7121,11 +7148,11 @@
       <c r="G207" s="14"/>
       <c r="H207" s="14"/>
       <c r="I207" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J207" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K207" s="16"/>
@@ -7143,11 +7170,11 @@
       <c r="G208" s="14"/>
       <c r="H208" s="14"/>
       <c r="I208" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J208" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K208" s="16"/>
@@ -7165,11 +7192,11 @@
       <c r="G209" s="14"/>
       <c r="H209" s="14"/>
       <c r="I209" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J209" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K209" s="16"/>
@@ -7187,11 +7214,11 @@
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J210" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K210" s="16"/>
@@ -7209,11 +7236,11 @@
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J211" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K211" s="16"/>
@@ -7231,11 +7258,11 @@
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J212" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K212" s="16"/>
@@ -7253,11 +7280,11 @@
       <c r="G213" s="14"/>
       <c r="H213" s="14"/>
       <c r="I213" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J213" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K213" s="16"/>
@@ -7275,11 +7302,11 @@
       <c r="G214" s="14"/>
       <c r="H214" s="14"/>
       <c r="I214" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J214" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K214" s="16"/>
@@ -7297,11 +7324,11 @@
       <c r="G215" s="14"/>
       <c r="H215" s="14"/>
       <c r="I215" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J215" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K215" s="16"/>
@@ -7319,11 +7346,11 @@
       <c r="G216" s="14"/>
       <c r="H216" s="14"/>
       <c r="I216" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J216" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K216" s="16"/>
@@ -7341,11 +7368,11 @@
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J217" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K217" s="16"/>
@@ -7363,11 +7390,11 @@
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J218" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K218" s="16"/>
@@ -7385,11 +7412,11 @@
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J219" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K219" s="16"/>
@@ -7407,11 +7434,11 @@
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J220" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K220" s="16"/>
@@ -7429,11 +7456,11 @@
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J221" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K221" s="16"/>
@@ -7451,11 +7478,11 @@
       <c r="G222" s="14"/>
       <c r="H222" s="14"/>
       <c r="I222" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J222" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K222" s="16"/>
@@ -7473,11 +7500,11 @@
       <c r="G223" s="14"/>
       <c r="H223" s="14"/>
       <c r="I223" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J223" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K223" s="16"/>
@@ -7495,11 +7522,11 @@
       <c r="G224" s="14"/>
       <c r="H224" s="14"/>
       <c r="I224" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J224" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K224" s="16"/>
@@ -7517,11 +7544,11 @@
       <c r="G225" s="14"/>
       <c r="H225" s="14"/>
       <c r="I225" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J225" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K225" s="16"/>
@@ -7539,11 +7566,11 @@
       <c r="G226" s="14"/>
       <c r="H226" s="14"/>
       <c r="I226" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J226" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K226" s="16"/>
@@ -7561,11 +7588,11 @@
       <c r="G227" s="14"/>
       <c r="H227" s="14"/>
       <c r="I227" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J227" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K227" s="16"/>
@@ -7583,11 +7610,11 @@
       <c r="G228" s="14"/>
       <c r="H228" s="14"/>
       <c r="I228" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J228" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K228" s="16"/>
@@ -7605,11 +7632,11 @@
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J229" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K229" s="16"/>
@@ -7627,11 +7654,11 @@
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J230" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K230" s="16"/>
@@ -7649,11 +7676,11 @@
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
       <c r="I231" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J231" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K231" s="16"/>
@@ -7671,11 +7698,11 @@
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
       <c r="I232" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J232" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K232" s="16"/>
@@ -7693,11 +7720,11 @@
       <c r="G233" s="14"/>
       <c r="H233" s="14"/>
       <c r="I233" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J233" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K233" s="16"/>
@@ -7715,11 +7742,11 @@
       <c r="G234" s="14"/>
       <c r="H234" s="14"/>
       <c r="I234" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J234" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K234" s="16"/>
@@ -7737,11 +7764,11 @@
       <c r="G235" s="14"/>
       <c r="H235" s="14"/>
       <c r="I235" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J235" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K235" s="16"/>
@@ -7759,11 +7786,11 @@
       <c r="G236" s="14"/>
       <c r="H236" s="14"/>
       <c r="I236" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J236" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K236" s="16"/>
@@ -7781,11 +7808,11 @@
       <c r="G237" s="14"/>
       <c r="H237" s="14"/>
       <c r="I237" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J237" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K237" s="16"/>
@@ -7803,11 +7830,11 @@
       <c r="G238" s="14"/>
       <c r="H238" s="14"/>
       <c r="I238" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J238" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K238" s="16"/>
@@ -7825,11 +7852,11 @@
       <c r="G239" s="14"/>
       <c r="H239" s="14"/>
       <c r="I239" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J239" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K239" s="16"/>
@@ -7847,11 +7874,11 @@
       <c r="G240" s="14"/>
       <c r="H240" s="14"/>
       <c r="I240" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J240" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K240" s="16"/>
@@ -7869,11 +7896,11 @@
       <c r="G241" s="14"/>
       <c r="H241" s="14"/>
       <c r="I241" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J241" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K241" s="16"/>
@@ -7891,11 +7918,11 @@
       <c r="G242" s="14"/>
       <c r="H242" s="14"/>
       <c r="I242" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J242" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K242" s="16"/>
@@ -7913,11 +7940,11 @@
       <c r="G243" s="14"/>
       <c r="H243" s="14"/>
       <c r="I243" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J243" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K243" s="16"/>
@@ -7935,11 +7962,11 @@
       <c r="G244" s="14"/>
       <c r="H244" s="14"/>
       <c r="I244" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J244" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K244" s="16"/>
@@ -7957,11 +7984,11 @@
       <c r="G245" s="14"/>
       <c r="H245" s="14"/>
       <c r="I245" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J245" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K245" s="16"/>
@@ -7979,11 +8006,11 @@
       <c r="G246" s="14"/>
       <c r="H246" s="14"/>
       <c r="I246" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J246" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K246" s="16"/>
@@ -8001,11 +8028,11 @@
       <c r="G247" s="14"/>
       <c r="H247" s="14"/>
       <c r="I247" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J247" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K247" s="16"/>
@@ -8023,11 +8050,11 @@
       <c r="G248" s="14"/>
       <c r="H248" s="14"/>
       <c r="I248" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J248" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K248" s="16"/>
@@ -8045,11 +8072,11 @@
       <c r="G249" s="14"/>
       <c r="H249" s="14"/>
       <c r="I249" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J249" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K249" s="16"/>
@@ -8067,11 +8094,11 @@
       <c r="G250" s="14"/>
       <c r="H250" s="14"/>
       <c r="I250" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J250" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K250" s="16"/>
@@ -8089,11 +8116,11 @@
       <c r="G251" s="14"/>
       <c r="H251" s="14"/>
       <c r="I251" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J251" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K251" s="16"/>
@@ -8111,11 +8138,11 @@
       <c r="G252" s="14"/>
       <c r="H252" s="14"/>
       <c r="I252" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J252" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K252" s="16"/>
@@ -8133,11 +8160,11 @@
       <c r="G253" s="14"/>
       <c r="H253" s="14"/>
       <c r="I253" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J253" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K253" s="16"/>
@@ -8155,11 +8182,11 @@
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
       <c r="I254" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J254" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K254" s="16"/>
@@ -8177,11 +8204,11 @@
       <c r="G255" s="14"/>
       <c r="H255" s="14"/>
       <c r="I255" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J255" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K255" s="16"/>
@@ -8199,11 +8226,11 @@
       <c r="G256" s="14"/>
       <c r="H256" s="14"/>
       <c r="I256" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J256" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K256" s="16"/>
@@ -8221,11 +8248,11 @@
       <c r="G257" s="14"/>
       <c r="H257" s="14"/>
       <c r="I257" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J257" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K257" s="16"/>
@@ -8243,11 +8270,11 @@
       <c r="G258" s="14"/>
       <c r="H258" s="14"/>
       <c r="I258" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J258" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K258" s="16"/>
@@ -8265,11 +8292,11 @@
       <c r="G259" s="14"/>
       <c r="H259" s="14"/>
       <c r="I259" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J259" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K259" s="16"/>
@@ -8287,11 +8314,11 @@
       <c r="G260" s="14"/>
       <c r="H260" s="14"/>
       <c r="I260" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J260" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K260" s="16"/>
@@ -8309,11 +8336,11 @@
       <c r="G261" s="14"/>
       <c r="H261" s="14"/>
       <c r="I261" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
       <c r="J261" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
       <c r="K261" s="16"/>
@@ -8331,11 +8358,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="28">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" ref="I262:I325" si="30">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="29">IF(I262="","",1440-I262)</f>
+        <f t="shared" ref="J262:J325" si="31">IF(I262="","",1440-I262)</f>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -8353,11 +8380,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8375,11 +8402,11 @@
       <c r="G264" s="14"/>
       <c r="H264" s="14"/>
       <c r="I264" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J264" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K264" s="16"/>
@@ -8397,11 +8424,11 @@
       <c r="G265" s="14"/>
       <c r="H265" s="14"/>
       <c r="I265" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J265" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K265" s="16"/>
@@ -8419,11 +8446,11 @@
       <c r="G266" s="14"/>
       <c r="H266" s="14"/>
       <c r="I266" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J266" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K266" s="16"/>
@@ -8441,11 +8468,11 @@
       <c r="G267" s="14"/>
       <c r="H267" s="14"/>
       <c r="I267" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J267" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K267" s="16"/>
@@ -8463,11 +8490,11 @@
       <c r="G268" s="14"/>
       <c r="H268" s="14"/>
       <c r="I268" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J268" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K268" s="16"/>
@@ -8485,11 +8512,11 @@
       <c r="G269" s="14"/>
       <c r="H269" s="14"/>
       <c r="I269" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J269" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K269" s="16"/>
@@ -8507,11 +8534,11 @@
       <c r="G270" s="14"/>
       <c r="H270" s="14"/>
       <c r="I270" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J270" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K270" s="16"/>
@@ -8529,11 +8556,11 @@
       <c r="G271" s="14"/>
       <c r="H271" s="14"/>
       <c r="I271" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J271" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K271" s="16"/>
@@ -8551,11 +8578,11 @@
       <c r="G272" s="14"/>
       <c r="H272" s="14"/>
       <c r="I272" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J272" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K272" s="16"/>
@@ -8573,11 +8600,11 @@
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
       <c r="I273" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J273" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K273" s="16"/>
@@ -8595,11 +8622,11 @@
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
       <c r="I274" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J274" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K274" s="16"/>
@@ -8617,11 +8644,11 @@
       <c r="G275" s="14"/>
       <c r="H275" s="14"/>
       <c r="I275" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J275" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K275" s="16"/>
@@ -8639,11 +8666,11 @@
       <c r="G276" s="14"/>
       <c r="H276" s="14"/>
       <c r="I276" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J276" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K276" s="16"/>
@@ -8661,11 +8688,11 @@
       <c r="G277" s="14"/>
       <c r="H277" s="14"/>
       <c r="I277" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J277" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K277" s="16"/>
@@ -8683,11 +8710,11 @@
       <c r="G278" s="14"/>
       <c r="H278" s="14"/>
       <c r="I278" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J278" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K278" s="16"/>
@@ -8705,11 +8732,11 @@
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
       <c r="I279" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J279" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K279" s="16"/>
@@ -8727,11 +8754,11 @@
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
       <c r="I280" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J280" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K280" s="16"/>
@@ -8749,11 +8776,11 @@
       <c r="G281" s="14"/>
       <c r="H281" s="14"/>
       <c r="I281" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J281" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K281" s="16"/>
@@ -8771,11 +8798,11 @@
       <c r="G282" s="14"/>
       <c r="H282" s="14"/>
       <c r="I282" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J282" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K282" s="16"/>
@@ -8793,11 +8820,11 @@
       <c r="G283" s="14"/>
       <c r="H283" s="14"/>
       <c r="I283" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J283" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K283" s="16"/>
@@ -8815,11 +8842,11 @@
       <c r="G284" s="14"/>
       <c r="H284" s="14"/>
       <c r="I284" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J284" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K284" s="16"/>
@@ -8837,11 +8864,11 @@
       <c r="G285" s="14"/>
       <c r="H285" s="14"/>
       <c r="I285" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J285" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K285" s="16"/>
@@ -8859,11 +8886,11 @@
       <c r="G286" s="14"/>
       <c r="H286" s="14"/>
       <c r="I286" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J286" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K286" s="16"/>
@@ -8881,11 +8908,11 @@
       <c r="G287" s="14"/>
       <c r="H287" s="14"/>
       <c r="I287" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J287" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K287" s="16"/>
@@ -8903,11 +8930,11 @@
       <c r="G288" s="14"/>
       <c r="H288" s="14"/>
       <c r="I288" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J288" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K288" s="16"/>
@@ -8925,11 +8952,11 @@
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
       <c r="I289" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J289" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K289" s="16"/>
@@ -8947,11 +8974,11 @@
       <c r="G290" s="14"/>
       <c r="H290" s="14"/>
       <c r="I290" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J290" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K290" s="16"/>
@@ -8969,11 +8996,11 @@
       <c r="G291" s="14"/>
       <c r="H291" s="14"/>
       <c r="I291" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J291" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K291" s="16"/>
@@ -8991,11 +9018,11 @@
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
       <c r="I292" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J292" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K292" s="16"/>
@@ -9013,11 +9040,11 @@
       <c r="G293" s="14"/>
       <c r="H293" s="14"/>
       <c r="I293" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J293" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K293" s="16"/>
@@ -9035,11 +9062,11 @@
       <c r="G294" s="14"/>
       <c r="H294" s="14"/>
       <c r="I294" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J294" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K294" s="16"/>
@@ -9057,11 +9084,11 @@
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
       <c r="I295" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J295" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K295" s="16"/>
@@ -9079,11 +9106,11 @@
       <c r="G296" s="14"/>
       <c r="H296" s="14"/>
       <c r="I296" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J296" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K296" s="16"/>
@@ -9101,11 +9128,11 @@
       <c r="G297" s="14"/>
       <c r="H297" s="14"/>
       <c r="I297" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J297" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K297" s="16"/>
@@ -9123,11 +9150,11 @@
       <c r="G298" s="14"/>
       <c r="H298" s="14"/>
       <c r="I298" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J298" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K298" s="16"/>
@@ -9145,11 +9172,11 @@
       <c r="G299" s="14"/>
       <c r="H299" s="14"/>
       <c r="I299" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J299" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K299" s="16"/>
@@ -9167,11 +9194,11 @@
       <c r="G300" s="14"/>
       <c r="H300" s="14"/>
       <c r="I300" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J300" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K300" s="16"/>
@@ -9189,11 +9216,11 @@
       <c r="G301" s="14"/>
       <c r="H301" s="14"/>
       <c r="I301" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J301" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K301" s="16"/>
@@ -9211,11 +9238,11 @@
       <c r="G302" s="14"/>
       <c r="H302" s="14"/>
       <c r="I302" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J302" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K302" s="16"/>
@@ -9233,11 +9260,11 @@
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
       <c r="I303" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J303" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K303" s="16"/>
@@ -9255,11 +9282,11 @@
       <c r="G304" s="14"/>
       <c r="H304" s="14"/>
       <c r="I304" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J304" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K304" s="16"/>
@@ -9277,11 +9304,11 @@
       <c r="G305" s="14"/>
       <c r="H305" s="14"/>
       <c r="I305" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J305" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K305" s="16"/>
@@ -9299,11 +9326,11 @@
       <c r="G306" s="14"/>
       <c r="H306" s="14"/>
       <c r="I306" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J306" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K306" s="16"/>
@@ -9321,11 +9348,11 @@
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
       <c r="I307" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J307" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K307" s="16"/>
@@ -9343,11 +9370,11 @@
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
       <c r="I308" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J308" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K308" s="16"/>
@@ -9365,11 +9392,11 @@
       <c r="G309" s="14"/>
       <c r="H309" s="14"/>
       <c r="I309" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J309" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K309" s="16"/>
@@ -9387,11 +9414,11 @@
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
       <c r="I310" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J310" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K310" s="16"/>
@@ -9409,11 +9436,11 @@
       <c r="G311" s="14"/>
       <c r="H311" s="14"/>
       <c r="I311" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J311" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K311" s="16"/>
@@ -9431,11 +9458,11 @@
       <c r="G312" s="14"/>
       <c r="H312" s="14"/>
       <c r="I312" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J312" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K312" s="16"/>
@@ -9453,11 +9480,11 @@
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
       <c r="I313" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J313" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K313" s="16"/>
@@ -9475,11 +9502,11 @@
       <c r="G314" s="14"/>
       <c r="H314" s="14"/>
       <c r="I314" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J314" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K314" s="16"/>
@@ -9497,11 +9524,11 @@
       <c r="G315" s="14"/>
       <c r="H315" s="14"/>
       <c r="I315" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J315" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K315" s="16"/>
@@ -9519,11 +9546,11 @@
       <c r="G316" s="14"/>
       <c r="H316" s="14"/>
       <c r="I316" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J316" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K316" s="16"/>
@@ -9541,11 +9568,11 @@
       <c r="G317" s="14"/>
       <c r="H317" s="14"/>
       <c r="I317" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J317" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K317" s="16"/>
@@ -9563,11 +9590,11 @@
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
       <c r="I318" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J318" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K318" s="16"/>
@@ -9585,11 +9612,11 @@
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
       <c r="I319" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J319" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K319" s="16"/>
@@ -9607,11 +9634,11 @@
       <c r="G320" s="14"/>
       <c r="H320" s="14"/>
       <c r="I320" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J320" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K320" s="16"/>
@@ -9629,11 +9656,11 @@
       <c r="G321" s="14"/>
       <c r="H321" s="14"/>
       <c r="I321" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J321" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K321" s="16"/>
@@ -9651,11 +9678,11 @@
       <c r="G322" s="14"/>
       <c r="H322" s="14"/>
       <c r="I322" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J322" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K322" s="16"/>
@@ -9673,11 +9700,11 @@
       <c r="G323" s="14"/>
       <c r="H323" s="14"/>
       <c r="I323" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J323" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K323" s="16"/>
@@ -9695,11 +9722,11 @@
       <c r="G324" s="14"/>
       <c r="H324" s="14"/>
       <c r="I324" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J324" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K324" s="16"/>
@@ -9717,11 +9744,11 @@
       <c r="G325" s="14"/>
       <c r="H325" s="14"/>
       <c r="I325" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
       <c r="J325" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="K325" s="16"/>
@@ -9739,11 +9766,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="30">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" ref="I326:I389" si="32">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="31">IF(I326="","",1440-I326)</f>
+        <f t="shared" ref="J326:J389" si="33">IF(I326="","",1440-I326)</f>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -9761,11 +9788,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -9783,11 +9810,11 @@
       <c r="G328" s="14"/>
       <c r="H328" s="14"/>
       <c r="I328" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J328" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K328" s="16"/>
@@ -9805,11 +9832,11 @@
       <c r="G329" s="14"/>
       <c r="H329" s="14"/>
       <c r="I329" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J329" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K329" s="16"/>
@@ -9827,11 +9854,11 @@
       <c r="G330" s="14"/>
       <c r="H330" s="14"/>
       <c r="I330" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J330" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K330" s="16"/>
@@ -9849,11 +9876,11 @@
       <c r="G331" s="14"/>
       <c r="H331" s="14"/>
       <c r="I331" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J331" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K331" s="16"/>
@@ -9871,11 +9898,11 @@
       <c r="G332" s="14"/>
       <c r="H332" s="14"/>
       <c r="I332" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J332" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K332" s="16"/>
@@ -9893,11 +9920,11 @@
       <c r="G333" s="14"/>
       <c r="H333" s="14"/>
       <c r="I333" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J333" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K333" s="16"/>
@@ -9915,11 +9942,11 @@
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
       <c r="I334" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J334" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K334" s="16"/>
@@ -9937,11 +9964,11 @@
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
       <c r="I335" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J335" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K335" s="16"/>
@@ -9959,11 +9986,11 @@
       <c r="G336" s="14"/>
       <c r="H336" s="14"/>
       <c r="I336" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J336" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K336" s="16"/>
@@ -9981,11 +10008,11 @@
       <c r="G337" s="14"/>
       <c r="H337" s="14"/>
       <c r="I337" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J337" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K337" s="16"/>
@@ -10003,11 +10030,11 @@
       <c r="G338" s="14"/>
       <c r="H338" s="14"/>
       <c r="I338" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J338" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K338" s="16"/>
@@ -10025,11 +10052,11 @@
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
       <c r="I339" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J339" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K339" s="16"/>
@@ -10047,11 +10074,11 @@
       <c r="G340" s="14"/>
       <c r="H340" s="14"/>
       <c r="I340" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J340" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K340" s="16"/>
@@ -10069,11 +10096,11 @@
       <c r="G341" s="14"/>
       <c r="H341" s="14"/>
       <c r="I341" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J341" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K341" s="16"/>
@@ -10091,11 +10118,11 @@
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
       <c r="I342" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J342" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K342" s="16"/>
@@ -10113,11 +10140,11 @@
       <c r="G343" s="14"/>
       <c r="H343" s="14"/>
       <c r="I343" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J343" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K343" s="16"/>
@@ -10135,11 +10162,11 @@
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
       <c r="I344" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J344" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K344" s="16"/>
@@ -10157,11 +10184,11 @@
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
       <c r="I345" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J345" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K345" s="16"/>
@@ -10179,11 +10206,11 @@
       <c r="G346" s="14"/>
       <c r="H346" s="14"/>
       <c r="I346" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J346" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K346" s="16"/>
@@ -10201,11 +10228,11 @@
       <c r="G347" s="14"/>
       <c r="H347" s="14"/>
       <c r="I347" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J347" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K347" s="16"/>
@@ -10223,11 +10250,11 @@
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
       <c r="I348" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J348" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K348" s="16"/>
@@ -10245,11 +10272,11 @@
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
       <c r="I349" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J349" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K349" s="16"/>
@@ -10267,11 +10294,11 @@
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
       <c r="I350" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J350" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K350" s="16"/>
@@ -10289,11 +10316,11 @@
       <c r="G351" s="14"/>
       <c r="H351" s="14"/>
       <c r="I351" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J351" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K351" s="16"/>
@@ -10311,11 +10338,11 @@
       <c r="G352" s="14"/>
       <c r="H352" s="14"/>
       <c r="I352" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J352" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K352" s="16"/>
@@ -10333,11 +10360,11 @@
       <c r="G353" s="14"/>
       <c r="H353" s="14"/>
       <c r="I353" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J353" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K353" s="16"/>
@@ -10355,11 +10382,11 @@
       <c r="G354" s="14"/>
       <c r="H354" s="14"/>
       <c r="I354" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J354" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K354" s="16"/>
@@ -10377,11 +10404,11 @@
       <c r="G355" s="14"/>
       <c r="H355" s="14"/>
       <c r="I355" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J355" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K355" s="16"/>
@@ -10399,11 +10426,11 @@
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
       <c r="I356" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J356" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K356" s="16"/>
@@ -10421,11 +10448,11 @@
       <c r="G357" s="14"/>
       <c r="H357" s="14"/>
       <c r="I357" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J357" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K357" s="16"/>
@@ -10443,11 +10470,11 @@
       <c r="G358" s="14"/>
       <c r="H358" s="14"/>
       <c r="I358" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J358" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K358" s="16"/>
@@ -10465,11 +10492,11 @@
       <c r="G359" s="14"/>
       <c r="H359" s="14"/>
       <c r="I359" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J359" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K359" s="16"/>
@@ -10487,11 +10514,11 @@
       <c r="G360" s="14"/>
       <c r="H360" s="14"/>
       <c r="I360" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J360" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K360" s="16"/>
@@ -10509,11 +10536,11 @@
       <c r="G361" s="14"/>
       <c r="H361" s="14"/>
       <c r="I361" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J361" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K361" s="16"/>
@@ -10531,11 +10558,11 @@
       <c r="G362" s="14"/>
       <c r="H362" s="14"/>
       <c r="I362" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J362" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K362" s="16"/>
@@ -10553,11 +10580,11 @@
       <c r="G363" s="14"/>
       <c r="H363" s="14"/>
       <c r="I363" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J363" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K363" s="16"/>
@@ -10575,11 +10602,11 @@
       <c r="G364" s="14"/>
       <c r="H364" s="14"/>
       <c r="I364" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J364" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K364" s="16"/>
@@ -10597,11 +10624,11 @@
       <c r="G365" s="14"/>
       <c r="H365" s="14"/>
       <c r="I365" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J365" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K365" s="16"/>
@@ -10619,11 +10646,11 @@
       <c r="G366" s="14"/>
       <c r="H366" s="14"/>
       <c r="I366" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J366" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K366" s="16"/>
@@ -10641,11 +10668,11 @@
       <c r="G367" s="14"/>
       <c r="H367" s="14"/>
       <c r="I367" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J367" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K367" s="16"/>
@@ -10663,11 +10690,11 @@
       <c r="G368" s="14"/>
       <c r="H368" s="14"/>
       <c r="I368" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J368" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K368" s="16"/>
@@ -10685,11 +10712,11 @@
       <c r="G369" s="14"/>
       <c r="H369" s="14"/>
       <c r="I369" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J369" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K369" s="16"/>
@@ -10707,11 +10734,11 @@
       <c r="G370" s="14"/>
       <c r="H370" s="14"/>
       <c r="I370" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J370" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K370" s="16"/>
@@ -10729,11 +10756,11 @@
       <c r="G371" s="14"/>
       <c r="H371" s="14"/>
       <c r="I371" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J371" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K371" s="16"/>
@@ -10751,11 +10778,11 @@
       <c r="G372" s="14"/>
       <c r="H372" s="14"/>
       <c r="I372" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J372" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K372" s="16"/>
@@ -10773,11 +10800,11 @@
       <c r="G373" s="14"/>
       <c r="H373" s="14"/>
       <c r="I373" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J373" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K373" s="16"/>
@@ -10795,11 +10822,11 @@
       <c r="G374" s="14"/>
       <c r="H374" s="14"/>
       <c r="I374" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J374" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K374" s="16"/>
@@ -10817,11 +10844,11 @@
       <c r="G375" s="14"/>
       <c r="H375" s="14"/>
       <c r="I375" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J375" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K375" s="16"/>
@@ -10839,11 +10866,11 @@
       <c r="G376" s="14"/>
       <c r="H376" s="14"/>
       <c r="I376" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J376" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K376" s="16"/>
@@ -10861,11 +10888,11 @@
       <c r="G377" s="14"/>
       <c r="H377" s="14"/>
       <c r="I377" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J377" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K377" s="16"/>
@@ -10883,11 +10910,11 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K378" s="16"/>
@@ -10905,11 +10932,11 @@
       <c r="G379" s="14"/>
       <c r="H379" s="14"/>
       <c r="I379" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J379" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K379" s="16"/>
@@ -10927,11 +10954,11 @@
       <c r="G380" s="14"/>
       <c r="H380" s="14"/>
       <c r="I380" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J380" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K380" s="16"/>
@@ -10949,11 +10976,11 @@
       <c r="G381" s="14"/>
       <c r="H381" s="14"/>
       <c r="I381" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J381" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K381" s="16"/>
@@ -10971,11 +10998,11 @@
       <c r="G382" s="14"/>
       <c r="H382" s="14"/>
       <c r="I382" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J382" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K382" s="16"/>
@@ -10993,11 +11020,11 @@
       <c r="G383" s="14"/>
       <c r="H383" s="14"/>
       <c r="I383" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J383" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K383" s="16"/>
@@ -11015,11 +11042,11 @@
       <c r="G384" s="14"/>
       <c r="H384" s="14"/>
       <c r="I384" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J384" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K384" s="16"/>
@@ -11037,11 +11064,11 @@
       <c r="G385" s="14"/>
       <c r="H385" s="14"/>
       <c r="I385" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J385" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K385" s="16"/>
@@ -11059,11 +11086,11 @@
       <c r="G386" s="14"/>
       <c r="H386" s="14"/>
       <c r="I386" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J386" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K386" s="16"/>
@@ -11081,11 +11108,11 @@
       <c r="G387" s="14"/>
       <c r="H387" s="14"/>
       <c r="I387" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J387" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K387" s="16"/>
@@ -11103,11 +11130,11 @@
       <c r="G388" s="14"/>
       <c r="H388" s="14"/>
       <c r="I388" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J388" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K388" s="16"/>
@@ -11125,11 +11152,11 @@
       <c r="G389" s="14"/>
       <c r="H389" s="14"/>
       <c r="I389" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J389" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K389" s="16"/>
@@ -11147,11 +11174,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="32">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="34">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="33">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="35">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -11169,11 +11196,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -11191,11 +11218,11 @@
       <c r="G392" s="14"/>
       <c r="H392" s="14"/>
       <c r="I392" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J392" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K392" s="16"/>
@@ -11213,11 +11240,11 @@
       <c r="G393" s="14"/>
       <c r="H393" s="14"/>
       <c r="I393" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J393" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K393" s="16"/>
@@ -11235,11 +11262,11 @@
       <c r="G394" s="14"/>
       <c r="H394" s="14"/>
       <c r="I394" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J394" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K394" s="16"/>
@@ -11257,11 +11284,11 @@
       <c r="G395" s="14"/>
       <c r="H395" s="14"/>
       <c r="I395" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J395" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K395" s="16"/>
@@ -11279,11 +11306,11 @@
       <c r="G396" s="14"/>
       <c r="H396" s="14"/>
       <c r="I396" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J396" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K396" s="16"/>
@@ -11301,11 +11328,11 @@
       <c r="G397" s="14"/>
       <c r="H397" s="14"/>
       <c r="I397" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J397" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K397" s="16"/>
@@ -11323,11 +11350,11 @@
       <c r="G398" s="14"/>
       <c r="H398" s="14"/>
       <c r="I398" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J398" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K398" s="16"/>
@@ -11345,11 +11372,11 @@
       <c r="G399" s="14"/>
       <c r="H399" s="14"/>
       <c r="I399" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J399" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K399" s="16"/>
@@ -11367,11 +11394,11 @@
       <c r="G400" s="14"/>
       <c r="H400" s="14"/>
       <c r="I400" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J400" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K400" s="16"/>
@@ -11389,11 +11416,11 @@
       <c r="G401" s="14"/>
       <c r="H401" s="14"/>
       <c r="I401" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J401" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K401" s="16"/>

</xml_diff>

<commit_message>
File Updated On 27/10/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A0AAD3F-634D-448C-A7C3-5D99A5BB58F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C123CA6-9F38-4660-9947-D4AD470F6ECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="612" yWindow="-108" windowWidth="22536" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="97">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -317,6 +317,15 @@
   </si>
   <si>
     <t>Feeling low</t>
+  </si>
+  <si>
+    <t>Started working on c++ project</t>
+  </si>
+  <si>
+    <t>Completed c++ project</t>
+  </si>
+  <si>
+    <t>Report submissions (C++)</t>
   </si>
 </sst>
 </file>
@@ -4169,92 +4178,188 @@
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A72" s="13"/>
-      <c r="B72" s="14"/>
-      <c r="C72" s="14"/>
-      <c r="D72" s="14"/>
-      <c r="E72" s="14"/>
-      <c r="F72" s="14"/>
-      <c r="G72" s="14"/>
-      <c r="H72" s="14"/>
-      <c r="I72" s="15" t="str">
-        <f t="shared" ref="I71:I133" si="24">IF(SUM(B72:F72,H72)=0,"",SUM(B72:F72,H72))</f>
-        <v/>
-      </c>
-      <c r="J72" s="15" t="str">
-        <f t="shared" ref="J71:J133" si="25">IF(I72="","",1440-I72)</f>
-        <v/>
-      </c>
-      <c r="K72" s="16"/>
-      <c r="L72" s="16"/>
-      <c r="M72" s="16"/>
-      <c r="N72" s="17"/>
+      <c r="A72" s="13">
+        <v>46319</v>
+      </c>
+      <c r="B72" s="14">
+        <v>480</v>
+      </c>
+      <c r="C72" s="14">
+        <v>0</v>
+      </c>
+      <c r="D72" s="14">
+        <v>150</v>
+      </c>
+      <c r="E72" s="14">
+        <v>100</v>
+      </c>
+      <c r="F72" s="14">
+        <v>0</v>
+      </c>
+      <c r="G72" s="14">
+        <v>0</v>
+      </c>
+      <c r="H72" s="14">
+        <v>50</v>
+      </c>
+      <c r="I72" s="15">
+        <f t="shared" ref="I72" si="24">IF(SUM(B72:F72,H72)=0,"",SUM(B72:F72,H72))</f>
+        <v>780</v>
+      </c>
+      <c r="J72" s="15">
+        <f t="shared" ref="J72" si="25">IF(I72="","",1440-I72)</f>
+        <v>660</v>
+      </c>
+      <c r="K72" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L72" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M72" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N72" s="17" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A73" s="13"/>
-      <c r="B73" s="14"/>
-      <c r="C73" s="14"/>
-      <c r="D73" s="14"/>
-      <c r="E73" s="14"/>
-      <c r="F73" s="14"/>
-      <c r="G73" s="14"/>
-      <c r="H73" s="14"/>
-      <c r="I73" s="15" t="str">
-        <f t="shared" si="24"/>
-        <v/>
-      </c>
-      <c r="J73" s="15" t="str">
-        <f t="shared" si="25"/>
-        <v/>
-      </c>
-      <c r="K73" s="16"/>
-      <c r="L73" s="16"/>
-      <c r="M73" s="16"/>
-      <c r="N73" s="17"/>
-    </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A74" s="13"/>
-      <c r="B74" s="14"/>
-      <c r="C74" s="14"/>
-      <c r="D74" s="14"/>
-      <c r="E74" s="14"/>
-      <c r="F74" s="14"/>
-      <c r="G74" s="14"/>
-      <c r="H74" s="14"/>
-      <c r="I74" s="15" t="str">
-        <f t="shared" si="24"/>
-        <v/>
-      </c>
-      <c r="J74" s="15" t="str">
-        <f t="shared" si="25"/>
-        <v/>
-      </c>
-      <c r="K74" s="16"/>
-      <c r="L74" s="16"/>
-      <c r="M74" s="16"/>
-      <c r="N74" s="17"/>
+      <c r="A73" s="13">
+        <v>46320</v>
+      </c>
+      <c r="B73" s="14">
+        <v>480</v>
+      </c>
+      <c r="C73" s="14">
+        <v>0</v>
+      </c>
+      <c r="D73" s="14">
+        <v>120</v>
+      </c>
+      <c r="E73" s="14">
+        <v>150</v>
+      </c>
+      <c r="F73" s="14">
+        <v>0</v>
+      </c>
+      <c r="G73" s="14">
+        <v>0</v>
+      </c>
+      <c r="H73" s="14">
+        <v>45</v>
+      </c>
+      <c r="I73" s="15">
+        <f t="shared" ref="I73" si="26">IF(SUM(B73:F73,H73)=0,"",SUM(B73:F73,H73))</f>
+        <v>795</v>
+      </c>
+      <c r="J73" s="15">
+        <f t="shared" ref="J73" si="27">IF(I73="","",1440-I73)</f>
+        <v>645</v>
+      </c>
+      <c r="K73" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L73" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M73" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N73" s="17" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A74" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B74" s="14">
+        <v>420</v>
+      </c>
+      <c r="C74" s="14">
+        <v>0</v>
+      </c>
+      <c r="D74" s="14">
+        <v>75</v>
+      </c>
+      <c r="E74" s="14">
+        <v>120</v>
+      </c>
+      <c r="F74" s="14">
+        <v>0</v>
+      </c>
+      <c r="G74" s="14">
+        <v>0</v>
+      </c>
+      <c r="H74" s="14">
+        <v>60</v>
+      </c>
+      <c r="I74" s="15">
+        <f t="shared" ref="I74" si="28">IF(SUM(B74:F74,H74)=0,"",SUM(B74:F74,H74))</f>
+        <v>675</v>
+      </c>
+      <c r="J74" s="15">
+        <f t="shared" ref="J74" si="29">IF(I74="","",1440-I74)</f>
+        <v>765</v>
+      </c>
+      <c r="K74" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L74" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M74" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N74" s="17" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A75" s="13"/>
-      <c r="B75" s="14"/>
-      <c r="C75" s="14"/>
-      <c r="D75" s="14"/>
-      <c r="E75" s="14"/>
-      <c r="F75" s="14"/>
-      <c r="G75" s="14"/>
-      <c r="H75" s="14"/>
-      <c r="I75" s="15" t="str">
-        <f t="shared" si="24"/>
-        <v/>
-      </c>
-      <c r="J75" s="15" t="str">
-        <f t="shared" si="25"/>
-        <v/>
-      </c>
-      <c r="K75" s="16"/>
-      <c r="L75" s="16"/>
-      <c r="M75" s="16"/>
-      <c r="N75" s="17"/>
+      <c r="A75" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B75" s="14">
+        <v>360</v>
+      </c>
+      <c r="C75" s="14">
+        <v>0</v>
+      </c>
+      <c r="D75" s="14">
+        <v>180</v>
+      </c>
+      <c r="E75" s="14">
+        <v>120</v>
+      </c>
+      <c r="F75" s="14">
+        <v>250</v>
+      </c>
+      <c r="G75" s="14">
+        <v>5</v>
+      </c>
+      <c r="H75" s="14">
+        <v>40</v>
+      </c>
+      <c r="I75" s="15">
+        <f t="shared" ref="I75" si="30">IF(SUM(B75:F75,H75)=0,"",SUM(B75:F75,H75))</f>
+        <v>950</v>
+      </c>
+      <c r="J75" s="15">
+        <f t="shared" ref="J75" si="31">IF(I75="","",1440-I75)</f>
+        <v>490</v>
+      </c>
+      <c r="K75" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L75" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M75" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N75" s="17" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76" s="13"/>
@@ -4266,11 +4371,11 @@
       <c r="G76" s="14"/>
       <c r="H76" s="14"/>
       <c r="I76" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" ref="I76:I133" si="32">IF(SUM(B76:F76,H76)=0,"",SUM(B76:F76,H76))</f>
         <v/>
       </c>
       <c r="J76" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" ref="J76:J133" si="33">IF(I76="","",1440-I76)</f>
         <v/>
       </c>
       <c r="K76" s="16"/>
@@ -4288,11 +4393,11 @@
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
       <c r="I77" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J77" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K77" s="16"/>
@@ -4310,11 +4415,11 @@
       <c r="G78" s="14"/>
       <c r="H78" s="14"/>
       <c r="I78" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J78" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K78" s="16"/>
@@ -4332,11 +4437,11 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J79" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K79" s="16"/>
@@ -4354,11 +4459,11 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J80" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K80" s="16"/>
@@ -4376,11 +4481,11 @@
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J81" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K81" s="16"/>
@@ -4398,11 +4503,11 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J82" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K82" s="16"/>
@@ -4420,11 +4525,11 @@
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
       <c r="I83" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J83" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K83" s="16"/>
@@ -4442,11 +4547,11 @@
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
       <c r="I84" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J84" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K84" s="16"/>
@@ -4464,11 +4569,11 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J85" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K85" s="16"/>
@@ -4486,11 +4591,11 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J86" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K86" s="16"/>
@@ -4508,11 +4613,11 @@
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
       <c r="I87" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J87" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K87" s="16"/>
@@ -4530,11 +4635,11 @@
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
       <c r="I88" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J88" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K88" s="16"/>
@@ -4552,11 +4657,11 @@
       <c r="G89" s="14"/>
       <c r="H89" s="14"/>
       <c r="I89" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J89" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K89" s="16"/>
@@ -4574,11 +4679,11 @@
       <c r="G90" s="14"/>
       <c r="H90" s="14"/>
       <c r="I90" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J90" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K90" s="16"/>
@@ -4596,11 +4701,11 @@
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
       <c r="I91" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J91" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K91" s="16"/>
@@ -4618,11 +4723,11 @@
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
       <c r="I92" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J92" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K92" s="16"/>
@@ -4640,11 +4745,11 @@
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J93" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K93" s="16"/>
@@ -4662,11 +4767,11 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J94" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K94" s="16"/>
@@ -4684,11 +4789,11 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J95" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K95" s="16"/>
@@ -4706,11 +4811,11 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J96" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K96" s="16"/>
@@ -4728,11 +4833,11 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J97" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K97" s="16"/>
@@ -4750,11 +4855,11 @@
       <c r="G98" s="14"/>
       <c r="H98" s="14"/>
       <c r="I98" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J98" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K98" s="16"/>
@@ -4772,11 +4877,11 @@
       <c r="G99" s="14"/>
       <c r="H99" s="14"/>
       <c r="I99" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J99" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K99" s="16"/>
@@ -4794,11 +4899,11 @@
       <c r="G100" s="14"/>
       <c r="H100" s="14"/>
       <c r="I100" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J100" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K100" s="16"/>
@@ -4816,11 +4921,11 @@
       <c r="G101" s="14"/>
       <c r="H101" s="14"/>
       <c r="I101" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J101" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K101" s="16"/>
@@ -4838,11 +4943,11 @@
       <c r="G102" s="14"/>
       <c r="H102" s="14"/>
       <c r="I102" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J102" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K102" s="16"/>
@@ -4860,11 +4965,11 @@
       <c r="G103" s="14"/>
       <c r="H103" s="14"/>
       <c r="I103" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J103" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K103" s="16"/>
@@ -4882,11 +4987,11 @@
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
       <c r="I104" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J104" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K104" s="16"/>
@@ -4904,11 +5009,11 @@
       <c r="G105" s="14"/>
       <c r="H105" s="14"/>
       <c r="I105" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J105" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K105" s="16"/>
@@ -4926,11 +5031,11 @@
       <c r="G106" s="14"/>
       <c r="H106" s="14"/>
       <c r="I106" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J106" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K106" s="16"/>
@@ -4948,11 +5053,11 @@
       <c r="G107" s="14"/>
       <c r="H107" s="14"/>
       <c r="I107" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J107" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K107" s="16"/>
@@ -4970,11 +5075,11 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J108" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K108" s="16"/>
@@ -4992,11 +5097,11 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J109" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K109" s="16"/>
@@ -5014,11 +5119,11 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J110" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K110" s="16"/>
@@ -5036,11 +5141,11 @@
       <c r="G111" s="14"/>
       <c r="H111" s="14"/>
       <c r="I111" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J111" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K111" s="16"/>
@@ -5058,11 +5163,11 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J112" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K112" s="16"/>
@@ -5080,11 +5185,11 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J113" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K113" s="16"/>
@@ -5102,11 +5207,11 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J114" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K114" s="16"/>
@@ -5124,11 +5229,11 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J115" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K115" s="16"/>
@@ -5146,11 +5251,11 @@
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
       <c r="I116" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J116" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K116" s="16"/>
@@ -5168,11 +5273,11 @@
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
       <c r="I117" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J117" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K117" s="16"/>
@@ -5190,11 +5295,11 @@
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
       <c r="I118" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J118" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K118" s="16"/>
@@ -5212,11 +5317,11 @@
       <c r="G119" s="14"/>
       <c r="H119" s="14"/>
       <c r="I119" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J119" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K119" s="16"/>
@@ -5234,11 +5339,11 @@
       <c r="G120" s="14"/>
       <c r="H120" s="14"/>
       <c r="I120" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J120" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K120" s="16"/>
@@ -5256,11 +5361,11 @@
       <c r="G121" s="14"/>
       <c r="H121" s="14"/>
       <c r="I121" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J121" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K121" s="16"/>
@@ -5278,11 +5383,11 @@
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
       <c r="I122" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J122" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K122" s="16"/>
@@ -5300,11 +5405,11 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J123" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K123" s="16"/>
@@ -5322,11 +5427,11 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J124" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K124" s="16"/>
@@ -5344,11 +5449,11 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J125" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K125" s="16"/>
@@ -5366,11 +5471,11 @@
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
       <c r="I126" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J126" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K126" s="16"/>
@@ -5388,11 +5493,11 @@
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J127" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K127" s="16"/>
@@ -5410,11 +5515,11 @@
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
       <c r="I128" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J128" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K128" s="16"/>
@@ -5432,11 +5537,11 @@
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
       <c r="I129" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J129" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K129" s="16"/>
@@ -5454,11 +5559,11 @@
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
       <c r="I130" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J130" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K130" s="16"/>
@@ -5476,11 +5581,11 @@
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
       <c r="I131" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J131" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K131" s="16"/>
@@ -5498,11 +5603,11 @@
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
       <c r="I132" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J132" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K132" s="16"/>
@@ -5520,11 +5625,11 @@
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
       <c r="I133" s="15" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="J133" s="15" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
       <c r="K133" s="16"/>
@@ -5542,11 +5647,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="26">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" ref="I134:I197" si="34">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="27">IF(I134="","",1440-I134)</f>
+        <f t="shared" ref="J134:J197" si="35">IF(I134="","",1440-I134)</f>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -5564,11 +5669,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5586,11 +5691,11 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J136" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K136" s="16"/>
@@ -5608,11 +5713,11 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J137" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K137" s="16"/>
@@ -5630,11 +5735,11 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J138" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K138" s="16"/>
@@ -5652,11 +5757,11 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J139" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K139" s="16"/>
@@ -5674,11 +5779,11 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J140" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K140" s="16"/>
@@ -5696,11 +5801,11 @@
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J141" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K141" s="16"/>
@@ -5718,11 +5823,11 @@
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J142" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K142" s="16"/>
@@ -5740,11 +5845,11 @@
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J143" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K143" s="16"/>
@@ -5762,11 +5867,11 @@
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J144" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K144" s="16"/>
@@ -5784,11 +5889,11 @@
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J145" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K145" s="16"/>
@@ -5806,11 +5911,11 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J146" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K146" s="16"/>
@@ -5828,11 +5933,11 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J147" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K147" s="16"/>
@@ -5850,11 +5955,11 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J148" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K148" s="16"/>
@@ -5872,11 +5977,11 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J149" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K149" s="16"/>
@@ -5894,11 +5999,11 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J150" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K150" s="16"/>
@@ -5916,11 +6021,11 @@
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
       <c r="I151" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J151" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K151" s="16"/>
@@ -5938,11 +6043,11 @@
       <c r="G152" s="14"/>
       <c r="H152" s="14"/>
       <c r="I152" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J152" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K152" s="16"/>
@@ -5960,11 +6065,11 @@
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J153" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K153" s="16"/>
@@ -5982,11 +6087,11 @@
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J154" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K154" s="16"/>
@@ -6004,11 +6109,11 @@
       <c r="G155" s="14"/>
       <c r="H155" s="14"/>
       <c r="I155" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J155" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K155" s="16"/>
@@ -6026,11 +6131,11 @@
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
       <c r="I156" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J156" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K156" s="16"/>
@@ -6048,11 +6153,11 @@
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J157" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K157" s="16"/>
@@ -6070,11 +6175,11 @@
       <c r="G158" s="14"/>
       <c r="H158" s="14"/>
       <c r="I158" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J158" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K158" s="16"/>
@@ -6092,11 +6197,11 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J159" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K159" s="16"/>
@@ -6114,11 +6219,11 @@
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
       <c r="I160" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J160" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K160" s="16"/>
@@ -6136,11 +6241,11 @@
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
       <c r="I161" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J161" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K161" s="16"/>
@@ -6158,11 +6263,11 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J162" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K162" s="16"/>
@@ -6180,11 +6285,11 @@
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
       <c r="I163" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J163" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K163" s="16"/>
@@ -6202,11 +6307,11 @@
       <c r="G164" s="14"/>
       <c r="H164" s="14"/>
       <c r="I164" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J164" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K164" s="16"/>
@@ -6224,11 +6329,11 @@
       <c r="G165" s="14"/>
       <c r="H165" s="14"/>
       <c r="I165" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J165" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K165" s="16"/>
@@ -6246,11 +6351,11 @@
       <c r="G166" s="14"/>
       <c r="H166" s="14"/>
       <c r="I166" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J166" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K166" s="16"/>
@@ -6268,11 +6373,11 @@
       <c r="G167" s="14"/>
       <c r="H167" s="14"/>
       <c r="I167" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J167" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K167" s="16"/>
@@ -6290,11 +6395,11 @@
       <c r="G168" s="14"/>
       <c r="H168" s="14"/>
       <c r="I168" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J168" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K168" s="16"/>
@@ -6312,11 +6417,11 @@
       <c r="G169" s="14"/>
       <c r="H169" s="14"/>
       <c r="I169" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J169" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K169" s="16"/>
@@ -6334,11 +6439,11 @@
       <c r="G170" s="14"/>
       <c r="H170" s="14"/>
       <c r="I170" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J170" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K170" s="16"/>
@@ -6356,11 +6461,11 @@
       <c r="G171" s="14"/>
       <c r="H171" s="14"/>
       <c r="I171" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J171" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K171" s="16"/>
@@ -6378,11 +6483,11 @@
       <c r="G172" s="14"/>
       <c r="H172" s="14"/>
       <c r="I172" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J172" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K172" s="16"/>
@@ -6400,11 +6505,11 @@
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
       <c r="I173" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J173" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K173" s="16"/>
@@ -6422,11 +6527,11 @@
       <c r="G174" s="14"/>
       <c r="H174" s="14"/>
       <c r="I174" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J174" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K174" s="16"/>
@@ -6444,11 +6549,11 @@
       <c r="G175" s="14"/>
       <c r="H175" s="14"/>
       <c r="I175" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J175" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K175" s="16"/>
@@ -6466,11 +6571,11 @@
       <c r="G176" s="14"/>
       <c r="H176" s="14"/>
       <c r="I176" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J176" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K176" s="16"/>
@@ -6488,11 +6593,11 @@
       <c r="G177" s="14"/>
       <c r="H177" s="14"/>
       <c r="I177" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J177" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K177" s="16"/>
@@ -6510,11 +6615,11 @@
       <c r="G178" s="14"/>
       <c r="H178" s="14"/>
       <c r="I178" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J178" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K178" s="16"/>
@@ -6532,11 +6637,11 @@
       <c r="G179" s="14"/>
       <c r="H179" s="14"/>
       <c r="I179" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J179" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K179" s="16"/>
@@ -6554,11 +6659,11 @@
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
       <c r="I180" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J180" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K180" s="16"/>
@@ -6576,11 +6681,11 @@
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J181" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K181" s="16"/>
@@ -6598,11 +6703,11 @@
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J182" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K182" s="16"/>
@@ -6620,11 +6725,11 @@
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J183" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K183" s="16"/>
@@ -6642,11 +6747,11 @@
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
       <c r="I184" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J184" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K184" s="16"/>
@@ -6664,11 +6769,11 @@
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
       <c r="I185" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J185" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K185" s="16"/>
@@ -6686,11 +6791,11 @@
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J186" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K186" s="16"/>
@@ -6708,11 +6813,11 @@
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J187" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K187" s="16"/>
@@ -6730,11 +6835,11 @@
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
       <c r="I188" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J188" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K188" s="16"/>
@@ -6752,11 +6857,11 @@
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
       <c r="I189" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J189" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K189" s="16"/>
@@ -6774,11 +6879,11 @@
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J190" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K190" s="16"/>
@@ -6796,11 +6901,11 @@
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J191" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K191" s="16"/>
@@ -6818,11 +6923,11 @@
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J192" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K192" s="16"/>
@@ -6840,11 +6945,11 @@
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
       <c r="I193" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J193" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K193" s="16"/>
@@ -6862,11 +6967,11 @@
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
       <c r="I194" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J194" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K194" s="16"/>
@@ -6884,11 +6989,11 @@
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J195" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K195" s="16"/>
@@ -6906,11 +7011,11 @@
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J196" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K196" s="16"/>
@@ -6928,11 +7033,11 @@
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="15" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J197" s="15" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K197" s="16"/>
@@ -6950,11 +7055,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="28">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" ref="I198:I261" si="36">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="29">IF(I198="","",1440-I198)</f>
+        <f t="shared" ref="J198:J261" si="37">IF(I198="","",1440-I198)</f>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -6972,11 +7077,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -6994,11 +7099,11 @@
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J200" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K200" s="16"/>
@@ -7016,11 +7121,11 @@
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
       <c r="I201" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J201" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K201" s="16"/>
@@ -7038,11 +7143,11 @@
       <c r="G202" s="14"/>
       <c r="H202" s="14"/>
       <c r="I202" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J202" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K202" s="16"/>
@@ -7060,11 +7165,11 @@
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
       <c r="I203" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J203" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K203" s="16"/>
@@ -7082,11 +7187,11 @@
       <c r="G204" s="14"/>
       <c r="H204" s="14"/>
       <c r="I204" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J204" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K204" s="16"/>
@@ -7104,11 +7209,11 @@
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J205" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K205" s="16"/>
@@ -7126,11 +7231,11 @@
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J206" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K206" s="16"/>
@@ -7148,11 +7253,11 @@
       <c r="G207" s="14"/>
       <c r="H207" s="14"/>
       <c r="I207" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J207" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K207" s="16"/>
@@ -7170,11 +7275,11 @@
       <c r="G208" s="14"/>
       <c r="H208" s="14"/>
       <c r="I208" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J208" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K208" s="16"/>
@@ -7192,11 +7297,11 @@
       <c r="G209" s="14"/>
       <c r="H209" s="14"/>
       <c r="I209" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J209" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K209" s="16"/>
@@ -7214,11 +7319,11 @@
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J210" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K210" s="16"/>
@@ -7236,11 +7341,11 @@
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J211" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K211" s="16"/>
@@ -7258,11 +7363,11 @@
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J212" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K212" s="16"/>
@@ -7280,11 +7385,11 @@
       <c r="G213" s="14"/>
       <c r="H213" s="14"/>
       <c r="I213" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J213" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K213" s="16"/>
@@ -7302,11 +7407,11 @@
       <c r="G214" s="14"/>
       <c r="H214" s="14"/>
       <c r="I214" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J214" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K214" s="16"/>
@@ -7324,11 +7429,11 @@
       <c r="G215" s="14"/>
       <c r="H215" s="14"/>
       <c r="I215" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J215" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K215" s="16"/>
@@ -7346,11 +7451,11 @@
       <c r="G216" s="14"/>
       <c r="H216" s="14"/>
       <c r="I216" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J216" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K216" s="16"/>
@@ -7368,11 +7473,11 @@
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J217" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K217" s="16"/>
@@ -7390,11 +7495,11 @@
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J218" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K218" s="16"/>
@@ -7412,11 +7517,11 @@
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J219" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K219" s="16"/>
@@ -7434,11 +7539,11 @@
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J220" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K220" s="16"/>
@@ -7456,11 +7561,11 @@
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J221" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K221" s="16"/>
@@ -7478,11 +7583,11 @@
       <c r="G222" s="14"/>
       <c r="H222" s="14"/>
       <c r="I222" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J222" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K222" s="16"/>
@@ -7500,11 +7605,11 @@
       <c r="G223" s="14"/>
       <c r="H223" s="14"/>
       <c r="I223" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J223" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K223" s="16"/>
@@ -7522,11 +7627,11 @@
       <c r="G224" s="14"/>
       <c r="H224" s="14"/>
       <c r="I224" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J224" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K224" s="16"/>
@@ -7544,11 +7649,11 @@
       <c r="G225" s="14"/>
       <c r="H225" s="14"/>
       <c r="I225" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J225" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K225" s="16"/>
@@ -7566,11 +7671,11 @@
       <c r="G226" s="14"/>
       <c r="H226" s="14"/>
       <c r="I226" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J226" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K226" s="16"/>
@@ -7588,11 +7693,11 @@
       <c r="G227" s="14"/>
       <c r="H227" s="14"/>
       <c r="I227" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J227" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K227" s="16"/>
@@ -7610,11 +7715,11 @@
       <c r="G228" s="14"/>
       <c r="H228" s="14"/>
       <c r="I228" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J228" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K228" s="16"/>
@@ -7632,11 +7737,11 @@
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J229" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K229" s="16"/>
@@ -7654,11 +7759,11 @@
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J230" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K230" s="16"/>
@@ -7676,11 +7781,11 @@
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
       <c r="I231" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J231" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K231" s="16"/>
@@ -7698,11 +7803,11 @@
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
       <c r="I232" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J232" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K232" s="16"/>
@@ -7720,11 +7825,11 @@
       <c r="G233" s="14"/>
       <c r="H233" s="14"/>
       <c r="I233" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J233" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K233" s="16"/>
@@ -7742,11 +7847,11 @@
       <c r="G234" s="14"/>
       <c r="H234" s="14"/>
       <c r="I234" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J234" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K234" s="16"/>
@@ -7764,11 +7869,11 @@
       <c r="G235" s="14"/>
       <c r="H235" s="14"/>
       <c r="I235" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J235" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K235" s="16"/>
@@ -7786,11 +7891,11 @@
       <c r="G236" s="14"/>
       <c r="H236" s="14"/>
       <c r="I236" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J236" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K236" s="16"/>
@@ -7808,11 +7913,11 @@
       <c r="G237" s="14"/>
       <c r="H237" s="14"/>
       <c r="I237" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J237" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K237" s="16"/>
@@ -7830,11 +7935,11 @@
       <c r="G238" s="14"/>
       <c r="H238" s="14"/>
       <c r="I238" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J238" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K238" s="16"/>
@@ -7852,11 +7957,11 @@
       <c r="G239" s="14"/>
       <c r="H239" s="14"/>
       <c r="I239" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J239" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K239" s="16"/>
@@ -7874,11 +7979,11 @@
       <c r="G240" s="14"/>
       <c r="H240" s="14"/>
       <c r="I240" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J240" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K240" s="16"/>
@@ -7896,11 +8001,11 @@
       <c r="G241" s="14"/>
       <c r="H241" s="14"/>
       <c r="I241" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J241" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K241" s="16"/>
@@ -7918,11 +8023,11 @@
       <c r="G242" s="14"/>
       <c r="H242" s="14"/>
       <c r="I242" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J242" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K242" s="16"/>
@@ -7940,11 +8045,11 @@
       <c r="G243" s="14"/>
       <c r="H243" s="14"/>
       <c r="I243" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J243" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K243" s="16"/>
@@ -7962,11 +8067,11 @@
       <c r="G244" s="14"/>
       <c r="H244" s="14"/>
       <c r="I244" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J244" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K244" s="16"/>
@@ -7984,11 +8089,11 @@
       <c r="G245" s="14"/>
       <c r="H245" s="14"/>
       <c r="I245" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J245" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K245" s="16"/>
@@ -8006,11 +8111,11 @@
       <c r="G246" s="14"/>
       <c r="H246" s="14"/>
       <c r="I246" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J246" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K246" s="16"/>
@@ -8028,11 +8133,11 @@
       <c r="G247" s="14"/>
       <c r="H247" s="14"/>
       <c r="I247" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J247" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K247" s="16"/>
@@ -8050,11 +8155,11 @@
       <c r="G248" s="14"/>
       <c r="H248" s="14"/>
       <c r="I248" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J248" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K248" s="16"/>
@@ -8072,11 +8177,11 @@
       <c r="G249" s="14"/>
       <c r="H249" s="14"/>
       <c r="I249" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J249" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K249" s="16"/>
@@ -8094,11 +8199,11 @@
       <c r="G250" s="14"/>
       <c r="H250" s="14"/>
       <c r="I250" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J250" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K250" s="16"/>
@@ -8116,11 +8221,11 @@
       <c r="G251" s="14"/>
       <c r="H251" s="14"/>
       <c r="I251" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J251" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K251" s="16"/>
@@ -8138,11 +8243,11 @@
       <c r="G252" s="14"/>
       <c r="H252" s="14"/>
       <c r="I252" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J252" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K252" s="16"/>
@@ -8160,11 +8265,11 @@
       <c r="G253" s="14"/>
       <c r="H253" s="14"/>
       <c r="I253" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J253" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K253" s="16"/>
@@ -8182,11 +8287,11 @@
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
       <c r="I254" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J254" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K254" s="16"/>
@@ -8204,11 +8309,11 @@
       <c r="G255" s="14"/>
       <c r="H255" s="14"/>
       <c r="I255" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J255" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K255" s="16"/>
@@ -8226,11 +8331,11 @@
       <c r="G256" s="14"/>
       <c r="H256" s="14"/>
       <c r="I256" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J256" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K256" s="16"/>
@@ -8248,11 +8353,11 @@
       <c r="G257" s="14"/>
       <c r="H257" s="14"/>
       <c r="I257" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J257" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K257" s="16"/>
@@ -8270,11 +8375,11 @@
       <c r="G258" s="14"/>
       <c r="H258" s="14"/>
       <c r="I258" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J258" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K258" s="16"/>
@@ -8292,11 +8397,11 @@
       <c r="G259" s="14"/>
       <c r="H259" s="14"/>
       <c r="I259" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J259" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K259" s="16"/>
@@ -8314,11 +8419,11 @@
       <c r="G260" s="14"/>
       <c r="H260" s="14"/>
       <c r="I260" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J260" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K260" s="16"/>
@@ -8336,11 +8441,11 @@
       <c r="G261" s="14"/>
       <c r="H261" s="14"/>
       <c r="I261" s="15" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J261" s="15" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K261" s="16"/>
@@ -8358,11 +8463,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="30">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" ref="I262:I325" si="38">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="31">IF(I262="","",1440-I262)</f>
+        <f t="shared" ref="J262:J325" si="39">IF(I262="","",1440-I262)</f>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -8380,11 +8485,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8402,11 +8507,11 @@
       <c r="G264" s="14"/>
       <c r="H264" s="14"/>
       <c r="I264" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J264" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K264" s="16"/>
@@ -8424,11 +8529,11 @@
       <c r="G265" s="14"/>
       <c r="H265" s="14"/>
       <c r="I265" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J265" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K265" s="16"/>
@@ -8446,11 +8551,11 @@
       <c r="G266" s="14"/>
       <c r="H266" s="14"/>
       <c r="I266" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J266" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K266" s="16"/>
@@ -8468,11 +8573,11 @@
       <c r="G267" s="14"/>
       <c r="H267" s="14"/>
       <c r="I267" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J267" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K267" s="16"/>
@@ -8490,11 +8595,11 @@
       <c r="G268" s="14"/>
       <c r="H268" s="14"/>
       <c r="I268" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J268" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K268" s="16"/>
@@ -8512,11 +8617,11 @@
       <c r="G269" s="14"/>
       <c r="H269" s="14"/>
       <c r="I269" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J269" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K269" s="16"/>
@@ -8534,11 +8639,11 @@
       <c r="G270" s="14"/>
       <c r="H270" s="14"/>
       <c r="I270" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J270" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K270" s="16"/>
@@ -8556,11 +8661,11 @@
       <c r="G271" s="14"/>
       <c r="H271" s="14"/>
       <c r="I271" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J271" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K271" s="16"/>
@@ -8578,11 +8683,11 @@
       <c r="G272" s="14"/>
       <c r="H272" s="14"/>
       <c r="I272" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J272" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K272" s="16"/>
@@ -8600,11 +8705,11 @@
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
       <c r="I273" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J273" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K273" s="16"/>
@@ -8622,11 +8727,11 @@
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
       <c r="I274" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J274" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K274" s="16"/>
@@ -8644,11 +8749,11 @@
       <c r="G275" s="14"/>
       <c r="H275" s="14"/>
       <c r="I275" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J275" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K275" s="16"/>
@@ -8666,11 +8771,11 @@
       <c r="G276" s="14"/>
       <c r="H276" s="14"/>
       <c r="I276" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J276" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K276" s="16"/>
@@ -8688,11 +8793,11 @@
       <c r="G277" s="14"/>
       <c r="H277" s="14"/>
       <c r="I277" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J277" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K277" s="16"/>
@@ -8710,11 +8815,11 @@
       <c r="G278" s="14"/>
       <c r="H278" s="14"/>
       <c r="I278" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J278" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K278" s="16"/>
@@ -8732,11 +8837,11 @@
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
       <c r="I279" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J279" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K279" s="16"/>
@@ -8754,11 +8859,11 @@
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
       <c r="I280" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J280" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K280" s="16"/>
@@ -8776,11 +8881,11 @@
       <c r="G281" s="14"/>
       <c r="H281" s="14"/>
       <c r="I281" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J281" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K281" s="16"/>
@@ -8798,11 +8903,11 @@
       <c r="G282" s="14"/>
       <c r="H282" s="14"/>
       <c r="I282" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J282" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K282" s="16"/>
@@ -8820,11 +8925,11 @@
       <c r="G283" s="14"/>
       <c r="H283" s="14"/>
       <c r="I283" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J283" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K283" s="16"/>
@@ -8842,11 +8947,11 @@
       <c r="G284" s="14"/>
       <c r="H284" s="14"/>
       <c r="I284" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J284" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K284" s="16"/>
@@ -8864,11 +8969,11 @@
       <c r="G285" s="14"/>
       <c r="H285" s="14"/>
       <c r="I285" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J285" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K285" s="16"/>
@@ -8886,11 +8991,11 @@
       <c r="G286" s="14"/>
       <c r="H286" s="14"/>
       <c r="I286" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J286" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K286" s="16"/>
@@ -8908,11 +9013,11 @@
       <c r="G287" s="14"/>
       <c r="H287" s="14"/>
       <c r="I287" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J287" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K287" s="16"/>
@@ -8930,11 +9035,11 @@
       <c r="G288" s="14"/>
       <c r="H288" s="14"/>
       <c r="I288" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J288" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K288" s="16"/>
@@ -8952,11 +9057,11 @@
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
       <c r="I289" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J289" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K289" s="16"/>
@@ -8974,11 +9079,11 @@
       <c r="G290" s="14"/>
       <c r="H290" s="14"/>
       <c r="I290" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J290" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K290" s="16"/>
@@ -8996,11 +9101,11 @@
       <c r="G291" s="14"/>
       <c r="H291" s="14"/>
       <c r="I291" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J291" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K291" s="16"/>
@@ -9018,11 +9123,11 @@
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
       <c r="I292" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J292" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K292" s="16"/>
@@ -9040,11 +9145,11 @@
       <c r="G293" s="14"/>
       <c r="H293" s="14"/>
       <c r="I293" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J293" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K293" s="16"/>
@@ -9062,11 +9167,11 @@
       <c r="G294" s="14"/>
       <c r="H294" s="14"/>
       <c r="I294" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J294" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K294" s="16"/>
@@ -9084,11 +9189,11 @@
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
       <c r="I295" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J295" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K295" s="16"/>
@@ -9106,11 +9211,11 @@
       <c r="G296" s="14"/>
       <c r="H296" s="14"/>
       <c r="I296" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J296" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K296" s="16"/>
@@ -9128,11 +9233,11 @@
       <c r="G297" s="14"/>
       <c r="H297" s="14"/>
       <c r="I297" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J297" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K297" s="16"/>
@@ -9150,11 +9255,11 @@
       <c r="G298" s="14"/>
       <c r="H298" s="14"/>
       <c r="I298" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J298" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K298" s="16"/>
@@ -9172,11 +9277,11 @@
       <c r="G299" s="14"/>
       <c r="H299" s="14"/>
       <c r="I299" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J299" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K299" s="16"/>
@@ -9194,11 +9299,11 @@
       <c r="G300" s="14"/>
       <c r="H300" s="14"/>
       <c r="I300" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J300" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K300" s="16"/>
@@ -9216,11 +9321,11 @@
       <c r="G301" s="14"/>
       <c r="H301" s="14"/>
       <c r="I301" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J301" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K301" s="16"/>
@@ -9238,11 +9343,11 @@
       <c r="G302" s="14"/>
       <c r="H302" s="14"/>
       <c r="I302" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J302" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K302" s="16"/>
@@ -9260,11 +9365,11 @@
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
       <c r="I303" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J303" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K303" s="16"/>
@@ -9282,11 +9387,11 @@
       <c r="G304" s="14"/>
       <c r="H304" s="14"/>
       <c r="I304" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J304" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K304" s="16"/>
@@ -9304,11 +9409,11 @@
       <c r="G305" s="14"/>
       <c r="H305" s="14"/>
       <c r="I305" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J305" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K305" s="16"/>
@@ -9326,11 +9431,11 @@
       <c r="G306" s="14"/>
       <c r="H306" s="14"/>
       <c r="I306" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J306" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K306" s="16"/>
@@ -9348,11 +9453,11 @@
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
       <c r="I307" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J307" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K307" s="16"/>
@@ -9370,11 +9475,11 @@
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
       <c r="I308" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J308" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K308" s="16"/>
@@ -9392,11 +9497,11 @@
       <c r="G309" s="14"/>
       <c r="H309" s="14"/>
       <c r="I309" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J309" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K309" s="16"/>
@@ -9414,11 +9519,11 @@
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
       <c r="I310" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J310" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K310" s="16"/>
@@ -9436,11 +9541,11 @@
       <c r="G311" s="14"/>
       <c r="H311" s="14"/>
       <c r="I311" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J311" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K311" s="16"/>
@@ -9458,11 +9563,11 @@
       <c r="G312" s="14"/>
       <c r="H312" s="14"/>
       <c r="I312" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J312" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K312" s="16"/>
@@ -9480,11 +9585,11 @@
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
       <c r="I313" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J313" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K313" s="16"/>
@@ -9502,11 +9607,11 @@
       <c r="G314" s="14"/>
       <c r="H314" s="14"/>
       <c r="I314" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J314" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K314" s="16"/>
@@ -9524,11 +9629,11 @@
       <c r="G315" s="14"/>
       <c r="H315" s="14"/>
       <c r="I315" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J315" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K315" s="16"/>
@@ -9546,11 +9651,11 @@
       <c r="G316" s="14"/>
       <c r="H316" s="14"/>
       <c r="I316" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J316" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K316" s="16"/>
@@ -9568,11 +9673,11 @@
       <c r="G317" s="14"/>
       <c r="H317" s="14"/>
       <c r="I317" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J317" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K317" s="16"/>
@@ -9590,11 +9695,11 @@
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
       <c r="I318" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J318" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K318" s="16"/>
@@ -9612,11 +9717,11 @@
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
       <c r="I319" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J319" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K319" s="16"/>
@@ -9634,11 +9739,11 @@
       <c r="G320" s="14"/>
       <c r="H320" s="14"/>
       <c r="I320" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J320" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K320" s="16"/>
@@ -9656,11 +9761,11 @@
       <c r="G321" s="14"/>
       <c r="H321" s="14"/>
       <c r="I321" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J321" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K321" s="16"/>
@@ -9678,11 +9783,11 @@
       <c r="G322" s="14"/>
       <c r="H322" s="14"/>
       <c r="I322" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J322" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K322" s="16"/>
@@ -9700,11 +9805,11 @@
       <c r="G323" s="14"/>
       <c r="H323" s="14"/>
       <c r="I323" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J323" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K323" s="16"/>
@@ -9722,11 +9827,11 @@
       <c r="G324" s="14"/>
       <c r="H324" s="14"/>
       <c r="I324" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J324" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K324" s="16"/>
@@ -9744,11 +9849,11 @@
       <c r="G325" s="14"/>
       <c r="H325" s="14"/>
       <c r="I325" s="15" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J325" s="15" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K325" s="16"/>
@@ -9766,11 +9871,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="32">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" ref="I326:I389" si="40">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="33">IF(I326="","",1440-I326)</f>
+        <f t="shared" ref="J326:J389" si="41">IF(I326="","",1440-I326)</f>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -9788,11 +9893,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -9810,11 +9915,11 @@
       <c r="G328" s="14"/>
       <c r="H328" s="14"/>
       <c r="I328" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J328" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K328" s="16"/>
@@ -9832,11 +9937,11 @@
       <c r="G329" s="14"/>
       <c r="H329" s="14"/>
       <c r="I329" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J329" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K329" s="16"/>
@@ -9854,11 +9959,11 @@
       <c r="G330" s="14"/>
       <c r="H330" s="14"/>
       <c r="I330" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J330" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K330" s="16"/>
@@ -9876,11 +9981,11 @@
       <c r="G331" s="14"/>
       <c r="H331" s="14"/>
       <c r="I331" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J331" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K331" s="16"/>
@@ -9898,11 +10003,11 @@
       <c r="G332" s="14"/>
       <c r="H332" s="14"/>
       <c r="I332" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J332" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K332" s="16"/>
@@ -9920,11 +10025,11 @@
       <c r="G333" s="14"/>
       <c r="H333" s="14"/>
       <c r="I333" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J333" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K333" s="16"/>
@@ -9942,11 +10047,11 @@
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
       <c r="I334" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J334" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K334" s="16"/>
@@ -9964,11 +10069,11 @@
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
       <c r="I335" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J335" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K335" s="16"/>
@@ -9986,11 +10091,11 @@
       <c r="G336" s="14"/>
       <c r="H336" s="14"/>
       <c r="I336" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J336" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K336" s="16"/>
@@ -10008,11 +10113,11 @@
       <c r="G337" s="14"/>
       <c r="H337" s="14"/>
       <c r="I337" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J337" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K337" s="16"/>
@@ -10030,11 +10135,11 @@
       <c r="G338" s="14"/>
       <c r="H338" s="14"/>
       <c r="I338" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J338" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K338" s="16"/>
@@ -10052,11 +10157,11 @@
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
       <c r="I339" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J339" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K339" s="16"/>
@@ -10074,11 +10179,11 @@
       <c r="G340" s="14"/>
       <c r="H340" s="14"/>
       <c r="I340" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J340" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K340" s="16"/>
@@ -10096,11 +10201,11 @@
       <c r="G341" s="14"/>
       <c r="H341" s="14"/>
       <c r="I341" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J341" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K341" s="16"/>
@@ -10118,11 +10223,11 @@
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
       <c r="I342" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J342" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K342" s="16"/>
@@ -10140,11 +10245,11 @@
       <c r="G343" s="14"/>
       <c r="H343" s="14"/>
       <c r="I343" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J343" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K343" s="16"/>
@@ -10162,11 +10267,11 @@
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
       <c r="I344" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J344" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K344" s="16"/>
@@ -10184,11 +10289,11 @@
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
       <c r="I345" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J345" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K345" s="16"/>
@@ -10206,11 +10311,11 @@
       <c r="G346" s="14"/>
       <c r="H346" s="14"/>
       <c r="I346" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J346" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K346" s="16"/>
@@ -10228,11 +10333,11 @@
       <c r="G347" s="14"/>
       <c r="H347" s="14"/>
       <c r="I347" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J347" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K347" s="16"/>
@@ -10250,11 +10355,11 @@
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
       <c r="I348" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J348" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K348" s="16"/>
@@ -10272,11 +10377,11 @@
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
       <c r="I349" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J349" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K349" s="16"/>
@@ -10294,11 +10399,11 @@
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
       <c r="I350" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J350" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K350" s="16"/>
@@ -10316,11 +10421,11 @@
       <c r="G351" s="14"/>
       <c r="H351" s="14"/>
       <c r="I351" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J351" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K351" s="16"/>
@@ -10338,11 +10443,11 @@
       <c r="G352" s="14"/>
       <c r="H352" s="14"/>
       <c r="I352" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J352" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K352" s="16"/>
@@ -10360,11 +10465,11 @@
       <c r="G353" s="14"/>
       <c r="H353" s="14"/>
       <c r="I353" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J353" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K353" s="16"/>
@@ -10382,11 +10487,11 @@
       <c r="G354" s="14"/>
       <c r="H354" s="14"/>
       <c r="I354" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J354" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K354" s="16"/>
@@ -10404,11 +10509,11 @@
       <c r="G355" s="14"/>
       <c r="H355" s="14"/>
       <c r="I355" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J355" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K355" s="16"/>
@@ -10426,11 +10531,11 @@
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
       <c r="I356" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J356" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K356" s="16"/>
@@ -10448,11 +10553,11 @@
       <c r="G357" s="14"/>
       <c r="H357" s="14"/>
       <c r="I357" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J357" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K357" s="16"/>
@@ -10470,11 +10575,11 @@
       <c r="G358" s="14"/>
       <c r="H358" s="14"/>
       <c r="I358" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J358" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K358" s="16"/>
@@ -10492,11 +10597,11 @@
       <c r="G359" s="14"/>
       <c r="H359" s="14"/>
       <c r="I359" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J359" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K359" s="16"/>
@@ -10514,11 +10619,11 @@
       <c r="G360" s="14"/>
       <c r="H360" s="14"/>
       <c r="I360" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J360" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K360" s="16"/>
@@ -10536,11 +10641,11 @@
       <c r="G361" s="14"/>
       <c r="H361" s="14"/>
       <c r="I361" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J361" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K361" s="16"/>
@@ -10558,11 +10663,11 @@
       <c r="G362" s="14"/>
       <c r="H362" s="14"/>
       <c r="I362" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J362" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K362" s="16"/>
@@ -10580,11 +10685,11 @@
       <c r="G363" s="14"/>
       <c r="H363" s="14"/>
       <c r="I363" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J363" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K363" s="16"/>
@@ -10602,11 +10707,11 @@
       <c r="G364" s="14"/>
       <c r="H364" s="14"/>
       <c r="I364" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J364" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K364" s="16"/>
@@ -10624,11 +10729,11 @@
       <c r="G365" s="14"/>
       <c r="H365" s="14"/>
       <c r="I365" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J365" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K365" s="16"/>
@@ -10646,11 +10751,11 @@
       <c r="G366" s="14"/>
       <c r="H366" s="14"/>
       <c r="I366" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J366" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K366" s="16"/>
@@ -10668,11 +10773,11 @@
       <c r="G367" s="14"/>
       <c r="H367" s="14"/>
       <c r="I367" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J367" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K367" s="16"/>
@@ -10690,11 +10795,11 @@
       <c r="G368" s="14"/>
       <c r="H368" s="14"/>
       <c r="I368" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J368" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K368" s="16"/>
@@ -10712,11 +10817,11 @@
       <c r="G369" s="14"/>
       <c r="H369" s="14"/>
       <c r="I369" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J369" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K369" s="16"/>
@@ -10734,11 +10839,11 @@
       <c r="G370" s="14"/>
       <c r="H370" s="14"/>
       <c r="I370" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J370" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K370" s="16"/>
@@ -10756,11 +10861,11 @@
       <c r="G371" s="14"/>
       <c r="H371" s="14"/>
       <c r="I371" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J371" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K371" s="16"/>
@@ -10778,11 +10883,11 @@
       <c r="G372" s="14"/>
       <c r="H372" s="14"/>
       <c r="I372" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J372" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K372" s="16"/>
@@ -10800,11 +10905,11 @@
       <c r="G373" s="14"/>
       <c r="H373" s="14"/>
       <c r="I373" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J373" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K373" s="16"/>
@@ -10822,11 +10927,11 @@
       <c r="G374" s="14"/>
       <c r="H374" s="14"/>
       <c r="I374" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J374" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K374" s="16"/>
@@ -10844,11 +10949,11 @@
       <c r="G375" s="14"/>
       <c r="H375" s="14"/>
       <c r="I375" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J375" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K375" s="16"/>
@@ -10866,11 +10971,11 @@
       <c r="G376" s="14"/>
       <c r="H376" s="14"/>
       <c r="I376" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J376" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K376" s="16"/>
@@ -10888,11 +10993,11 @@
       <c r="G377" s="14"/>
       <c r="H377" s="14"/>
       <c r="I377" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J377" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K377" s="16"/>
@@ -10910,11 +11015,11 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K378" s="16"/>
@@ -10932,11 +11037,11 @@
       <c r="G379" s="14"/>
       <c r="H379" s="14"/>
       <c r="I379" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J379" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K379" s="16"/>
@@ -10954,11 +11059,11 @@
       <c r="G380" s="14"/>
       <c r="H380" s="14"/>
       <c r="I380" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J380" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K380" s="16"/>
@@ -10976,11 +11081,11 @@
       <c r="G381" s="14"/>
       <c r="H381" s="14"/>
       <c r="I381" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J381" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K381" s="16"/>
@@ -10998,11 +11103,11 @@
       <c r="G382" s="14"/>
       <c r="H382" s="14"/>
       <c r="I382" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J382" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K382" s="16"/>
@@ -11020,11 +11125,11 @@
       <c r="G383" s="14"/>
       <c r="H383" s="14"/>
       <c r="I383" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J383" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K383" s="16"/>
@@ -11042,11 +11147,11 @@
       <c r="G384" s="14"/>
       <c r="H384" s="14"/>
       <c r="I384" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J384" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K384" s="16"/>
@@ -11064,11 +11169,11 @@
       <c r="G385" s="14"/>
       <c r="H385" s="14"/>
       <c r="I385" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J385" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K385" s="16"/>
@@ -11086,11 +11191,11 @@
       <c r="G386" s="14"/>
       <c r="H386" s="14"/>
       <c r="I386" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J386" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K386" s="16"/>
@@ -11108,11 +11213,11 @@
       <c r="G387" s="14"/>
       <c r="H387" s="14"/>
       <c r="I387" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J387" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K387" s="16"/>
@@ -11130,11 +11235,11 @@
       <c r="G388" s="14"/>
       <c r="H388" s="14"/>
       <c r="I388" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J388" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K388" s="16"/>
@@ -11152,11 +11257,11 @@
       <c r="G389" s="14"/>
       <c r="H389" s="14"/>
       <c r="I389" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J389" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K389" s="16"/>
@@ -11174,11 +11279,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="34">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="42">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="35">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="43">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -11196,11 +11301,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -11218,11 +11323,11 @@
       <c r="G392" s="14"/>
       <c r="H392" s="14"/>
       <c r="I392" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J392" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K392" s="16"/>
@@ -11240,11 +11345,11 @@
       <c r="G393" s="14"/>
       <c r="H393" s="14"/>
       <c r="I393" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J393" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K393" s="16"/>
@@ -11262,11 +11367,11 @@
       <c r="G394" s="14"/>
       <c r="H394" s="14"/>
       <c r="I394" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J394" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K394" s="16"/>
@@ -11284,11 +11389,11 @@
       <c r="G395" s="14"/>
       <c r="H395" s="14"/>
       <c r="I395" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J395" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K395" s="16"/>
@@ -11306,11 +11411,11 @@
       <c r="G396" s="14"/>
       <c r="H396" s="14"/>
       <c r="I396" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J396" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K396" s="16"/>
@@ -11328,11 +11433,11 @@
       <c r="G397" s="14"/>
       <c r="H397" s="14"/>
       <c r="I397" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J397" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K397" s="16"/>
@@ -11350,11 +11455,11 @@
       <c r="G398" s="14"/>
       <c r="H398" s="14"/>
       <c r="I398" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J398" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K398" s="16"/>
@@ -11372,11 +11477,11 @@
       <c r="G399" s="14"/>
       <c r="H399" s="14"/>
       <c r="I399" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J399" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K399" s="16"/>
@@ -11394,11 +11499,11 @@
       <c r="G400" s="14"/>
       <c r="H400" s="14"/>
       <c r="I400" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J400" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K400" s="16"/>
@@ -11416,11 +11521,11 @@
       <c r="G401" s="14"/>
       <c r="H401" s="14"/>
       <c r="I401" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J401" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K401" s="16"/>

</xml_diff>

<commit_message>
File Updated On 28/10/2028
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C123CA6-9F38-4660-9947-D4AD470F6ECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A95B3402-AF96-464E-973E-BA6670B80344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="612" yWindow="-108" windowWidth="22536" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
     <sheet name="Daily Log" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="98">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -326,6 +326,9 @@
   </si>
   <si>
     <t>Report submissions (C++)</t>
+  </si>
+  <si>
+    <t>Started working on c++ CA 2 project</t>
   </si>
 </sst>
 </file>
@@ -4361,27 +4364,51 @@
         <v>96</v>
       </c>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A76" s="13"/>
-      <c r="B76" s="14"/>
-      <c r="C76" s="14"/>
-      <c r="D76" s="14"/>
-      <c r="E76" s="14"/>
-      <c r="F76" s="14"/>
-      <c r="G76" s="14"/>
-      <c r="H76" s="14"/>
-      <c r="I76" s="15" t="str">
-        <f t="shared" ref="I76:I133" si="32">IF(SUM(B76:F76,H76)=0,"",SUM(B76:F76,H76))</f>
-        <v/>
-      </c>
-      <c r="J76" s="15" t="str">
-        <f t="shared" ref="J76:J133" si="33">IF(I76="","",1440-I76)</f>
-        <v/>
-      </c>
-      <c r="K76" s="16"/>
-      <c r="L76" s="16"/>
-      <c r="M76" s="16"/>
-      <c r="N76" s="17"/>
+    <row r="76" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A76" s="13">
+        <v>46323</v>
+      </c>
+      <c r="B76" s="14">
+        <v>380</v>
+      </c>
+      <c r="C76" s="14">
+        <v>0</v>
+      </c>
+      <c r="D76" s="14">
+        <v>170</v>
+      </c>
+      <c r="E76" s="14">
+        <v>100</v>
+      </c>
+      <c r="F76" s="14">
+        <v>300</v>
+      </c>
+      <c r="G76" s="14">
+        <v>6</v>
+      </c>
+      <c r="H76" s="14">
+        <v>50</v>
+      </c>
+      <c r="I76" s="15">
+        <f t="shared" ref="I76" si="32">IF(SUM(B76:F76,H76)=0,"",SUM(B76:F76,H76))</f>
+        <v>1000</v>
+      </c>
+      <c r="J76" s="15">
+        <f t="shared" ref="J76" si="33">IF(I76="","",1440-I76)</f>
+        <v>440</v>
+      </c>
+      <c r="K76" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L76" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M76" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N76" s="17" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77" s="13"/>
@@ -4393,11 +4420,11 @@
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
       <c r="I77" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" ref="I76:I133" si="34">IF(SUM(B77:F77,H77)=0,"",SUM(B77:F77,H77))</f>
         <v/>
       </c>
       <c r="J77" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" ref="J76:J133" si="35">IF(I77="","",1440-I77)</f>
         <v/>
       </c>
       <c r="K77" s="16"/>
@@ -4415,11 +4442,11 @@
       <c r="G78" s="14"/>
       <c r="H78" s="14"/>
       <c r="I78" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J78" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K78" s="16"/>
@@ -4437,11 +4464,11 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J79" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K79" s="16"/>
@@ -4459,11 +4486,11 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J80" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K80" s="16"/>
@@ -4481,11 +4508,11 @@
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J81" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K81" s="16"/>
@@ -4503,11 +4530,11 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J82" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K82" s="16"/>
@@ -4525,11 +4552,11 @@
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
       <c r="I83" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J83" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K83" s="16"/>
@@ -4547,11 +4574,11 @@
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
       <c r="I84" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J84" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K84" s="16"/>
@@ -4569,11 +4596,11 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J85" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K85" s="16"/>
@@ -4591,11 +4618,11 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J86" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K86" s="16"/>
@@ -4613,11 +4640,11 @@
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
       <c r="I87" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J87" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K87" s="16"/>
@@ -4635,11 +4662,11 @@
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
       <c r="I88" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J88" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K88" s="16"/>
@@ -4657,11 +4684,11 @@
       <c r="G89" s="14"/>
       <c r="H89" s="14"/>
       <c r="I89" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J89" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K89" s="16"/>
@@ -4679,11 +4706,11 @@
       <c r="G90" s="14"/>
       <c r="H90" s="14"/>
       <c r="I90" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J90" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K90" s="16"/>
@@ -4701,11 +4728,11 @@
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
       <c r="I91" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J91" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K91" s="16"/>
@@ -4723,11 +4750,11 @@
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
       <c r="I92" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J92" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K92" s="16"/>
@@ -4745,11 +4772,11 @@
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J93" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K93" s="16"/>
@@ -4767,11 +4794,11 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J94" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K94" s="16"/>
@@ -4789,11 +4816,11 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J95" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K95" s="16"/>
@@ -4811,11 +4838,11 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J96" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K96" s="16"/>
@@ -4833,11 +4860,11 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J97" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K97" s="16"/>
@@ -4855,11 +4882,11 @@
       <c r="G98" s="14"/>
       <c r="H98" s="14"/>
       <c r="I98" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J98" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K98" s="16"/>
@@ -4877,11 +4904,11 @@
       <c r="G99" s="14"/>
       <c r="H99" s="14"/>
       <c r="I99" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J99" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K99" s="16"/>
@@ -4899,11 +4926,11 @@
       <c r="G100" s="14"/>
       <c r="H100" s="14"/>
       <c r="I100" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J100" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K100" s="16"/>
@@ -4921,11 +4948,11 @@
       <c r="G101" s="14"/>
       <c r="H101" s="14"/>
       <c r="I101" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J101" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K101" s="16"/>
@@ -4943,11 +4970,11 @@
       <c r="G102" s="14"/>
       <c r="H102" s="14"/>
       <c r="I102" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J102" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K102" s="16"/>
@@ -4965,11 +4992,11 @@
       <c r="G103" s="14"/>
       <c r="H103" s="14"/>
       <c r="I103" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J103" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K103" s="16"/>
@@ -4987,11 +5014,11 @@
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
       <c r="I104" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J104" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K104" s="16"/>
@@ -5009,11 +5036,11 @@
       <c r="G105" s="14"/>
       <c r="H105" s="14"/>
       <c r="I105" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J105" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K105" s="16"/>
@@ -5031,11 +5058,11 @@
       <c r="G106" s="14"/>
       <c r="H106" s="14"/>
       <c r="I106" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J106" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K106" s="16"/>
@@ -5053,11 +5080,11 @@
       <c r="G107" s="14"/>
       <c r="H107" s="14"/>
       <c r="I107" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J107" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K107" s="16"/>
@@ -5075,11 +5102,11 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J108" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K108" s="16"/>
@@ -5097,11 +5124,11 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J109" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K109" s="16"/>
@@ -5119,11 +5146,11 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J110" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K110" s="16"/>
@@ -5141,11 +5168,11 @@
       <c r="G111" s="14"/>
       <c r="H111" s="14"/>
       <c r="I111" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J111" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K111" s="16"/>
@@ -5163,11 +5190,11 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J112" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K112" s="16"/>
@@ -5185,11 +5212,11 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J113" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K113" s="16"/>
@@ -5207,11 +5234,11 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J114" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K114" s="16"/>
@@ -5229,11 +5256,11 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J115" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K115" s="16"/>
@@ -5251,11 +5278,11 @@
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
       <c r="I116" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J116" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K116" s="16"/>
@@ -5273,11 +5300,11 @@
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
       <c r="I117" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J117" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K117" s="16"/>
@@ -5295,11 +5322,11 @@
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
       <c r="I118" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J118" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K118" s="16"/>
@@ -5317,11 +5344,11 @@
       <c r="G119" s="14"/>
       <c r="H119" s="14"/>
       <c r="I119" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J119" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K119" s="16"/>
@@ -5339,11 +5366,11 @@
       <c r="G120" s="14"/>
       <c r="H120" s="14"/>
       <c r="I120" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J120" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K120" s="16"/>
@@ -5361,11 +5388,11 @@
       <c r="G121" s="14"/>
       <c r="H121" s="14"/>
       <c r="I121" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J121" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K121" s="16"/>
@@ -5383,11 +5410,11 @@
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
       <c r="I122" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J122" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K122" s="16"/>
@@ -5405,11 +5432,11 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J123" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K123" s="16"/>
@@ -5427,11 +5454,11 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J124" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K124" s="16"/>
@@ -5449,11 +5476,11 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J125" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K125" s="16"/>
@@ -5471,11 +5498,11 @@
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
       <c r="I126" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J126" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K126" s="16"/>
@@ -5493,11 +5520,11 @@
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J127" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K127" s="16"/>
@@ -5515,11 +5542,11 @@
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
       <c r="I128" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J128" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K128" s="16"/>
@@ -5537,11 +5564,11 @@
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
       <c r="I129" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J129" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K129" s="16"/>
@@ -5559,11 +5586,11 @@
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
       <c r="I130" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J130" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K130" s="16"/>
@@ -5581,11 +5608,11 @@
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
       <c r="I131" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J131" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K131" s="16"/>
@@ -5603,11 +5630,11 @@
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
       <c r="I132" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J132" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K132" s="16"/>
@@ -5625,11 +5652,11 @@
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
       <c r="I133" s="15" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
       <c r="J133" s="15" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
       <c r="K133" s="16"/>
@@ -5647,11 +5674,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="34">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" ref="I134:I197" si="36">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="35">IF(I134="","",1440-I134)</f>
+        <f t="shared" ref="J134:J197" si="37">IF(I134="","",1440-I134)</f>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -5669,11 +5696,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5691,11 +5718,11 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J136" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K136" s="16"/>
@@ -5713,11 +5740,11 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J137" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K137" s="16"/>
@@ -5735,11 +5762,11 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J138" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K138" s="16"/>
@@ -5757,11 +5784,11 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J139" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K139" s="16"/>
@@ -5779,11 +5806,11 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J140" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K140" s="16"/>
@@ -5801,11 +5828,11 @@
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J141" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K141" s="16"/>
@@ -5823,11 +5850,11 @@
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J142" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K142" s="16"/>
@@ -5845,11 +5872,11 @@
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J143" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K143" s="16"/>
@@ -5867,11 +5894,11 @@
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J144" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K144" s="16"/>
@@ -5889,11 +5916,11 @@
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J145" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K145" s="16"/>
@@ -5911,11 +5938,11 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J146" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K146" s="16"/>
@@ -5933,11 +5960,11 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J147" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K147" s="16"/>
@@ -5955,11 +5982,11 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J148" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K148" s="16"/>
@@ -5977,11 +6004,11 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J149" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K149" s="16"/>
@@ -5999,11 +6026,11 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J150" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K150" s="16"/>
@@ -6021,11 +6048,11 @@
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
       <c r="I151" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J151" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K151" s="16"/>
@@ -6043,11 +6070,11 @@
       <c r="G152" s="14"/>
       <c r="H152" s="14"/>
       <c r="I152" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J152" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K152" s="16"/>
@@ -6065,11 +6092,11 @@
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J153" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K153" s="16"/>
@@ -6087,11 +6114,11 @@
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J154" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K154" s="16"/>
@@ -6109,11 +6136,11 @@
       <c r="G155" s="14"/>
       <c r="H155" s="14"/>
       <c r="I155" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J155" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K155" s="16"/>
@@ -6131,11 +6158,11 @@
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
       <c r="I156" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J156" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K156" s="16"/>
@@ -6153,11 +6180,11 @@
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J157" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K157" s="16"/>
@@ -6175,11 +6202,11 @@
       <c r="G158" s="14"/>
       <c r="H158" s="14"/>
       <c r="I158" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J158" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K158" s="16"/>
@@ -6197,11 +6224,11 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J159" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K159" s="16"/>
@@ -6219,11 +6246,11 @@
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
       <c r="I160" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J160" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K160" s="16"/>
@@ -6241,11 +6268,11 @@
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
       <c r="I161" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J161" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K161" s="16"/>
@@ -6263,11 +6290,11 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J162" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K162" s="16"/>
@@ -6285,11 +6312,11 @@
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
       <c r="I163" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J163" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K163" s="16"/>
@@ -6307,11 +6334,11 @@
       <c r="G164" s="14"/>
       <c r="H164" s="14"/>
       <c r="I164" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J164" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K164" s="16"/>
@@ -6329,11 +6356,11 @@
       <c r="G165" s="14"/>
       <c r="H165" s="14"/>
       <c r="I165" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J165" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K165" s="16"/>
@@ -6351,11 +6378,11 @@
       <c r="G166" s="14"/>
       <c r="H166" s="14"/>
       <c r="I166" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J166" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K166" s="16"/>
@@ -6373,11 +6400,11 @@
       <c r="G167" s="14"/>
       <c r="H167" s="14"/>
       <c r="I167" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J167" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K167" s="16"/>
@@ -6395,11 +6422,11 @@
       <c r="G168" s="14"/>
       <c r="H168" s="14"/>
       <c r="I168" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J168" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K168" s="16"/>
@@ -6417,11 +6444,11 @@
       <c r="G169" s="14"/>
       <c r="H169" s="14"/>
       <c r="I169" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J169" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K169" s="16"/>
@@ -6439,11 +6466,11 @@
       <c r="G170" s="14"/>
       <c r="H170" s="14"/>
       <c r="I170" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J170" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K170" s="16"/>
@@ -6461,11 +6488,11 @@
       <c r="G171" s="14"/>
       <c r="H171" s="14"/>
       <c r="I171" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J171" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K171" s="16"/>
@@ -6483,11 +6510,11 @@
       <c r="G172" s="14"/>
       <c r="H172" s="14"/>
       <c r="I172" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J172" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K172" s="16"/>
@@ -6505,11 +6532,11 @@
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
       <c r="I173" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J173" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K173" s="16"/>
@@ -6527,11 +6554,11 @@
       <c r="G174" s="14"/>
       <c r="H174" s="14"/>
       <c r="I174" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J174" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K174" s="16"/>
@@ -6549,11 +6576,11 @@
       <c r="G175" s="14"/>
       <c r="H175" s="14"/>
       <c r="I175" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J175" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K175" s="16"/>
@@ -6571,11 +6598,11 @@
       <c r="G176" s="14"/>
       <c r="H176" s="14"/>
       <c r="I176" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J176" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K176" s="16"/>
@@ -6593,11 +6620,11 @@
       <c r="G177" s="14"/>
       <c r="H177" s="14"/>
       <c r="I177" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J177" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K177" s="16"/>
@@ -6615,11 +6642,11 @@
       <c r="G178" s="14"/>
       <c r="H178" s="14"/>
       <c r="I178" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J178" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K178" s="16"/>
@@ -6637,11 +6664,11 @@
       <c r="G179" s="14"/>
       <c r="H179" s="14"/>
       <c r="I179" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J179" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K179" s="16"/>
@@ -6659,11 +6686,11 @@
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
       <c r="I180" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J180" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K180" s="16"/>
@@ -6681,11 +6708,11 @@
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J181" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K181" s="16"/>
@@ -6703,11 +6730,11 @@
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J182" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K182" s="16"/>
@@ -6725,11 +6752,11 @@
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J183" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K183" s="16"/>
@@ -6747,11 +6774,11 @@
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
       <c r="I184" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J184" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K184" s="16"/>
@@ -6769,11 +6796,11 @@
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
       <c r="I185" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J185" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K185" s="16"/>
@@ -6791,11 +6818,11 @@
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J186" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K186" s="16"/>
@@ -6813,11 +6840,11 @@
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J187" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K187" s="16"/>
@@ -6835,11 +6862,11 @@
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
       <c r="I188" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J188" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K188" s="16"/>
@@ -6857,11 +6884,11 @@
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
       <c r="I189" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J189" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K189" s="16"/>
@@ -6879,11 +6906,11 @@
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J190" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K190" s="16"/>
@@ -6901,11 +6928,11 @@
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J191" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K191" s="16"/>
@@ -6923,11 +6950,11 @@
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J192" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K192" s="16"/>
@@ -6945,11 +6972,11 @@
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
       <c r="I193" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J193" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K193" s="16"/>
@@ -6967,11 +6994,11 @@
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
       <c r="I194" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J194" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K194" s="16"/>
@@ -6989,11 +7016,11 @@
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J195" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K195" s="16"/>
@@ -7011,11 +7038,11 @@
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J196" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K196" s="16"/>
@@ -7033,11 +7060,11 @@
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="15" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
       <c r="J197" s="15" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
       <c r="K197" s="16"/>
@@ -7055,11 +7082,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="36">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" ref="I198:I261" si="38">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="37">IF(I198="","",1440-I198)</f>
+        <f t="shared" ref="J198:J261" si="39">IF(I198="","",1440-I198)</f>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -7077,11 +7104,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -7099,11 +7126,11 @@
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J200" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K200" s="16"/>
@@ -7121,11 +7148,11 @@
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
       <c r="I201" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J201" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K201" s="16"/>
@@ -7143,11 +7170,11 @@
       <c r="G202" s="14"/>
       <c r="H202" s="14"/>
       <c r="I202" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J202" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K202" s="16"/>
@@ -7165,11 +7192,11 @@
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
       <c r="I203" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J203" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K203" s="16"/>
@@ -7187,11 +7214,11 @@
       <c r="G204" s="14"/>
       <c r="H204" s="14"/>
       <c r="I204" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J204" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K204" s="16"/>
@@ -7209,11 +7236,11 @@
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J205" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K205" s="16"/>
@@ -7231,11 +7258,11 @@
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J206" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K206" s="16"/>
@@ -7253,11 +7280,11 @@
       <c r="G207" s="14"/>
       <c r="H207" s="14"/>
       <c r="I207" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J207" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K207" s="16"/>
@@ -7275,11 +7302,11 @@
       <c r="G208" s="14"/>
       <c r="H208" s="14"/>
       <c r="I208" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J208" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K208" s="16"/>
@@ -7297,11 +7324,11 @@
       <c r="G209" s="14"/>
       <c r="H209" s="14"/>
       <c r="I209" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J209" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K209" s="16"/>
@@ -7319,11 +7346,11 @@
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J210" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K210" s="16"/>
@@ -7341,11 +7368,11 @@
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J211" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K211" s="16"/>
@@ -7363,11 +7390,11 @@
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J212" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K212" s="16"/>
@@ -7385,11 +7412,11 @@
       <c r="G213" s="14"/>
       <c r="H213" s="14"/>
       <c r="I213" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J213" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K213" s="16"/>
@@ -7407,11 +7434,11 @@
       <c r="G214" s="14"/>
       <c r="H214" s="14"/>
       <c r="I214" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J214" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K214" s="16"/>
@@ -7429,11 +7456,11 @@
       <c r="G215" s="14"/>
       <c r="H215" s="14"/>
       <c r="I215" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J215" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K215" s="16"/>
@@ -7451,11 +7478,11 @@
       <c r="G216" s="14"/>
       <c r="H216" s="14"/>
       <c r="I216" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J216" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K216" s="16"/>
@@ -7473,11 +7500,11 @@
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J217" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K217" s="16"/>
@@ -7495,11 +7522,11 @@
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J218" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K218" s="16"/>
@@ -7517,11 +7544,11 @@
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J219" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K219" s="16"/>
@@ -7539,11 +7566,11 @@
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J220" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K220" s="16"/>
@@ -7561,11 +7588,11 @@
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J221" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K221" s="16"/>
@@ -7583,11 +7610,11 @@
       <c r="G222" s="14"/>
       <c r="H222" s="14"/>
       <c r="I222" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J222" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K222" s="16"/>
@@ -7605,11 +7632,11 @@
       <c r="G223" s="14"/>
       <c r="H223" s="14"/>
       <c r="I223" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J223" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K223" s="16"/>
@@ -7627,11 +7654,11 @@
       <c r="G224" s="14"/>
       <c r="H224" s="14"/>
       <c r="I224" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J224" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K224" s="16"/>
@@ -7649,11 +7676,11 @@
       <c r="G225" s="14"/>
       <c r="H225" s="14"/>
       <c r="I225" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J225" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K225" s="16"/>
@@ -7671,11 +7698,11 @@
       <c r="G226" s="14"/>
       <c r="H226" s="14"/>
       <c r="I226" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J226" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K226" s="16"/>
@@ -7693,11 +7720,11 @@
       <c r="G227" s="14"/>
       <c r="H227" s="14"/>
       <c r="I227" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J227" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K227" s="16"/>
@@ -7715,11 +7742,11 @@
       <c r="G228" s="14"/>
       <c r="H228" s="14"/>
       <c r="I228" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J228" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K228" s="16"/>
@@ -7737,11 +7764,11 @@
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J229" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K229" s="16"/>
@@ -7759,11 +7786,11 @@
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J230" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K230" s="16"/>
@@ -7781,11 +7808,11 @@
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
       <c r="I231" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J231" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K231" s="16"/>
@@ -7803,11 +7830,11 @@
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
       <c r="I232" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J232" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K232" s="16"/>
@@ -7825,11 +7852,11 @@
       <c r="G233" s="14"/>
       <c r="H233" s="14"/>
       <c r="I233" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J233" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K233" s="16"/>
@@ -7847,11 +7874,11 @@
       <c r="G234" s="14"/>
       <c r="H234" s="14"/>
       <c r="I234" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J234" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K234" s="16"/>
@@ -7869,11 +7896,11 @@
       <c r="G235" s="14"/>
       <c r="H235" s="14"/>
       <c r="I235" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J235" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K235" s="16"/>
@@ -7891,11 +7918,11 @@
       <c r="G236" s="14"/>
       <c r="H236" s="14"/>
       <c r="I236" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J236" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K236" s="16"/>
@@ -7913,11 +7940,11 @@
       <c r="G237" s="14"/>
       <c r="H237" s="14"/>
       <c r="I237" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J237" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K237" s="16"/>
@@ -7935,11 +7962,11 @@
       <c r="G238" s="14"/>
       <c r="H238" s="14"/>
       <c r="I238" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J238" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K238" s="16"/>
@@ -7957,11 +7984,11 @@
       <c r="G239" s="14"/>
       <c r="H239" s="14"/>
       <c r="I239" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J239" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K239" s="16"/>
@@ -7979,11 +8006,11 @@
       <c r="G240" s="14"/>
       <c r="H240" s="14"/>
       <c r="I240" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J240" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K240" s="16"/>
@@ -8001,11 +8028,11 @@
       <c r="G241" s="14"/>
       <c r="H241" s="14"/>
       <c r="I241" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J241" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K241" s="16"/>
@@ -8023,11 +8050,11 @@
       <c r="G242" s="14"/>
       <c r="H242" s="14"/>
       <c r="I242" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J242" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K242" s="16"/>
@@ -8045,11 +8072,11 @@
       <c r="G243" s="14"/>
       <c r="H243" s="14"/>
       <c r="I243" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J243" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K243" s="16"/>
@@ -8067,11 +8094,11 @@
       <c r="G244" s="14"/>
       <c r="H244" s="14"/>
       <c r="I244" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J244" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K244" s="16"/>
@@ -8089,11 +8116,11 @@
       <c r="G245" s="14"/>
       <c r="H245" s="14"/>
       <c r="I245" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J245" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K245" s="16"/>
@@ -8111,11 +8138,11 @@
       <c r="G246" s="14"/>
       <c r="H246" s="14"/>
       <c r="I246" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J246" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K246" s="16"/>
@@ -8133,11 +8160,11 @@
       <c r="G247" s="14"/>
       <c r="H247" s="14"/>
       <c r="I247" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J247" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K247" s="16"/>
@@ -8155,11 +8182,11 @@
       <c r="G248" s="14"/>
       <c r="H248" s="14"/>
       <c r="I248" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J248" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K248" s="16"/>
@@ -8177,11 +8204,11 @@
       <c r="G249" s="14"/>
       <c r="H249" s="14"/>
       <c r="I249" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J249" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K249" s="16"/>
@@ -8199,11 +8226,11 @@
       <c r="G250" s="14"/>
       <c r="H250" s="14"/>
       <c r="I250" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J250" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K250" s="16"/>
@@ -8221,11 +8248,11 @@
       <c r="G251" s="14"/>
       <c r="H251" s="14"/>
       <c r="I251" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J251" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K251" s="16"/>
@@ -8243,11 +8270,11 @@
       <c r="G252" s="14"/>
       <c r="H252" s="14"/>
       <c r="I252" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J252" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K252" s="16"/>
@@ -8265,11 +8292,11 @@
       <c r="G253" s="14"/>
       <c r="H253" s="14"/>
       <c r="I253" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J253" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K253" s="16"/>
@@ -8287,11 +8314,11 @@
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
       <c r="I254" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J254" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K254" s="16"/>
@@ -8309,11 +8336,11 @@
       <c r="G255" s="14"/>
       <c r="H255" s="14"/>
       <c r="I255" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J255" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K255" s="16"/>
@@ -8331,11 +8358,11 @@
       <c r="G256" s="14"/>
       <c r="H256" s="14"/>
       <c r="I256" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J256" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K256" s="16"/>
@@ -8353,11 +8380,11 @@
       <c r="G257" s="14"/>
       <c r="H257" s="14"/>
       <c r="I257" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J257" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K257" s="16"/>
@@ -8375,11 +8402,11 @@
       <c r="G258" s="14"/>
       <c r="H258" s="14"/>
       <c r="I258" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J258" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K258" s="16"/>
@@ -8397,11 +8424,11 @@
       <c r="G259" s="14"/>
       <c r="H259" s="14"/>
       <c r="I259" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J259" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K259" s="16"/>
@@ -8419,11 +8446,11 @@
       <c r="G260" s="14"/>
       <c r="H260" s="14"/>
       <c r="I260" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J260" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K260" s="16"/>
@@ -8441,11 +8468,11 @@
       <c r="G261" s="14"/>
       <c r="H261" s="14"/>
       <c r="I261" s="15" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
       <c r="J261" s="15" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="K261" s="16"/>
@@ -8463,11 +8490,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="38">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" ref="I262:I325" si="40">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="39">IF(I262="","",1440-I262)</f>
+        <f t="shared" ref="J262:J325" si="41">IF(I262="","",1440-I262)</f>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -8485,11 +8512,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8507,11 +8534,11 @@
       <c r="G264" s="14"/>
       <c r="H264" s="14"/>
       <c r="I264" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J264" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K264" s="16"/>
@@ -8529,11 +8556,11 @@
       <c r="G265" s="14"/>
       <c r="H265" s="14"/>
       <c r="I265" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J265" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K265" s="16"/>
@@ -8551,11 +8578,11 @@
       <c r="G266" s="14"/>
       <c r="H266" s="14"/>
       <c r="I266" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J266" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K266" s="16"/>
@@ -8573,11 +8600,11 @@
       <c r="G267" s="14"/>
       <c r="H267" s="14"/>
       <c r="I267" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J267" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K267" s="16"/>
@@ -8595,11 +8622,11 @@
       <c r="G268" s="14"/>
       <c r="H268" s="14"/>
       <c r="I268" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J268" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K268" s="16"/>
@@ -8617,11 +8644,11 @@
       <c r="G269" s="14"/>
       <c r="H269" s="14"/>
       <c r="I269" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J269" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K269" s="16"/>
@@ -8639,11 +8666,11 @@
       <c r="G270" s="14"/>
       <c r="H270" s="14"/>
       <c r="I270" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J270" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K270" s="16"/>
@@ -8661,11 +8688,11 @@
       <c r="G271" s="14"/>
       <c r="H271" s="14"/>
       <c r="I271" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J271" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K271" s="16"/>
@@ -8683,11 +8710,11 @@
       <c r="G272" s="14"/>
       <c r="H272" s="14"/>
       <c r="I272" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J272" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K272" s="16"/>
@@ -8705,11 +8732,11 @@
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
       <c r="I273" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J273" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K273" s="16"/>
@@ -8727,11 +8754,11 @@
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
       <c r="I274" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J274" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K274" s="16"/>
@@ -8749,11 +8776,11 @@
       <c r="G275" s="14"/>
       <c r="H275" s="14"/>
       <c r="I275" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J275" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K275" s="16"/>
@@ -8771,11 +8798,11 @@
       <c r="G276" s="14"/>
       <c r="H276" s="14"/>
       <c r="I276" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J276" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K276" s="16"/>
@@ -8793,11 +8820,11 @@
       <c r="G277" s="14"/>
       <c r="H277" s="14"/>
       <c r="I277" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J277" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K277" s="16"/>
@@ -8815,11 +8842,11 @@
       <c r="G278" s="14"/>
       <c r="H278" s="14"/>
       <c r="I278" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J278" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K278" s="16"/>
@@ -8837,11 +8864,11 @@
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
       <c r="I279" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J279" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K279" s="16"/>
@@ -8859,11 +8886,11 @@
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
       <c r="I280" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J280" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K280" s="16"/>
@@ -8881,11 +8908,11 @@
       <c r="G281" s="14"/>
       <c r="H281" s="14"/>
       <c r="I281" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J281" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K281" s="16"/>
@@ -8903,11 +8930,11 @@
       <c r="G282" s="14"/>
       <c r="H282" s="14"/>
       <c r="I282" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J282" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K282" s="16"/>
@@ -8925,11 +8952,11 @@
       <c r="G283" s="14"/>
       <c r="H283" s="14"/>
       <c r="I283" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J283" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K283" s="16"/>
@@ -8947,11 +8974,11 @@
       <c r="G284" s="14"/>
       <c r="H284" s="14"/>
       <c r="I284" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J284" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K284" s="16"/>
@@ -8969,11 +8996,11 @@
       <c r="G285" s="14"/>
       <c r="H285" s="14"/>
       <c r="I285" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J285" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K285" s="16"/>
@@ -8991,11 +9018,11 @@
       <c r="G286" s="14"/>
       <c r="H286" s="14"/>
       <c r="I286" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J286" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K286" s="16"/>
@@ -9013,11 +9040,11 @@
       <c r="G287" s="14"/>
       <c r="H287" s="14"/>
       <c r="I287" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J287" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K287" s="16"/>
@@ -9035,11 +9062,11 @@
       <c r="G288" s="14"/>
       <c r="H288" s="14"/>
       <c r="I288" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J288" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K288" s="16"/>
@@ -9057,11 +9084,11 @@
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
       <c r="I289" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J289" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K289" s="16"/>
@@ -9079,11 +9106,11 @@
       <c r="G290" s="14"/>
       <c r="H290" s="14"/>
       <c r="I290" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J290" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K290" s="16"/>
@@ -9101,11 +9128,11 @@
       <c r="G291" s="14"/>
       <c r="H291" s="14"/>
       <c r="I291" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J291" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K291" s="16"/>
@@ -9123,11 +9150,11 @@
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
       <c r="I292" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J292" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K292" s="16"/>
@@ -9145,11 +9172,11 @@
       <c r="G293" s="14"/>
       <c r="H293" s="14"/>
       <c r="I293" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J293" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K293" s="16"/>
@@ -9167,11 +9194,11 @@
       <c r="G294" s="14"/>
       <c r="H294" s="14"/>
       <c r="I294" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J294" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K294" s="16"/>
@@ -9189,11 +9216,11 @@
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
       <c r="I295" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J295" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K295" s="16"/>
@@ -9211,11 +9238,11 @@
       <c r="G296" s="14"/>
       <c r="H296" s="14"/>
       <c r="I296" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J296" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K296" s="16"/>
@@ -9233,11 +9260,11 @@
       <c r="G297" s="14"/>
       <c r="H297" s="14"/>
       <c r="I297" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J297" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K297" s="16"/>
@@ -9255,11 +9282,11 @@
       <c r="G298" s="14"/>
       <c r="H298" s="14"/>
       <c r="I298" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J298" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K298" s="16"/>
@@ -9277,11 +9304,11 @@
       <c r="G299" s="14"/>
       <c r="H299" s="14"/>
       <c r="I299" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J299" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K299" s="16"/>
@@ -9299,11 +9326,11 @@
       <c r="G300" s="14"/>
       <c r="H300" s="14"/>
       <c r="I300" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J300" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K300" s="16"/>
@@ -9321,11 +9348,11 @@
       <c r="G301" s="14"/>
       <c r="H301" s="14"/>
       <c r="I301" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J301" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K301" s="16"/>
@@ -9343,11 +9370,11 @@
       <c r="G302" s="14"/>
       <c r="H302" s="14"/>
       <c r="I302" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J302" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K302" s="16"/>
@@ -9365,11 +9392,11 @@
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
       <c r="I303" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J303" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K303" s="16"/>
@@ -9387,11 +9414,11 @@
       <c r="G304" s="14"/>
       <c r="H304" s="14"/>
       <c r="I304" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J304" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K304" s="16"/>
@@ -9409,11 +9436,11 @@
       <c r="G305" s="14"/>
       <c r="H305" s="14"/>
       <c r="I305" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J305" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K305" s="16"/>
@@ -9431,11 +9458,11 @@
       <c r="G306" s="14"/>
       <c r="H306" s="14"/>
       <c r="I306" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J306" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K306" s="16"/>
@@ -9453,11 +9480,11 @@
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
       <c r="I307" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J307" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K307" s="16"/>
@@ -9475,11 +9502,11 @@
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
       <c r="I308" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J308" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K308" s="16"/>
@@ -9497,11 +9524,11 @@
       <c r="G309" s="14"/>
       <c r="H309" s="14"/>
       <c r="I309" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J309" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K309" s="16"/>
@@ -9519,11 +9546,11 @@
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
       <c r="I310" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J310" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K310" s="16"/>
@@ -9541,11 +9568,11 @@
       <c r="G311" s="14"/>
       <c r="H311" s="14"/>
       <c r="I311" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J311" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K311" s="16"/>
@@ -9563,11 +9590,11 @@
       <c r="G312" s="14"/>
       <c r="H312" s="14"/>
       <c r="I312" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J312" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K312" s="16"/>
@@ -9585,11 +9612,11 @@
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
       <c r="I313" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J313" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K313" s="16"/>
@@ -9607,11 +9634,11 @@
       <c r="G314" s="14"/>
       <c r="H314" s="14"/>
       <c r="I314" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J314" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K314" s="16"/>
@@ -9629,11 +9656,11 @@
       <c r="G315" s="14"/>
       <c r="H315" s="14"/>
       <c r="I315" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J315" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K315" s="16"/>
@@ -9651,11 +9678,11 @@
       <c r="G316" s="14"/>
       <c r="H316" s="14"/>
       <c r="I316" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J316" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K316" s="16"/>
@@ -9673,11 +9700,11 @@
       <c r="G317" s="14"/>
       <c r="H317" s="14"/>
       <c r="I317" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J317" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K317" s="16"/>
@@ -9695,11 +9722,11 @@
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
       <c r="I318" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J318" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K318" s="16"/>
@@ -9717,11 +9744,11 @@
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
       <c r="I319" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J319" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K319" s="16"/>
@@ -9739,11 +9766,11 @@
       <c r="G320" s="14"/>
       <c r="H320" s="14"/>
       <c r="I320" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J320" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K320" s="16"/>
@@ -9761,11 +9788,11 @@
       <c r="G321" s="14"/>
       <c r="H321" s="14"/>
       <c r="I321" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J321" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K321" s="16"/>
@@ -9783,11 +9810,11 @@
       <c r="G322" s="14"/>
       <c r="H322" s="14"/>
       <c r="I322" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J322" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K322" s="16"/>
@@ -9805,11 +9832,11 @@
       <c r="G323" s="14"/>
       <c r="H323" s="14"/>
       <c r="I323" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J323" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K323" s="16"/>
@@ -9827,11 +9854,11 @@
       <c r="G324" s="14"/>
       <c r="H324" s="14"/>
       <c r="I324" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J324" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K324" s="16"/>
@@ -9849,11 +9876,11 @@
       <c r="G325" s="14"/>
       <c r="H325" s="14"/>
       <c r="I325" s="15" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
       <c r="J325" s="15" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
       <c r="K325" s="16"/>
@@ -9871,11 +9898,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="40">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" ref="I326:I389" si="42">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="41">IF(I326="","",1440-I326)</f>
+        <f t="shared" ref="J326:J389" si="43">IF(I326="","",1440-I326)</f>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -9893,11 +9920,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -9915,11 +9942,11 @@
       <c r="G328" s="14"/>
       <c r="H328" s="14"/>
       <c r="I328" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J328" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K328" s="16"/>
@@ -9937,11 +9964,11 @@
       <c r="G329" s="14"/>
       <c r="H329" s="14"/>
       <c r="I329" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J329" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K329" s="16"/>
@@ -9959,11 +9986,11 @@
       <c r="G330" s="14"/>
       <c r="H330" s="14"/>
       <c r="I330" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J330" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K330" s="16"/>
@@ -9981,11 +10008,11 @@
       <c r="G331" s="14"/>
       <c r="H331" s="14"/>
       <c r="I331" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J331" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K331" s="16"/>
@@ -10003,11 +10030,11 @@
       <c r="G332" s="14"/>
       <c r="H332" s="14"/>
       <c r="I332" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J332" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K332" s="16"/>
@@ -10025,11 +10052,11 @@
       <c r="G333" s="14"/>
       <c r="H333" s="14"/>
       <c r="I333" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J333" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K333" s="16"/>
@@ -10047,11 +10074,11 @@
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
       <c r="I334" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J334" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K334" s="16"/>
@@ -10069,11 +10096,11 @@
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
       <c r="I335" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J335" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K335" s="16"/>
@@ -10091,11 +10118,11 @@
       <c r="G336" s="14"/>
       <c r="H336" s="14"/>
       <c r="I336" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J336" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K336" s="16"/>
@@ -10113,11 +10140,11 @@
       <c r="G337" s="14"/>
       <c r="H337" s="14"/>
       <c r="I337" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J337" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K337" s="16"/>
@@ -10135,11 +10162,11 @@
       <c r="G338" s="14"/>
       <c r="H338" s="14"/>
       <c r="I338" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J338" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K338" s="16"/>
@@ -10157,11 +10184,11 @@
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
       <c r="I339" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J339" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K339" s="16"/>
@@ -10179,11 +10206,11 @@
       <c r="G340" s="14"/>
       <c r="H340" s="14"/>
       <c r="I340" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J340" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K340" s="16"/>
@@ -10201,11 +10228,11 @@
       <c r="G341" s="14"/>
       <c r="H341" s="14"/>
       <c r="I341" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J341" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K341" s="16"/>
@@ -10223,11 +10250,11 @@
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
       <c r="I342" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J342" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K342" s="16"/>
@@ -10245,11 +10272,11 @@
       <c r="G343" s="14"/>
       <c r="H343" s="14"/>
       <c r="I343" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J343" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K343" s="16"/>
@@ -10267,11 +10294,11 @@
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
       <c r="I344" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J344" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K344" s="16"/>
@@ -10289,11 +10316,11 @@
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
       <c r="I345" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J345" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K345" s="16"/>
@@ -10311,11 +10338,11 @@
       <c r="G346" s="14"/>
       <c r="H346" s="14"/>
       <c r="I346" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J346" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K346" s="16"/>
@@ -10333,11 +10360,11 @@
       <c r="G347" s="14"/>
       <c r="H347" s="14"/>
       <c r="I347" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J347" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K347" s="16"/>
@@ -10355,11 +10382,11 @@
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
       <c r="I348" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J348" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K348" s="16"/>
@@ -10377,11 +10404,11 @@
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
       <c r="I349" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J349" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K349" s="16"/>
@@ -10399,11 +10426,11 @@
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
       <c r="I350" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J350" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K350" s="16"/>
@@ -10421,11 +10448,11 @@
       <c r="G351" s="14"/>
       <c r="H351" s="14"/>
       <c r="I351" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J351" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K351" s="16"/>
@@ -10443,11 +10470,11 @@
       <c r="G352" s="14"/>
       <c r="H352" s="14"/>
       <c r="I352" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J352" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K352" s="16"/>
@@ -10465,11 +10492,11 @@
       <c r="G353" s="14"/>
       <c r="H353" s="14"/>
       <c r="I353" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J353" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K353" s="16"/>
@@ -10487,11 +10514,11 @@
       <c r="G354" s="14"/>
       <c r="H354" s="14"/>
       <c r="I354" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J354" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K354" s="16"/>
@@ -10509,11 +10536,11 @@
       <c r="G355" s="14"/>
       <c r="H355" s="14"/>
       <c r="I355" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J355" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K355" s="16"/>
@@ -10531,11 +10558,11 @@
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
       <c r="I356" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J356" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K356" s="16"/>
@@ -10553,11 +10580,11 @@
       <c r="G357" s="14"/>
       <c r="H357" s="14"/>
       <c r="I357" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J357" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K357" s="16"/>
@@ -10575,11 +10602,11 @@
       <c r="G358" s="14"/>
       <c r="H358" s="14"/>
       <c r="I358" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J358" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K358" s="16"/>
@@ -10597,11 +10624,11 @@
       <c r="G359" s="14"/>
       <c r="H359" s="14"/>
       <c r="I359" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J359" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K359" s="16"/>
@@ -10619,11 +10646,11 @@
       <c r="G360" s="14"/>
       <c r="H360" s="14"/>
       <c r="I360" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J360" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K360" s="16"/>
@@ -10641,11 +10668,11 @@
       <c r="G361" s="14"/>
       <c r="H361" s="14"/>
       <c r="I361" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J361" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K361" s="16"/>
@@ -10663,11 +10690,11 @@
       <c r="G362" s="14"/>
       <c r="H362" s="14"/>
       <c r="I362" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J362" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K362" s="16"/>
@@ -10685,11 +10712,11 @@
       <c r="G363" s="14"/>
       <c r="H363" s="14"/>
       <c r="I363" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J363" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K363" s="16"/>
@@ -10707,11 +10734,11 @@
       <c r="G364" s="14"/>
       <c r="H364" s="14"/>
       <c r="I364" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J364" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K364" s="16"/>
@@ -10729,11 +10756,11 @@
       <c r="G365" s="14"/>
       <c r="H365" s="14"/>
       <c r="I365" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J365" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K365" s="16"/>
@@ -10751,11 +10778,11 @@
       <c r="G366" s="14"/>
       <c r="H366" s="14"/>
       <c r="I366" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J366" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K366" s="16"/>
@@ -10773,11 +10800,11 @@
       <c r="G367" s="14"/>
       <c r="H367" s="14"/>
       <c r="I367" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J367" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K367" s="16"/>
@@ -10795,11 +10822,11 @@
       <c r="G368" s="14"/>
       <c r="H368" s="14"/>
       <c r="I368" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J368" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K368" s="16"/>
@@ -10817,11 +10844,11 @@
       <c r="G369" s="14"/>
       <c r="H369" s="14"/>
       <c r="I369" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J369" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K369" s="16"/>
@@ -10839,11 +10866,11 @@
       <c r="G370" s="14"/>
       <c r="H370" s="14"/>
       <c r="I370" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J370" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K370" s="16"/>
@@ -10861,11 +10888,11 @@
       <c r="G371" s="14"/>
       <c r="H371" s="14"/>
       <c r="I371" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J371" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K371" s="16"/>
@@ -10883,11 +10910,11 @@
       <c r="G372" s="14"/>
       <c r="H372" s="14"/>
       <c r="I372" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J372" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K372" s="16"/>
@@ -10905,11 +10932,11 @@
       <c r="G373" s="14"/>
       <c r="H373" s="14"/>
       <c r="I373" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J373" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K373" s="16"/>
@@ -10927,11 +10954,11 @@
       <c r="G374" s="14"/>
       <c r="H374" s="14"/>
       <c r="I374" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J374" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K374" s="16"/>
@@ -10949,11 +10976,11 @@
       <c r="G375" s="14"/>
       <c r="H375" s="14"/>
       <c r="I375" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J375" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K375" s="16"/>
@@ -10971,11 +10998,11 @@
       <c r="G376" s="14"/>
       <c r="H376" s="14"/>
       <c r="I376" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J376" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K376" s="16"/>
@@ -10993,11 +11020,11 @@
       <c r="G377" s="14"/>
       <c r="H377" s="14"/>
       <c r="I377" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J377" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K377" s="16"/>
@@ -11015,11 +11042,11 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K378" s="16"/>
@@ -11037,11 +11064,11 @@
       <c r="G379" s="14"/>
       <c r="H379" s="14"/>
       <c r="I379" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J379" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K379" s="16"/>
@@ -11059,11 +11086,11 @@
       <c r="G380" s="14"/>
       <c r="H380" s="14"/>
       <c r="I380" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J380" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K380" s="16"/>
@@ -11081,11 +11108,11 @@
       <c r="G381" s="14"/>
       <c r="H381" s="14"/>
       <c r="I381" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J381" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K381" s="16"/>
@@ -11103,11 +11130,11 @@
       <c r="G382" s="14"/>
       <c r="H382" s="14"/>
       <c r="I382" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J382" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K382" s="16"/>
@@ -11125,11 +11152,11 @@
       <c r="G383" s="14"/>
       <c r="H383" s="14"/>
       <c r="I383" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J383" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K383" s="16"/>
@@ -11147,11 +11174,11 @@
       <c r="G384" s="14"/>
       <c r="H384" s="14"/>
       <c r="I384" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J384" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K384" s="16"/>
@@ -11169,11 +11196,11 @@
       <c r="G385" s="14"/>
       <c r="H385" s="14"/>
       <c r="I385" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J385" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K385" s="16"/>
@@ -11191,11 +11218,11 @@
       <c r="G386" s="14"/>
       <c r="H386" s="14"/>
       <c r="I386" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J386" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K386" s="16"/>
@@ -11213,11 +11240,11 @@
       <c r="G387" s="14"/>
       <c r="H387" s="14"/>
       <c r="I387" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J387" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K387" s="16"/>
@@ -11235,11 +11262,11 @@
       <c r="G388" s="14"/>
       <c r="H388" s="14"/>
       <c r="I388" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J388" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K388" s="16"/>
@@ -11257,11 +11284,11 @@
       <c r="G389" s="14"/>
       <c r="H389" s="14"/>
       <c r="I389" s="15" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
       <c r="J389" s="15" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
       <c r="K389" s="16"/>
@@ -11279,11 +11306,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="42">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="44">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="43">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="45">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -11301,11 +11328,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="44"/>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="45"/>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -11323,11 +11350,11 @@
       <c r="G392" s="14"/>
       <c r="H392" s="14"/>
       <c r="I392" s="15" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="44"/>
         <v/>
       </c>
       <c r="J392" s="15" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="45"/>
         <v/>
       </c>
       <c r="K392" s="16"/>
@@ -11345,11 +11372,11 @@
       <c r="G393" s="14"/>
       <c r="H393" s="14"/>
       <c r="I393" s="15" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="44"/>
         <v/>
       </c>
       <c r="J393" s="15" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="45"/>
         <v/>
       </c>
       <c r="K393" s="16"/>
@@ -11367,11 +11394,11 @@
       <c r="G394" s="14"/>
       <c r="H394" s="14"/>
       <c r="I394" s="15" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="44"/>
         <v/>
       </c>
       <c r="J394" s="15" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="45"/>
         <v/>
       </c>
       <c r="K394" s="16"/>
@@ -11389,11 +11416,11 @@
       <c r="G395" s="14"/>
       <c r="H395" s="14"/>
       <c r="I395" s="15" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="44"/>
         <v/>
       </c>
       <c r="J395" s="15" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="45"/>
         <v/>
       </c>
       <c r="K395" s="16"/>
@@ -11411,11 +11438,11 @@
       <c r="G396" s="14"/>
       <c r="H396" s="14"/>
       <c r="I396" s="15" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="44"/>
         <v/>
       </c>
       <c r="J396" s="15" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="45"/>
         <v/>
       </c>
       <c r="K396" s="16"/>
@@ -11433,11 +11460,11 @@
       <c r="G397" s="14"/>
       <c r="H397" s="14"/>
       <c r="I397" s="15" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="44"/>
         <v/>
       </c>
       <c r="J397" s="15" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="45"/>
         <v/>
       </c>
       <c r="K397" s="16"/>
@@ -11455,11 +11482,11 @@
       <c r="G398" s="14"/>
       <c r="H398" s="14"/>
       <c r="I398" s="15" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="44"/>
         <v/>
       </c>
       <c r="J398" s="15" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="45"/>
         <v/>
       </c>
       <c r="K398" s="16"/>
@@ -11477,11 +11504,11 @@
       <c r="G399" s="14"/>
       <c r="H399" s="14"/>
       <c r="I399" s="15" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="44"/>
         <v/>
       </c>
       <c r="J399" s="15" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="45"/>
         <v/>
       </c>
       <c r="K399" s="16"/>
@@ -11499,11 +11526,11 @@
       <c r="G400" s="14"/>
       <c r="H400" s="14"/>
       <c r="I400" s="15" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="44"/>
         <v/>
       </c>
       <c r="J400" s="15" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="45"/>
         <v/>
       </c>
       <c r="K400" s="16"/>
@@ -11521,11 +11548,11 @@
       <c r="G401" s="14"/>
       <c r="H401" s="14"/>
       <c r="I401" s="15" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="44"/>
         <v/>
       </c>
       <c r="J401" s="15" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="45"/>
         <v/>
       </c>
       <c r="K401" s="16"/>

</xml_diff>